<commit_message>
added LES, BS for TX and CSS, EV for GA
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43B746B-6B8A-4CE2-85A5-A1A9B4B34F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B29284A6-FF55-4972-B120-EA539E7721BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="998">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="1009">
   <si>
     <t>Name</t>
   </si>
@@ -2967,9 +2967,6 @@
     <t>CSS_ICWStudentStatus</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>RCV</t>
   </si>
   <si>
@@ -3034,6 +3031,42 @@
   </si>
   <si>
     <t>RCV_SupportingDocInIAQ</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>BS</t>
+  </si>
+  <si>
+    <t>Bank Statements</t>
+  </si>
+  <si>
+    <t>LES</t>
+  </si>
+  <si>
+    <t>Leave and Earnings Statement</t>
+  </si>
+  <si>
+    <t>BSExists</t>
+  </si>
+  <si>
+    <t>BS_FindingError</t>
+  </si>
+  <si>
+    <t>LESExists</t>
+  </si>
+  <si>
+    <t>LES_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Bank Statements. Needs manual review.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Statements are present in the application, manual review required. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leave and Earnings Statement is present in the application, manual review required. </t>
   </si>
 </sst>
 </file>
@@ -3502,7 +3535,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>975</v>
+        <v>997</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3851,14 +3884,28 @@
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
+        <v>975</v>
+      </c>
+      <c r="B50" t="s">
         <v>976</v>
       </c>
-      <c r="B50" t="s">
-        <v>977</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="51" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A51" t="s">
+        <v>998</v>
+      </c>
+      <c r="B51" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1001</v>
+      </c>
+    </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7785,7 +7832,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C434"/>
+  <dimension ref="A1:C440"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -11186,86 +11233,118 @@
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B425" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B426" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B427" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B428" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B429" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B430" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B431" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B432" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B433" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B434" t="s">
-        <v>987</v>
+        <v>986</v>
+      </c>
+    </row>
+    <row r="436" spans="1:2">
+      <c r="A436" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B436" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2">
+      <c r="A437" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B437" t="s">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2">
+      <c r="A439" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B439" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2">
+      <c r="A440" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B440" t="s">
+        <v>986</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A425:A434">
+  <conditionalFormatting sqref="A425:A434 A436:A437 A439:A440">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added RCF to the code
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B29284A6-FF55-4972-B120-EA539E7721BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF18531-0EEE-4844-B78B-F3D1D74152B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1234" uniqueCount="1009">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="1034">
   <si>
     <t>Name</t>
   </si>
@@ -3051,22 +3051,97 @@
     <t>BSExists</t>
   </si>
   <si>
+    <t>LESExists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Statements are present in the application, manual review required. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leave and Earnings Statement is present in the application, manual review required. </t>
+  </si>
+  <si>
+    <t>VABL</t>
+  </si>
+  <si>
+    <t>VABL_FindingError</t>
+  </si>
+  <si>
+    <t>Date on the Veterans Affairs Benefit Letter is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>Gross Benefit Amount listed on the Veterans Affairs Benefit Letter does not match the $/Period on the ICW. </t>
+  </si>
+  <si>
+    <t>VABL_CheckDateMoveIn</t>
+  </si>
+  <si>
+    <t>VABL_ICWCheck</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Veterans Affairs Benefits Letter. Manual review required.</t>
+  </si>
+  <si>
     <t>BS_FindingError</t>
   </si>
   <si>
-    <t>LESExists</t>
+    <t>Unable to validate findings for Bank Statements. Needs manual review.</t>
   </si>
   <si>
     <t>LES_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Bank Statements. Needs manual review.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank Statements are present in the application, manual review required. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leave and Earnings Statement is present in the application, manual review required. </t>
+    <t>Unable to validate findings for Leave and Earnings Statement. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Veterans Benefits Letter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Release and Consent for is missing from the application. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">All adults have not been listed on the Applicant/Resident Name line of the Release and Consent Form. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">All adults have not been listed on the I/We line of the Release and Consent Form. </t>
+  </si>
+  <si>
+    <t>Not all adults have signed the Release and Consent Form.  </t>
+  </si>
+  <si>
+    <t>Not all adults have dated the Release and Consent Form.  </t>
+  </si>
+  <si>
+    <t>Date on the Release and Consent Form is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Release and Consent Form. Needs manual review. </t>
+  </si>
+  <si>
+    <t>RCFExists</t>
+  </si>
+  <si>
+    <t>RCF_ApplicantName</t>
+  </si>
+  <si>
+    <t>RCF_WeLine</t>
+  </si>
+  <si>
+    <t>RDC_Signed</t>
+  </si>
+  <si>
+    <t>RCF_Dated</t>
+  </si>
+  <si>
+    <t>RCF_DateCheckMoveIn</t>
+  </si>
+  <si>
+    <t>RCF_FindingError</t>
+  </si>
+  <si>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>Release and Consent Form</t>
   </si>
 </sst>
 </file>
@@ -3906,8 +3981,22 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A53" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A54" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1033</v>
+      </c>
+    </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7832,7 +7921,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C440"/>
+  <dimension ref="A1:C452"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -11316,36 +11405,116 @@
         <v>1002</v>
       </c>
       <c r="B436" t="s">
-        <v>1007</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>1003</v>
+        <v>1013</v>
       </c>
       <c r="B437" t="s">
-        <v>1006</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B439" t="s">
-        <v>1008</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>1005</v>
+        <v>1015</v>
       </c>
       <c r="B440" t="s">
-        <v>986</v>
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2">
+      <c r="A442" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B442" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2">
+      <c r="A443" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B444" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2">
+      <c r="A446" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2">
+      <c r="A447" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B447" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="448" spans="1:2">
+      <c r="A448" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B448" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="449" spans="1:2">
+      <c r="A449" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B449" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2">
+      <c r="A450" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B451" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="452" spans="1:2">
+      <c r="A452" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B452" t="s">
+        <v>1024</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A425:A434 A436:A437 A439:A440">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A442:A443 A439:A440 A425:A434 A436:A437">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added the TSAHC, TRRG for TX, and started VSA for TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CF18531-0EEE-4844-B78B-F3D1D74152B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596B2485-964D-4823-AD5D-538944FFF87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="1034">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="1073">
   <si>
     <t>Name</t>
   </si>
@@ -2313,9 +2313,6 @@
     <t>RDC</t>
   </si>
   <si>
-    <t>Rounded Day Calculator</t>
-  </si>
-  <si>
     <t>CSEI_SupportingDocInIAQ</t>
   </si>
   <si>
@@ -3142,6 +3139,126 @@
   </si>
   <si>
     <t>Release and Consent Form</t>
+  </si>
+  <si>
+    <t>Day Calculator</t>
+  </si>
+  <si>
+    <t>TRRG</t>
+  </si>
+  <si>
+    <t>A Tenant Rights and Resource Guide (TRRG)</t>
+  </si>
+  <si>
+    <t>Household name listed on the Tenant Rights and Resource Guide (TRRG) does not match the Head of Household listed on the ICW. </t>
+  </si>
+  <si>
+    <t>Unit Number listed on the Tenant Rights and Resource Guide (TRRG) does not match the Unit Number listed on the Application Summary. </t>
+  </si>
+  <si>
+    <t>All adults have not signed the Tenant Rights and Resource Guide (TRRG). </t>
+  </si>
+  <si>
+    <t>All adults have not dated the Tenant Rights and Resource Guide (TRRG). </t>
+  </si>
+  <si>
+    <t>Date on the Tenant Rights and Resource Guide (TRRG) is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>Unable to validate findings for the Tenant Rights and Resource Guide (TRRG). Manual review required. </t>
+  </si>
+  <si>
+    <t>TRRG_HeadOfHousehold</t>
+  </si>
+  <si>
+    <t>TRRG_Signed</t>
+  </si>
+  <si>
+    <t>TRRG_Dated</t>
+  </si>
+  <si>
+    <t>TRRG_FindingError</t>
+  </si>
+  <si>
+    <t>TRRG_CheckDateMoveIn</t>
+  </si>
+  <si>
+    <t>TRRG_UnitNumber</t>
+  </si>
+  <si>
+    <t>TSAHC document is missing from the application, and it is a required document for this property. </t>
+  </si>
+  <si>
+    <t>Property name listed on the TSAHC does not match the property listed on the Application Summary. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The TSAHC has not been signed. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The TSAHC has not been dated. </t>
+  </si>
+  <si>
+    <t>The date on the TSAHC is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>Unable to validate findings for the TSAHC. Manual review required. </t>
+  </si>
+  <si>
+    <t>TSAHC</t>
+  </si>
+  <si>
+    <t>TSAHC_PropertyName</t>
+  </si>
+  <si>
+    <t>TSAHC_Signed</t>
+  </si>
+  <si>
+    <t>TSAHC_Dated</t>
+  </si>
+  <si>
+    <t>TSAHC_CheckDateMoveIn</t>
+  </si>
+  <si>
+    <t>TSAHC_FindingError</t>
+  </si>
+  <si>
+    <t>TSAHCExists</t>
+  </si>
+  <si>
+    <t>VSAExists</t>
+  </si>
+  <si>
+    <t>Verification Services (Assets) is missing from the application and this property requires asset verification. Manual review required.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Account Type listed on Verification Services does not match the ICW. </t>
+  </si>
+  <si>
+    <t>Asset Institution Name listed on Verification Services does not match the ICW. </t>
+  </si>
+  <si>
+    <t>Asset Current Balance listed on Verification Services does not match the ICW. </t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Verification Services. Needs manual review. </t>
+  </si>
+  <si>
+    <t>VSA_AssetAccount</t>
+  </si>
+  <si>
+    <t>VSA_ICWInstitutionName</t>
+  </si>
+  <si>
+    <t>VSA_ICWCurrentBalance</t>
+  </si>
+  <si>
+    <t>VSA_FindingError</t>
+  </si>
+  <si>
+    <t>VSA</t>
+  </si>
+  <si>
+    <t>Verification Services (Assets)</t>
   </si>
 </sst>
 </file>
@@ -3610,7 +3727,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3759,7 +3876,7 @@
         <v>412</v>
       </c>
       <c r="B25" t="s">
-        <v>234</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
@@ -3914,99 +4031,123 @@
         <v>756</v>
       </c>
       <c r="B44" t="s">
-        <v>757</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>847</v>
+      </c>
+      <c r="B45" t="s">
         <v>848</v>
-      </c>
-      <c r="B45" t="s">
-        <v>849</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
+        <v>858</v>
+      </c>
+      <c r="B46" t="s">
         <v>859</v>
-      </c>
-      <c r="B46" t="s">
-        <v>860</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
+        <v>860</v>
+      </c>
+      <c r="B47" t="s">
         <v>861</v>
-      </c>
-      <c r="B47" t="s">
-        <v>862</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
+        <v>889</v>
+      </c>
+      <c r="B48" t="s">
         <v>890</v>
       </c>
-      <c r="B48" t="s">
-        <v>891</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="14.25" customHeight="1">
+    </row>
+    <row r="49" spans="1:3" ht="14.25" customHeight="1">
       <c r="A49" t="s">
+        <v>930</v>
+      </c>
+      <c r="B49" t="s">
         <v>931</v>
       </c>
-      <c r="B49" t="s">
-        <v>932</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="14.25" customHeight="1">
+    </row>
+    <row r="50" spans="1:3" ht="14.25" customHeight="1">
       <c r="A50" t="s">
+        <v>974</v>
+      </c>
+      <c r="B50" t="s">
         <v>975</v>
       </c>
-      <c r="B50" t="s">
-        <v>976</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="14.25" customHeight="1">
+    </row>
+    <row r="51" spans="1:3" ht="14.25" customHeight="1">
       <c r="A51" t="s">
+        <v>997</v>
+      </c>
+      <c r="B51" t="s">
         <v>998</v>
       </c>
-      <c r="B51" t="s">
+    </row>
+    <row r="52" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
         <v>999</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A52" t="s">
+      <c r="B52" t="s">
         <v>1000</v>
       </c>
-      <c r="B52" t="s">
-        <v>1001</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1">
+    </row>
+    <row r="53" spans="1:3" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B53" t="s">
-        <v>1017</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="14.25" customHeight="1">
       <c r="A54" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B54" t="s">
         <v>1032</v>
       </c>
-      <c r="B54" t="s">
-        <v>1033</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="55" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A55" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A56" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A57" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B57" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -7921,7 +8062,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C452"/>
+  <dimension ref="A1:C472"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8130,7 +8271,7 @@
         <v>741</v>
       </c>
       <c r="B24" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C24" t="s">
         <v>629</v>
@@ -8138,10 +8279,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>891</v>
+      </c>
+      <c r="B25" t="s">
         <v>892</v>
-      </c>
-      <c r="B25" t="s">
-        <v>893</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -8756,10 +8897,10 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
+        <v>924</v>
+      </c>
+      <c r="B99" t="s">
         <v>925</v>
-      </c>
-      <c r="B99" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -8805,34 +8946,34 @@
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
+        <v>920</v>
+      </c>
+      <c r="B104" t="s">
         <v>921</v>
-      </c>
-      <c r="B104" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
+        <v>922</v>
+      </c>
+      <c r="B105" t="s">
         <v>923</v>
-      </c>
-      <c r="B105" t="s">
-        <v>924</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
+        <v>927</v>
+      </c>
+      <c r="B106" t="s">
         <v>928</v>
-      </c>
-      <c r="B106" t="s">
-        <v>929</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B107" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -9236,7 +9377,7 @@
         <v>593</v>
       </c>
       <c r="B160" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="C160" t="s">
         <v>594</v>
@@ -9258,7 +9399,7 @@
         <v>753</v>
       </c>
       <c r="B162" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C162" t="s">
         <v>629</v>
@@ -9269,7 +9410,7 @@
         <v>754</v>
       </c>
       <c r="B163" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C163" t="s">
         <v>629</v>
@@ -9291,7 +9432,7 @@
         <v>468</v>
       </c>
       <c r="B166" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -9321,7 +9462,7 @@
         <v>239</v>
       </c>
       <c r="B169" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C169" t="s">
         <v>533</v>
@@ -9332,7 +9473,7 @@
         <v>240</v>
       </c>
       <c r="B170" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -9340,7 +9481,7 @@
         <v>248</v>
       </c>
       <c r="B171" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C171" t="s">
         <v>591</v>
@@ -9351,7 +9492,7 @@
         <v>719</v>
       </c>
       <c r="B172" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C172" t="s">
         <v>629</v>
@@ -9378,7 +9519,7 @@
         <v>243</v>
       </c>
       <c r="B175" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -9386,7 +9527,7 @@
         <v>244</v>
       </c>
       <c r="B176" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -9394,7 +9535,7 @@
         <v>245</v>
       </c>
       <c r="B177" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -9402,7 +9543,7 @@
         <v>246</v>
       </c>
       <c r="B178" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -9410,7 +9551,7 @@
         <v>247</v>
       </c>
       <c r="B179" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -9418,7 +9559,7 @@
         <v>279</v>
       </c>
       <c r="B180" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -9442,7 +9583,7 @@
         <v>638</v>
       </c>
       <c r="B183" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -9469,10 +9610,10 @@
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
+        <v>918</v>
+      </c>
+      <c r="B186" t="s">
         <v>919</v>
-      </c>
-      <c r="B186" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="187" spans="1:3">
@@ -9499,7 +9640,7 @@
         <v>469</v>
       </c>
       <c r="B190" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -9507,7 +9648,7 @@
         <v>249</v>
       </c>
       <c r="B191" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C191" t="s">
         <v>599</v>
@@ -9518,7 +9659,7 @@
         <v>251</v>
       </c>
       <c r="B192" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="C192" t="s">
         <v>633</v>
@@ -9529,7 +9670,7 @@
         <v>250</v>
       </c>
       <c r="B193" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -9572,7 +9713,7 @@
         <v>258</v>
       </c>
       <c r="B198" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="199" spans="1:3">
@@ -9588,7 +9729,7 @@
         <v>264</v>
       </c>
       <c r="B200" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="201" spans="1:3">
@@ -9596,7 +9737,7 @@
         <v>265</v>
       </c>
       <c r="B201" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="202" spans="1:3">
@@ -9604,7 +9745,7 @@
         <v>266</v>
       </c>
       <c r="B202" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="C202" t="s">
         <v>599</v>
@@ -9615,7 +9756,7 @@
         <v>267</v>
       </c>
       <c r="B203" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -9623,7 +9764,7 @@
         <v>268</v>
       </c>
       <c r="B204" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="C204" t="s">
         <v>599</v>
@@ -9634,7 +9775,7 @@
         <v>269</v>
       </c>
       <c r="B205" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -9650,7 +9791,7 @@
         <v>278</v>
       </c>
       <c r="B207" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -9666,7 +9807,7 @@
         <v>639</v>
       </c>
       <c r="B209" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -9693,7 +9834,7 @@
         <v>470</v>
       </c>
       <c r="B213" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -9709,7 +9850,7 @@
         <v>274</v>
       </c>
       <c r="B215" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="216" spans="1:3">
@@ -9717,7 +9858,7 @@
         <v>275</v>
       </c>
       <c r="B216" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="217" spans="1:3">
@@ -9725,7 +9866,7 @@
         <v>283</v>
       </c>
       <c r="B217" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -9733,7 +9874,7 @@
         <v>282</v>
       </c>
       <c r="B218" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="219" spans="1:3">
@@ -9741,7 +9882,7 @@
         <v>284</v>
       </c>
       <c r="B219" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -9749,7 +9890,7 @@
         <v>640</v>
       </c>
       <c r="B220" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -9765,7 +9906,7 @@
         <v>471</v>
       </c>
       <c r="B223" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -9781,7 +9922,7 @@
         <v>287</v>
       </c>
       <c r="B225" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="226" spans="1:3">
@@ -9797,7 +9938,7 @@
         <v>289</v>
       </c>
       <c r="B227" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -9805,7 +9946,7 @@
         <v>291</v>
       </c>
       <c r="B228" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="229" spans="1:3">
@@ -9813,7 +9954,7 @@
         <v>292</v>
       </c>
       <c r="B229" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -9821,7 +9962,7 @@
         <v>293</v>
       </c>
       <c r="B230" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="231" spans="1:3">
@@ -9829,7 +9970,7 @@
         <v>294</v>
       </c>
       <c r="B231" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -9837,7 +9978,7 @@
         <v>641</v>
       </c>
       <c r="B232" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="233" spans="1:3">
@@ -9853,7 +9994,7 @@
         <v>472</v>
       </c>
       <c r="B235" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -9880,7 +10021,7 @@
         <v>298</v>
       </c>
       <c r="B238" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="C238" t="s">
         <v>533</v>
@@ -9891,7 +10032,7 @@
         <v>299</v>
       </c>
       <c r="B239" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -9899,7 +10040,7 @@
         <v>455</v>
       </c>
       <c r="B240" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -9907,7 +10048,7 @@
         <v>301</v>
       </c>
       <c r="B241" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="242" spans="1:3">
@@ -9915,7 +10056,7 @@
         <v>302</v>
       </c>
       <c r="B242" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -9923,7 +10064,7 @@
         <v>303</v>
       </c>
       <c r="B243" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -9931,7 +10072,7 @@
         <v>304</v>
       </c>
       <c r="B244" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -9939,7 +10080,7 @@
         <v>305</v>
       </c>
       <c r="B245" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -9947,7 +10088,7 @@
         <v>642</v>
       </c>
       <c r="B246" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -10642,207 +10783,207 @@
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
+        <v>757</v>
+      </c>
+      <c r="B333" t="s">
         <v>758</v>
-      </c>
-      <c r="B333" t="s">
-        <v>759</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
+        <v>759</v>
+      </c>
+      <c r="B334" t="s">
         <v>760</v>
-      </c>
-      <c r="B334" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
+        <v>761</v>
+      </c>
+      <c r="B335" t="s">
         <v>762</v>
-      </c>
-      <c r="B335" t="s">
-        <v>763</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
+        <v>763</v>
+      </c>
+      <c r="B336" t="s">
         <v>764</v>
-      </c>
-      <c r="B336" t="s">
-        <v>765</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="A337" t="s">
+        <v>765</v>
+      </c>
+      <c r="B337" t="s">
         <v>766</v>
-      </c>
-      <c r="B337" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="A338" t="s">
+        <v>767</v>
+      </c>
+      <c r="B338" t="s">
         <v>768</v>
-      </c>
-      <c r="B338" t="s">
-        <v>769</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="A339" t="s">
+        <v>769</v>
+      </c>
+      <c r="B339" t="s">
         <v>770</v>
-      </c>
-      <c r="B339" t="s">
-        <v>771</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="A340" t="s">
+        <v>771</v>
+      </c>
+      <c r="B340" t="s">
         <v>772</v>
-      </c>
-      <c r="B340" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="A341" t="s">
+        <v>773</v>
+      </c>
+      <c r="B341" t="s">
         <v>774</v>
-      </c>
-      <c r="B341" t="s">
-        <v>775</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="A342" t="s">
+        <v>775</v>
+      </c>
+      <c r="B342" t="s">
         <v>776</v>
-      </c>
-      <c r="B342" t="s">
-        <v>777</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="A343" t="s">
+        <v>777</v>
+      </c>
+      <c r="B343" t="s">
         <v>778</v>
-      </c>
-      <c r="B343" t="s">
-        <v>779</v>
       </c>
     </row>
     <row r="344" spans="1:2">
       <c r="A344" t="s">
+        <v>779</v>
+      </c>
+      <c r="B344" t="s">
         <v>780</v>
-      </c>
-      <c r="B344" t="s">
-        <v>781</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="A345" t="s">
+        <v>781</v>
+      </c>
+      <c r="B345" t="s">
         <v>782</v>
-      </c>
-      <c r="B345" t="s">
-        <v>783</v>
       </c>
     </row>
     <row r="346" spans="1:2">
       <c r="A346" t="s">
+        <v>783</v>
+      </c>
+      <c r="B346" t="s">
         <v>784</v>
-      </c>
-      <c r="B346" t="s">
-        <v>785</v>
       </c>
     </row>
     <row r="347" spans="1:2">
       <c r="A347" t="s">
+        <v>785</v>
+      </c>
+      <c r="B347" t="s">
         <v>786</v>
-      </c>
-      <c r="B347" t="s">
-        <v>787</v>
       </c>
     </row>
     <row r="348" spans="1:2">
       <c r="A348" t="s">
+        <v>787</v>
+      </c>
+      <c r="B348" t="s">
         <v>788</v>
-      </c>
-      <c r="B348" t="s">
-        <v>789</v>
       </c>
     </row>
     <row r="349" spans="1:2">
       <c r="A349" t="s">
+        <v>789</v>
+      </c>
+      <c r="B349" t="s">
         <v>790</v>
-      </c>
-      <c r="B349" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="350" spans="1:2">
       <c r="A350" t="s">
+        <v>791</v>
+      </c>
+      <c r="B350" t="s">
         <v>792</v>
-      </c>
-      <c r="B350" t="s">
-        <v>793</v>
       </c>
     </row>
     <row r="352" spans="1:2">
       <c r="A352" t="s">
+        <v>793</v>
+      </c>
+      <c r="B352" t="s">
         <v>794</v>
-      </c>
-      <c r="B352" t="s">
-        <v>795</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
+        <v>795</v>
+      </c>
+      <c r="B353" t="s">
         <v>796</v>
-      </c>
-      <c r="B353" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
+        <v>797</v>
+      </c>
+      <c r="B354" t="s">
         <v>798</v>
-      </c>
-      <c r="B354" t="s">
-        <v>799</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
+        <v>799</v>
+      </c>
+      <c r="B355" t="s">
         <v>800</v>
-      </c>
-      <c r="B355" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
+        <v>801</v>
+      </c>
+      <c r="B356" t="s">
         <v>802</v>
-      </c>
-      <c r="B356" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
+        <v>803</v>
+      </c>
+      <c r="B357" t="s">
         <v>804</v>
-      </c>
-      <c r="B357" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
+        <v>805</v>
+      </c>
+      <c r="B358" t="s">
         <v>806</v>
-      </c>
-      <c r="B358" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B359" t="s">
         <v>321</v>
@@ -10850,39 +10991,39 @@
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
+        <v>808</v>
+      </c>
+      <c r="B360" t="s">
         <v>809</v>
-      </c>
-      <c r="B360" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
+        <v>810</v>
+      </c>
+      <c r="B361" t="s">
         <v>811</v>
-      </c>
-      <c r="B361" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
+        <v>812</v>
+      </c>
+      <c r="B362" t="s">
         <v>813</v>
-      </c>
-      <c r="B362" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
+        <v>814</v>
+      </c>
+      <c r="B363" t="s">
         <v>815</v>
-      </c>
-      <c r="B363" t="s">
-        <v>816</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B365" t="s">
         <v>314</v>
@@ -10890,15 +11031,15 @@
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
+        <v>817</v>
+      </c>
+      <c r="B366" t="s">
         <v>818</v>
-      </c>
-      <c r="B366" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B367" t="s">
         <v>316</v>
@@ -10906,7 +11047,7 @@
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="B368" t="s">
         <v>317</v>
@@ -10914,119 +11055,119 @@
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
+        <v>845</v>
+      </c>
+      <c r="B370" t="s">
         <v>846</v>
-      </c>
-      <c r="B370" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B371" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
+        <v>837</v>
+      </c>
+      <c r="B372" t="s">
         <v>838</v>
-      </c>
-      <c r="B372" t="s">
-        <v>839</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B373" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B374" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B375" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B377" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B378" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B379" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B380" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B381" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B382" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
+        <v>862</v>
+      </c>
+      <c r="B384" t="s">
         <v>863</v>
-      </c>
-      <c r="B384" t="s">
-        <v>864</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
+        <v>864</v>
+      </c>
+      <c r="B385" t="s">
         <v>865</v>
-      </c>
-      <c r="B385" t="s">
-        <v>866</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B386" t="s">
         <v>717</v>
@@ -11034,15 +11175,15 @@
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B387" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B388" t="s">
         <v>252</v>
@@ -11050,7 +11191,7 @@
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B389" t="s">
         <v>255</v>
@@ -11058,23 +11199,23 @@
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B390" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B391" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B392" t="s">
         <v>260</v>
@@ -11082,39 +11223,39 @@
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B393" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B394" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B395" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B396" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B397" t="s">
         <v>277</v>
@@ -11122,7 +11263,7 @@
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B398" t="s">
         <v>281</v>
@@ -11130,15 +11271,15 @@
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B399" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B400" t="s">
         <v>635</v>
@@ -11146,7 +11287,7 @@
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B401" t="s">
         <v>617</v>
@@ -11154,362 +11295,498 @@
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B403" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B404" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B405" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B406" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B407" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B408" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B409" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B410" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B411" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B412" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B413" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B414" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B415" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B416" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B417" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B418" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B419" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B420" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B421" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B422" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B423" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B425" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B426" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B427" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B428" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B429" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B430" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B431" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B432" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B433" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B434" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B436" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B437" t="s">
         <v>1013</v>
-      </c>
-      <c r="B437" t="s">
-        <v>1014</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B439" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B440" t="s">
         <v>1015</v>
-      </c>
-      <c r="B440" t="s">
-        <v>1016</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B442" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B443" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B444" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B446" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B447" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B448" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B449" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B450" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B451" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B452" t="s">
-        <v>1024</v>
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2">
+      <c r="A454" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B454" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2">
+      <c r="A455" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B455" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2">
+      <c r="A456" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B457" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B459" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B461" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B462" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2">
+      <c r="A463" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B463" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2">
+      <c r="A464" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B464" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B465" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B466" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B468" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2">
+      <c r="A469" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B470" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2">
+      <c r="A471" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B471" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2">
+      <c r="A472" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1066</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
found a mistake within the Config file and corrected it
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596B2485-964D-4823-AD5D-538944FFF87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0B9927-F6DD-416C-9931-63840F329573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5640" yWindow="1515" windowWidth="21060" windowHeight="9615" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3123,9 +3123,6 @@
     <t>RCF_WeLine</t>
   </si>
   <si>
-    <t>RDC_Signed</t>
-  </si>
-  <si>
     <t>RCF_Dated</t>
   </si>
   <si>
@@ -3259,6 +3256,9 @@
   </si>
   <si>
     <t>Verification Services (Assets)</t>
+  </si>
+  <si>
+    <t>RCF_Signed</t>
   </si>
 </sst>
 </file>
@@ -3876,7 +3876,7 @@
         <v>412</v>
       </c>
       <c r="B25" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
@@ -4031,7 +4031,7 @@
         <v>756</v>
       </c>
       <c r="B44" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
@@ -4108,37 +4108,37 @@
     </row>
     <row r="54" spans="1:3" ht="14.25" customHeight="1">
       <c r="A54" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B54" t="s">
         <v>1031</v>
-      </c>
-      <c r="B54" t="s">
-        <v>1032</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="14.25" customHeight="1">
       <c r="A55" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C55" t="s">
         <v>1034</v>
-      </c>
-      <c r="B55" t="s">
-        <v>1034</v>
-      </c>
-      <c r="C55" t="s">
-        <v>1035</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="14.25" customHeight="1">
       <c r="A56" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B56" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="14.25" customHeight="1">
       <c r="A57" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B57" t="s">
         <v>1071</v>
-      </c>
-      <c r="B57" t="s">
-        <v>1072</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1"/>
@@ -11623,7 +11623,7 @@
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>1027</v>
+        <v>1072</v>
       </c>
       <c r="B449" t="s">
         <v>1020</v>
@@ -11631,7 +11631,7 @@
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B450" t="s">
         <v>1021</v>
@@ -11639,7 +11639,7 @@
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B451" t="s">
         <v>1022</v>
@@ -11647,7 +11647,7 @@
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B452" t="s">
         <v>1023</v>
@@ -11655,138 +11655,138 @@
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B454" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B455" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B456" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B457" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B458" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B459" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B461" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B462" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B463" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B464" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B465" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B466" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B468" t="s">
         <v>1061</v>
-      </c>
-      <c r="B468" t="s">
-        <v>1062</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B469" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B470" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B471" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B472" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updateded CSPH and added CSC - TX workflow
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9609CC5-FFC0-4638-9FD3-2EAC75919003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C792B698-9E05-43A4-B382-EE789041A5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3780" yWindow="3015" windowWidth="21060" windowHeight="9615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="1073">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1317" uniqueCount="1086">
   <si>
     <t>Name</t>
   </si>
@@ -3258,7 +3258,46 @@
     <t>RCF_Signed</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>CSC_120days</t>
+  </si>
+  <si>
+    <t>Both 120 days of pay history available and 120 days of pay history not available data is populated on the Child Support Calcs. Achie cannot determine which data to use, manual review is required. </t>
+  </si>
+  <si>
+    <t>TX - Newly added by Raluca</t>
+  </si>
+  <si>
+    <t>CSC_ConsistentPayments</t>
+  </si>
+  <si>
+    <t>The consistent payments data is populated on Child Support Calcs but additional data tables are populated as well. Archie cannot determine which data to use, manual review is required. </t>
+  </si>
+  <si>
+    <t>CSC_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Child Support Calcs. Needs manual review.</t>
+  </si>
+  <si>
+    <t>CSPH_PaymentGenerationDate</t>
+  </si>
+  <si>
+    <t>Payment Generation Date listed on the Child Support Payment History is not with in 120 days of Move-In date. </t>
+  </si>
+  <si>
+    <t>CSPH_LessThan120</t>
+  </si>
+  <si>
+    <t>Less than 120 days of payment data is available but the oldest payment date on the Child Support Payment History does not match the Start Date on Child Support Calcs. </t>
+  </si>
+  <si>
+    <t>CSPH_PaymentAndEndDateCheck</t>
+  </si>
+  <si>
+    <t>Payment Generation Date listed on the Child Support Payment History does not match the End Date listed on Child Support Calcs. </t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3727,7 +3766,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>1072</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -8062,7 +8101,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C472"/>
+  <dimension ref="A1:C478"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -10392,1405 +10431,1471 @@
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>482</v>
+        <v>1079</v>
       </c>
       <c r="B283" t="s">
-        <v>621</v>
+        <v>1080</v>
+      </c>
+      <c r="C283" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3">
+      <c r="A284" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B284" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C284" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>678</v>
+        <v>1083</v>
       </c>
       <c r="B285" t="s">
-        <v>697</v>
+        <v>1084</v>
       </c>
       <c r="C285" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="287" spans="1:3">
-      <c r="A287" t="s">
-        <v>674</v>
-      </c>
-      <c r="B287" t="s">
-        <v>675</v>
-      </c>
-      <c r="C287" t="s">
-        <v>629</v>
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3">
+      <c r="A286" t="s">
+        <v>482</v>
+      </c>
+      <c r="B286" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>473</v>
+        <v>678</v>
       </c>
       <c r="B288" t="s">
-        <v>474</v>
+        <v>697</v>
+      </c>
+      <c r="C288" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>368</v>
+        <v>1072</v>
       </c>
       <c r="B289" t="s">
-        <v>379</v>
+        <v>1073</v>
+      </c>
+      <c r="C289" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>369</v>
+        <v>1075</v>
       </c>
       <c r="B290" t="s">
-        <v>380</v>
+        <v>1076</v>
       </c>
       <c r="C290" t="s">
-        <v>533</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>521</v>
+        <v>1077</v>
       </c>
       <c r="B291" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="292" spans="1:3">
-      <c r="A292" t="s">
-        <v>370</v>
-      </c>
-      <c r="B292" t="s">
-        <v>381</v>
-      </c>
-      <c r="C292" t="s">
-        <v>533</v>
+        <v>1078</v>
+      </c>
+      <c r="C291" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>371</v>
+        <v>674</v>
       </c>
       <c r="B293" t="s">
-        <v>382</v>
+        <v>675</v>
       </c>
       <c r="C293" t="s">
-        <v>533</v>
+        <v>629</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>372</v>
+        <v>473</v>
       </c>
       <c r="B294" t="s">
-        <v>534</v>
+        <v>474</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="B295" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="B296" t="s">
-        <v>384</v>
+        <v>380</v>
+      </c>
+      <c r="C296" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>375</v>
+        <v>521</v>
       </c>
       <c r="B297" t="s">
-        <v>385</v>
+        <v>522</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
       <c r="B298" t="s">
-        <v>386</v>
+        <v>381</v>
+      </c>
+      <c r="C298" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="B299" t="s">
-        <v>387</v>
+        <v>382</v>
+      </c>
+      <c r="C299" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="B300" t="s">
-        <v>388</v>
+        <v>534</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>733</v>
+        <v>373</v>
       </c>
       <c r="B301" t="s">
-        <v>734</v>
-      </c>
-      <c r="C301" t="s">
-        <v>629</v>
+        <v>383</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>480</v>
+        <v>374</v>
       </c>
       <c r="B302" t="s">
-        <v>622</v>
+        <v>384</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>557</v>
+        <v>375</v>
       </c>
       <c r="B303" t="s">
-        <v>558</v>
+        <v>385</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3">
+      <c r="A304" t="s">
+        <v>376</v>
+      </c>
+      <c r="B304" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>475</v>
+        <v>377</v>
       </c>
       <c r="B305" t="s">
-        <v>474</v>
+        <v>387</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>395</v>
+        <v>378</v>
       </c>
       <c r="B306" t="s">
-        <v>406</v>
+        <v>388</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>396</v>
+        <v>733</v>
       </c>
       <c r="B307" t="s">
-        <v>407</v>
+        <v>734</v>
       </c>
       <c r="C307" t="s">
-        <v>533</v>
+        <v>629</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="B308" t="s">
-        <v>523</v>
+        <v>622</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>397</v>
+        <v>557</v>
       </c>
       <c r="B309" t="s">
-        <v>408</v>
-      </c>
-      <c r="C309" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="310" spans="1:3">
-      <c r="A310" t="s">
-        <v>398</v>
-      </c>
-      <c r="B310" t="s">
-        <v>409</v>
-      </c>
-      <c r="C310" t="s">
-        <v>533</v>
+        <v>558</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>399</v>
+        <v>475</v>
       </c>
       <c r="B311" t="s">
-        <v>535</v>
+        <v>474</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B312" t="s">
-        <v>383</v>
+        <v>406</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
       <c r="B313" t="s">
-        <v>384</v>
+        <v>407</v>
+      </c>
+      <c r="C313" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>402</v>
+        <v>465</v>
       </c>
       <c r="B314" t="s">
-        <v>410</v>
+        <v>523</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="B315" t="s">
-        <v>411</v>
+        <v>408</v>
+      </c>
+      <c r="C315" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="B316" t="s">
-        <v>387</v>
+        <v>409</v>
+      </c>
+      <c r="C316" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="B317" t="s">
-        <v>388</v>
+        <v>535</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>479</v>
+        <v>400</v>
       </c>
       <c r="B318" t="s">
-        <v>622</v>
+        <v>383</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>564</v>
+        <v>401</v>
       </c>
       <c r="B319" t="s">
-        <v>558</v>
+        <v>384</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3">
+      <c r="A320" t="s">
+        <v>402</v>
+      </c>
+      <c r="B320" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>672</v>
+        <v>403</v>
       </c>
       <c r="B321" t="s">
-        <v>673</v>
-      </c>
-      <c r="C321" t="s">
-        <v>629</v>
+        <v>411</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
       <c r="B322" t="s">
-        <v>565</v>
+        <v>387</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="B323" t="s">
-        <v>566</v>
-      </c>
-      <c r="C323" t="s">
-        <v>533</v>
+        <v>388</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>466</v>
+        <v>479</v>
       </c>
       <c r="B324" t="s">
-        <v>567</v>
+        <v>622</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>391</v>
+        <v>564</v>
       </c>
       <c r="B325" t="s">
-        <v>592</v>
-      </c>
-    </row>
-    <row r="326" spans="1:3">
-      <c r="A326" t="s">
-        <v>392</v>
-      </c>
-      <c r="B326" t="s">
-        <v>568</v>
+        <v>558</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>393</v>
+        <v>672</v>
       </c>
       <c r="B327" t="s">
-        <v>569</v>
+        <v>673</v>
+      </c>
+      <c r="C327" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>478</v>
+        <v>389</v>
       </c>
       <c r="B328" t="s">
-        <v>623</v>
+        <v>565</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3">
+      <c r="A329" t="s">
+        <v>390</v>
+      </c>
+      <c r="B329" t="s">
+        <v>566</v>
+      </c>
+      <c r="C329" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>749</v>
+        <v>466</v>
       </c>
       <c r="B330" t="s">
-        <v>750</v>
-      </c>
-      <c r="C330" t="s">
-        <v>629</v>
+        <v>567</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>751</v>
+        <v>391</v>
       </c>
       <c r="B331" t="s">
-        <v>752</v>
-      </c>
-      <c r="C331" t="s">
-        <v>629</v>
+        <v>592</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3">
+      <c r="A332" t="s">
+        <v>392</v>
+      </c>
+      <c r="B332" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>757</v>
+        <v>393</v>
       </c>
       <c r="B333" t="s">
-        <v>758</v>
+        <v>569</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>759</v>
+        <v>478</v>
       </c>
       <c r="B334" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="335" spans="1:3">
-      <c r="A335" t="s">
-        <v>761</v>
-      </c>
-      <c r="B335" t="s">
-        <v>762</v>
+        <v>623</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
+        <v>749</v>
+      </c>
+      <c r="B336" t="s">
+        <v>750</v>
+      </c>
+      <c r="C336" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3">
+      <c r="A337" t="s">
+        <v>751</v>
+      </c>
+      <c r="B337" t="s">
+        <v>752</v>
+      </c>
+      <c r="C337" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3">
+      <c r="A339" t="s">
+        <v>757</v>
+      </c>
+      <c r="B339" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3">
+      <c r="A340" t="s">
+        <v>759</v>
+      </c>
+      <c r="B340" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3">
+      <c r="A341" t="s">
+        <v>761</v>
+      </c>
+      <c r="B341" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="342" spans="1:3">
+      <c r="A342" t="s">
         <v>763</v>
       </c>
-      <c r="B336" t="s">
+      <c r="B342" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="337" spans="1:2">
-      <c r="A337" t="s">
+    <row r="343" spans="1:3">
+      <c r="A343" t="s">
         <v>765</v>
       </c>
-      <c r="B337" t="s">
+      <c r="B343" t="s">
         <v>766</v>
       </c>
     </row>
-    <row r="338" spans="1:2">
-      <c r="A338" t="s">
+    <row r="344" spans="1:3">
+      <c r="A344" t="s">
         <v>767</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B344" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="339" spans="1:2">
-      <c r="A339" t="s">
+    <row r="345" spans="1:3">
+      <c r="A345" t="s">
         <v>769</v>
       </c>
-      <c r="B339" t="s">
+      <c r="B345" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="340" spans="1:2">
-      <c r="A340" t="s">
+    <row r="346" spans="1:3">
+      <c r="A346" t="s">
         <v>771</v>
       </c>
-      <c r="B340" t="s">
+      <c r="B346" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="341" spans="1:2">
-      <c r="A341" t="s">
+    <row r="347" spans="1:3">
+      <c r="A347" t="s">
         <v>773</v>
       </c>
-      <c r="B341" t="s">
+      <c r="B347" t="s">
         <v>774</v>
       </c>
     </row>
-    <row r="342" spans="1:2">
-      <c r="A342" t="s">
+    <row r="348" spans="1:3">
+      <c r="A348" t="s">
         <v>775</v>
       </c>
-      <c r="B342" t="s">
+      <c r="B348" t="s">
         <v>776</v>
       </c>
     </row>
-    <row r="343" spans="1:2">
-      <c r="A343" t="s">
+    <row r="349" spans="1:3">
+      <c r="A349" t="s">
         <v>777</v>
       </c>
-      <c r="B343" t="s">
+      <c r="B349" t="s">
         <v>778</v>
       </c>
     </row>
-    <row r="344" spans="1:2">
-      <c r="A344" t="s">
+    <row r="350" spans="1:3">
+      <c r="A350" t="s">
         <v>779</v>
       </c>
-      <c r="B344" t="s">
+      <c r="B350" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="345" spans="1:2">
-      <c r="A345" t="s">
+    <row r="351" spans="1:3">
+      <c r="A351" t="s">
         <v>781</v>
       </c>
-      <c r="B345" t="s">
+      <c r="B351" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="346" spans="1:2">
-      <c r="A346" t="s">
+    <row r="352" spans="1:3">
+      <c r="A352" t="s">
         <v>783</v>
       </c>
-      <c r="B346" t="s">
+      <c r="B352" t="s">
         <v>784</v>
-      </c>
-    </row>
-    <row r="347" spans="1:2">
-      <c r="A347" t="s">
-        <v>785</v>
-      </c>
-      <c r="B347" t="s">
-        <v>786</v>
-      </c>
-    </row>
-    <row r="348" spans="1:2">
-      <c r="A348" t="s">
-        <v>787</v>
-      </c>
-      <c r="B348" t="s">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="349" spans="1:2">
-      <c r="A349" t="s">
-        <v>789</v>
-      </c>
-      <c r="B349" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="350" spans="1:2">
-      <c r="A350" t="s">
-        <v>791</v>
-      </c>
-      <c r="B350" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="352" spans="1:2">
-      <c r="A352" t="s">
-        <v>793</v>
-      </c>
-      <c r="B352" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>795</v>
+        <v>785</v>
       </c>
       <c r="B353" t="s">
-        <v>796</v>
+        <v>786</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>797</v>
+        <v>787</v>
       </c>
       <c r="B354" t="s">
-        <v>798</v>
+        <v>788</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>799</v>
+        <v>789</v>
       </c>
       <c r="B355" t="s">
-        <v>800</v>
+        <v>790</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>801</v>
+        <v>791</v>
       </c>
       <c r="B356" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="357" spans="1:2">
-      <c r="A357" t="s">
-        <v>803</v>
-      </c>
-      <c r="B357" t="s">
-        <v>804</v>
+        <v>792</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>805</v>
+        <v>793</v>
       </c>
       <c r="B358" t="s">
-        <v>806</v>
+        <v>794</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>807</v>
+        <v>795</v>
       </c>
       <c r="B359" t="s">
-        <v>321</v>
+        <v>796</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>808</v>
+        <v>797</v>
       </c>
       <c r="B360" t="s">
-        <v>809</v>
+        <v>798</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>810</v>
+        <v>799</v>
       </c>
       <c r="B361" t="s">
-        <v>811</v>
+        <v>800</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>812</v>
+        <v>801</v>
       </c>
       <c r="B362" t="s">
-        <v>813</v>
+        <v>802</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>814</v>
+        <v>803</v>
       </c>
       <c r="B363" t="s">
-        <v>815</v>
+        <v>804</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" t="s">
+        <v>805</v>
+      </c>
+      <c r="B364" t="s">
+        <v>806</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
       <c r="B365" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>817</v>
+        <v>808</v>
       </c>
       <c r="B366" t="s">
-        <v>818</v>
+        <v>809</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>819</v>
+        <v>810</v>
       </c>
       <c r="B367" t="s">
-        <v>316</v>
+        <v>811</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>820</v>
+        <v>812</v>
       </c>
       <c r="B368" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="370" spans="1:2">
-      <c r="A370" t="s">
-        <v>845</v>
-      </c>
-      <c r="B370" t="s">
-        <v>846</v>
+        <v>813</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" t="s">
+        <v>814</v>
+      </c>
+      <c r="B369" t="s">
+        <v>815</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>844</v>
+        <v>816</v>
       </c>
       <c r="B371" t="s">
-        <v>843</v>
+        <v>314</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>837</v>
+        <v>817</v>
       </c>
       <c r="B372" t="s">
-        <v>838</v>
+        <v>818</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>835</v>
+        <v>819</v>
       </c>
       <c r="B373" t="s">
-        <v>839</v>
+        <v>316</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>836</v>
+        <v>820</v>
       </c>
       <c r="B374" t="s">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="375" spans="1:2">
-      <c r="A375" t="s">
-        <v>842</v>
-      </c>
-      <c r="B375" t="s">
-        <v>841</v>
+        <v>317</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" t="s">
+        <v>845</v>
+      </c>
+      <c r="B376" t="s">
+        <v>846</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="B377" t="s">
-        <v>854</v>
+        <v>843</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>857</v>
+        <v>837</v>
       </c>
       <c r="B378" t="s">
-        <v>855</v>
+        <v>838</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>850</v>
+        <v>835</v>
       </c>
       <c r="B379" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>851</v>
+        <v>836</v>
       </c>
       <c r="B380" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>852</v>
+        <v>842</v>
       </c>
       <c r="B381" t="s">
-        <v>840</v>
-      </c>
-    </row>
-    <row r="382" spans="1:2">
-      <c r="A382" t="s">
-        <v>853</v>
-      </c>
-      <c r="B382" t="s">
-        <v>856</v>
+        <v>841</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" t="s">
+        <v>849</v>
+      </c>
+      <c r="B383" t="s">
+        <v>854</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="B384" t="s">
-        <v>863</v>
+        <v>855</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>864</v>
+        <v>850</v>
       </c>
       <c r="B385" t="s">
-        <v>865</v>
+        <v>838</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>866</v>
+        <v>851</v>
       </c>
       <c r="B386" t="s">
-        <v>717</v>
+        <v>839</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>868</v>
+        <v>852</v>
       </c>
       <c r="B387" t="s">
-        <v>867</v>
+        <v>840</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>875</v>
+        <v>853</v>
       </c>
       <c r="B388" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="389" spans="1:2">
-      <c r="A389" t="s">
-        <v>876</v>
-      </c>
-      <c r="B389" t="s">
-        <v>255</v>
+        <v>856</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>877</v>
+        <v>862</v>
       </c>
       <c r="B390" t="s">
-        <v>869</v>
+        <v>863</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>880</v>
+        <v>864</v>
       </c>
       <c r="B391" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>881</v>
+        <v>866</v>
       </c>
       <c r="B392" t="s">
-        <v>260</v>
+        <v>717</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>882</v>
+        <v>868</v>
       </c>
       <c r="B393" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>883</v>
+        <v>875</v>
       </c>
       <c r="B394" t="s">
-        <v>872</v>
+        <v>252</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>884</v>
+        <v>876</v>
       </c>
       <c r="B395" t="s">
-        <v>873</v>
+        <v>255</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>885</v>
+        <v>877</v>
       </c>
       <c r="B396" t="s">
-        <v>874</v>
+        <v>869</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>886</v>
+        <v>880</v>
       </c>
       <c r="B397" t="s">
-        <v>277</v>
+        <v>870</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>887</v>
+        <v>881</v>
       </c>
       <c r="B398" t="s">
-        <v>281</v>
+        <v>260</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>888</v>
+        <v>882</v>
       </c>
       <c r="B399" t="s">
-        <v>828</v>
+        <v>871</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="B400" t="s">
-        <v>635</v>
+        <v>872</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="B401" t="s">
-        <v>617</v>
+        <v>873</v>
+      </c>
+    </row>
+    <row r="402" spans="1:2">
+      <c r="A402" t="s">
+        <v>885</v>
+      </c>
+      <c r="B402" t="s">
+        <v>874</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>953</v>
+        <v>886</v>
       </c>
       <c r="B403" t="s">
-        <v>932</v>
+        <v>277</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>972</v>
+        <v>887</v>
       </c>
       <c r="B404" t="s">
-        <v>933</v>
+        <v>281</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>971</v>
+        <v>888</v>
       </c>
       <c r="B405" t="s">
-        <v>934</v>
+        <v>828</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>970</v>
+        <v>879</v>
       </c>
       <c r="B406" t="s">
-        <v>935</v>
+        <v>635</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>969</v>
+        <v>878</v>
       </c>
       <c r="B407" t="s">
-        <v>936</v>
-      </c>
-    </row>
-    <row r="408" spans="1:2">
-      <c r="A408" t="s">
-        <v>968</v>
-      </c>
-      <c r="B408" t="s">
-        <v>937</v>
+        <v>617</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>967</v>
+        <v>953</v>
       </c>
       <c r="B409" t="s">
-        <v>938</v>
+        <v>932</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="B410" t="s">
-        <v>939</v>
+        <v>933</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="B411" t="s">
-        <v>940</v>
+        <v>934</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="B412" t="s">
-        <v>941</v>
+        <v>935</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="B413" t="s">
-        <v>942</v>
+        <v>936</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="B414" t="s">
-        <v>943</v>
+        <v>937</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>962</v>
+        <v>967</v>
       </c>
       <c r="B415" t="s">
-        <v>944</v>
+        <v>938</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="B416" t="s">
-        <v>945</v>
+        <v>939</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
       <c r="B417" t="s">
-        <v>946</v>
+        <v>940</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>959</v>
+        <v>964</v>
       </c>
       <c r="B418" t="s">
-        <v>947</v>
+        <v>941</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="B419" t="s">
-        <v>948</v>
+        <v>942</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>957</v>
+        <v>973</v>
       </c>
       <c r="B420" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="B421" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="B422" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="B423" t="s">
-        <v>952</v>
+        <v>946</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2">
+      <c r="A424" t="s">
+        <v>959</v>
+      </c>
+      <c r="B424" t="s">
+        <v>947</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>995</v>
+        <v>958</v>
       </c>
       <c r="B425" t="s">
-        <v>976</v>
+        <v>948</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>986</v>
+        <v>957</v>
       </c>
       <c r="B426" t="s">
-        <v>977</v>
+        <v>949</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>987</v>
+        <v>956</v>
       </c>
       <c r="B427" t="s">
-        <v>978</v>
+        <v>950</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>988</v>
+        <v>955</v>
       </c>
       <c r="B428" t="s">
-        <v>979</v>
+        <v>951</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>991</v>
+        <v>954</v>
       </c>
       <c r="B429" t="s">
-        <v>980</v>
-      </c>
-    </row>
-    <row r="430" spans="1:2">
-      <c r="A430" t="s">
-        <v>989</v>
-      </c>
-      <c r="B430" t="s">
-        <v>981</v>
+        <v>952</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>992</v>
+        <v>995</v>
       </c>
       <c r="B431" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="B432" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>994</v>
+        <v>987</v>
       </c>
       <c r="B433" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="B434" t="s">
-        <v>985</v>
+        <v>979</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2">
+      <c r="A435" t="s">
+        <v>991</v>
+      </c>
+      <c r="B435" t="s">
+        <v>980</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>1000</v>
+        <v>989</v>
       </c>
       <c r="B436" t="s">
-        <v>1002</v>
+        <v>981</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>1011</v>
+        <v>992</v>
       </c>
       <c r="B437" t="s">
-        <v>1012</v>
+        <v>982</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2">
+      <c r="A438" t="s">
+        <v>990</v>
+      </c>
+      <c r="B438" t="s">
+        <v>983</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>1001</v>
+        <v>994</v>
       </c>
       <c r="B439" t="s">
-        <v>1003</v>
+        <v>984</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>1013</v>
+        <v>993</v>
       </c>
       <c r="B440" t="s">
-        <v>1014</v>
+        <v>985</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>1008</v>
+        <v>1000</v>
       </c>
       <c r="B442" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
       <c r="B443" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="444" spans="1:2">
-      <c r="A444" t="s">
-        <v>1005</v>
-      </c>
-      <c r="B444" t="s">
-        <v>1010</v>
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="445" spans="1:2">
+      <c r="A445" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B445" t="s">
+        <v>1003</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>1023</v>
+        <v>1013</v>
       </c>
       <c r="B446" t="s">
-        <v>1016</v>
-      </c>
-    </row>
-    <row r="447" spans="1:2">
-      <c r="A447" t="s">
-        <v>1024</v>
-      </c>
-      <c r="B447" t="s">
-        <v>1017</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>1025</v>
+        <v>1008</v>
       </c>
       <c r="B448" t="s">
-        <v>1018</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>1071</v>
+        <v>1009</v>
       </c>
       <c r="B449" t="s">
-        <v>1019</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>1026</v>
+        <v>1005</v>
       </c>
       <c r="B450" t="s">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="451" spans="1:2">
-      <c r="A451" t="s">
-        <v>1027</v>
-      </c>
-      <c r="B451" t="s">
-        <v>1021</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>1028</v>
+        <v>1023</v>
       </c>
       <c r="B452" t="s">
-        <v>1022</v>
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="453" spans="1:2">
+      <c r="A453" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B453" t="s">
+        <v>1017</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>1040</v>
+        <v>1025</v>
       </c>
       <c r="B454" t="s">
-        <v>1034</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>1045</v>
+        <v>1071</v>
       </c>
       <c r="B455" t="s">
-        <v>1035</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>1041</v>
+        <v>1026</v>
       </c>
       <c r="B456" t="s">
-        <v>1036</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>1042</v>
+        <v>1027</v>
       </c>
       <c r="B457" t="s">
-        <v>1037</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
-        <v>1044</v>
+        <v>1028</v>
       </c>
       <c r="B458" t="s">
-        <v>1038</v>
-      </c>
-    </row>
-    <row r="459" spans="1:2">
-      <c r="A459" t="s">
-        <v>1043</v>
-      </c>
-      <c r="B459" t="s">
-        <v>1039</v>
+        <v>1022</v>
+      </c>
+    </row>
+    <row r="460" spans="1:2">
+      <c r="A460" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B460" t="s">
+        <v>1034</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>1058</v>
+        <v>1045</v>
       </c>
       <c r="B461" t="s">
-        <v>1046</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>1053</v>
+        <v>1041</v>
       </c>
       <c r="B462" t="s">
-        <v>1047</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1054</v>
+        <v>1042</v>
       </c>
       <c r="B463" t="s">
-        <v>1048</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1055</v>
+        <v>1044</v>
       </c>
       <c r="B464" t="s">
-        <v>1049</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1056</v>
+        <v>1043</v>
       </c>
       <c r="B465" t="s">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="466" spans="1:2">
-      <c r="A466" t="s">
-        <v>1057</v>
-      </c>
-      <c r="B466" t="s">
-        <v>1051</v>
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="467" spans="1:2">
+      <c r="A467" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B467" t="s">
+        <v>1046</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1059</v>
+        <v>1053</v>
       </c>
       <c r="B468" t="s">
-        <v>1060</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1065</v>
+        <v>1054</v>
       </c>
       <c r="B469" t="s">
-        <v>1061</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1066</v>
+        <v>1055</v>
       </c>
       <c r="B470" t="s">
-        <v>1062</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1067</v>
+        <v>1056</v>
       </c>
       <c r="B471" t="s">
-        <v>1063</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2">
+      <c r="A474" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B474" t="s">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2">
+      <c r="A475" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B475" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B476" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2">
+      <c r="A477" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B477" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="478" spans="1:2">
+      <c r="A478" t="s">
         <v>1068</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B478" t="s">
         <v>1064</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A442:A443 A439:A440 A425:A434 A436:A437">
+  <conditionalFormatting sqref="A448:A449 A445:A446 A431:A440 A442:A443">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates for AS, IAQ logic
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C792B698-9E05-43A4-B382-EE789041A5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08DEABB-C2A6-4DB8-B8F3-06EB33734E24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3780" yWindow="3015" windowWidth="21060" windowHeight="9615" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3297,7 +3297,7 @@
     <t>Payment Generation Date listed on the Child Support Payment History does not match the End Date listed on Child Support Calcs. </t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updates with all the invalid findings in User story 2658
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519B1CAF-F499-4E28-8F70-41AB4C7667E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D10BA5B-67B4-41AE-8920-6740B6B7A51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4455" yWindow="3720" windowWidth="21510" windowHeight="9900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3297,7 +3297,7 @@
     <t>Payment Generation Date listed on the Child Support Payment History does not match the End Date listed on Child Support Calcs. </t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updates to CSS to fix Student Status check
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D10BA5B-67B4-41AE-8920-6740B6B7A51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FF775A-B8BC-42F5-85BF-0E2C18FC45C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4455" yWindow="3720" windowWidth="21510" windowHeight="9900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="300" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
MID - TX added
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FF775A-B8BC-42F5-85BF-0E2C18FC45C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB9088E-40C8-41A7-87AB-7AA7E94E6A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="300" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1317" uniqueCount="1086">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1319" uniqueCount="1088">
   <si>
     <t>Name</t>
   </si>
@@ -3297,7 +3297,13 @@
     <t>Payment Generation Date listed on the Child Support Payment History does not match the End Date listed on Child Support Calcs. </t>
   </si>
   <si>
-    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>MID_VeteranCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Veteran of the United States Military question was not documented appropriately. </t>
   </si>
 </sst>
 </file>
@@ -8101,7 +8107,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C478"/>
+  <dimension ref="A1:C479"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8551,18 +8557,18 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>495</v>
+        <v>720</v>
       </c>
       <c r="B55" t="s">
-        <v>607</v>
+        <v>721</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>720</v>
+        <v>1086</v>
       </c>
       <c r="B56" t="s">
-        <v>721</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -8576,31 +8582,28 @@
         <v>629</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
-      <c r="A59" t="s">
-        <v>183</v>
-      </c>
-      <c r="B59" t="s">
-        <v>536</v>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>495</v>
+      </c>
+      <c r="B58" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>106</v>
+        <v>183</v>
       </c>
       <c r="B60" t="s">
-        <v>107</v>
-      </c>
-      <c r="C60" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B61" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C61" t="s">
         <v>533</v>
@@ -8608,10 +8611,10 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C62" t="s">
         <v>533</v>
@@ -8619,10 +8622,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B63" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C63" t="s">
         <v>533</v>
@@ -8630,10 +8633,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B64" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C64" t="s">
         <v>533</v>
@@ -8641,10 +8644,10 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B65" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C65" t="s">
         <v>533</v>
@@ -8652,123 +8655,123 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B66" t="s">
-        <v>111</v>
+        <v>110</v>
+      </c>
+      <c r="C66" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>201</v>
+        <v>115</v>
       </c>
       <c r="B67" t="s">
-        <v>722</v>
+        <v>111</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B68" t="s">
-        <v>723</v>
-      </c>
-      <c r="C68" t="s">
-        <v>533</v>
+        <v>722</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>524</v>
+        <v>202</v>
       </c>
       <c r="B69" t="s">
-        <v>724</v>
+        <v>723</v>
+      </c>
+      <c r="C69" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>497</v>
+        <v>524</v>
       </c>
       <c r="B70" t="s">
-        <v>498</v>
+        <v>724</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="B71" t="s">
-        <v>725</v>
+        <v>498</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="B72" t="s">
-        <v>608</v>
+        <v>725</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
+        <v>494</v>
+      </c>
+      <c r="B73" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
         <v>680</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>679</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C74" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" t="s">
-        <v>157</v>
-      </c>
-      <c r="B75" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>121</v>
+        <v>157</v>
       </c>
       <c r="B76" t="s">
-        <v>537</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B77" t="s">
-        <v>122</v>
+        <v>537</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>576</v>
+        <v>123</v>
       </c>
       <c r="B78" t="s">
-        <v>577</v>
+        <v>122</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>690</v>
+        <v>576</v>
       </c>
       <c r="B79" t="s">
-        <v>691</v>
-      </c>
-      <c r="C79" t="s">
-        <v>629</v>
+        <v>577</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>710</v>
+        <v>690</v>
       </c>
       <c r="B80" t="s">
-        <v>711</v>
+        <v>691</v>
       </c>
       <c r="C80" t="s">
         <v>629</v>
@@ -8776,10 +8779,10 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B81" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C81" t="s">
         <v>629</v>
@@ -8787,10 +8790,10 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B82" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C82" t="s">
         <v>629</v>
@@ -8798,37 +8801,37 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
+        <v>708</v>
+      </c>
+      <c r="B83" t="s">
+        <v>713</v>
+      </c>
+      <c r="C83" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" t="s">
         <v>493</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B84" t="s">
         <v>609</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3">
-      <c r="A85" t="s">
-        <v>185</v>
-      </c>
-      <c r="B85" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>689</v>
+        <v>185</v>
       </c>
       <c r="B86" t="s">
-        <v>704</v>
-      </c>
-      <c r="C86" t="s">
-        <v>629</v>
+        <v>186</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B87" t="s">
-        <v>688</v>
+        <v>704</v>
       </c>
       <c r="C87" t="s">
         <v>629</v>
@@ -8836,80 +8839,80 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>124</v>
+        <v>687</v>
       </c>
       <c r="B88" t="s">
-        <v>126</v>
+        <v>688</v>
+      </c>
+      <c r="C88" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="B90" t="s">
-        <v>538</v>
+        <v>127</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B91" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B92" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B93" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B94" t="s">
-        <v>451</v>
-      </c>
-      <c r="C94" t="s">
-        <v>624</v>
+        <v>541</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B95" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C95" t="s">
-        <v>506</v>
+        <v>624</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B96" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C96" t="s">
         <v>506</v>
@@ -8917,48 +8920,48 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>578</v>
+        <v>143</v>
       </c>
       <c r="B97" t="s">
-        <v>579</v>
+        <v>454</v>
+      </c>
+      <c r="C97" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>654</v>
+        <v>578</v>
       </c>
       <c r="B98" t="s">
-        <v>655</v>
-      </c>
-      <c r="C98" t="s">
-        <v>629</v>
+        <v>579</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>924</v>
+        <v>654</v>
       </c>
       <c r="B99" t="s">
-        <v>925</v>
+        <v>655</v>
+      </c>
+      <c r="C99" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>681</v>
+        <v>924</v>
       </c>
       <c r="B100" t="s">
-        <v>682</v>
-      </c>
-      <c r="C100" t="s">
-        <v>629</v>
+        <v>925</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B101" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="C101" t="s">
         <v>629</v>
@@ -8966,10 +8969,10 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B102" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C102" t="s">
         <v>629</v>
@@ -8977,381 +8980,381 @@
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>492</v>
+        <v>686</v>
       </c>
       <c r="B103" t="s">
-        <v>610</v>
+        <v>685</v>
+      </c>
+      <c r="C103" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>920</v>
+        <v>492</v>
       </c>
       <c r="B104" t="s">
-        <v>921</v>
+        <v>610</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="B105" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="B106" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
+        <v>927</v>
+      </c>
+      <c r="B107" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" t="s">
         <v>929</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B108" t="s">
         <v>926</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3">
-      <c r="A109" t="s">
-        <v>146</v>
-      </c>
-      <c r="B109" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B110" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B111" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B112" t="s">
-        <v>525</v>
-      </c>
-      <c r="C112" t="s">
-        <v>628</v>
+        <v>151</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>627</v>
+        <v>144</v>
       </c>
       <c r="B113" t="s">
         <v>525</v>
       </c>
+      <c r="C113" t="s">
+        <v>628</v>
+      </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>145</v>
+        <v>627</v>
       </c>
       <c r="B114" t="s">
-        <v>128</v>
+        <v>525</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="B115" t="s">
-        <v>542</v>
+        <v>128</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B116" t="s">
-        <v>129</v>
+        <v>542</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>580</v>
+        <v>131</v>
       </c>
       <c r="B117" t="s">
-        <v>581</v>
+        <v>129</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
+        <v>580</v>
+      </c>
+      <c r="B118" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" t="s">
         <v>491</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B119" t="s">
         <v>611</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3">
-      <c r="A120" t="s">
-        <v>187</v>
-      </c>
-      <c r="B120" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="B121" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B122" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B123" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>740</v>
+        <v>133</v>
       </c>
       <c r="B124" t="s">
-        <v>739</v>
-      </c>
-      <c r="C124" t="s">
-        <v>629</v>
+        <v>154</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>135</v>
+        <v>740</v>
       </c>
       <c r="B125" t="s">
-        <v>155</v>
+        <v>739</v>
+      </c>
+      <c r="C125" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B126" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>571</v>
+        <v>136</v>
       </c>
       <c r="B127" t="s">
-        <v>632</v>
-      </c>
-      <c r="C127" t="s">
-        <v>636</v>
+        <v>156</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>582</v>
+        <v>571</v>
       </c>
       <c r="B128" t="s">
-        <v>583</v>
+        <v>632</v>
+      </c>
+      <c r="C128" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>656</v>
+        <v>582</v>
       </c>
       <c r="B129" t="s">
-        <v>657</v>
-      </c>
-      <c r="C129" t="s">
-        <v>629</v>
+        <v>583</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
+        <v>656</v>
+      </c>
+      <c r="B130" t="s">
+        <v>657</v>
+      </c>
+      <c r="C130" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" t="s">
         <v>490</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B131" t="s">
         <v>612</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" t="s">
-        <v>645</v>
-      </c>
-      <c r="B132" t="s">
-        <v>646</v>
-      </c>
-      <c r="C132" t="s">
-        <v>647</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="B133" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="C133" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
-      <c r="A135" t="s">
-        <v>158</v>
-      </c>
-      <c r="B135" t="s">
-        <v>162</v>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
+        <v>648</v>
+      </c>
+      <c r="B134" t="s">
+        <v>649</v>
+      </c>
+      <c r="C134" t="s">
+        <v>647</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B136" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B137" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B138" t="s">
-        <v>543</v>
+        <v>164</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>507</v>
+        <v>161</v>
       </c>
       <c r="B139" t="s">
-        <v>670</v>
-      </c>
-      <c r="C139" t="s">
-        <v>671</v>
+        <v>543</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>588</v>
+        <v>507</v>
       </c>
       <c r="B140" t="s">
-        <v>589</v>
+        <v>670</v>
+      </c>
+      <c r="C140" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
+        <v>588</v>
+      </c>
+      <c r="B141" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3">
+      <c r="A142" t="s">
         <v>489</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B142" t="s">
         <v>613</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" t="s">
-        <v>191</v>
-      </c>
-      <c r="B143" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="B144" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B145" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>584</v>
+        <v>166</v>
       </c>
       <c r="B146" t="s">
-        <v>585</v>
+        <v>168</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>488</v>
+        <v>584</v>
       </c>
       <c r="B147" t="s">
-        <v>614</v>
+        <v>585</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
+        <v>488</v>
+      </c>
+      <c r="B148" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" t="s">
         <v>658</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B149" t="s">
         <v>659</v>
       </c>
-      <c r="C148" t="s">
+      <c r="C149" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3">
-      <c r="A150" t="s">
-        <v>189</v>
-      </c>
-      <c r="B150" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B151" t="s">
-        <v>171</v>
-      </c>
-      <c r="C151" t="s">
-        <v>533</v>
+        <v>190</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B152" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C152" t="s">
         <v>533</v>
@@ -9359,10 +9362,10 @@
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B153" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C153" t="s">
         <v>533</v>
@@ -9370,75 +9373,75 @@
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="B154" t="s">
-        <v>199</v>
+        <v>173</v>
+      </c>
+      <c r="C154" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B155" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="B156" t="s">
-        <v>176</v>
-      </c>
-      <c r="C156" t="s">
-        <v>533</v>
+        <v>198</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>586</v>
+        <v>175</v>
       </c>
       <c r="B157" t="s">
-        <v>587</v>
+        <v>176</v>
+      </c>
+      <c r="C157" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
+        <v>586</v>
+      </c>
+      <c r="B158" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3">
+      <c r="A159" t="s">
         <v>477</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B159" t="s">
         <v>615</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3">
-      <c r="A160" t="s">
-        <v>593</v>
-      </c>
-      <c r="B160" t="s">
-        <v>896</v>
-      </c>
-      <c r="C160" t="s">
-        <v>594</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>661</v>
+        <v>593</v>
       </c>
       <c r="B161" t="s">
-        <v>662</v>
+        <v>896</v>
       </c>
       <c r="C161" t="s">
-        <v>629</v>
+        <v>594</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>753</v>
+        <v>661</v>
       </c>
       <c r="B162" t="s">
-        <v>897</v>
+        <v>662</v>
       </c>
       <c r="C162" t="s">
         <v>629</v>
@@ -9446,10 +9449,10 @@
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B163" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C163" t="s">
         <v>629</v>
@@ -9457,40 +9460,40 @@
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B164" t="s">
-        <v>736</v>
+        <v>898</v>
       </c>
       <c r="C164" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
-      <c r="A166" t="s">
-        <v>468</v>
-      </c>
-      <c r="B166" t="s">
-        <v>899</v>
+    <row r="165" spans="1:3">
+      <c r="A165" t="s">
+        <v>755</v>
+      </c>
+      <c r="B165" t="s">
+        <v>736</v>
+      </c>
+      <c r="C165" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>600</v>
+        <v>468</v>
       </c>
       <c r="B167" t="s">
-        <v>604</v>
-      </c>
-      <c r="C167" t="s">
-        <v>602</v>
+        <v>899</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B168" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C168" t="s">
         <v>602</v>
@@ -9498,150 +9501,150 @@
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>239</v>
+        <v>601</v>
       </c>
       <c r="B169" t="s">
-        <v>900</v>
+        <v>603</v>
       </c>
       <c r="C169" t="s">
-        <v>533</v>
+        <v>602</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B170" t="s">
-        <v>901</v>
+        <v>900</v>
+      </c>
+      <c r="C170" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="B171" t="s">
-        <v>902</v>
-      </c>
-      <c r="C171" t="s">
-        <v>591</v>
+        <v>901</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>719</v>
+        <v>248</v>
       </c>
       <c r="B172" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C172" t="s">
-        <v>629</v>
+        <v>591</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>242</v>
+        <v>719</v>
       </c>
       <c r="B173" t="s">
-        <v>241</v>
+        <v>903</v>
+      </c>
+      <c r="C173" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>458</v>
+        <v>242</v>
       </c>
       <c r="B174" t="s">
-        <v>467</v>
+        <v>241</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>243</v>
+        <v>458</v>
       </c>
       <c r="B175" t="s">
-        <v>904</v>
+        <v>467</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B176" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B177" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B178" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B179" t="s">
-        <v>827</v>
+        <v>907</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>279</v>
+        <v>247</v>
       </c>
       <c r="B180" t="s">
-        <v>904</v>
+        <v>827</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>306</v>
+        <v>279</v>
       </c>
       <c r="B181" t="s">
-        <v>307</v>
+        <v>904</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>596</v>
+        <v>306</v>
       </c>
       <c r="B182" t="s">
-        <v>597</v>
+        <v>307</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>638</v>
+        <v>596</v>
       </c>
       <c r="B183" t="s">
-        <v>828</v>
+        <v>597</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>705</v>
+        <v>638</v>
       </c>
       <c r="B184" t="s">
-        <v>706</v>
-      </c>
-      <c r="C184" t="s">
-        <v>629</v>
+        <v>828</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="B185" t="s">
-        <v>738</v>
+        <v>706</v>
       </c>
       <c r="C185" t="s">
         <v>629</v>
@@ -9649,803 +9652,803 @@
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>918</v>
+        <v>718</v>
       </c>
       <c r="B186" t="s">
-        <v>919</v>
+        <v>738</v>
+      </c>
+      <c r="C186" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
+        <v>918</v>
+      </c>
+      <c r="B187" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3">
+      <c r="A188" t="s">
         <v>476</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B188" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3">
-      <c r="A189" t="s">
-        <v>716</v>
-      </c>
-      <c r="B189" t="s">
-        <v>717</v>
-      </c>
-      <c r="C189" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>469</v>
+        <v>716</v>
       </c>
       <c r="B190" t="s">
-        <v>908</v>
+        <v>717</v>
+      </c>
+      <c r="C190" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
+        <v>469</v>
+      </c>
+      <c r="B191" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3">
+      <c r="A192" t="s">
         <v>249</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>909</v>
       </c>
-      <c r="C191" t="s">
+      <c r="C192" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A192" t="s">
+    <row r="193" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A193" t="s">
         <v>251</v>
       </c>
-      <c r="B192" t="s">
+      <c r="B193" t="s">
         <v>910</v>
       </c>
-      <c r="C192" t="s">
+      <c r="C193" t="s">
         <v>633</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3">
-      <c r="A193" t="s">
-        <v>250</v>
-      </c>
-      <c r="B193" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B194" t="s">
-        <v>252</v>
+        <v>867</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B195" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B196" t="s">
-        <v>256</v>
-      </c>
-      <c r="C196" t="s">
-        <v>599</v>
+        <v>255</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>459</v>
+        <v>257</v>
       </c>
       <c r="B197" t="s">
-        <v>515</v>
+        <v>256</v>
+      </c>
+      <c r="C197" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>258</v>
+        <v>459</v>
       </c>
       <c r="B198" t="s">
-        <v>870</v>
+        <v>515</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B199" t="s">
-        <v>260</v>
+        <v>870</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B200" t="s">
-        <v>871</v>
+        <v>260</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B201" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B202" t="s">
-        <v>911</v>
-      </c>
-      <c r="C202" t="s">
-        <v>599</v>
+        <v>872</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B203" t="s">
-        <v>873</v>
+        <v>911</v>
+      </c>
+      <c r="C203" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B204" t="s">
-        <v>912</v>
-      </c>
-      <c r="C204" t="s">
-        <v>599</v>
+        <v>873</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B205" t="s">
-        <v>874</v>
+        <v>912</v>
+      </c>
+      <c r="C205" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B206" t="s">
-        <v>277</v>
+        <v>874</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B207" t="s">
-        <v>904</v>
+        <v>277</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B208" t="s">
-        <v>281</v>
+        <v>904</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>639</v>
+        <v>280</v>
       </c>
       <c r="B209" t="s">
-        <v>828</v>
+        <v>281</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>487</v>
+        <v>639</v>
       </c>
       <c r="B210" t="s">
-        <v>617</v>
+        <v>828</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
+        <v>487</v>
+      </c>
+      <c r="B211" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3">
+      <c r="A212" t="s">
         <v>634</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B212" t="s">
         <v>635</v>
       </c>
-      <c r="C211" t="s">
+      <c r="C212" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="213" spans="1:3">
-      <c r="A213" t="s">
-        <v>470</v>
-      </c>
-      <c r="B213" t="s">
-        <v>829</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="B214" t="s">
-        <v>516</v>
+        <v>829</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>274</v>
+        <v>460</v>
       </c>
       <c r="B215" t="s">
-        <v>830</v>
+        <v>516</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B216" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="B217" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B218" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B219" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>640</v>
+        <v>284</v>
       </c>
       <c r="B220" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
+        <v>640</v>
+      </c>
+      <c r="B221" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3">
+      <c r="A222" t="s">
         <v>486</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B222" t="s">
         <v>618</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3">
-      <c r="A223" t="s">
-        <v>471</v>
-      </c>
-      <c r="B223" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="B224" t="s">
-        <v>517</v>
+        <v>821</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>287</v>
+        <v>461</v>
       </c>
       <c r="B225" t="s">
-        <v>822</v>
+        <v>517</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B226" t="s">
-        <v>290</v>
+        <v>822</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B227" t="s">
-        <v>823</v>
+        <v>290</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B228" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B229" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B230" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B231" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>641</v>
+        <v>294</v>
       </c>
       <c r="B232" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
+        <v>641</v>
+      </c>
+      <c r="B233" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3">
+      <c r="A234" t="s">
         <v>485</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B234" t="s">
         <v>619</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3">
-      <c r="A235" t="s">
-        <v>472</v>
-      </c>
-      <c r="B235" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>456</v>
+        <v>472</v>
       </c>
       <c r="B236" t="s">
-        <v>300</v>
-      </c>
-      <c r="C236" t="s">
-        <v>533</v>
+        <v>913</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="B237" t="s">
-        <v>518</v>
+        <v>300</v>
+      </c>
+      <c r="C237" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>298</v>
+        <v>462</v>
       </c>
       <c r="B238" t="s">
-        <v>914</v>
-      </c>
-      <c r="C238" t="s">
-        <v>533</v>
+        <v>518</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B239" t="s">
-        <v>894</v>
+        <v>914</v>
+      </c>
+      <c r="C239" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>455</v>
+        <v>299</v>
       </c>
       <c r="B240" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>301</v>
+        <v>455</v>
       </c>
       <c r="B241" t="s">
-        <v>904</v>
+        <v>895</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B242" t="s">
-        <v>915</v>
+        <v>904</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B243" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B244" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B245" t="s">
-        <v>827</v>
+        <v>917</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>642</v>
+        <v>305</v>
       </c>
       <c r="B246" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
+        <v>642</v>
+      </c>
+      <c r="B247" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3">
+      <c r="A248" t="s">
         <v>484</v>
       </c>
-      <c r="B247" t="s">
+      <c r="B248" t="s">
         <v>620</v>
-      </c>
-    </row>
-    <row r="249" spans="1:3">
-      <c r="A249" t="s">
-        <v>676</v>
-      </c>
-      <c r="B249" t="s">
-        <v>677</v>
-      </c>
-      <c r="C249" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>501</v>
+        <v>676</v>
       </c>
       <c r="B250" t="s">
-        <v>504</v>
+        <v>677</v>
       </c>
       <c r="C250" t="s">
-        <v>531</v>
+        <v>629</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B251" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C251" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>530</v>
+        <v>502</v>
       </c>
       <c r="B252" t="s">
-        <v>544</v>
+        <v>503</v>
+      </c>
+      <c r="C252" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>322</v>
+        <v>530</v>
       </c>
       <c r="B253" t="s">
-        <v>308</v>
+        <v>544</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B254" t="s">
-        <v>309</v>
-      </c>
-      <c r="C254" t="s">
-        <v>533</v>
+        <v>308</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>463</v>
+        <v>323</v>
       </c>
       <c r="B255" t="s">
-        <v>519</v>
+        <v>309</v>
+      </c>
+      <c r="C255" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>324</v>
+        <v>463</v>
       </c>
       <c r="B256" t="s">
-        <v>310</v>
+        <v>519</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B257" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B258" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B259" t="s">
-        <v>313</v>
-      </c>
-      <c r="C259" t="s">
-        <v>533</v>
+        <v>312</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B260" t="s">
-        <v>314</v>
+        <v>313</v>
+      </c>
+      <c r="C260" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B261" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B262" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B263" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B264" t="s">
-        <v>318</v>
-      </c>
-      <c r="C264" t="s">
-        <v>533</v>
+        <v>317</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B265" t="s">
-        <v>319</v>
+        <v>318</v>
+      </c>
+      <c r="C265" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B266" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B267" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
+        <v>335</v>
+      </c>
+      <c r="B268" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3">
+      <c r="A269" t="s">
         <v>483</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B269" t="s">
         <v>605</v>
-      </c>
-    </row>
-    <row r="270" spans="1:3">
-      <c r="A270" t="s">
-        <v>548</v>
-      </c>
-      <c r="B270" t="s">
-        <v>549</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>342</v>
+        <v>548</v>
       </c>
       <c r="B271" t="s">
-        <v>360</v>
+        <v>549</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B272" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B273" t="s">
-        <v>358</v>
-      </c>
-      <c r="C273" t="s">
-        <v>533</v>
+        <v>357</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>464</v>
+        <v>344</v>
       </c>
       <c r="B274" t="s">
-        <v>520</v>
+        <v>358</v>
+      </c>
+      <c r="C274" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>361</v>
+        <v>464</v>
       </c>
       <c r="B275" t="s">
-        <v>359</v>
-      </c>
-      <c r="C275" t="s">
-        <v>533</v>
+        <v>520</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="B276" t="s">
-        <v>351</v>
+        <v>359</v>
+      </c>
+      <c r="C276" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>362</v>
+        <v>345</v>
       </c>
       <c r="B277" t="s">
-        <v>352</v>
-      </c>
-      <c r="C277" t="s">
-        <v>510</v>
+        <v>351</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="B278" t="s">
-        <v>353</v>
+        <v>352</v>
+      </c>
+      <c r="C278" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B279" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B280" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B281" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B282" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>1079</v>
+        <v>350</v>
       </c>
       <c r="B283" t="s">
-        <v>1080</v>
-      </c>
-      <c r="C283" t="s">
-        <v>1074</v>
+        <v>353</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="B284" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="C284" t="s">
         <v>1074</v>
@@ -10453,10 +10456,10 @@
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="B285" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="C285" t="s">
         <v>1074</v>
@@ -10464,40 +10467,40 @@
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B286" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C286" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3">
+      <c r="A287" t="s">
         <v>482</v>
       </c>
-      <c r="B286" t="s">
+      <c r="B287" t="s">
         <v>621</v>
-      </c>
-    </row>
-    <row r="288" spans="1:3">
-      <c r="A288" t="s">
-        <v>678</v>
-      </c>
-      <c r="B288" t="s">
-        <v>697</v>
-      </c>
-      <c r="C288" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>1072</v>
+        <v>678</v>
       </c>
       <c r="B289" t="s">
-        <v>1073</v>
+        <v>697</v>
       </c>
       <c r="C289" t="s">
-        <v>1074</v>
+        <v>629</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="B290" t="s">
-        <v>1076</v>
+        <v>1073</v>
       </c>
       <c r="C290" t="s">
         <v>1074</v>
@@ -10505,78 +10508,78 @@
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="B291" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C291" t="s">
         <v>1074</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
-      <c r="A293" t="s">
-        <v>674</v>
-      </c>
-      <c r="B293" t="s">
-        <v>675</v>
-      </c>
-      <c r="C293" t="s">
-        <v>629</v>
+    <row r="292" spans="1:3">
+      <c r="A292" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B292" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C292" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>473</v>
+        <v>674</v>
       </c>
       <c r="B294" t="s">
-        <v>474</v>
+        <v>675</v>
+      </c>
+      <c r="C294" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>368</v>
+        <v>473</v>
       </c>
       <c r="B295" t="s">
-        <v>379</v>
+        <v>474</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B296" t="s">
-        <v>380</v>
-      </c>
-      <c r="C296" t="s">
-        <v>533</v>
+        <v>379</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>521</v>
+        <v>369</v>
       </c>
       <c r="B297" t="s">
-        <v>522</v>
+        <v>380</v>
+      </c>
+      <c r="C297" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>370</v>
+        <v>521</v>
       </c>
       <c r="B298" t="s">
-        <v>381</v>
-      </c>
-      <c r="C298" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B299" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C299" t="s">
         <v>533</v>
@@ -10584,139 +10587,139 @@
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B300" t="s">
-        <v>534</v>
+        <v>382</v>
+      </c>
+      <c r="C300" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B301" t="s">
-        <v>383</v>
+        <v>534</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B302" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B303" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B304" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B305" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B306" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>733</v>
+        <v>378</v>
       </c>
       <c r="B307" t="s">
-        <v>734</v>
-      </c>
-      <c r="C307" t="s">
-        <v>629</v>
+        <v>388</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>480</v>
+        <v>733</v>
       </c>
       <c r="B308" t="s">
-        <v>622</v>
+        <v>734</v>
+      </c>
+      <c r="C308" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
+        <v>480</v>
+      </c>
+      <c r="B309" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3">
+      <c r="A310" t="s">
         <v>557</v>
       </c>
-      <c r="B309" t="s">
+      <c r="B310" t="s">
         <v>558</v>
-      </c>
-    </row>
-    <row r="311" spans="1:3">
-      <c r="A311" t="s">
-        <v>475</v>
-      </c>
-      <c r="B311" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>395</v>
+        <v>475</v>
       </c>
       <c r="B312" t="s">
-        <v>406</v>
+        <v>474</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B313" t="s">
-        <v>407</v>
-      </c>
-      <c r="C313" t="s">
-        <v>533</v>
+        <v>406</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>465</v>
+        <v>396</v>
       </c>
       <c r="B314" t="s">
-        <v>523</v>
+        <v>407</v>
+      </c>
+      <c r="C314" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>397</v>
+        <v>465</v>
       </c>
       <c r="B315" t="s">
-        <v>408</v>
-      </c>
-      <c r="C315" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B316" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C316" t="s">
         <v>533</v>
@@ -10724,1178 +10727,1189 @@
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B317" t="s">
-        <v>535</v>
+        <v>409</v>
+      </c>
+      <c r="C317" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B318" t="s">
-        <v>383</v>
+        <v>535</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B319" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B320" t="s">
-        <v>410</v>
+        <v>384</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B321" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B322" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B323" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>479</v>
+        <v>405</v>
       </c>
       <c r="B324" t="s">
-        <v>622</v>
+        <v>388</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
+        <v>479</v>
+      </c>
+      <c r="B325" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3">
+      <c r="A326" t="s">
         <v>564</v>
       </c>
-      <c r="B325" t="s">
+      <c r="B326" t="s">
         <v>558</v>
-      </c>
-    </row>
-    <row r="327" spans="1:3">
-      <c r="A327" t="s">
-        <v>672</v>
-      </c>
-      <c r="B327" t="s">
-        <v>673</v>
-      </c>
-      <c r="C327" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>389</v>
+        <v>672</v>
       </c>
       <c r="B328" t="s">
-        <v>565</v>
+        <v>673</v>
+      </c>
+      <c r="C328" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B329" t="s">
-        <v>566</v>
-      </c>
-      <c r="C329" t="s">
-        <v>533</v>
+        <v>565</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>466</v>
+        <v>390</v>
       </c>
       <c r="B330" t="s">
-        <v>567</v>
+        <v>566</v>
+      </c>
+      <c r="C330" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>391</v>
+        <v>466</v>
       </c>
       <c r="B331" t="s">
-        <v>592</v>
+        <v>567</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B332" t="s">
-        <v>568</v>
+        <v>592</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B333" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
+        <v>393</v>
+      </c>
+      <c r="B334" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3">
+      <c r="A335" t="s">
         <v>478</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B335" t="s">
         <v>623</v>
-      </c>
-    </row>
-    <row r="336" spans="1:3">
-      <c r="A336" t="s">
-        <v>749</v>
-      </c>
-      <c r="B336" t="s">
-        <v>750</v>
-      </c>
-      <c r="C336" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="B337" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C337" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="339" spans="1:3">
-      <c r="A339" t="s">
-        <v>757</v>
-      </c>
-      <c r="B339" t="s">
-        <v>758</v>
+    <row r="338" spans="1:3">
+      <c r="A338" t="s">
+        <v>751</v>
+      </c>
+      <c r="B338" t="s">
+        <v>752</v>
+      </c>
+      <c r="C338" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="340" spans="1:3">
       <c r="A340" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B340" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="B341" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B342" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B343" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B344" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B345" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B346" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B347" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B348" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B349" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="B350" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="B351" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B352" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="B353" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B354" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="B355" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
+        <v>789</v>
+      </c>
+      <c r="B356" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" t="s">
         <v>791</v>
       </c>
-      <c r="B356" t="s">
+      <c r="B357" t="s">
         <v>792</v>
-      </c>
-    </row>
-    <row r="358" spans="1:2">
-      <c r="A358" t="s">
-        <v>793</v>
-      </c>
-      <c r="B358" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="B359" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="B360" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="B361" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="B362" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="B363" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="B364" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B365" t="s">
-        <v>321</v>
+        <v>806</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B366" t="s">
-        <v>809</v>
+        <v>321</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="B367" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="B368" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
+        <v>812</v>
+      </c>
+      <c r="B369" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" t="s">
         <v>814</v>
       </c>
-      <c r="B369" t="s">
+      <c r="B370" t="s">
         <v>815</v>
-      </c>
-    </row>
-    <row r="371" spans="1:2">
-      <c r="A371" t="s">
-        <v>816</v>
-      </c>
-      <c r="B371" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B372" t="s">
-        <v>818</v>
+        <v>314</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="B373" t="s">
-        <v>316</v>
+        <v>818</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
+        <v>819</v>
+      </c>
+      <c r="B374" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" t="s">
         <v>820</v>
       </c>
-      <c r="B374" t="s">
+      <c r="B375" t="s">
         <v>317</v>
-      </c>
-    </row>
-    <row r="376" spans="1:2">
-      <c r="A376" t="s">
-        <v>845</v>
-      </c>
-      <c r="B376" t="s">
-        <v>846</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B377" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>837</v>
+        <v>844</v>
       </c>
       <c r="B378" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="B379" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B380" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
+        <v>836</v>
+      </c>
+      <c r="B381" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" t="s">
         <v>842</v>
       </c>
-      <c r="B381" t="s">
+      <c r="B382" t="s">
         <v>841</v>
-      </c>
-    </row>
-    <row r="383" spans="1:2">
-      <c r="A383" t="s">
-        <v>849</v>
-      </c>
-      <c r="B383" t="s">
-        <v>854</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="B384" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="B385" t="s">
-        <v>838</v>
+        <v>855</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B386" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B387" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
+        <v>852</v>
+      </c>
+      <c r="B388" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" t="s">
         <v>853</v>
       </c>
-      <c r="B388" t="s">
+      <c r="B389" t="s">
         <v>856</v>
-      </c>
-    </row>
-    <row r="390" spans="1:2">
-      <c r="A390" t="s">
-        <v>862</v>
-      </c>
-      <c r="B390" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B391" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="B392" t="s">
-        <v>717</v>
+        <v>865</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="B393" t="s">
-        <v>867</v>
+        <v>717</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>875</v>
+        <v>868</v>
       </c>
       <c r="B394" t="s">
-        <v>252</v>
+        <v>867</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B395" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B396" t="s">
-        <v>869</v>
+        <v>255</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="B397" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B398" t="s">
-        <v>260</v>
+        <v>870</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B399" t="s">
-        <v>871</v>
+        <v>260</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B400" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B401" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B402" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B403" t="s">
-        <v>277</v>
+        <v>874</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B404" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B405" t="s">
-        <v>828</v>
+        <v>281</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>879</v>
+        <v>888</v>
       </c>
       <c r="B406" t="s">
-        <v>635</v>
+        <v>828</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
+        <v>879</v>
+      </c>
+      <c r="B407" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2">
+      <c r="A408" t="s">
         <v>878</v>
       </c>
-      <c r="B407" t="s">
+      <c r="B408" t="s">
         <v>617</v>
-      </c>
-    </row>
-    <row r="409" spans="1:2">
-      <c r="A409" t="s">
-        <v>953</v>
-      </c>
-      <c r="B409" t="s">
-        <v>932</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>972</v>
+        <v>953</v>
       </c>
       <c r="B410" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B411" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B412" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="B413" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B414" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B415" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B416" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B417" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B418" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="B419" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>973</v>
+        <v>963</v>
       </c>
       <c r="B420" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>962</v>
+        <v>973</v>
       </c>
       <c r="B421" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B422" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B423" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="B424" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B425" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B426" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="B427" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B428" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
+        <v>955</v>
+      </c>
+      <c r="B429" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2">
+      <c r="A430" t="s">
         <v>954</v>
       </c>
-      <c r="B429" t="s">
+      <c r="B430" t="s">
         <v>952</v>
-      </c>
-    </row>
-    <row r="431" spans="1:2">
-      <c r="A431" t="s">
-        <v>995</v>
-      </c>
-      <c r="B431" t="s">
-        <v>976</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>986</v>
+        <v>995</v>
       </c>
       <c r="B432" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B433" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B434" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>991</v>
+        <v>988</v>
       </c>
       <c r="B435" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
       <c r="B436" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="B437" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="B438" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="B439" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
+        <v>994</v>
+      </c>
+      <c r="B440" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2">
+      <c r="A441" t="s">
         <v>993</v>
       </c>
-      <c r="B440" t="s">
+      <c r="B441" t="s">
         <v>985</v>
-      </c>
-    </row>
-    <row r="442" spans="1:2">
-      <c r="A442" t="s">
-        <v>1000</v>
-      </c>
-      <c r="B442" t="s">
-        <v>1002</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" t="s">
         <v>1011</v>
       </c>
-      <c r="B443" t="s">
+      <c r="B444" t="s">
         <v>1012</v>
-      </c>
-    </row>
-    <row r="445" spans="1:2">
-      <c r="A445" t="s">
-        <v>1001</v>
-      </c>
-      <c r="B445" t="s">
-        <v>1003</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2">
+      <c r="A447" t="s">
         <v>1013</v>
       </c>
-      <c r="B446" t="s">
+      <c r="B447" t="s">
         <v>1014</v>
-      </c>
-    </row>
-    <row r="448" spans="1:2">
-      <c r="A448" t="s">
-        <v>1008</v>
-      </c>
-      <c r="B448" t="s">
-        <v>1006</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B449" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" t="s">
         <v>1005</v>
       </c>
-      <c r="B450" t="s">
+      <c r="B451" t="s">
         <v>1010</v>
-      </c>
-    </row>
-    <row r="452" spans="1:2">
-      <c r="A452" t="s">
-        <v>1023</v>
-      </c>
-      <c r="B452" t="s">
-        <v>1016</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B453" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B454" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>1071</v>
+        <v>1025</v>
       </c>
       <c r="B455" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>1026</v>
+        <v>1071</v>
       </c>
       <c r="B456" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B457" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" t="s">
         <v>1028</v>
       </c>
-      <c r="B458" t="s">
+      <c r="B459" t="s">
         <v>1022</v>
-      </c>
-    </row>
-    <row r="460" spans="1:2">
-      <c r="A460" t="s">
-        <v>1040</v>
-      </c>
-      <c r="B460" t="s">
-        <v>1034</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>1045</v>
+        <v>1040</v>
       </c>
       <c r="B461" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="B462" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B463" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="B464" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B465" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" t="s">
         <v>1043</v>
       </c>
-      <c r="B465" t="s">
+      <c r="B466" t="s">
         <v>1039</v>
-      </c>
-    </row>
-    <row r="467" spans="1:2">
-      <c r="A467" t="s">
-        <v>1058</v>
-      </c>
-      <c r="B467" t="s">
-        <v>1046</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="B468" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B469" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B470" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B471" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" t="s">
         <v>1057</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B473" t="s">
         <v>1051</v>
-      </c>
-    </row>
-    <row r="474" spans="1:2">
-      <c r="A474" t="s">
-        <v>1059</v>
-      </c>
-      <c r="B474" t="s">
-        <v>1060</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
-        <v>1065</v>
+        <v>1059</v>
       </c>
       <c r="B475" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B476" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B477" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B478" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="479" spans="1:2">
+      <c r="A479" t="s">
         <v>1068</v>
       </c>
-      <c r="B478" t="s">
+      <c r="B479" t="s">
         <v>1064</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A448:A449 A445:A446 A431:A440 A442:A443">
+  <conditionalFormatting sqref="A449:A450 A446:A447 A432:A441 A443:A444">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates to Raluca's latest changes for MID TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FF775A-B8BC-42F5-85BF-0E2C18FC45C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB9088E-40C8-41A7-87AB-7AA7E94E6A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="300" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1317" uniqueCount="1086">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1319" uniqueCount="1088">
   <si>
     <t>Name</t>
   </si>
@@ -3297,7 +3297,13 @@
     <t>Payment Generation Date listed on the Child Support Payment History does not match the End Date listed on Child Support Calcs. </t>
   </si>
   <si>
-    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>MID_VeteranCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Veteran of the United States Military question was not documented appropriately. </t>
   </si>
 </sst>
 </file>
@@ -8101,7 +8107,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C478"/>
+  <dimension ref="A1:C479"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8551,18 +8557,18 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>495</v>
+        <v>720</v>
       </c>
       <c r="B55" t="s">
-        <v>607</v>
+        <v>721</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>720</v>
+        <v>1086</v>
       </c>
       <c r="B56" t="s">
-        <v>721</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -8576,31 +8582,28 @@
         <v>629</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
-      <c r="A59" t="s">
-        <v>183</v>
-      </c>
-      <c r="B59" t="s">
-        <v>536</v>
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
+        <v>495</v>
+      </c>
+      <c r="B58" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>106</v>
+        <v>183</v>
       </c>
       <c r="B60" t="s">
-        <v>107</v>
-      </c>
-      <c r="C60" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B61" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C61" t="s">
         <v>533</v>
@@ -8608,10 +8611,10 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C62" t="s">
         <v>533</v>
@@ -8619,10 +8622,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B63" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C63" t="s">
         <v>533</v>
@@ -8630,10 +8633,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B64" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C64" t="s">
         <v>533</v>
@@ -8641,10 +8644,10 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B65" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C65" t="s">
         <v>533</v>
@@ -8652,123 +8655,123 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B66" t="s">
-        <v>111</v>
+        <v>110</v>
+      </c>
+      <c r="C66" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>201</v>
+        <v>115</v>
       </c>
       <c r="B67" t="s">
-        <v>722</v>
+        <v>111</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B68" t="s">
-        <v>723</v>
-      </c>
-      <c r="C68" t="s">
-        <v>533</v>
+        <v>722</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>524</v>
+        <v>202</v>
       </c>
       <c r="B69" t="s">
-        <v>724</v>
+        <v>723</v>
+      </c>
+      <c r="C69" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>497</v>
+        <v>524</v>
       </c>
       <c r="B70" t="s">
-        <v>498</v>
+        <v>724</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="B71" t="s">
-        <v>725</v>
+        <v>498</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="B72" t="s">
-        <v>608</v>
+        <v>725</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
+        <v>494</v>
+      </c>
+      <c r="B73" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
         <v>680</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>679</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C74" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3">
-      <c r="A75" t="s">
-        <v>157</v>
-      </c>
-      <c r="B75" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>121</v>
+        <v>157</v>
       </c>
       <c r="B76" t="s">
-        <v>537</v>
+        <v>120</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B77" t="s">
-        <v>122</v>
+        <v>537</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>576</v>
+        <v>123</v>
       </c>
       <c r="B78" t="s">
-        <v>577</v>
+        <v>122</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>690</v>
+        <v>576</v>
       </c>
       <c r="B79" t="s">
-        <v>691</v>
-      </c>
-      <c r="C79" t="s">
-        <v>629</v>
+        <v>577</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>710</v>
+        <v>690</v>
       </c>
       <c r="B80" t="s">
-        <v>711</v>
+        <v>691</v>
       </c>
       <c r="C80" t="s">
         <v>629</v>
@@ -8776,10 +8779,10 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B81" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C81" t="s">
         <v>629</v>
@@ -8787,10 +8790,10 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B82" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C82" t="s">
         <v>629</v>
@@ -8798,37 +8801,37 @@
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
+        <v>708</v>
+      </c>
+      <c r="B83" t="s">
+        <v>713</v>
+      </c>
+      <c r="C83" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" t="s">
         <v>493</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B84" t="s">
         <v>609</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3">
-      <c r="A85" t="s">
-        <v>185</v>
-      </c>
-      <c r="B85" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>689</v>
+        <v>185</v>
       </c>
       <c r="B86" t="s">
-        <v>704</v>
-      </c>
-      <c r="C86" t="s">
-        <v>629</v>
+        <v>186</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B87" t="s">
-        <v>688</v>
+        <v>704</v>
       </c>
       <c r="C87" t="s">
         <v>629</v>
@@ -8836,80 +8839,80 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>124</v>
+        <v>687</v>
       </c>
       <c r="B88" t="s">
-        <v>126</v>
+        <v>688</v>
+      </c>
+      <c r="C88" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="B90" t="s">
-        <v>538</v>
+        <v>127</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B91" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B92" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B93" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B94" t="s">
-        <v>451</v>
-      </c>
-      <c r="C94" t="s">
-        <v>624</v>
+        <v>541</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B95" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C95" t="s">
-        <v>506</v>
+        <v>624</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B96" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C96" t="s">
         <v>506</v>
@@ -8917,48 +8920,48 @@
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>578</v>
+        <v>143</v>
       </c>
       <c r="B97" t="s">
-        <v>579</v>
+        <v>454</v>
+      </c>
+      <c r="C97" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>654</v>
+        <v>578</v>
       </c>
       <c r="B98" t="s">
-        <v>655</v>
-      </c>
-      <c r="C98" t="s">
-        <v>629</v>
+        <v>579</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>924</v>
+        <v>654</v>
       </c>
       <c r="B99" t="s">
-        <v>925</v>
+        <v>655</v>
+      </c>
+      <c r="C99" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>681</v>
+        <v>924</v>
       </c>
       <c r="B100" t="s">
-        <v>682</v>
-      </c>
-      <c r="C100" t="s">
-        <v>629</v>
+        <v>925</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="B101" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="C101" t="s">
         <v>629</v>
@@ -8966,10 +8969,10 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="B102" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="C102" t="s">
         <v>629</v>
@@ -8977,381 +8980,381 @@
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>492</v>
+        <v>686</v>
       </c>
       <c r="B103" t="s">
-        <v>610</v>
+        <v>685</v>
+      </c>
+      <c r="C103" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>920</v>
+        <v>492</v>
       </c>
       <c r="B104" t="s">
-        <v>921</v>
+        <v>610</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="B105" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="B106" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
+        <v>927</v>
+      </c>
+      <c r="B107" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3">
+      <c r="A108" t="s">
         <v>929</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B108" t="s">
         <v>926</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3">
-      <c r="A109" t="s">
-        <v>146</v>
-      </c>
-      <c r="B109" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B110" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B111" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B112" t="s">
-        <v>525</v>
-      </c>
-      <c r="C112" t="s">
-        <v>628</v>
+        <v>151</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>627</v>
+        <v>144</v>
       </c>
       <c r="B113" t="s">
         <v>525</v>
       </c>
+      <c r="C113" t="s">
+        <v>628</v>
+      </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>145</v>
+        <v>627</v>
       </c>
       <c r="B114" t="s">
-        <v>128</v>
+        <v>525</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="B115" t="s">
-        <v>542</v>
+        <v>128</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B116" t="s">
-        <v>129</v>
+        <v>542</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>580</v>
+        <v>131</v>
       </c>
       <c r="B117" t="s">
-        <v>581</v>
+        <v>129</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
+        <v>580</v>
+      </c>
+      <c r="B118" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3">
+      <c r="A119" t="s">
         <v>491</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B119" t="s">
         <v>611</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3">
-      <c r="A120" t="s">
-        <v>187</v>
-      </c>
-      <c r="B120" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="B121" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B122" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B123" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>740</v>
+        <v>133</v>
       </c>
       <c r="B124" t="s">
-        <v>739</v>
-      </c>
-      <c r="C124" t="s">
-        <v>629</v>
+        <v>154</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>135</v>
+        <v>740</v>
       </c>
       <c r="B125" t="s">
-        <v>155</v>
+        <v>739</v>
+      </c>
+      <c r="C125" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B126" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>571</v>
+        <v>136</v>
       </c>
       <c r="B127" t="s">
-        <v>632</v>
-      </c>
-      <c r="C127" t="s">
-        <v>636</v>
+        <v>156</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>582</v>
+        <v>571</v>
       </c>
       <c r="B128" t="s">
-        <v>583</v>
+        <v>632</v>
+      </c>
+      <c r="C128" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>656</v>
+        <v>582</v>
       </c>
       <c r="B129" t="s">
-        <v>657</v>
-      </c>
-      <c r="C129" t="s">
-        <v>629</v>
+        <v>583</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
+        <v>656</v>
+      </c>
+      <c r="B130" t="s">
+        <v>657</v>
+      </c>
+      <c r="C130" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3">
+      <c r="A131" t="s">
         <v>490</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B131" t="s">
         <v>612</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3">
-      <c r="A132" t="s">
-        <v>645</v>
-      </c>
-      <c r="B132" t="s">
-        <v>646</v>
-      </c>
-      <c r="C132" t="s">
-        <v>647</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="B133" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="C133" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
-      <c r="A135" t="s">
-        <v>158</v>
-      </c>
-      <c r="B135" t="s">
-        <v>162</v>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
+        <v>648</v>
+      </c>
+      <c r="B134" t="s">
+        <v>649</v>
+      </c>
+      <c r="C134" t="s">
+        <v>647</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B136" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B137" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B138" t="s">
-        <v>543</v>
+        <v>164</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>507</v>
+        <v>161</v>
       </c>
       <c r="B139" t="s">
-        <v>670</v>
-      </c>
-      <c r="C139" t="s">
-        <v>671</v>
+        <v>543</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>588</v>
+        <v>507</v>
       </c>
       <c r="B140" t="s">
-        <v>589</v>
+        <v>670</v>
+      </c>
+      <c r="C140" t="s">
+        <v>671</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
+        <v>588</v>
+      </c>
+      <c r="B141" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3">
+      <c r="A142" t="s">
         <v>489</v>
       </c>
-      <c r="B141" t="s">
+      <c r="B142" t="s">
         <v>613</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3">
-      <c r="A143" t="s">
-        <v>191</v>
-      </c>
-      <c r="B143" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="B144" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B145" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>584</v>
+        <v>166</v>
       </c>
       <c r="B146" t="s">
-        <v>585</v>
+        <v>168</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>488</v>
+        <v>584</v>
       </c>
       <c r="B147" t="s">
-        <v>614</v>
+        <v>585</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
+        <v>488</v>
+      </c>
+      <c r="B148" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" t="s">
         <v>658</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B149" t="s">
         <v>659</v>
       </c>
-      <c r="C148" t="s">
+      <c r="C149" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3">
-      <c r="A150" t="s">
-        <v>189</v>
-      </c>
-      <c r="B150" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B151" t="s">
-        <v>171</v>
-      </c>
-      <c r="C151" t="s">
-        <v>533</v>
+        <v>190</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B152" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C152" t="s">
         <v>533</v>
@@ -9359,10 +9362,10 @@
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B153" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C153" t="s">
         <v>533</v>
@@ -9370,75 +9373,75 @@
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="B154" t="s">
-        <v>199</v>
+        <v>173</v>
+      </c>
+      <c r="C154" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B155" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="B156" t="s">
-        <v>176</v>
-      </c>
-      <c r="C156" t="s">
-        <v>533</v>
+        <v>198</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>586</v>
+        <v>175</v>
       </c>
       <c r="B157" t="s">
-        <v>587</v>
+        <v>176</v>
+      </c>
+      <c r="C157" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
+        <v>586</v>
+      </c>
+      <c r="B158" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3">
+      <c r="A159" t="s">
         <v>477</v>
       </c>
-      <c r="B158" t="s">
+      <c r="B159" t="s">
         <v>615</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3">
-      <c r="A160" t="s">
-        <v>593</v>
-      </c>
-      <c r="B160" t="s">
-        <v>896</v>
-      </c>
-      <c r="C160" t="s">
-        <v>594</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>661</v>
+        <v>593</v>
       </c>
       <c r="B161" t="s">
-        <v>662</v>
+        <v>896</v>
       </c>
       <c r="C161" t="s">
-        <v>629</v>
+        <v>594</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>753</v>
+        <v>661</v>
       </c>
       <c r="B162" t="s">
-        <v>897</v>
+        <v>662</v>
       </c>
       <c r="C162" t="s">
         <v>629</v>
@@ -9446,10 +9449,10 @@
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B163" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C163" t="s">
         <v>629</v>
@@ -9457,40 +9460,40 @@
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B164" t="s">
-        <v>736</v>
+        <v>898</v>
       </c>
       <c r="C164" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
-      <c r="A166" t="s">
-        <v>468</v>
-      </c>
-      <c r="B166" t="s">
-        <v>899</v>
+    <row r="165" spans="1:3">
+      <c r="A165" t="s">
+        <v>755</v>
+      </c>
+      <c r="B165" t="s">
+        <v>736</v>
+      </c>
+      <c r="C165" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>600</v>
+        <v>468</v>
       </c>
       <c r="B167" t="s">
-        <v>604</v>
-      </c>
-      <c r="C167" t="s">
-        <v>602</v>
+        <v>899</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B168" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C168" t="s">
         <v>602</v>
@@ -9498,150 +9501,150 @@
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>239</v>
+        <v>601</v>
       </c>
       <c r="B169" t="s">
-        <v>900</v>
+        <v>603</v>
       </c>
       <c r="C169" t="s">
-        <v>533</v>
+        <v>602</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B170" t="s">
-        <v>901</v>
+        <v>900</v>
+      </c>
+      <c r="C170" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="B171" t="s">
-        <v>902</v>
-      </c>
-      <c r="C171" t="s">
-        <v>591</v>
+        <v>901</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>719</v>
+        <v>248</v>
       </c>
       <c r="B172" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C172" t="s">
-        <v>629</v>
+        <v>591</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>242</v>
+        <v>719</v>
       </c>
       <c r="B173" t="s">
-        <v>241</v>
+        <v>903</v>
+      </c>
+      <c r="C173" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>458</v>
+        <v>242</v>
       </c>
       <c r="B174" t="s">
-        <v>467</v>
+        <v>241</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>243</v>
+        <v>458</v>
       </c>
       <c r="B175" t="s">
-        <v>904</v>
+        <v>467</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B176" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B177" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B178" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B179" t="s">
-        <v>827</v>
+        <v>907</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>279</v>
+        <v>247</v>
       </c>
       <c r="B180" t="s">
-        <v>904</v>
+        <v>827</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>306</v>
+        <v>279</v>
       </c>
       <c r="B181" t="s">
-        <v>307</v>
+        <v>904</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>596</v>
+        <v>306</v>
       </c>
       <c r="B182" t="s">
-        <v>597</v>
+        <v>307</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>638</v>
+        <v>596</v>
       </c>
       <c r="B183" t="s">
-        <v>828</v>
+        <v>597</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>705</v>
+        <v>638</v>
       </c>
       <c r="B184" t="s">
-        <v>706</v>
-      </c>
-      <c r="C184" t="s">
-        <v>629</v>
+        <v>828</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>718</v>
+        <v>705</v>
       </c>
       <c r="B185" t="s">
-        <v>738</v>
+        <v>706</v>
       </c>
       <c r="C185" t="s">
         <v>629</v>
@@ -9649,803 +9652,803 @@
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>918</v>
+        <v>718</v>
       </c>
       <c r="B186" t="s">
-        <v>919</v>
+        <v>738</v>
+      </c>
+      <c r="C186" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
+        <v>918</v>
+      </c>
+      <c r="B187" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3">
+      <c r="A188" t="s">
         <v>476</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B188" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3">
-      <c r="A189" t="s">
-        <v>716</v>
-      </c>
-      <c r="B189" t="s">
-        <v>717</v>
-      </c>
-      <c r="C189" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>469</v>
+        <v>716</v>
       </c>
       <c r="B190" t="s">
-        <v>908</v>
+        <v>717</v>
+      </c>
+      <c r="C190" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
+        <v>469</v>
+      </c>
+      <c r="B191" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3">
+      <c r="A192" t="s">
         <v>249</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>909</v>
       </c>
-      <c r="C191" t="s">
+      <c r="C192" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="192" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A192" t="s">
+    <row r="193" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A193" t="s">
         <v>251</v>
       </c>
-      <c r="B192" t="s">
+      <c r="B193" t="s">
         <v>910</v>
       </c>
-      <c r="C192" t="s">
+      <c r="C193" t="s">
         <v>633</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3">
-      <c r="A193" t="s">
-        <v>250</v>
-      </c>
-      <c r="B193" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B194" t="s">
-        <v>252</v>
+        <v>867</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B195" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B196" t="s">
-        <v>256</v>
-      </c>
-      <c r="C196" t="s">
-        <v>599</v>
+        <v>255</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>459</v>
+        <v>257</v>
       </c>
       <c r="B197" t="s">
-        <v>515</v>
+        <v>256</v>
+      </c>
+      <c r="C197" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>258</v>
+        <v>459</v>
       </c>
       <c r="B198" t="s">
-        <v>870</v>
+        <v>515</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B199" t="s">
-        <v>260</v>
+        <v>870</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B200" t="s">
-        <v>871</v>
+        <v>260</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B201" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B202" t="s">
-        <v>911</v>
-      </c>
-      <c r="C202" t="s">
-        <v>599</v>
+        <v>872</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B203" t="s">
-        <v>873</v>
+        <v>911</v>
+      </c>
+      <c r="C203" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B204" t="s">
-        <v>912</v>
-      </c>
-      <c r="C204" t="s">
-        <v>599</v>
+        <v>873</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B205" t="s">
-        <v>874</v>
+        <v>912</v>
+      </c>
+      <c r="C205" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B206" t="s">
-        <v>277</v>
+        <v>874</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B207" t="s">
-        <v>904</v>
+        <v>277</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B208" t="s">
-        <v>281</v>
+        <v>904</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>639</v>
+        <v>280</v>
       </c>
       <c r="B209" t="s">
-        <v>828</v>
+        <v>281</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>487</v>
+        <v>639</v>
       </c>
       <c r="B210" t="s">
-        <v>617</v>
+        <v>828</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
+        <v>487</v>
+      </c>
+      <c r="B211" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3">
+      <c r="A212" t="s">
         <v>634</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B212" t="s">
         <v>635</v>
       </c>
-      <c r="C211" t="s">
+      <c r="C212" t="s">
         <v>629</v>
-      </c>
-    </row>
-    <row r="213" spans="1:3">
-      <c r="A213" t="s">
-        <v>470</v>
-      </c>
-      <c r="B213" t="s">
-        <v>829</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="B214" t="s">
-        <v>516</v>
+        <v>829</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>274</v>
+        <v>460</v>
       </c>
       <c r="B215" t="s">
-        <v>830</v>
+        <v>516</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B216" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="B217" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B218" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B219" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>640</v>
+        <v>284</v>
       </c>
       <c r="B220" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
+        <v>640</v>
+      </c>
+      <c r="B221" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3">
+      <c r="A222" t="s">
         <v>486</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B222" t="s">
         <v>618</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3">
-      <c r="A223" t="s">
-        <v>471</v>
-      </c>
-      <c r="B223" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>461</v>
+        <v>471</v>
       </c>
       <c r="B224" t="s">
-        <v>517</v>
+        <v>821</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>287</v>
+        <v>461</v>
       </c>
       <c r="B225" t="s">
-        <v>822</v>
+        <v>517</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B226" t="s">
-        <v>290</v>
+        <v>822</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B227" t="s">
-        <v>823</v>
+        <v>290</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B228" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B229" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B230" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B231" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>641</v>
+        <v>294</v>
       </c>
       <c r="B232" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
+        <v>641</v>
+      </c>
+      <c r="B233" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3">
+      <c r="A234" t="s">
         <v>485</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B234" t="s">
         <v>619</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3">
-      <c r="A235" t="s">
-        <v>472</v>
-      </c>
-      <c r="B235" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>456</v>
+        <v>472</v>
       </c>
       <c r="B236" t="s">
-        <v>300</v>
-      </c>
-      <c r="C236" t="s">
-        <v>533</v>
+        <v>913</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>462</v>
+        <v>456</v>
       </c>
       <c r="B237" t="s">
-        <v>518</v>
+        <v>300</v>
+      </c>
+      <c r="C237" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>298</v>
+        <v>462</v>
       </c>
       <c r="B238" t="s">
-        <v>914</v>
-      </c>
-      <c r="C238" t="s">
-        <v>533</v>
+        <v>518</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B239" t="s">
-        <v>894</v>
+        <v>914</v>
+      </c>
+      <c r="C239" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>455</v>
+        <v>299</v>
       </c>
       <c r="B240" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>301</v>
+        <v>455</v>
       </c>
       <c r="B241" t="s">
-        <v>904</v>
+        <v>895</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B242" t="s">
-        <v>915</v>
+        <v>904</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B243" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B244" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B245" t="s">
-        <v>827</v>
+        <v>917</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>642</v>
+        <v>305</v>
       </c>
       <c r="B246" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
+        <v>642</v>
+      </c>
+      <c r="B247" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3">
+      <c r="A248" t="s">
         <v>484</v>
       </c>
-      <c r="B247" t="s">
+      <c r="B248" t="s">
         <v>620</v>
-      </c>
-    </row>
-    <row r="249" spans="1:3">
-      <c r="A249" t="s">
-        <v>676</v>
-      </c>
-      <c r="B249" t="s">
-        <v>677</v>
-      </c>
-      <c r="C249" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>501</v>
+        <v>676</v>
       </c>
       <c r="B250" t="s">
-        <v>504</v>
+        <v>677</v>
       </c>
       <c r="C250" t="s">
-        <v>531</v>
+        <v>629</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B251" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C251" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>530</v>
+        <v>502</v>
       </c>
       <c r="B252" t="s">
-        <v>544</v>
+        <v>503</v>
+      </c>
+      <c r="C252" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>322</v>
+        <v>530</v>
       </c>
       <c r="B253" t="s">
-        <v>308</v>
+        <v>544</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B254" t="s">
-        <v>309</v>
-      </c>
-      <c r="C254" t="s">
-        <v>533</v>
+        <v>308</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>463</v>
+        <v>323</v>
       </c>
       <c r="B255" t="s">
-        <v>519</v>
+        <v>309</v>
+      </c>
+      <c r="C255" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>324</v>
+        <v>463</v>
       </c>
       <c r="B256" t="s">
-        <v>310</v>
+        <v>519</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B257" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B258" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B259" t="s">
-        <v>313</v>
-      </c>
-      <c r="C259" t="s">
-        <v>533</v>
+        <v>312</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B260" t="s">
-        <v>314</v>
+        <v>313</v>
+      </c>
+      <c r="C260" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B261" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B262" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B263" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B264" t="s">
-        <v>318</v>
-      </c>
-      <c r="C264" t="s">
-        <v>533</v>
+        <v>317</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B265" t="s">
-        <v>319</v>
+        <v>318</v>
+      </c>
+      <c r="C265" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B266" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B267" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
+        <v>335</v>
+      </c>
+      <c r="B268" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3">
+      <c r="A269" t="s">
         <v>483</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B269" t="s">
         <v>605</v>
-      </c>
-    </row>
-    <row r="270" spans="1:3">
-      <c r="A270" t="s">
-        <v>548</v>
-      </c>
-      <c r="B270" t="s">
-        <v>549</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>342</v>
+        <v>548</v>
       </c>
       <c r="B271" t="s">
-        <v>360</v>
+        <v>549</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B272" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B273" t="s">
-        <v>358</v>
-      </c>
-      <c r="C273" t="s">
-        <v>533</v>
+        <v>357</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>464</v>
+        <v>344</v>
       </c>
       <c r="B274" t="s">
-        <v>520</v>
+        <v>358</v>
+      </c>
+      <c r="C274" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>361</v>
+        <v>464</v>
       </c>
       <c r="B275" t="s">
-        <v>359</v>
-      </c>
-      <c r="C275" t="s">
-        <v>533</v>
+        <v>520</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="B276" t="s">
-        <v>351</v>
+        <v>359</v>
+      </c>
+      <c r="C276" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>362</v>
+        <v>345</v>
       </c>
       <c r="B277" t="s">
-        <v>352</v>
-      </c>
-      <c r="C277" t="s">
-        <v>510</v>
+        <v>351</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="B278" t="s">
-        <v>353</v>
+        <v>352</v>
+      </c>
+      <c r="C278" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B279" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B280" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B281" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B282" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>1079</v>
+        <v>350</v>
       </c>
       <c r="B283" t="s">
-        <v>1080</v>
-      </c>
-      <c r="C283" t="s">
-        <v>1074</v>
+        <v>353</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="B284" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="C284" t="s">
         <v>1074</v>
@@ -10453,10 +10456,10 @@
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="B285" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="C285" t="s">
         <v>1074</v>
@@ -10464,40 +10467,40 @@
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B286" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C286" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3">
+      <c r="A287" t="s">
         <v>482</v>
       </c>
-      <c r="B286" t="s">
+      <c r="B287" t="s">
         <v>621</v>
-      </c>
-    </row>
-    <row r="288" spans="1:3">
-      <c r="A288" t="s">
-        <v>678</v>
-      </c>
-      <c r="B288" t="s">
-        <v>697</v>
-      </c>
-      <c r="C288" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>1072</v>
+        <v>678</v>
       </c>
       <c r="B289" t="s">
-        <v>1073</v>
+        <v>697</v>
       </c>
       <c r="C289" t="s">
-        <v>1074</v>
+        <v>629</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>1075</v>
+        <v>1072</v>
       </c>
       <c r="B290" t="s">
-        <v>1076</v>
+        <v>1073</v>
       </c>
       <c r="C290" t="s">
         <v>1074</v>
@@ -10505,78 +10508,78 @@
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="B291" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C291" t="s">
         <v>1074</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
-      <c r="A293" t="s">
-        <v>674</v>
-      </c>
-      <c r="B293" t="s">
-        <v>675</v>
-      </c>
-      <c r="C293" t="s">
-        <v>629</v>
+    <row r="292" spans="1:3">
+      <c r="A292" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B292" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C292" t="s">
+        <v>1074</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>473</v>
+        <v>674</v>
       </c>
       <c r="B294" t="s">
-        <v>474</v>
+        <v>675</v>
+      </c>
+      <c r="C294" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>368</v>
+        <v>473</v>
       </c>
       <c r="B295" t="s">
-        <v>379</v>
+        <v>474</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B296" t="s">
-        <v>380</v>
-      </c>
-      <c r="C296" t="s">
-        <v>533</v>
+        <v>379</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>521</v>
+        <v>369</v>
       </c>
       <c r="B297" t="s">
-        <v>522</v>
+        <v>380</v>
+      </c>
+      <c r="C297" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>370</v>
+        <v>521</v>
       </c>
       <c r="B298" t="s">
-        <v>381</v>
-      </c>
-      <c r="C298" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B299" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C299" t="s">
         <v>533</v>
@@ -10584,139 +10587,139 @@
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B300" t="s">
-        <v>534</v>
+        <v>382</v>
+      </c>
+      <c r="C300" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B301" t="s">
-        <v>383</v>
+        <v>534</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B302" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B303" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B304" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B305" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B306" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>733</v>
+        <v>378</v>
       </c>
       <c r="B307" t="s">
-        <v>734</v>
-      </c>
-      <c r="C307" t="s">
-        <v>629</v>
+        <v>388</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>480</v>
+        <v>733</v>
       </c>
       <c r="B308" t="s">
-        <v>622</v>
+        <v>734</v>
+      </c>
+      <c r="C308" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
+        <v>480</v>
+      </c>
+      <c r="B309" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3">
+      <c r="A310" t="s">
         <v>557</v>
       </c>
-      <c r="B309" t="s">
+      <c r="B310" t="s">
         <v>558</v>
-      </c>
-    </row>
-    <row r="311" spans="1:3">
-      <c r="A311" t="s">
-        <v>475</v>
-      </c>
-      <c r="B311" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>395</v>
+        <v>475</v>
       </c>
       <c r="B312" t="s">
-        <v>406</v>
+        <v>474</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B313" t="s">
-        <v>407</v>
-      </c>
-      <c r="C313" t="s">
-        <v>533</v>
+        <v>406</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>465</v>
+        <v>396</v>
       </c>
       <c r="B314" t="s">
-        <v>523</v>
+        <v>407</v>
+      </c>
+      <c r="C314" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>397</v>
+        <v>465</v>
       </c>
       <c r="B315" t="s">
-        <v>408</v>
-      </c>
-      <c r="C315" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B316" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C316" t="s">
         <v>533</v>
@@ -10724,1178 +10727,1189 @@
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B317" t="s">
-        <v>535</v>
+        <v>409</v>
+      </c>
+      <c r="C317" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B318" t="s">
-        <v>383</v>
+        <v>535</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B319" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B320" t="s">
-        <v>410</v>
+        <v>384</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B321" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B322" t="s">
-        <v>387</v>
+        <v>411</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B323" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>479</v>
+        <v>405</v>
       </c>
       <c r="B324" t="s">
-        <v>622</v>
+        <v>388</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
+        <v>479</v>
+      </c>
+      <c r="B325" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3">
+      <c r="A326" t="s">
         <v>564</v>
       </c>
-      <c r="B325" t="s">
+      <c r="B326" t="s">
         <v>558</v>
-      </c>
-    </row>
-    <row r="327" spans="1:3">
-      <c r="A327" t="s">
-        <v>672</v>
-      </c>
-      <c r="B327" t="s">
-        <v>673</v>
-      </c>
-      <c r="C327" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>389</v>
+        <v>672</v>
       </c>
       <c r="B328" t="s">
-        <v>565</v>
+        <v>673</v>
+      </c>
+      <c r="C328" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B329" t="s">
-        <v>566</v>
-      </c>
-      <c r="C329" t="s">
-        <v>533</v>
+        <v>565</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>466</v>
+        <v>390</v>
       </c>
       <c r="B330" t="s">
-        <v>567</v>
+        <v>566</v>
+      </c>
+      <c r="C330" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>391</v>
+        <v>466</v>
       </c>
       <c r="B331" t="s">
-        <v>592</v>
+        <v>567</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B332" t="s">
-        <v>568</v>
+        <v>592</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B333" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
+        <v>393</v>
+      </c>
+      <c r="B334" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3">
+      <c r="A335" t="s">
         <v>478</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B335" t="s">
         <v>623</v>
-      </c>
-    </row>
-    <row r="336" spans="1:3">
-      <c r="A336" t="s">
-        <v>749</v>
-      </c>
-      <c r="B336" t="s">
-        <v>750</v>
-      </c>
-      <c r="C336" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="B337" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C337" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="339" spans="1:3">
-      <c r="A339" t="s">
-        <v>757</v>
-      </c>
-      <c r="B339" t="s">
-        <v>758</v>
+    <row r="338" spans="1:3">
+      <c r="A338" t="s">
+        <v>751</v>
+      </c>
+      <c r="B338" t="s">
+        <v>752</v>
+      </c>
+      <c r="C338" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="340" spans="1:3">
       <c r="A340" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B340" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="B341" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B342" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B343" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B344" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B345" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B346" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B347" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B348" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B349" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="B350" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="B351" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B352" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="B353" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B354" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="B355" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
+        <v>789</v>
+      </c>
+      <c r="B356" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" t="s">
         <v>791</v>
       </c>
-      <c r="B356" t="s">
+      <c r="B357" t="s">
         <v>792</v>
-      </c>
-    </row>
-    <row r="358" spans="1:2">
-      <c r="A358" t="s">
-        <v>793</v>
-      </c>
-      <c r="B358" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="B359" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="B360" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="B361" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="B362" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="B363" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="B364" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B365" t="s">
-        <v>321</v>
+        <v>806</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B366" t="s">
-        <v>809</v>
+        <v>321</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="B367" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="B368" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
+        <v>812</v>
+      </c>
+      <c r="B369" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" t="s">
         <v>814</v>
       </c>
-      <c r="B369" t="s">
+      <c r="B370" t="s">
         <v>815</v>
-      </c>
-    </row>
-    <row r="371" spans="1:2">
-      <c r="A371" t="s">
-        <v>816</v>
-      </c>
-      <c r="B371" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B372" t="s">
-        <v>818</v>
+        <v>314</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="B373" t="s">
-        <v>316</v>
+        <v>818</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
+        <v>819</v>
+      </c>
+      <c r="B374" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" t="s">
         <v>820</v>
       </c>
-      <c r="B374" t="s">
+      <c r="B375" t="s">
         <v>317</v>
-      </c>
-    </row>
-    <row r="376" spans="1:2">
-      <c r="A376" t="s">
-        <v>845</v>
-      </c>
-      <c r="B376" t="s">
-        <v>846</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B377" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>837</v>
+        <v>844</v>
       </c>
       <c r="B378" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="B379" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B380" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
+        <v>836</v>
+      </c>
+      <c r="B381" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" t="s">
         <v>842</v>
       </c>
-      <c r="B381" t="s">
+      <c r="B382" t="s">
         <v>841</v>
-      </c>
-    </row>
-    <row r="383" spans="1:2">
-      <c r="A383" t="s">
-        <v>849</v>
-      </c>
-      <c r="B383" t="s">
-        <v>854</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>857</v>
+        <v>849</v>
       </c>
       <c r="B384" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="B385" t="s">
-        <v>838</v>
+        <v>855</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B386" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B387" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
+        <v>852</v>
+      </c>
+      <c r="B388" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" t="s">
         <v>853</v>
       </c>
-      <c r="B388" t="s">
+      <c r="B389" t="s">
         <v>856</v>
-      </c>
-    </row>
-    <row r="390" spans="1:2">
-      <c r="A390" t="s">
-        <v>862</v>
-      </c>
-      <c r="B390" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B391" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="B392" t="s">
-        <v>717</v>
+        <v>865</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="B393" t="s">
-        <v>867</v>
+        <v>717</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>875</v>
+        <v>868</v>
       </c>
       <c r="B394" t="s">
-        <v>252</v>
+        <v>867</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B395" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B396" t="s">
-        <v>869</v>
+        <v>255</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="B397" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B398" t="s">
-        <v>260</v>
+        <v>870</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B399" t="s">
-        <v>871</v>
+        <v>260</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B400" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B401" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B402" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B403" t="s">
-        <v>277</v>
+        <v>874</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B404" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B405" t="s">
-        <v>828</v>
+        <v>281</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>879</v>
+        <v>888</v>
       </c>
       <c r="B406" t="s">
-        <v>635</v>
+        <v>828</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
+        <v>879</v>
+      </c>
+      <c r="B407" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2">
+      <c r="A408" t="s">
         <v>878</v>
       </c>
-      <c r="B407" t="s">
+      <c r="B408" t="s">
         <v>617</v>
-      </c>
-    </row>
-    <row r="409" spans="1:2">
-      <c r="A409" t="s">
-        <v>953</v>
-      </c>
-      <c r="B409" t="s">
-        <v>932</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>972</v>
+        <v>953</v>
       </c>
       <c r="B410" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B411" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B412" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="B413" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="B414" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="B415" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B416" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B417" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B418" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="B419" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>973</v>
+        <v>963</v>
       </c>
       <c r="B420" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>962</v>
+        <v>973</v>
       </c>
       <c r="B421" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B422" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B423" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="B424" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B425" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B426" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="B427" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B428" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
+        <v>955</v>
+      </c>
+      <c r="B429" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2">
+      <c r="A430" t="s">
         <v>954</v>
       </c>
-      <c r="B429" t="s">
+      <c r="B430" t="s">
         <v>952</v>
-      </c>
-    </row>
-    <row r="431" spans="1:2">
-      <c r="A431" t="s">
-        <v>995</v>
-      </c>
-      <c r="B431" t="s">
-        <v>976</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>986</v>
+        <v>995</v>
       </c>
       <c r="B432" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B433" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B434" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>991</v>
+        <v>988</v>
       </c>
       <c r="B435" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
       <c r="B436" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="B437" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="B438" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="B439" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
+        <v>994</v>
+      </c>
+      <c r="B440" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2">
+      <c r="A441" t="s">
         <v>993</v>
       </c>
-      <c r="B440" t="s">
+      <c r="B441" t="s">
         <v>985</v>
-      </c>
-    </row>
-    <row r="442" spans="1:2">
-      <c r="A442" t="s">
-        <v>1000</v>
-      </c>
-      <c r="B442" t="s">
-        <v>1002</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" t="s">
         <v>1011</v>
       </c>
-      <c r="B443" t="s">
+      <c r="B444" t="s">
         <v>1012</v>
-      </c>
-    </row>
-    <row r="445" spans="1:2">
-      <c r="A445" t="s">
-        <v>1001</v>
-      </c>
-      <c r="B445" t="s">
-        <v>1003</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2">
+      <c r="A447" t="s">
         <v>1013</v>
       </c>
-      <c r="B446" t="s">
+      <c r="B447" t="s">
         <v>1014</v>
-      </c>
-    </row>
-    <row r="448" spans="1:2">
-      <c r="A448" t="s">
-        <v>1008</v>
-      </c>
-      <c r="B448" t="s">
-        <v>1006</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B449" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" t="s">
         <v>1005</v>
       </c>
-      <c r="B450" t="s">
+      <c r="B451" t="s">
         <v>1010</v>
-      </c>
-    </row>
-    <row r="452" spans="1:2">
-      <c r="A452" t="s">
-        <v>1023</v>
-      </c>
-      <c r="B452" t="s">
-        <v>1016</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B453" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B454" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>1071</v>
+        <v>1025</v>
       </c>
       <c r="B455" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>1026</v>
+        <v>1071</v>
       </c>
       <c r="B456" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B457" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" t="s">
         <v>1028</v>
       </c>
-      <c r="B458" t="s">
+      <c r="B459" t="s">
         <v>1022</v>
-      </c>
-    </row>
-    <row r="460" spans="1:2">
-      <c r="A460" t="s">
-        <v>1040</v>
-      </c>
-      <c r="B460" t="s">
-        <v>1034</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>1045</v>
+        <v>1040</v>
       </c>
       <c r="B461" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="B462" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B463" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="B464" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B465" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" t="s">
         <v>1043</v>
       </c>
-      <c r="B465" t="s">
+      <c r="B466" t="s">
         <v>1039</v>
-      </c>
-    </row>
-    <row r="467" spans="1:2">
-      <c r="A467" t="s">
-        <v>1058</v>
-      </c>
-      <c r="B467" t="s">
-        <v>1046</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="B468" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B469" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B470" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B471" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" t="s">
         <v>1057</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B473" t="s">
         <v>1051</v>
-      </c>
-    </row>
-    <row r="474" spans="1:2">
-      <c r="A474" t="s">
-        <v>1059</v>
-      </c>
-      <c r="B474" t="s">
-        <v>1060</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
-        <v>1065</v>
+        <v>1059</v>
       </c>
       <c r="B475" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B476" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B477" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B478" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="479" spans="1:2">
+      <c r="A479" t="s">
         <v>1068</v>
       </c>
-      <c r="B478" t="s">
+      <c r="B479" t="s">
         <v>1064</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A448:A449 A445:A446 A431:A440 A442:A443">
+  <conditionalFormatting sqref="A449:A450 A446:A447 A432:A441 A443:A444">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updates to fix ICW Adults FT questions, CSS Student Status Check in CSS, HAB Signature check
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB9088E-40C8-41A7-87AB-7AA7E94E6A62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58AC5248-0F30-416A-992F-5884C210A048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1319" uniqueCount="1088">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="1092">
   <si>
     <t>Name</t>
   </si>
@@ -3297,13 +3297,25 @@
     <t>Payment Generation Date listed on the Child Support Payment History does not match the End Date listed on Child Support Calcs. </t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>MID_VeteranCheck</t>
   </si>
   <si>
     <t xml:space="preserve">The Veteran of the United States Military question was not documented appropriately. </t>
+  </si>
+  <si>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>ShortTimeDelay</t>
+  </si>
+  <si>
+    <t>MediumTimeDelay</t>
+  </si>
+  <si>
+    <t>LongTimeDelay</t>
+  </si>
+  <si>
+    <t>DU_TimeOut</t>
   </si>
 </sst>
 </file>
@@ -3355,7 +3367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3365,6 +3377,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3772,7 +3785,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>1085</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7129,10 +7142,38 @@
         <v>714</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A44" s="5" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A45" s="5" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>1089</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A46" s="5" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A47" s="5" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>1091</v>
+      </c>
+    </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
@@ -8565,10 +8606,10 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
+        <v>1085</v>
+      </c>
+      <c r="B56" t="s">
         <v>1086</v>
-      </c>
-      <c r="B56" t="s">
-        <v>1087</v>
       </c>
     </row>
     <row r="57" spans="1:3">

</xml_diff>

<commit_message>
changes for ACNFA - TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58AC5248-0F30-416A-992F-5884C210A048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D3C510-7FFE-4B88-A848-15206B8058F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="1092">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1357" uniqueCount="1122">
   <si>
     <t>Name</t>
   </si>
@@ -3316,6 +3316,96 @@
   </si>
   <si>
     <t>DU_TimeOut</t>
+  </si>
+  <si>
+    <t>ACNFA</t>
+  </si>
+  <si>
+    <t>Asset Certification of Net Family Assets</t>
+  </si>
+  <si>
+    <t>ACNFAExists</t>
+  </si>
+  <si>
+    <t>The Asset Certification of Net Family Assets is missing from the application. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Head of Household listed on the Asset Certification of Net Family Assets does not match the ICW </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash Value for all sources on the Asset Certification of Net Family Assets has not been documented with either a value or N/A. </t>
+  </si>
+  <si>
+    <t>Cash Value listed for a source on the Asset Certification of Net Family Assets does not match the sum of the same asset source listed on the ICW. </t>
+  </si>
+  <si>
+    <t>Interest Rate is populated for a source on the Asset Certification of Net Family Assets but the corresponding Annual Income is not documented.  </t>
+  </si>
+  <si>
+    <t>None of the Fair Market Value checkboxes on the Asset Certification of Net Family Assets have been documented appropriately. </t>
+  </si>
+  <si>
+    <t>Multiple of the Fair Market Value checkboxes on the Asset Certification of Net Family Assets have been documented but only one should be. </t>
+  </si>
+  <si>
+    <t>Checkbox 4 on the Asset Certification of Net Family Assets has been documented claiming no assets, but not all sources have listed N/A for Cash Value. </t>
+  </si>
+  <si>
+    <t>The net family assets listed on the Asset Certification of Net Family Assets is blank. (Can be 0 or N/A but can’t be blank.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The net family assets listed on the Asset Certification of Net Family Assets does not equal the sum of all the sources Annual Income values. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Asset Certification of Net Family Assets has not been signed by all adults in the household. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Asset Certification of Net Family Assets has not been dated by all adults in the household. </t>
+  </si>
+  <si>
+    <t>The date on the Asset Certification of Net Family Assets is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Asset Certification of Net Family Assets. Needs manual review. </t>
+  </si>
+  <si>
+    <t>ACNFA_FindingError</t>
+  </si>
+  <si>
+    <t>ACNFA_ICWHeadOfHousehold</t>
+  </si>
+  <si>
+    <t>ACNFA_CashValue</t>
+  </si>
+  <si>
+    <t>ACNFA_ICWAssetSource</t>
+  </si>
+  <si>
+    <t>ACNFA_InteresrRate</t>
+  </si>
+  <si>
+    <t>ACNFA_FairMarket</t>
+  </si>
+  <si>
+    <t>ACNFA_MultipleFairMarketValue</t>
+  </si>
+  <si>
+    <t>ACNFA_Checkbox4</t>
+  </si>
+  <si>
+    <t>ACNFA_NetFamilyIncomeBlank</t>
+  </si>
+  <si>
+    <t>ACNFA_NetFamilySumSources</t>
+  </si>
+  <si>
+    <t>ACNFA_Signed</t>
+  </si>
+  <si>
+    <t>ACNFA_Dated</t>
+  </si>
+  <si>
+    <t>ACNFA_CheckMoveInDate</t>
   </si>
 </sst>
 </file>
@@ -3367,7 +3457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3377,7 +3467,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4199,7 +4288,14 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A58" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1093</v>
+      </c>
+    </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="60" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
@@ -7143,34 +7239,34 @@
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A44" s="5" t="s">
+      <c r="A44" t="s">
         <v>1088</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" t="s">
         <v>1088</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A45" s="5" t="s">
+      <c r="A45" t="s">
         <v>1089</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" t="s">
         <v>1089</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A46" s="5" t="s">
+      <c r="A46" t="s">
         <v>1090</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" t="s">
         <v>1090</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A47" s="5" t="s">
+      <c r="A47" t="s">
         <v>1091</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" t="s">
         <v>1091</v>
       </c>
     </row>
@@ -8148,7 +8244,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C479"/>
+  <dimension ref="A1:C494"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -11949,6 +12045,118 @@
         <v>1064</v>
       </c>
     </row>
+    <row r="481" spans="1:2">
+      <c r="A481" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B481" t="s">
+        <v>1095</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2">
+      <c r="A482" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B482" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2">
+      <c r="A483" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B483" t="s">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="484" spans="1:2">
+      <c r="A484" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B484" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="485" spans="1:2">
+      <c r="A485" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B485" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="486" spans="1:2">
+      <c r="A486" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B486" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="487" spans="1:2">
+      <c r="A487" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2">
+      <c r="A488" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B488" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B489" t="s">
+        <v>1103</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2">
+      <c r="A490" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B490" t="s">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="491" spans="1:2">
+      <c r="A491" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B491" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="492" spans="1:2">
+      <c r="A492" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B492" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="493" spans="1:2">
+      <c r="A493" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="494" spans="1:2">
+      <c r="A494" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B494" t="s">
+        <v>1108</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A449:A450 A446:A447 A432:A441 A443:A444">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>

</xml_diff>

<commit_message>
Update to CSS, and RCV
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC38452-053C-42E6-98B4-09955C96B3BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143D50AB-6373-42E9-9D12-0E14BCD44CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3405,7 +3405,7 @@
     <t>ACNFA_InterestRate</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added the parallel processing LLM and DU exception handling, replaced the property name in the AS code for AZ, updated the SCNE and ACNFA
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143D50AB-6373-42E9-9D12-0E14BCD44CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BEDA7C-960D-4DC0-9E73-20BC478EE360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3405,7 +3405,7 @@
     <t>ACNFA_InterestRate</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updates to OL, VS, and PS, RCV verbaige change
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9097D3B3-B1C2-47AD-96D2-A1AAC22850A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28059B1-05D8-4D8D-9DB1-13E4B6808259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3396,9 +3396,6 @@
     <t>ACNFA_InterestRate</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Presently Employed has been listed as No on the Employment Verification. Needs manual review.  </t>
   </si>
   <si>
@@ -3487,6 +3484,9 @@
   </si>
   <si>
     <t>Asset Self Certification is missing from the application.</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3955,7 +3955,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1118</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -9041,7 +9041,7 @@
         <v>185</v>
       </c>
       <c r="B86" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -11499,7 +11499,7 @@
         <v>863</v>
       </c>
       <c r="B392" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="393" spans="1:2">
@@ -11507,7 +11507,7 @@
         <v>864</v>
       </c>
       <c r="B393" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="394" spans="1:2">
@@ -11515,7 +11515,7 @@
         <v>866</v>
       </c>
       <c r="B394" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="395" spans="1:2">
@@ -11523,7 +11523,7 @@
         <v>872</v>
       </c>
       <c r="B395" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="396" spans="1:2">
@@ -11531,7 +11531,7 @@
         <v>873</v>
       </c>
       <c r="B396" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="397" spans="1:2">
@@ -11539,7 +11539,7 @@
         <v>874</v>
       </c>
       <c r="B397" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="398" spans="1:2">
@@ -11547,7 +11547,7 @@
         <v>877</v>
       </c>
       <c r="B398" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="399" spans="1:2">
@@ -11555,7 +11555,7 @@
         <v>878</v>
       </c>
       <c r="B399" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="400" spans="1:2">
@@ -11563,7 +11563,7 @@
         <v>879</v>
       </c>
       <c r="B400" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="401" spans="1:2">
@@ -11571,7 +11571,7 @@
         <v>880</v>
       </c>
       <c r="B401" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="402" spans="1:2">
@@ -11579,7 +11579,7 @@
         <v>881</v>
       </c>
       <c r="B402" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="403" spans="1:2">
@@ -11595,7 +11595,7 @@
         <v>883</v>
       </c>
       <c r="B404" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="405" spans="1:2">
@@ -11627,71 +11627,71 @@
         <v>875</v>
       </c>
       <c r="B408" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B409" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B410" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B411" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B412" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="B413" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="B414" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B415" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B416" t="s">
         <v>1146</v>
-      </c>
-      <c r="B416" t="s">
-        <v>1147</v>
       </c>
     </row>
     <row r="418" spans="1:2">

</xml_diff>

<commit_message>
changes in IAQ for TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28059B1-05D8-4D8D-9DB1-13E4B6808259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23A9635-911A-4569-91F9-DB7C85C4675D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3486,7 +3486,7 @@
     <t>Asset Self Certification is missing from the application.</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
minor change in TRRG
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6949A955-DC89-4954-897D-AD9F90B0898B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776592C2-80DA-457D-9863-3F177DEB496C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3483,10 +3483,10 @@
     <t>Asset Self Certification is missing from the application.</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Social Security Benefits Letter is missing at least one page. Manual Review is required.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3955,7 +3955,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -10875,7 +10875,7 @@
         <v>732</v>
       </c>
       <c r="B308" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="C308" t="s">
         <v>628</v>

</xml_diff>

<commit_message>
Updates to Paystubs, Employment Verification, to use separate prompts for each state for classification, MID, ICW
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776592C2-80DA-457D-9863-3F177DEB496C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227897AD-0408-40C3-A865-1B03F89FF160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -1830,9 +1830,6 @@
     <t>PS_PaystubsMatchEDC</t>
   </si>
   <si>
-    <t>Paystubs do not match EDC with Employee Name, End date and Gross pay</t>
-  </si>
-  <si>
     <t>Business asked to remove</t>
   </si>
   <si>
@@ -2709,9 +2706,6 @@
     <t xml:space="preserve">This application is a Section 811 unit, manual review is required. </t>
   </si>
   <si>
-    <t>The Anuual Income is listd as zero. Manual review required.</t>
-  </si>
-  <si>
     <t>Employee Name listed on Verification Services, Day Calculator, and ICW do not match.</t>
   </si>
   <si>
@@ -3487,6 +3481,12 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>Paystubs do not match Day Calculator with Employee Name, End date and Gross pay</t>
+  </si>
+  <si>
+    <t>The Annual Income is listed as zero. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -3955,7 +3955,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4001,10 +4001,10 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
+        <v>641</v>
+      </c>
+      <c r="B14" t="s">
         <v>642</v>
-      </c>
-      <c r="B14" t="s">
-        <v>643</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -4104,7 +4104,7 @@
         <v>411</v>
       </c>
       <c r="B25" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
@@ -4248,133 +4248,133 @@
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B43" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B44" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>844</v>
+      </c>
+      <c r="B45" t="s">
         <v>845</v>
-      </c>
-      <c r="B45" t="s">
-        <v>846</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
+        <v>855</v>
+      </c>
+      <c r="B46" t="s">
         <v>856</v>
-      </c>
-      <c r="B46" t="s">
-        <v>857</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
+        <v>857</v>
+      </c>
+      <c r="B47" t="s">
         <v>858</v>
-      </c>
-      <c r="B47" t="s">
-        <v>859</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
+        <v>884</v>
+      </c>
+      <c r="B48" t="s">
         <v>885</v>
-      </c>
-      <c r="B48" t="s">
-        <v>886</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="B49" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="B50" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1">
       <c r="A51" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B51" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="B52" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
       <c r="B53" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="B54" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="14.25" customHeight="1">
       <c r="A55" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="B55" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="C55" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="14.25" customHeight="1">
       <c r="A56" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="B56" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="B57" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="B58" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5668,7 +5668,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B42" t="s">
         <v>438</v>
@@ -5871,10 +5871,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B20" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -5887,10 +5887,10 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B22" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -6993,10 +6993,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B3" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -7281,74 +7281,74 @@
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="B39" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B40" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B41" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B42" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="B43" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="B44" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="B45" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="B46" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="B47" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8351,79 +8351,79 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="B5" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
       <c r="C5" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="B6" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="C6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="B7" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="C7" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B8" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C8" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="B9" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C9" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>727</v>
+      </c>
+      <c r="B10" t="s">
         <v>728</v>
       </c>
-      <c r="B10" t="s">
-        <v>729</v>
-      </c>
       <c r="C10" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
+        <v>693</v>
+      </c>
+      <c r="B11" t="s">
         <v>694</v>
       </c>
-      <c r="B11" t="s">
-        <v>695</v>
-      </c>
       <c r="C11" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -8455,7 +8455,7 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -8466,7 +8466,7 @@
         <v>203</v>
       </c>
       <c r="C17" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -8479,73 +8479,73 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B19" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B20" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="C20" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
+        <v>648</v>
+      </c>
+      <c r="B21" t="s">
         <v>649</v>
       </c>
-      <c r="B21" t="s">
-        <v>650</v>
-      </c>
       <c r="C21" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="B22" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="C22" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="B23" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="C23" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B24" t="s">
-        <v>889</v>
+        <v>1148</v>
       </c>
       <c r="C24" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>886</v>
+      </c>
+      <c r="B25" t="s">
         <v>887</v>
-      </c>
-      <c r="B25" t="s">
-        <v>888</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -8553,7 +8553,7 @@
         <v>480</v>
       </c>
       <c r="B26" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -8601,7 +8601,7 @@
         <v>194</v>
       </c>
       <c r="B33" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -8609,7 +8609,7 @@
         <v>195</v>
       </c>
       <c r="B34" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="35" spans="1:3">
@@ -8657,29 +8657,29 @@
         <v>594</v>
       </c>
       <c r="B40" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>650</v>
+      </c>
+      <c r="B41" t="s">
         <v>651</v>
       </c>
-      <c r="B41" t="s">
-        <v>652</v>
-      </c>
       <c r="C41" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>729</v>
+      </c>
+      <c r="B42" t="s">
         <v>730</v>
       </c>
-      <c r="B42" t="s">
-        <v>731</v>
-      </c>
       <c r="C42" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="43" spans="1:3">
@@ -8687,7 +8687,7 @@
         <v>495</v>
       </c>
       <c r="B43" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -8775,29 +8775,29 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>718</v>
+      </c>
+      <c r="B55" t="s">
         <v>719</v>
-      </c>
-      <c r="B55" t="s">
-        <v>720</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="B56" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
+        <v>628</v>
+      </c>
+      <c r="B57" t="s">
         <v>629</v>
       </c>
-      <c r="B57" t="s">
-        <v>630</v>
-      </c>
       <c r="C57" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -8805,7 +8805,7 @@
         <v>494</v>
       </c>
       <c r="B58" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -8895,7 +8895,7 @@
         <v>200</v>
       </c>
       <c r="B68" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -8903,7 +8903,7 @@
         <v>201</v>
       </c>
       <c r="B69" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C69" t="s">
         <v>532</v>
@@ -8914,7 +8914,7 @@
         <v>523</v>
       </c>
       <c r="B70" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -8930,7 +8930,7 @@
         <v>504</v>
       </c>
       <c r="B72" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -8938,18 +8938,18 @@
         <v>493</v>
       </c>
       <c r="B73" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B74" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="C74" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -8986,46 +8986,46 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
+        <v>688</v>
+      </c>
+      <c r="B80" t="s">
         <v>689</v>
       </c>
-      <c r="B80" t="s">
-        <v>690</v>
-      </c>
       <c r="C80" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
+        <v>708</v>
+      </c>
+      <c r="B81" t="s">
         <v>709</v>
       </c>
-      <c r="B81" t="s">
-        <v>710</v>
-      </c>
       <c r="C81" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="B82" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="C82" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="B83" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C83" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -9033,7 +9033,7 @@
         <v>492</v>
       </c>
       <c r="B84" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -9041,29 +9041,29 @@
         <v>185</v>
       </c>
       <c r="B86" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B87" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C87" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
+        <v>685</v>
+      </c>
+      <c r="B88" t="s">
         <v>686</v>
       </c>
-      <c r="B88" t="s">
-        <v>687</v>
-      </c>
       <c r="C88" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -9122,7 +9122,7 @@
         <v>450</v>
       </c>
       <c r="C95" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="96" spans="1:3">
@@ -9157,54 +9157,54 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
+        <v>652</v>
+      </c>
+      <c r="B99" t="s">
         <v>653</v>
       </c>
-      <c r="B99" t="s">
-        <v>654</v>
-      </c>
       <c r="C99" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="B100" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
+        <v>679</v>
+      </c>
+      <c r="B101" t="s">
         <v>680</v>
       </c>
-      <c r="B101" t="s">
-        <v>681</v>
-      </c>
       <c r="C101" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B102" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="C102" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="B103" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C103" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="104" spans="1:3">
@@ -9212,39 +9212,39 @@
         <v>491</v>
       </c>
       <c r="B104" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="B105" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="B106" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="B107" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="B108" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -9279,12 +9279,12 @@
         <v>524</v>
       </c>
       <c r="C113" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B114" t="s">
         <v>524</v>
@@ -9327,7 +9327,7 @@
         <v>490</v>
       </c>
       <c r="B119" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="121" spans="1:3">
@@ -9364,13 +9364,13 @@
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B125" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C125" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -9394,10 +9394,10 @@
         <v>570</v>
       </c>
       <c r="B128" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C128" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -9410,13 +9410,13 @@
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
+        <v>654</v>
+      </c>
+      <c r="B130" t="s">
         <v>655</v>
       </c>
-      <c r="B130" t="s">
-        <v>656</v>
-      </c>
       <c r="C130" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -9424,29 +9424,29 @@
         <v>489</v>
       </c>
       <c r="B131" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
+        <v>643</v>
+      </c>
+      <c r="B133" t="s">
         <v>644</v>
       </c>
-      <c r="B133" t="s">
+      <c r="C133" t="s">
         <v>645</v>
-      </c>
-      <c r="C133" t="s">
-        <v>646</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
+        <v>646</v>
+      </c>
+      <c r="B134" t="s">
         <v>647</v>
       </c>
-      <c r="B134" t="s">
-        <v>648</v>
-      </c>
       <c r="C134" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="136" spans="1:3">
@@ -9486,10 +9486,10 @@
         <v>506</v>
       </c>
       <c r="B140" t="s">
+        <v>668</v>
+      </c>
+      <c r="C140" t="s">
         <v>669</v>
-      </c>
-      <c r="C140" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -9505,7 +9505,7 @@
         <v>488</v>
       </c>
       <c r="B142" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -9545,18 +9545,18 @@
         <v>487</v>
       </c>
       <c r="B148" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
+        <v>656</v>
+      </c>
+      <c r="B149" t="s">
         <v>657</v>
       </c>
-      <c r="B149" t="s">
-        <v>658</v>
-      </c>
       <c r="C149" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -9640,7 +9640,7 @@
         <v>476</v>
       </c>
       <c r="B159" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -9648,7 +9648,7 @@
         <v>592</v>
       </c>
       <c r="B161" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="C161" t="s">
         <v>593</v>
@@ -9656,46 +9656,46 @@
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
+        <v>659</v>
+      </c>
+      <c r="B162" t="s">
         <v>660</v>
       </c>
-      <c r="B162" t="s">
-        <v>661</v>
-      </c>
       <c r="C162" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B163" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="C163" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B164" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="C164" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B165" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C165" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -9703,29 +9703,29 @@
         <v>467</v>
       </c>
       <c r="B167" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B168" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C168" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
+        <v>599</v>
+      </c>
+      <c r="B169" t="s">
+        <v>601</v>
+      </c>
+      <c r="C169" t="s">
         <v>600</v>
-      </c>
-      <c r="B169" t="s">
-        <v>602</v>
-      </c>
-      <c r="C169" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="170" spans="1:3">
@@ -9733,7 +9733,7 @@
         <v>238</v>
       </c>
       <c r="B170" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="C170" t="s">
         <v>532</v>
@@ -9744,7 +9744,7 @@
         <v>239</v>
       </c>
       <c r="B171" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -9752,7 +9752,7 @@
         <v>247</v>
       </c>
       <c r="B172" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="C172" t="s">
         <v>590</v>
@@ -9760,13 +9760,13 @@
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B173" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="C173" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="174" spans="1:3">
@@ -9790,7 +9790,7 @@
         <v>242</v>
       </c>
       <c r="B176" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -9798,7 +9798,7 @@
         <v>243</v>
       </c>
       <c r="B177" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -9806,7 +9806,7 @@
         <v>244</v>
       </c>
       <c r="B178" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -9814,7 +9814,7 @@
         <v>245</v>
       </c>
       <c r="B179" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -9822,7 +9822,7 @@
         <v>246</v>
       </c>
       <c r="B180" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -9830,7 +9830,7 @@
         <v>278</v>
       </c>
       <c r="B181" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -9846,45 +9846,45 @@
         <v>595</v>
       </c>
       <c r="B183" t="s">
-        <v>596</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B184" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
+        <v>703</v>
+      </c>
+      <c r="B185" t="s">
         <v>704</v>
       </c>
-      <c r="B185" t="s">
-        <v>705</v>
-      </c>
       <c r="C185" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B186" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C186" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="B187" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -9892,18 +9892,18 @@
         <v>475</v>
       </c>
       <c r="B188" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
+        <v>714</v>
+      </c>
+      <c r="B190" t="s">
         <v>715</v>
       </c>
-      <c r="B190" t="s">
-        <v>716</v>
-      </c>
       <c r="C190" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -9911,7 +9911,7 @@
         <v>468</v>
       </c>
       <c r="B191" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
     </row>
     <row r="192" spans="1:3">
@@ -9919,10 +9919,10 @@
         <v>248</v>
       </c>
       <c r="B192" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="C192" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="193" spans="1:3" ht="13.5" customHeight="1">
@@ -9930,10 +9930,10 @@
         <v>250</v>
       </c>
       <c r="B193" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="C193" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -9941,7 +9941,7 @@
         <v>249</v>
       </c>
       <c r="B194" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -9968,7 +9968,7 @@
         <v>255</v>
       </c>
       <c r="C197" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -9984,7 +9984,7 @@
         <v>257</v>
       </c>
       <c r="B199" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="200" spans="1:3">
@@ -10000,7 +10000,7 @@
         <v>263</v>
       </c>
       <c r="B201" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="202" spans="1:3">
@@ -10008,7 +10008,7 @@
         <v>264</v>
       </c>
       <c r="B202" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="203" spans="1:3">
@@ -10016,10 +10016,10 @@
         <v>265</v>
       </c>
       <c r="B203" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="C203" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -10027,7 +10027,7 @@
         <v>266</v>
       </c>
       <c r="B204" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="205" spans="1:3">
@@ -10035,10 +10035,10 @@
         <v>267</v>
       </c>
       <c r="B205" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="C205" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -10046,7 +10046,7 @@
         <v>268</v>
       </c>
       <c r="B206" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="207" spans="1:3">
@@ -10062,7 +10062,7 @@
         <v>277</v>
       </c>
       <c r="B208" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
     </row>
     <row r="209" spans="1:3">
@@ -10075,10 +10075,10 @@
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B210" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="211" spans="1:3">
@@ -10086,18 +10086,18 @@
         <v>486</v>
       </c>
       <c r="B211" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
+        <v>632</v>
+      </c>
+      <c r="B212" t="s">
         <v>633</v>
       </c>
-      <c r="B212" t="s">
-        <v>634</v>
-      </c>
       <c r="C212" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -10105,7 +10105,7 @@
         <v>469</v>
       </c>
       <c r="B214" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="215" spans="1:3">
@@ -10121,7 +10121,7 @@
         <v>273</v>
       </c>
       <c r="B216" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="217" spans="1:3">
@@ -10129,7 +10129,7 @@
         <v>274</v>
       </c>
       <c r="B217" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -10137,7 +10137,7 @@
         <v>282</v>
       </c>
       <c r="B218" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="219" spans="1:3">
@@ -10145,7 +10145,7 @@
         <v>281</v>
       </c>
       <c r="B219" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -10153,15 +10153,15 @@
         <v>283</v>
       </c>
       <c r="B220" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B221" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -10169,7 +10169,7 @@
         <v>485</v>
       </c>
       <c r="B222" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -10177,7 +10177,7 @@
         <v>470</v>
       </c>
       <c r="B224" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -10193,7 +10193,7 @@
         <v>286</v>
       </c>
       <c r="B226" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
     <row r="227" spans="1:3">
@@ -10209,7 +10209,7 @@
         <v>288</v>
       </c>
       <c r="B228" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="229" spans="1:3">
@@ -10217,7 +10217,7 @@
         <v>290</v>
       </c>
       <c r="B229" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -10225,7 +10225,7 @@
         <v>291</v>
       </c>
       <c r="B230" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="231" spans="1:3">
@@ -10233,7 +10233,7 @@
         <v>292</v>
       </c>
       <c r="B231" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -10241,15 +10241,15 @@
         <v>293</v>
       </c>
       <c r="B232" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B233" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -10257,7 +10257,7 @@
         <v>484</v>
       </c>
       <c r="B234" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -10265,7 +10265,7 @@
         <v>471</v>
       </c>
       <c r="B236" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
     </row>
     <row r="237" spans="1:3">
@@ -10292,7 +10292,7 @@
         <v>297</v>
       </c>
       <c r="B239" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="C239" t="s">
         <v>532</v>
@@ -10303,7 +10303,7 @@
         <v>298</v>
       </c>
       <c r="B240" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -10311,7 +10311,7 @@
         <v>454</v>
       </c>
       <c r="B241" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
     </row>
     <row r="242" spans="1:3">
@@ -10319,7 +10319,7 @@
         <v>300</v>
       </c>
       <c r="B242" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -10327,7 +10327,7 @@
         <v>301</v>
       </c>
       <c r="B243" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -10335,7 +10335,7 @@
         <v>302</v>
       </c>
       <c r="B244" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -10343,7 +10343,7 @@
         <v>303</v>
       </c>
       <c r="B245" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -10351,15 +10351,15 @@
         <v>304</v>
       </c>
       <c r="B246" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B247" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -10367,18 +10367,18 @@
         <v>483</v>
       </c>
       <c r="B248" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
+        <v>674</v>
+      </c>
+      <c r="B250" t="s">
         <v>675</v>
       </c>
-      <c r="B250" t="s">
-        <v>676</v>
-      </c>
       <c r="C250" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -10545,7 +10545,7 @@
         <v>482</v>
       </c>
       <c r="B269" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="271" spans="1:3">
@@ -10663,35 +10663,35 @@
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="B284" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="C284" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="B285" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C285" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="B286" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="C286" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="287" spans="1:3">
@@ -10699,62 +10699,62 @@
         <v>481</v>
       </c>
       <c r="B287" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="B289" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="C289" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B290" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C290" t="s">
         <v>1068</v>
-      </c>
-      <c r="B290" t="s">
-        <v>1069</v>
-      </c>
-      <c r="C290" t="s">
-        <v>1070</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="B291" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="C291" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="B292" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="C292" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
+        <v>672</v>
+      </c>
+      <c r="B294" t="s">
         <v>673</v>
       </c>
-      <c r="B294" t="s">
-        <v>674</v>
-      </c>
       <c r="C294" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="295" spans="1:3">
@@ -10872,13 +10872,13 @@
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B308" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="C308" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="309" spans="1:3">
@@ -10886,7 +10886,7 @@
         <v>479</v>
       </c>
       <c r="B309" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="310" spans="1:3">
@@ -11015,7 +11015,7 @@
         <v>478</v>
       </c>
       <c r="B325" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="326" spans="1:3">
@@ -11028,13 +11028,13 @@
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
+        <v>670</v>
+      </c>
+      <c r="B328" t="s">
         <v>671</v>
       </c>
-      <c r="B328" t="s">
-        <v>672</v>
-      </c>
       <c r="C328" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="329" spans="1:3">
@@ -11093,234 +11093,234 @@
         <v>477</v>
       </c>
       <c r="B335" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
+        <v>746</v>
+      </c>
+      <c r="B337" t="s">
         <v>747</v>
       </c>
-      <c r="B337" t="s">
-        <v>748</v>
-      </c>
       <c r="C337" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="338" spans="1:3">
       <c r="A338" t="s">
+        <v>748</v>
+      </c>
+      <c r="B338" t="s">
         <v>749</v>
       </c>
-      <c r="B338" t="s">
-        <v>750</v>
-      </c>
       <c r="C338" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="340" spans="1:3">
       <c r="A340" t="s">
+        <v>754</v>
+      </c>
+      <c r="B340" t="s">
         <v>755</v>
-      </c>
-      <c r="B340" t="s">
-        <v>756</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
+        <v>756</v>
+      </c>
+      <c r="B341" t="s">
         <v>757</v>
-      </c>
-      <c r="B341" t="s">
-        <v>758</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
+        <v>758</v>
+      </c>
+      <c r="B342" t="s">
         <v>759</v>
-      </c>
-      <c r="B342" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
+        <v>760</v>
+      </c>
+      <c r="B343" t="s">
         <v>761</v>
-      </c>
-      <c r="B343" t="s">
-        <v>762</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
+        <v>762</v>
+      </c>
+      <c r="B344" t="s">
         <v>763</v>
-      </c>
-      <c r="B344" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
+        <v>764</v>
+      </c>
+      <c r="B345" t="s">
         <v>765</v>
-      </c>
-      <c r="B345" t="s">
-        <v>766</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
+        <v>766</v>
+      </c>
+      <c r="B346" t="s">
         <v>767</v>
-      </c>
-      <c r="B346" t="s">
-        <v>768</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
+        <v>768</v>
+      </c>
+      <c r="B347" t="s">
         <v>769</v>
-      </c>
-      <c r="B347" t="s">
-        <v>770</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
+        <v>770</v>
+      </c>
+      <c r="B348" t="s">
         <v>771</v>
-      </c>
-      <c r="B348" t="s">
-        <v>772</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
+        <v>772</v>
+      </c>
+      <c r="B349" t="s">
         <v>773</v>
-      </c>
-      <c r="B349" t="s">
-        <v>774</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
+        <v>774</v>
+      </c>
+      <c r="B350" t="s">
         <v>775</v>
-      </c>
-      <c r="B350" t="s">
-        <v>776</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
+        <v>776</v>
+      </c>
+      <c r="B351" t="s">
         <v>777</v>
-      </c>
-      <c r="B351" t="s">
-        <v>778</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
+        <v>778</v>
+      </c>
+      <c r="B352" t="s">
         <v>779</v>
-      </c>
-      <c r="B352" t="s">
-        <v>780</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
+        <v>780</v>
+      </c>
+      <c r="B353" t="s">
         <v>781</v>
-      </c>
-      <c r="B353" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
+        <v>782</v>
+      </c>
+      <c r="B354" t="s">
         <v>783</v>
-      </c>
-      <c r="B354" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
+        <v>784</v>
+      </c>
+      <c r="B355" t="s">
         <v>785</v>
-      </c>
-      <c r="B355" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
+        <v>786</v>
+      </c>
+      <c r="B356" t="s">
         <v>787</v>
-      </c>
-      <c r="B356" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
+        <v>788</v>
+      </c>
+      <c r="B357" t="s">
         <v>789</v>
-      </c>
-      <c r="B357" t="s">
-        <v>790</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
+        <v>790</v>
+      </c>
+      <c r="B359" t="s">
         <v>791</v>
-      </c>
-      <c r="B359" t="s">
-        <v>792</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
+        <v>792</v>
+      </c>
+      <c r="B360" t="s">
         <v>793</v>
-      </c>
-      <c r="B360" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
+        <v>794</v>
+      </c>
+      <c r="B361" t="s">
         <v>795</v>
-      </c>
-      <c r="B361" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
+        <v>796</v>
+      </c>
+      <c r="B362" t="s">
         <v>797</v>
-      </c>
-      <c r="B362" t="s">
-        <v>798</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
+        <v>798</v>
+      </c>
+      <c r="B363" t="s">
         <v>799</v>
-      </c>
-      <c r="B363" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
+        <v>800</v>
+      </c>
+      <c r="B364" t="s">
         <v>801</v>
-      </c>
-      <c r="B364" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
+        <v>802</v>
+      </c>
+      <c r="B365" t="s">
         <v>803</v>
-      </c>
-      <c r="B365" t="s">
-        <v>804</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B366" t="s">
         <v>320</v>
@@ -11328,39 +11328,39 @@
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
+        <v>805</v>
+      </c>
+      <c r="B367" t="s">
         <v>806</v>
-      </c>
-      <c r="B367" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
+        <v>807</v>
+      </c>
+      <c r="B368" t="s">
         <v>808</v>
-      </c>
-      <c r="B368" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
+        <v>809</v>
+      </c>
+      <c r="B369" t="s">
         <v>810</v>
-      </c>
-      <c r="B369" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
+        <v>811</v>
+      </c>
+      <c r="B370" t="s">
         <v>812</v>
-      </c>
-      <c r="B370" t="s">
-        <v>813</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B372" t="s">
         <v>313</v>
@@ -11368,15 +11368,15 @@
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
+        <v>814</v>
+      </c>
+      <c r="B373" t="s">
         <v>815</v>
-      </c>
-      <c r="B373" t="s">
-        <v>816</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B374" t="s">
         <v>315</v>
@@ -11384,7 +11384,7 @@
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="B375" t="s">
         <v>316</v>
@@ -11392,215 +11392,215 @@
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
+        <v>842</v>
+      </c>
+      <c r="B377" t="s">
         <v>843</v>
-      </c>
-      <c r="B377" t="s">
-        <v>844</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B378" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
+        <v>834</v>
+      </c>
+      <c r="B379" t="s">
         <v>835</v>
-      </c>
-      <c r="B379" t="s">
-        <v>836</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B380" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B381" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B382" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="B384" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B385" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B386" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B387" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="B388" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B389" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
+        <v>859</v>
+      </c>
+      <c r="B391" t="s">
         <v>860</v>
-      </c>
-      <c r="B391" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B392" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B393" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B394" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B395" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B396" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B397" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B398" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B399" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B400" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B401" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B402" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B403" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B404" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B405" t="s">
         <v>280</v>
@@ -11608,698 +11608,698 @@
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B406" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B407" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B408" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="B409" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="B410" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="B411" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="B412" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="B413" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="B414" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="B415" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="B416" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="B418" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="B419" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="B420" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="B421" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="B422" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B423" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="B424" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="B425" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="B426" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="B427" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="B428" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="B429" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="B430" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="B431" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="B432" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="B433" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="B434" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="B435" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="B436" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="B437" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="B438" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="B440" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="B441" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="B442" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="B443" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="B444" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="B445" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="B446" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="B447" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="B448" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="B449" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
+        <v>994</v>
+      </c>
+      <c r="B451" t="s">
         <v>996</v>
-      </c>
-      <c r="B451" t="s">
-        <v>998</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="B452" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
+        <v>995</v>
+      </c>
+      <c r="B454" t="s">
         <v>997</v>
-      </c>
-      <c r="B454" t="s">
-        <v>999</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="B455" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B457" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="B458" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="B459" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="B461" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="B462" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
       <c r="B463" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="B464" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="B465" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="B466" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B467" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="B469" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="B470" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="B471" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B472" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="B473" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="474" spans="1:2">
       <c r="A474" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="B474" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="B476" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="B477" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="B478" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B479" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="B480" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="B481" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="B483" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="B484" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="B485" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="B486" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="B487" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="489" spans="1:2">
       <c r="A489" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="B489" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="B490" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="B491" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="B492" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="B493" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B494" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="B495" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
       <c r="B496" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="B497" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
       <c r="B498" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="B499" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="B500" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="B501" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="B502" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update to fix the UAT invalid findings
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227897AD-0408-40C3-A865-1B03F89FF160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D3308D-FEAA-4133-AE4B-06B118FAB872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3480,13 +3480,13 @@
     <t>Social Security Benefits Letter is missing at least one page. Manual Review is required.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Paystubs do not match Day Calculator with Employee Name, End date and Gross pay</t>
   </si>
   <si>
     <t>The Annual Income is listed as zero. Manual review required.</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3955,7 +3955,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1146</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -8534,7 +8534,7 @@
         <v>738</v>
       </c>
       <c r="B24" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="C24" t="s">
         <v>627</v>
@@ -9846,7 +9846,7 @@
         <v>595</v>
       </c>
       <c r="B183" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="184" spans="1:3">

</xml_diff>

<commit_message>
removing the YTD from each file and adding it just for EDC for AZ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D3308D-FEAA-4133-AE4B-06B118FAB872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE59049-4A7D-4951-9F72-96C344290B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1373" uniqueCount="1149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="1153">
   <si>
     <t>Name</t>
   </si>
@@ -3486,7 +3486,19 @@
     <t>The Annual Income is listed as zero. Manual review required.</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>Implementing whis only in EDC.</t>
+  </si>
+  <si>
+    <t>DC_YTDIncome</t>
+  </si>
+  <si>
+    <t>Newly added by Bagi</t>
+  </si>
+  <si>
+    <t>Implementing this only in EDC.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3955,7 +3967,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1148</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -8325,7 +8337,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C502"/>
+  <dimension ref="A1:C503"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -9698,31 +9710,31 @@
         <v>627</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
-      <c r="A167" t="s">
-        <v>467</v>
-      </c>
-      <c r="B167" t="s">
-        <v>893</v>
+    <row r="166" spans="1:3">
+      <c r="A166" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B166" t="s">
+        <v>898</v>
+      </c>
+      <c r="C166" t="s">
+        <v>1150</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>598</v>
+        <v>467</v>
       </c>
       <c r="B168" t="s">
-        <v>602</v>
-      </c>
-      <c r="C168" t="s">
-        <v>600</v>
+        <v>893</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B169" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C169" t="s">
         <v>600</v>
@@ -9730,150 +9742,156 @@
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>238</v>
+        <v>599</v>
       </c>
       <c r="B170" t="s">
-        <v>894</v>
+        <v>601</v>
       </c>
       <c r="C170" t="s">
-        <v>532</v>
+        <v>600</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B171" t="s">
-        <v>895</v>
+        <v>894</v>
+      </c>
+      <c r="C171" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="B172" t="s">
-        <v>896</v>
-      </c>
-      <c r="C172" t="s">
-        <v>590</v>
+        <v>895</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>717</v>
+        <v>247</v>
       </c>
       <c r="B173" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="C173" t="s">
-        <v>627</v>
+        <v>590</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>241</v>
+        <v>717</v>
       </c>
       <c r="B174" t="s">
-        <v>240</v>
+        <v>897</v>
+      </c>
+      <c r="C174" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>457</v>
+        <v>241</v>
       </c>
       <c r="B175" t="s">
-        <v>466</v>
+        <v>240</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>242</v>
+        <v>457</v>
       </c>
       <c r="B176" t="s">
-        <v>898</v>
+        <v>466</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B177" t="s">
-        <v>899</v>
+        <v>898</v>
+      </c>
+      <c r="C177" t="s">
+        <v>1151</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B178" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B179" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B180" t="s">
-        <v>824</v>
+        <v>901</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>278</v>
+        <v>246</v>
       </c>
       <c r="B181" t="s">
-        <v>898</v>
+        <v>824</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>305</v>
+        <v>278</v>
       </c>
       <c r="B182" t="s">
-        <v>306</v>
+        <v>898</v>
+      </c>
+      <c r="C182" t="s">
+        <v>1151</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>595</v>
+        <v>305</v>
       </c>
       <c r="B183" t="s">
-        <v>1146</v>
+        <v>306</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>636</v>
+        <v>595</v>
       </c>
       <c r="B184" t="s">
-        <v>825</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>703</v>
+        <v>636</v>
       </c>
       <c r="B185" t="s">
-        <v>704</v>
-      </c>
-      <c r="C185" t="s">
-        <v>627</v>
+        <v>825</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>716</v>
+        <v>703</v>
       </c>
       <c r="B186" t="s">
-        <v>735</v>
+        <v>704</v>
       </c>
       <c r="C186" t="s">
         <v>627</v>
@@ -9881,803 +9899,809 @@
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>912</v>
+        <v>716</v>
       </c>
       <c r="B187" t="s">
-        <v>913</v>
+        <v>735</v>
+      </c>
+      <c r="C187" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
+        <v>912</v>
+      </c>
+      <c r="B188" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3">
+      <c r="A189" t="s">
         <v>475</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B189" t="s">
         <v>614</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3">
-      <c r="A190" t="s">
-        <v>714</v>
-      </c>
-      <c r="B190" t="s">
-        <v>715</v>
-      </c>
-      <c r="C190" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>468</v>
+        <v>714</v>
       </c>
       <c r="B191" t="s">
-        <v>902</v>
+        <v>715</v>
+      </c>
+      <c r="C191" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
+        <v>468</v>
+      </c>
+      <c r="B192" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3">
+      <c r="A193" t="s">
         <v>248</v>
       </c>
-      <c r="B192" t="s">
+      <c r="B193" t="s">
         <v>903</v>
       </c>
-      <c r="C192" t="s">
+      <c r="C193" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="193" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A193" t="s">
+    <row r="194" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A194" t="s">
         <v>250</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B194" t="s">
         <v>904</v>
       </c>
-      <c r="C193" t="s">
+      <c r="C194" t="s">
         <v>631</v>
-      </c>
-    </row>
-    <row r="194" spans="1:3">
-      <c r="A194" t="s">
-        <v>249</v>
-      </c>
-      <c r="B194" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B195" t="s">
-        <v>251</v>
+        <v>863</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B196" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B197" t="s">
-        <v>255</v>
-      </c>
-      <c r="C197" t="s">
-        <v>597</v>
+        <v>254</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>458</v>
+        <v>256</v>
       </c>
       <c r="B198" t="s">
-        <v>514</v>
+        <v>255</v>
+      </c>
+      <c r="C198" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>257</v>
+        <v>458</v>
       </c>
       <c r="B199" t="s">
-        <v>865</v>
+        <v>514</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B200" t="s">
-        <v>259</v>
+        <v>865</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B201" t="s">
-        <v>866</v>
+        <v>259</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B202" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B203" t="s">
-        <v>905</v>
-      </c>
-      <c r="C203" t="s">
-        <v>597</v>
+        <v>867</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B204" t="s">
-        <v>868</v>
+        <v>905</v>
+      </c>
+      <c r="C204" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B205" t="s">
-        <v>906</v>
-      </c>
-      <c r="C205" t="s">
-        <v>597</v>
+        <v>868</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B206" t="s">
-        <v>869</v>
+        <v>906</v>
+      </c>
+      <c r="C206" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B207" t="s">
-        <v>276</v>
+        <v>869</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B208" t="s">
-        <v>898</v>
+        <v>276</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B209" t="s">
-        <v>280</v>
+        <v>898</v>
+      </c>
+      <c r="C209" t="s">
+        <v>1151</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>637</v>
+        <v>279</v>
       </c>
       <c r="B210" t="s">
-        <v>825</v>
+        <v>280</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>486</v>
+        <v>637</v>
       </c>
       <c r="B211" t="s">
-        <v>615</v>
+        <v>825</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
+        <v>486</v>
+      </c>
+      <c r="B212" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3">
+      <c r="A213" t="s">
         <v>632</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B213" t="s">
         <v>633</v>
       </c>
-      <c r="C212" t="s">
+      <c r="C213" t="s">
         <v>627</v>
-      </c>
-    </row>
-    <row r="214" spans="1:3">
-      <c r="A214" t="s">
-        <v>469</v>
-      </c>
-      <c r="B214" t="s">
-        <v>826</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="B215" t="s">
-        <v>515</v>
+        <v>826</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>273</v>
+        <v>459</v>
       </c>
       <c r="B216" t="s">
-        <v>827</v>
+        <v>515</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B217" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="B218" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B219" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B220" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>638</v>
+        <v>283</v>
       </c>
       <c r="B221" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
+        <v>638</v>
+      </c>
+      <c r="B222" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3">
+      <c r="A223" t="s">
         <v>485</v>
       </c>
-      <c r="B222" t="s">
+      <c r="B223" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="224" spans="1:3">
-      <c r="A224" t="s">
-        <v>470</v>
-      </c>
-      <c r="B224" t="s">
-        <v>818</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="B225" t="s">
-        <v>516</v>
+        <v>818</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>286</v>
+        <v>460</v>
       </c>
       <c r="B226" t="s">
-        <v>819</v>
+        <v>516</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B227" t="s">
-        <v>289</v>
+        <v>819</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B228" t="s">
-        <v>820</v>
+        <v>289</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B229" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B230" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B231" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B232" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>639</v>
+        <v>293</v>
       </c>
       <c r="B233" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
+        <v>639</v>
+      </c>
+      <c r="B234" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3">
+      <c r="A235" t="s">
         <v>484</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B235" t="s">
         <v>617</v>
-      </c>
-    </row>
-    <row r="236" spans="1:3">
-      <c r="A236" t="s">
-        <v>471</v>
-      </c>
-      <c r="B236" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>455</v>
+        <v>471</v>
       </c>
       <c r="B237" t="s">
-        <v>299</v>
-      </c>
-      <c r="C237" t="s">
-        <v>532</v>
+        <v>907</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="B238" t="s">
-        <v>517</v>
+        <v>299</v>
+      </c>
+      <c r="C238" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>297</v>
+        <v>461</v>
       </c>
       <c r="B239" t="s">
-        <v>908</v>
-      </c>
-      <c r="C239" t="s">
-        <v>532</v>
+        <v>517</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B240" t="s">
-        <v>888</v>
+        <v>908</v>
+      </c>
+      <c r="C240" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>454</v>
+        <v>298</v>
       </c>
       <c r="B241" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>300</v>
+        <v>454</v>
       </c>
       <c r="B242" t="s">
-        <v>898</v>
+        <v>889</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B243" t="s">
-        <v>909</v>
+        <v>898</v>
+      </c>
+      <c r="C243" t="s">
+        <v>1148</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B244" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B245" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B246" t="s">
-        <v>824</v>
+        <v>911</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>640</v>
+        <v>304</v>
       </c>
       <c r="B247" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
+        <v>640</v>
+      </c>
+      <c r="B248" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3">
+      <c r="A249" t="s">
         <v>483</v>
       </c>
-      <c r="B248" t="s">
+      <c r="B249" t="s">
         <v>618</v>
-      </c>
-    </row>
-    <row r="250" spans="1:3">
-      <c r="A250" t="s">
-        <v>674</v>
-      </c>
-      <c r="B250" t="s">
-        <v>675</v>
-      </c>
-      <c r="C250" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>500</v>
+        <v>674</v>
       </c>
       <c r="B251" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="C251" t="s">
-        <v>530</v>
+        <v>627</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B252" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C252" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>529</v>
+        <v>501</v>
       </c>
       <c r="B253" t="s">
-        <v>543</v>
+        <v>502</v>
+      </c>
+      <c r="C253" t="s">
+        <v>531</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>321</v>
+        <v>529</v>
       </c>
       <c r="B254" t="s">
-        <v>307</v>
+        <v>543</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B255" t="s">
-        <v>308</v>
-      </c>
-      <c r="C255" t="s">
-        <v>532</v>
+        <v>307</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>462</v>
+        <v>322</v>
       </c>
       <c r="B256" t="s">
-        <v>518</v>
+        <v>308</v>
+      </c>
+      <c r="C256" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>323</v>
+        <v>462</v>
       </c>
       <c r="B257" t="s">
-        <v>309</v>
+        <v>518</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B258" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B259" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B260" t="s">
-        <v>312</v>
-      </c>
-      <c r="C260" t="s">
-        <v>532</v>
+        <v>311</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B261" t="s">
-        <v>313</v>
+        <v>312</v>
+      </c>
+      <c r="C261" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B262" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B263" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B264" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B265" t="s">
-        <v>317</v>
-      </c>
-      <c r="C265" t="s">
-        <v>532</v>
+        <v>316</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B266" t="s">
-        <v>318</v>
+        <v>317</v>
+      </c>
+      <c r="C266" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B267" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B268" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
+        <v>334</v>
+      </c>
+      <c r="B269" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3">
+      <c r="A270" t="s">
         <v>482</v>
       </c>
-      <c r="B269" t="s">
+      <c r="B270" t="s">
         <v>603</v>
-      </c>
-    </row>
-    <row r="271" spans="1:3">
-      <c r="A271" t="s">
-        <v>547</v>
-      </c>
-      <c r="B271" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>341</v>
+        <v>547</v>
       </c>
       <c r="B272" t="s">
-        <v>359</v>
+        <v>548</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B273" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B274" t="s">
-        <v>357</v>
-      </c>
-      <c r="C274" t="s">
-        <v>532</v>
+        <v>356</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>463</v>
+        <v>343</v>
       </c>
       <c r="B275" t="s">
-        <v>519</v>
+        <v>357</v>
+      </c>
+      <c r="C275" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>360</v>
+        <v>463</v>
       </c>
       <c r="B276" t="s">
-        <v>358</v>
-      </c>
-      <c r="C276" t="s">
-        <v>532</v>
+        <v>519</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="B277" t="s">
-        <v>350</v>
+        <v>358</v>
+      </c>
+      <c r="C277" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>361</v>
+        <v>344</v>
       </c>
       <c r="B278" t="s">
-        <v>351</v>
-      </c>
-      <c r="C278" t="s">
-        <v>509</v>
+        <v>350</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="B279" t="s">
-        <v>352</v>
+        <v>351</v>
+      </c>
+      <c r="C279" t="s">
+        <v>509</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B280" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B281" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B282" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B283" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>1073</v>
+        <v>349</v>
       </c>
       <c r="B284" t="s">
-        <v>1074</v>
-      </c>
-      <c r="C284" t="s">
-        <v>1068</v>
+        <v>352</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="B285" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="C285" t="s">
         <v>1068</v>
@@ -10685,10 +10709,10 @@
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="B286" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C286" t="s">
         <v>1068</v>
@@ -10696,40 +10720,40 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B287" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C287" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3">
+      <c r="A288" t="s">
         <v>481</v>
       </c>
-      <c r="B287" t="s">
+      <c r="B288" t="s">
         <v>619</v>
-      </c>
-    </row>
-    <row r="289" spans="1:3">
-      <c r="A289" t="s">
-        <v>676</v>
-      </c>
-      <c r="B289" t="s">
-        <v>695</v>
-      </c>
-      <c r="C289" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>1066</v>
+        <v>676</v>
       </c>
       <c r="B290" t="s">
-        <v>1067</v>
+        <v>695</v>
       </c>
       <c r="C290" t="s">
-        <v>1068</v>
+        <v>627</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="B291" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="C291" t="s">
         <v>1068</v>
@@ -10737,78 +10761,78 @@
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="B292" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="C292" t="s">
         <v>1068</v>
       </c>
     </row>
-    <row r="294" spans="1:3">
-      <c r="A294" t="s">
-        <v>672</v>
-      </c>
-      <c r="B294" t="s">
-        <v>673</v>
-      </c>
-      <c r="C294" t="s">
-        <v>627</v>
+    <row r="293" spans="1:3">
+      <c r="A293" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B293" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C293" t="s">
+        <v>1068</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>472</v>
+        <v>672</v>
       </c>
       <c r="B295" t="s">
-        <v>473</v>
+        <v>673</v>
+      </c>
+      <c r="C295" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>367</v>
+        <v>472</v>
       </c>
       <c r="B296" t="s">
-        <v>378</v>
+        <v>473</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B297" t="s">
-        <v>379</v>
-      </c>
-      <c r="C297" t="s">
-        <v>532</v>
+        <v>378</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>520</v>
+        <v>368</v>
       </c>
       <c r="B298" t="s">
-        <v>521</v>
+        <v>379</v>
+      </c>
+      <c r="C298" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>369</v>
+        <v>520</v>
       </c>
       <c r="B299" t="s">
-        <v>380</v>
-      </c>
-      <c r="C299" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B300" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C300" t="s">
         <v>532</v>
@@ -10816,139 +10840,139 @@
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B301" t="s">
-        <v>533</v>
+        <v>381</v>
+      </c>
+      <c r="C301" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B302" t="s">
-        <v>382</v>
+        <v>533</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B303" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B304" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B305" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B306" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B307" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>731</v>
+        <v>377</v>
       </c>
       <c r="B308" t="s">
-        <v>1145</v>
-      </c>
-      <c r="C308" t="s">
-        <v>627</v>
+        <v>387</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>479</v>
+        <v>731</v>
       </c>
       <c r="B309" t="s">
-        <v>620</v>
+        <v>1145</v>
+      </c>
+      <c r="C309" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
+        <v>479</v>
+      </c>
+      <c r="B310" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3">
+      <c r="A311" t="s">
         <v>556</v>
       </c>
-      <c r="B310" t="s">
+      <c r="B311" t="s">
         <v>557</v>
-      </c>
-    </row>
-    <row r="312" spans="1:3">
-      <c r="A312" t="s">
-        <v>474</v>
-      </c>
-      <c r="B312" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>394</v>
+        <v>474</v>
       </c>
       <c r="B313" t="s">
-        <v>405</v>
+        <v>473</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B314" t="s">
-        <v>406</v>
-      </c>
-      <c r="C314" t="s">
-        <v>532</v>
+        <v>405</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>464</v>
+        <v>395</v>
       </c>
       <c r="B315" t="s">
-        <v>522</v>
+        <v>406</v>
+      </c>
+      <c r="C315" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>396</v>
+        <v>464</v>
       </c>
       <c r="B316" t="s">
-        <v>407</v>
-      </c>
-      <c r="C316" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B317" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C317" t="s">
         <v>532</v>
@@ -10956,1354 +10980,1365 @@
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B318" t="s">
-        <v>534</v>
+        <v>408</v>
+      </c>
+      <c r="C318" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B319" t="s">
-        <v>382</v>
+        <v>534</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B320" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B321" t="s">
-        <v>409</v>
+        <v>383</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B322" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B323" t="s">
-        <v>386</v>
+        <v>410</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B324" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>478</v>
+        <v>404</v>
       </c>
       <c r="B325" t="s">
-        <v>620</v>
+        <v>387</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
+        <v>478</v>
+      </c>
+      <c r="B326" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3">
+      <c r="A327" t="s">
         <v>563</v>
       </c>
-      <c r="B326" t="s">
+      <c r="B327" t="s">
         <v>557</v>
-      </c>
-    </row>
-    <row r="328" spans="1:3">
-      <c r="A328" t="s">
-        <v>670</v>
-      </c>
-      <c r="B328" t="s">
-        <v>671</v>
-      </c>
-      <c r="C328" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>388</v>
+        <v>670</v>
       </c>
       <c r="B329" t="s">
-        <v>564</v>
+        <v>671</v>
+      </c>
+      <c r="C329" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B330" t="s">
-        <v>565</v>
-      </c>
-      <c r="C330" t="s">
-        <v>532</v>
+        <v>564</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>465</v>
+        <v>389</v>
       </c>
       <c r="B331" t="s">
-        <v>566</v>
+        <v>565</v>
+      </c>
+      <c r="C331" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>390</v>
+        <v>465</v>
       </c>
       <c r="B332" t="s">
-        <v>591</v>
+        <v>566</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B333" t="s">
-        <v>567</v>
+        <v>591</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B334" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
+        <v>392</v>
+      </c>
+      <c r="B335" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3">
+      <c r="A336" t="s">
         <v>477</v>
       </c>
-      <c r="B335" t="s">
+      <c r="B336" t="s">
         <v>621</v>
-      </c>
-    </row>
-    <row r="337" spans="1:3">
-      <c r="A337" t="s">
-        <v>746</v>
-      </c>
-      <c r="B337" t="s">
-        <v>747</v>
-      </c>
-      <c r="C337" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="338" spans="1:3">
       <c r="A338" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B338" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="C338" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="340" spans="1:3">
-      <c r="A340" t="s">
-        <v>754</v>
-      </c>
-      <c r="B340" t="s">
-        <v>755</v>
+    <row r="339" spans="1:3">
+      <c r="A339" t="s">
+        <v>748</v>
+      </c>
+      <c r="B339" t="s">
+        <v>749</v>
+      </c>
+      <c r="C339" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="B341" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="B342" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B343" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="B344" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="B345" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B346" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B347" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B348" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B349" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="B350" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B351" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="B352" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="B353" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="B354" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B355" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="B356" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
+        <v>786</v>
+      </c>
+      <c r="B357" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" t="s">
         <v>788</v>
       </c>
-      <c r="B357" t="s">
+      <c r="B358" t="s">
         <v>789</v>
-      </c>
-    </row>
-    <row r="359" spans="1:2">
-      <c r="A359" t="s">
-        <v>790</v>
-      </c>
-      <c r="B359" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B360" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="B361" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B362" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B363" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B364" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="B365" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="B366" t="s">
-        <v>320</v>
+        <v>803</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B367" t="s">
-        <v>806</v>
+        <v>320</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B368" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="B369" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
+        <v>809</v>
+      </c>
+      <c r="B370" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2">
+      <c r="A371" t="s">
         <v>811</v>
       </c>
-      <c r="B370" t="s">
+      <c r="B371" t="s">
         <v>812</v>
-      </c>
-    </row>
-    <row r="372" spans="1:2">
-      <c r="A372" t="s">
-        <v>813</v>
-      </c>
-      <c r="B372" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B373" t="s">
-        <v>815</v>
+        <v>313</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="B374" t="s">
-        <v>315</v>
+        <v>815</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
+        <v>816</v>
+      </c>
+      <c r="B375" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" t="s">
         <v>817</v>
       </c>
-      <c r="B375" t="s">
+      <c r="B376" t="s">
         <v>316</v>
-      </c>
-    </row>
-    <row r="377" spans="1:2">
-      <c r="A377" t="s">
-        <v>842</v>
-      </c>
-      <c r="B377" t="s">
-        <v>843</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="B378" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="B379" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B380" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B381" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
+        <v>833</v>
+      </c>
+      <c r="B382" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" t="s">
         <v>839</v>
       </c>
-      <c r="B382" t="s">
+      <c r="B383" t="s">
         <v>838</v>
-      </c>
-    </row>
-    <row r="384" spans="1:2">
-      <c r="A384" t="s">
-        <v>846</v>
-      </c>
-      <c r="B384" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>854</v>
+        <v>846</v>
       </c>
       <c r="B385" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
       <c r="B386" t="s">
-        <v>835</v>
+        <v>852</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B387" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B388" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
+        <v>849</v>
+      </c>
+      <c r="B389" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2">
+      <c r="A390" t="s">
         <v>850</v>
       </c>
-      <c r="B389" t="s">
+      <c r="B390" t="s">
         <v>853</v>
-      </c>
-    </row>
-    <row r="391" spans="1:2">
-      <c r="A391" t="s">
-        <v>859</v>
-      </c>
-      <c r="B391" t="s">
-        <v>860</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="B392" t="s">
-        <v>1137</v>
+        <v>860</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B393" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B394" t="s">
-        <v>1129</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
       <c r="B395" t="s">
-        <v>1115</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B396" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B397" t="s">
-        <v>1135</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="B398" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B399" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B400" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B401" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B402" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B403" t="s">
-        <v>869</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B404" t="s">
-        <v>1138</v>
+        <v>869</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B405" t="s">
-        <v>280</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B406" t="s">
-        <v>825</v>
+        <v>280</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="B407" t="s">
-        <v>633</v>
+        <v>825</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B408" t="s">
-        <v>1139</v>
+        <v>633</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>1119</v>
+        <v>873</v>
       </c>
       <c r="B409" t="s">
-        <v>1117</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="B410" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="B411" t="s">
-        <v>1121</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
       <c r="B412" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B413" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B414" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1141</v>
+        <v>1128</v>
       </c>
       <c r="B415" t="s">
-        <v>1140</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B416" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="417" spans="1:2">
+      <c r="A417" t="s">
         <v>1142</v>
       </c>
-      <c r="B416" t="s">
+      <c r="B417" t="s">
         <v>1143</v>
-      </c>
-    </row>
-    <row r="418" spans="1:2">
-      <c r="A418" t="s">
-        <v>947</v>
-      </c>
-      <c r="B418" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>966</v>
+        <v>947</v>
       </c>
       <c r="B419" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B420" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B421" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="B422" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B423" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B424" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B425" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="B426" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B427" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B428" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>967</v>
+        <v>957</v>
       </c>
       <c r="B429" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>956</v>
+        <v>967</v>
       </c>
       <c r="B430" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B431" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B432" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B433" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B434" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B435" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B436" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B437" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
+        <v>949</v>
+      </c>
+      <c r="B438" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2">
+      <c r="A439" t="s">
         <v>948</v>
       </c>
-      <c r="B438" t="s">
+      <c r="B439" t="s">
         <v>946</v>
-      </c>
-    </row>
-    <row r="440" spans="1:2">
-      <c r="A440" t="s">
-        <v>989</v>
-      </c>
-      <c r="B440" t="s">
-        <v>970</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>980</v>
+        <v>989</v>
       </c>
       <c r="B441" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B442" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B443" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="B444" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="B445" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="B446" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="B447" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="B448" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
+        <v>988</v>
+      </c>
+      <c r="B449" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2">
+      <c r="A450" t="s">
         <v>987</v>
       </c>
-      <c r="B449" t="s">
+      <c r="B450" t="s">
         <v>979</v>
-      </c>
-    </row>
-    <row r="451" spans="1:2">
-      <c r="A451" t="s">
-        <v>994</v>
-      </c>
-      <c r="B451" t="s">
-        <v>996</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
+        <v>994</v>
+      </c>
+      <c r="B452" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="453" spans="1:2">
+      <c r="A453" t="s">
         <v>1005</v>
       </c>
-      <c r="B452" t="s">
+      <c r="B453" t="s">
         <v>1006</v>
-      </c>
-    </row>
-    <row r="454" spans="1:2">
-      <c r="A454" t="s">
-        <v>995</v>
-      </c>
-      <c r="B454" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
+        <v>995</v>
+      </c>
+      <c r="B455" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2">
+      <c r="A456" t="s">
         <v>1007</v>
       </c>
-      <c r="B455" t="s">
+      <c r="B456" t="s">
         <v>1008</v>
-      </c>
-    </row>
-    <row r="457" spans="1:2">
-      <c r="A457" t="s">
-        <v>1002</v>
-      </c>
-      <c r="B457" t="s">
-        <v>1000</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B458" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B459" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="460" spans="1:2">
+      <c r="A460" t="s">
         <v>999</v>
       </c>
-      <c r="B459" t="s">
+      <c r="B460" t="s">
         <v>1004</v>
-      </c>
-    </row>
-    <row r="461" spans="1:2">
-      <c r="A461" t="s">
-        <v>1017</v>
-      </c>
-      <c r="B461" t="s">
-        <v>1010</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B462" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="B463" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1065</v>
+        <v>1019</v>
       </c>
       <c r="B464" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1020</v>
+        <v>1065</v>
       </c>
       <c r="B465" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B466" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B467" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" t="s">
         <v>1022</v>
       </c>
-      <c r="B467" t="s">
+      <c r="B468" t="s">
         <v>1016</v>
-      </c>
-    </row>
-    <row r="469" spans="1:2">
-      <c r="A469" t="s">
-        <v>1034</v>
-      </c>
-      <c r="B469" t="s">
-        <v>1028</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1039</v>
+        <v>1034</v>
       </c>
       <c r="B470" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="B471" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B472" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B473" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="474" spans="1:2">
       <c r="A474" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B474" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2">
+      <c r="A475" t="s">
         <v>1037</v>
       </c>
-      <c r="B474" t="s">
+      <c r="B475" t="s">
         <v>1033</v>
-      </c>
-    </row>
-    <row r="476" spans="1:2">
-      <c r="A476" t="s">
-        <v>1052</v>
-      </c>
-      <c r="B476" t="s">
-        <v>1040</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="B477" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B478" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B479" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B480" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B481" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2">
+      <c r="A482" t="s">
         <v>1051</v>
       </c>
-      <c r="B481" t="s">
+      <c r="B482" t="s">
         <v>1045</v>
-      </c>
-    </row>
-    <row r="483" spans="1:2">
-      <c r="A483" t="s">
-        <v>1053</v>
-      </c>
-      <c r="B483" t="s">
-        <v>1054</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>1059</v>
+        <v>1053</v>
       </c>
       <c r="B484" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B485" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B486" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2">
+      <c r="A488" t="s">
         <v>1062</v>
       </c>
-      <c r="B487" t="s">
+      <c r="B488" t="s">
         <v>1058</v>
-      </c>
-    </row>
-    <row r="489" spans="1:2">
-      <c r="A489" t="s">
-        <v>1087</v>
-      </c>
-      <c r="B489" t="s">
-        <v>1088</v>
       </c>
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
-        <v>1103</v>
+        <v>1087</v>
       </c>
       <c r="B490" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B491" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B492" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1114</v>
+        <v>1105</v>
       </c>
       <c r="B493" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1106</v>
+        <v>1114</v>
       </c>
       <c r="B494" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B495" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B496" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B497" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B498" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B499" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B500" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B501" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B502" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="503" spans="1:2">
+      <c r="A503" t="s">
         <v>1102</v>
       </c>
-      <c r="B502" t="s">
+      <c r="B503" t="s">
         <v>1101</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A457:A458 A454:A455 A440:A449 A451:A452">
+  <conditionalFormatting sqref="A458:A459 A455:A456 A441:A450 A452:A453">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated the config file
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE59049-4A7D-4951-9F72-96C344290B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C43836E-C948-4CDD-A47C-6E3CABE3FF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3234,9 +3234,6 @@
     <t>VSA</t>
   </si>
   <si>
-    <t>Verification Services (Assets)</t>
-  </si>
-  <si>
     <t>RCF_Signed</t>
   </si>
   <si>
@@ -3499,6 +3496,9 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>Verification Services Assets</t>
   </si>
 </sst>
 </file>
@@ -3967,7 +3967,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4378,15 +4378,15 @@
         <v>1063</v>
       </c>
       <c r="B57" t="s">
-        <v>1064</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B58" t="s">
         <v>1085</v>
-      </c>
-      <c r="B58" t="s">
-        <v>1086</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
@@ -7333,34 +7333,34 @@
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B44" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B45" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B46" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B47" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8546,7 +8546,7 @@
         <v>738</v>
       </c>
       <c r="B24" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="C24" t="s">
         <v>627</v>
@@ -8795,10 +8795,10 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B56" t="s">
         <v>1079</v>
-      </c>
-      <c r="B56" t="s">
-        <v>1080</v>
       </c>
     </row>
     <row r="57" spans="1:3">
@@ -9053,7 +9053,7 @@
         <v>185</v>
       </c>
       <c r="B86" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -9712,13 +9712,13 @@
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="B166" t="s">
         <v>898</v>
       </c>
       <c r="C166" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="168" spans="1:3">
@@ -9816,7 +9816,7 @@
         <v>898</v>
       </c>
       <c r="C177" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -9859,7 +9859,7 @@
         <v>898</v>
       </c>
       <c r="C182" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -9875,7 +9875,7 @@
         <v>595</v>
       </c>
       <c r="B184" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -10094,7 +10094,7 @@
         <v>898</v>
       </c>
       <c r="C209" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -10354,7 +10354,7 @@
         <v>898</v>
       </c>
       <c r="C243" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -10698,35 +10698,35 @@
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B285" t="s">
         <v>1073</v>
       </c>
-      <c r="B285" t="s">
-        <v>1074</v>
-      </c>
       <c r="C285" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B286" t="s">
         <v>1075</v>
       </c>
-      <c r="B286" t="s">
-        <v>1076</v>
-      </c>
       <c r="C286" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B287" t="s">
         <v>1077</v>
       </c>
-      <c r="B287" t="s">
-        <v>1078</v>
-      </c>
       <c r="C287" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="288" spans="1:3">
@@ -10750,35 +10750,35 @@
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B291" t="s">
         <v>1066</v>
       </c>
-      <c r="B291" t="s">
+      <c r="C291" t="s">
         <v>1067</v>
-      </c>
-      <c r="C291" t="s">
-        <v>1068</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B292" t="s">
         <v>1069</v>
       </c>
-      <c r="B292" t="s">
-        <v>1070</v>
-      </c>
       <c r="C292" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B293" t="s">
         <v>1071</v>
       </c>
-      <c r="B293" t="s">
-        <v>1072</v>
-      </c>
       <c r="C293" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="295" spans="1:3">
@@ -10910,7 +10910,7 @@
         <v>731</v>
       </c>
       <c r="B309" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="C309" t="s">
         <v>627</v>
@@ -11534,7 +11534,7 @@
         <v>861</v>
       </c>
       <c r="B393" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="394" spans="1:2">
@@ -11542,7 +11542,7 @@
         <v>862</v>
       </c>
       <c r="B394" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="395" spans="1:2">
@@ -11550,7 +11550,7 @@
         <v>864</v>
       </c>
       <c r="B395" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="396" spans="1:2">
@@ -11558,7 +11558,7 @@
         <v>870</v>
       </c>
       <c r="B396" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="397" spans="1:2">
@@ -11566,7 +11566,7 @@
         <v>871</v>
       </c>
       <c r="B397" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="398" spans="1:2">
@@ -11574,7 +11574,7 @@
         <v>872</v>
       </c>
       <c r="B398" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="399" spans="1:2">
@@ -11582,7 +11582,7 @@
         <v>875</v>
       </c>
       <c r="B399" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="400" spans="1:2">
@@ -11590,7 +11590,7 @@
         <v>876</v>
       </c>
       <c r="B400" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="401" spans="1:2">
@@ -11598,7 +11598,7 @@
         <v>877</v>
       </c>
       <c r="B401" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="402" spans="1:2">
@@ -11606,7 +11606,7 @@
         <v>878</v>
       </c>
       <c r="B402" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="403" spans="1:2">
@@ -11614,7 +11614,7 @@
         <v>879</v>
       </c>
       <c r="B403" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="404" spans="1:2">
@@ -11630,7 +11630,7 @@
         <v>881</v>
       </c>
       <c r="B405" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="406" spans="1:2">
@@ -11662,71 +11662,71 @@
         <v>873</v>
       </c>
       <c r="B409" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B410" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="B411" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B412" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B413" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B414" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B415" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B416" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
+        <v>1141</v>
+      </c>
+      <c r="B417" t="s">
         <v>1142</v>
-      </c>
-      <c r="B417" t="s">
-        <v>1143</v>
       </c>
     </row>
     <row r="419" spans="1:2">
@@ -12059,7 +12059,7 @@
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B465" t="s">
         <v>1013</v>
@@ -12227,114 +12227,114 @@
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B490" t="s">
         <v>1087</v>
-      </c>
-      <c r="B490" t="s">
-        <v>1088</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B491" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B492" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B493" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B494" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B495" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B496" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B497" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B498" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B499" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B500" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B501" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="B502" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B503" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update to CZI DU replacement, HHD
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C43836E-C948-4CDD-A47C-6E3CABE3FF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144BF75E-F8A8-42D4-BCB2-40BB639D3BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3495,10 +3495,10 @@
     <t>Implementing this only in EDC.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Verification Services Assets</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3967,7 +3967,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4378,7 +4378,7 @@
         <v>1063</v>
       </c>
       <c r="B57" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
changes to AS, HHD, and DU TXSpecificAll - IAQ, MID, ACNFA, and EV
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144BF75E-F8A8-42D4-BCB2-40BB639D3BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7E911AA-79E9-4EF2-B859-8DFFED2CBDFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="28260" windowHeight="13665" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3498,7 +3498,7 @@
     <t>Verification Services Assets</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
updated VSA and a check in ScheduleC
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A11D5C9-D271-42B2-91BE-F5E3B9D60A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2DD4DE-F87F-4A0E-AE00-0127DEC5F757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="1153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="1155">
   <si>
     <t>Name</t>
   </si>
@@ -3499,6 +3499,12 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>TX_VSACheck</t>
+  </si>
+  <si>
+    <t>TX_TSAHCCheck</t>
   </si>
 </sst>
 </file>
@@ -7363,23 +7369,37 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
+    <row r="48" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A48" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A49" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Updtated CSS and CSEI check
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2DD4DE-F87F-4A0E-AE00-0127DEC5F757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E313ABC-C580-4E6E-B72D-4FE96AD6A4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="1155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="1157">
   <si>
     <t>Name</t>
   </si>
@@ -3498,13 +3498,19 @@
     <t>Verification Services Assets</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>TX_VSACheck</t>
   </si>
   <si>
     <t>TX_TSAHCCheck</t>
+  </si>
+  <si>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>CSEI_ScheduleCCountCheck</t>
+  </si>
+  <si>
+    <t>There are more Schedule Cs than CSEI</t>
   </si>
 </sst>
 </file>
@@ -3973,7 +3979,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1152</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7371,18 +7377,18 @@
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B48" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B49" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8357,7 +8363,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C503"/>
+  <dimension ref="A1:C504"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -11303,1062 +11309,1070 @@
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>786</v>
+        <v>1155</v>
       </c>
       <c r="B357" t="s">
-        <v>787</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
+        <v>786</v>
+      </c>
+      <c r="B358" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="A359" t="s">
         <v>788</v>
       </c>
-      <c r="B358" t="s">
+      <c r="B359" t="s">
         <v>789</v>
-      </c>
-    </row>
-    <row r="360" spans="1:2">
-      <c r="A360" t="s">
-        <v>790</v>
-      </c>
-      <c r="B360" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B361" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="B362" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B363" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B364" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B365" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="B366" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="B367" t="s">
-        <v>320</v>
+        <v>803</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B368" t="s">
-        <v>806</v>
+        <v>320</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B369" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="B370" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
+        <v>809</v>
+      </c>
+      <c r="B371" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2">
+      <c r="A372" t="s">
         <v>811</v>
       </c>
-      <c r="B371" t="s">
+      <c r="B372" t="s">
         <v>812</v>
-      </c>
-    </row>
-    <row r="373" spans="1:2">
-      <c r="A373" t="s">
-        <v>813</v>
-      </c>
-      <c r="B373" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B374" t="s">
-        <v>815</v>
+        <v>313</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="B375" t="s">
-        <v>315</v>
+        <v>815</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
+        <v>816</v>
+      </c>
+      <c r="B376" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2">
+      <c r="A377" t="s">
         <v>817</v>
       </c>
-      <c r="B376" t="s">
+      <c r="B377" t="s">
         <v>316</v>
-      </c>
-    </row>
-    <row r="378" spans="1:2">
-      <c r="A378" t="s">
-        <v>842</v>
-      </c>
-      <c r="B378" t="s">
-        <v>843</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="B379" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="B380" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B381" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B382" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
+        <v>833</v>
+      </c>
+      <c r="B383" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2">
+      <c r="A384" t="s">
         <v>839</v>
       </c>
-      <c r="B383" t="s">
+      <c r="B384" t="s">
         <v>838</v>
-      </c>
-    </row>
-    <row r="385" spans="1:2">
-      <c r="A385" t="s">
-        <v>846</v>
-      </c>
-      <c r="B385" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>854</v>
+        <v>846</v>
       </c>
       <c r="B386" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
       <c r="B387" t="s">
-        <v>835</v>
+        <v>852</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B388" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B389" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
+        <v>849</v>
+      </c>
+      <c r="B390" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" t="s">
         <v>850</v>
       </c>
-      <c r="B390" t="s">
+      <c r="B391" t="s">
         <v>853</v>
-      </c>
-    </row>
-    <row r="392" spans="1:2">
-      <c r="A392" t="s">
-        <v>859</v>
-      </c>
-      <c r="B392" t="s">
-        <v>860</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="B393" t="s">
-        <v>1136</v>
+        <v>860</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B394" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B395" t="s">
-        <v>1128</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
       <c r="B396" t="s">
-        <v>1114</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B397" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B398" t="s">
-        <v>1134</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="B399" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B400" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B401" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B402" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B403" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B404" t="s">
-        <v>869</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B405" t="s">
-        <v>1137</v>
+        <v>869</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B406" t="s">
-        <v>280</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B407" t="s">
-        <v>825</v>
+        <v>280</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="B408" t="s">
-        <v>633</v>
+        <v>825</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B409" t="s">
-        <v>1138</v>
+        <v>633</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>1118</v>
+        <v>873</v>
       </c>
       <c r="B410" t="s">
-        <v>1116</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B411" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="B412" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
       <c r="B413" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B414" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B415" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1140</v>
+        <v>1127</v>
       </c>
       <c r="B416" t="s">
-        <v>1139</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B417" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="418" spans="1:2">
+      <c r="A418" t="s">
         <v>1141</v>
       </c>
-      <c r="B417" t="s">
+      <c r="B418" t="s">
         <v>1142</v>
-      </c>
-    </row>
-    <row r="419" spans="1:2">
-      <c r="A419" t="s">
-        <v>947</v>
-      </c>
-      <c r="B419" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>966</v>
+        <v>947</v>
       </c>
       <c r="B420" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B421" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B422" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="B423" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B424" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B425" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B426" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="B427" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B428" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B429" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>967</v>
+        <v>957</v>
       </c>
       <c r="B430" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>956</v>
+        <v>967</v>
       </c>
       <c r="B431" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B432" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B433" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B434" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B435" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B436" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B437" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B438" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
+        <v>949</v>
+      </c>
+      <c r="B439" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2">
+      <c r="A440" t="s">
         <v>948</v>
       </c>
-      <c r="B439" t="s">
+      <c r="B440" t="s">
         <v>946</v>
-      </c>
-    </row>
-    <row r="441" spans="1:2">
-      <c r="A441" t="s">
-        <v>989</v>
-      </c>
-      <c r="B441" t="s">
-        <v>970</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>980</v>
+        <v>989</v>
       </c>
       <c r="B442" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B443" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B444" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="B445" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="B446" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="B447" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="B448" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="B449" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
+        <v>988</v>
+      </c>
+      <c r="B450" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" t="s">
         <v>987</v>
       </c>
-      <c r="B450" t="s">
+      <c r="B451" t="s">
         <v>979</v>
-      </c>
-    </row>
-    <row r="452" spans="1:2">
-      <c r="A452" t="s">
-        <v>994</v>
-      </c>
-      <c r="B452" t="s">
-        <v>996</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
+        <v>994</v>
+      </c>
+      <c r="B453" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2">
+      <c r="A454" t="s">
         <v>1005</v>
       </c>
-      <c r="B453" t="s">
+      <c r="B454" t="s">
         <v>1006</v>
-      </c>
-    </row>
-    <row r="455" spans="1:2">
-      <c r="A455" t="s">
-        <v>995</v>
-      </c>
-      <c r="B455" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
+        <v>995</v>
+      </c>
+      <c r="B456" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
         <v>1007</v>
       </c>
-      <c r="B456" t="s">
+      <c r="B457" t="s">
         <v>1008</v>
-      </c>
-    </row>
-    <row r="458" spans="1:2">
-      <c r="A458" t="s">
-        <v>1002</v>
-      </c>
-      <c r="B458" t="s">
-        <v>1000</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B459" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B460" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" t="s">
         <v>999</v>
       </c>
-      <c r="B460" t="s">
+      <c r="B461" t="s">
         <v>1004</v>
-      </c>
-    </row>
-    <row r="462" spans="1:2">
-      <c r="A462" t="s">
-        <v>1017</v>
-      </c>
-      <c r="B462" t="s">
-        <v>1010</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B463" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="B464" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1064</v>
+        <v>1019</v>
       </c>
       <c r="B465" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>1020</v>
+        <v>1064</v>
       </c>
       <c r="B466" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B467" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B468" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2">
+      <c r="A469" t="s">
         <v>1022</v>
       </c>
-      <c r="B468" t="s">
+      <c r="B469" t="s">
         <v>1016</v>
-      </c>
-    </row>
-    <row r="470" spans="1:2">
-      <c r="A470" t="s">
-        <v>1034</v>
-      </c>
-      <c r="B470" t="s">
-        <v>1028</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1039</v>
+        <v>1034</v>
       </c>
       <c r="B471" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="B472" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B473" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="474" spans="1:2">
       <c r="A474" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B474" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B475" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" t="s">
         <v>1037</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B476" t="s">
         <v>1033</v>
-      </c>
-    </row>
-    <row r="477" spans="1:2">
-      <c r="A477" t="s">
-        <v>1052</v>
-      </c>
-      <c r="B477" t="s">
-        <v>1040</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="B478" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B479" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B480" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B481" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B482" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2">
+      <c r="A483" t="s">
         <v>1051</v>
       </c>
-      <c r="B482" t="s">
+      <c r="B483" t="s">
         <v>1045</v>
-      </c>
-    </row>
-    <row r="484" spans="1:2">
-      <c r="A484" t="s">
-        <v>1053</v>
-      </c>
-      <c r="B484" t="s">
-        <v>1054</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1059</v>
+        <v>1053</v>
       </c>
       <c r="B485" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B486" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B487" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B488" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" t="s">
         <v>1062</v>
       </c>
-      <c r="B488" t="s">
+      <c r="B489" t="s">
         <v>1058</v>
-      </c>
-    </row>
-    <row r="490" spans="1:2">
-      <c r="A490" t="s">
-        <v>1086</v>
-      </c>
-      <c r="B490" t="s">
-        <v>1087</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1102</v>
+        <v>1086</v>
       </c>
       <c r="B491" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B492" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B493" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1113</v>
+        <v>1104</v>
       </c>
       <c r="B494" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1105</v>
+        <v>1113</v>
       </c>
       <c r="B495" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B496" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B497" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B498" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B499" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B500" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B501" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B502" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B503" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="504" spans="1:2">
+      <c r="A504" t="s">
         <v>1101</v>
       </c>
-      <c r="B503" t="s">
+      <c r="B504" t="s">
         <v>1100</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A458:A459 A455:A456 A441:A450 A452:A453">
+  <conditionalFormatting sqref="A459:A460 A456:A457 A442:A451 A453:A454">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
changes for VSA and BS
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E313ABC-C580-4E6E-B72D-4FE96AD6A4EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A775C07F-0F6E-4E90-8583-9A8E9677489D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3504,13 +3504,13 @@
     <t>TX_TSAHCCheck</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>CSEI_ScheduleCCountCheck</t>
   </si>
   <si>
     <t>There are more Schedule Cs than CSEI</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3979,7 +3979,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1154</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -11309,10 +11309,10 @@
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B357" t="s">
         <v>1155</v>
-      </c>
-      <c r="B357" t="s">
-        <v>1156</v>
       </c>
     </row>
     <row r="358" spans="1:2">

</xml_diff>

<commit_message>
changed the VS to not add the finding
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A775C07F-0F6E-4E90-8583-9A8E9677489D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F24B81-8DFA-43DB-B6C5-BCB0EAE0CAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="1157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="1159">
   <si>
     <t>Name</t>
   </si>
@@ -3511,6 +3511,12 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>VSI</t>
+  </si>
+  <si>
+    <t>Verification Services Income</t>
   </si>
 </sst>
 </file>
@@ -3897,7 +3903,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1003"/>
+  <dimension ref="A1:Z1004"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -4395,13 +4401,20 @@
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1158</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A59" t="s">
         <v>1084</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B59" t="s">
         <v>1085</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="60" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5346,6 +5359,7 @@
     <row r="1001" ht="14.25" customHeight="1"/>
     <row r="1002" ht="14.25" customHeight="1"/>
     <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated the CZI and IAQ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66F24B81-8DFA-43DB-B6C5-BCB0EAE0CAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBBFCB9-F16F-415F-80B5-D5BE983FDE59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="1159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="1161">
   <si>
     <t>Name</t>
   </si>
@@ -3517,6 +3517,12 @@
   </si>
   <si>
     <t>Verification Services Income</t>
+  </si>
+  <si>
+    <t>CZI_PartAYes</t>
+  </si>
+  <si>
+    <t>One adult answered "Yes" to a question in section A.</t>
   </si>
 </sst>
 </file>
@@ -8377,7 +8383,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C504"/>
+  <dimension ref="A1:C505"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -9546,96 +9552,96 @@
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>587</v>
+        <v>1159</v>
       </c>
       <c r="B141" t="s">
-        <v>588</v>
+        <v>1160</v>
+      </c>
+      <c r="C141" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
+        <v>587</v>
+      </c>
+      <c r="B142" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3">
+      <c r="A143" t="s">
         <v>488</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B143" t="s">
         <v>611</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3">
-      <c r="A144" t="s">
-        <v>190</v>
-      </c>
-      <c r="B144" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>165</v>
+        <v>190</v>
       </c>
       <c r="B145" t="s">
-        <v>167</v>
+        <v>191</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B146" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>583</v>
+        <v>166</v>
       </c>
       <c r="B147" t="s">
-        <v>584</v>
+        <v>168</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>487</v>
+        <v>583</v>
       </c>
       <c r="B148" t="s">
-        <v>612</v>
+        <v>584</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
+        <v>487</v>
+      </c>
+      <c r="B149" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3">
+      <c r="A150" t="s">
         <v>656</v>
       </c>
-      <c r="B149" t="s">
+      <c r="B150" t="s">
         <v>657</v>
       </c>
-      <c r="C149" t="s">
+      <c r="C150" t="s">
         <v>627</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3">
-      <c r="A151" t="s">
-        <v>188</v>
-      </c>
-      <c r="B151" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="B152" t="s">
-        <v>171</v>
-      </c>
-      <c r="C152" t="s">
-        <v>532</v>
+        <v>189</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B153" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C153" t="s">
         <v>532</v>
@@ -9643,10 +9649,10 @@
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B154" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C154" t="s">
         <v>532</v>
@@ -9654,75 +9660,75 @@
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="B155" t="s">
-        <v>198</v>
+        <v>173</v>
+      </c>
+      <c r="C155" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B156" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
       <c r="B157" t="s">
-        <v>176</v>
-      </c>
-      <c r="C157" t="s">
-        <v>532</v>
+        <v>197</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>585</v>
+        <v>175</v>
       </c>
       <c r="B158" t="s">
-        <v>586</v>
+        <v>176</v>
+      </c>
+      <c r="C158" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
+        <v>585</v>
+      </c>
+      <c r="B159" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3">
+      <c r="A160" t="s">
         <v>476</v>
       </c>
-      <c r="B159" t="s">
+      <c r="B160" t="s">
         <v>613</v>
-      </c>
-    </row>
-    <row r="161" spans="1:3">
-      <c r="A161" t="s">
-        <v>592</v>
-      </c>
-      <c r="B161" t="s">
-        <v>890</v>
-      </c>
-      <c r="C161" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>659</v>
+        <v>592</v>
       </c>
       <c r="B162" t="s">
-        <v>660</v>
+        <v>890</v>
       </c>
       <c r="C162" t="s">
-        <v>627</v>
+        <v>593</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>750</v>
+        <v>659</v>
       </c>
       <c r="B163" t="s">
-        <v>891</v>
+        <v>660</v>
       </c>
       <c r="C163" t="s">
         <v>627</v>
@@ -9730,10 +9736,10 @@
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B164" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="C164" t="s">
         <v>627</v>
@@ -9741,10 +9747,10 @@
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B165" t="s">
-        <v>733</v>
+        <v>892</v>
       </c>
       <c r="C165" t="s">
         <v>627</v>
@@ -9752,40 +9758,40 @@
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
+        <v>752</v>
+      </c>
+      <c r="B166" t="s">
+        <v>733</v>
+      </c>
+      <c r="C166" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3">
+      <c r="A167" t="s">
         <v>1148</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B167" t="s">
         <v>898</v>
       </c>
-      <c r="C166" t="s">
+      <c r="C167" t="s">
         <v>1149</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3">
-      <c r="A168" t="s">
-        <v>467</v>
-      </c>
-      <c r="B168" t="s">
-        <v>893</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>598</v>
+        <v>467</v>
       </c>
       <c r="B169" t="s">
-        <v>602</v>
-      </c>
-      <c r="C169" t="s">
-        <v>600</v>
+        <v>893</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B170" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C170" t="s">
         <v>600</v>
@@ -9793,156 +9799,156 @@
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>238</v>
+        <v>599</v>
       </c>
       <c r="B171" t="s">
-        <v>894</v>
+        <v>601</v>
       </c>
       <c r="C171" t="s">
-        <v>532</v>
+        <v>600</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B172" t="s">
-        <v>895</v>
+        <v>894</v>
+      </c>
+      <c r="C172" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="B173" t="s">
-        <v>896</v>
-      </c>
-      <c r="C173" t="s">
-        <v>590</v>
+        <v>895</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>717</v>
+        <v>247</v>
       </c>
       <c r="B174" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="C174" t="s">
-        <v>627</v>
+        <v>590</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>241</v>
+        <v>717</v>
       </c>
       <c r="B175" t="s">
-        <v>240</v>
+        <v>897</v>
+      </c>
+      <c r="C175" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>457</v>
+        <v>241</v>
       </c>
       <c r="B176" t="s">
-        <v>466</v>
+        <v>240</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>242</v>
+        <v>457</v>
       </c>
       <c r="B177" t="s">
-        <v>898</v>
-      </c>
-      <c r="C177" t="s">
-        <v>1150</v>
+        <v>466</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B178" t="s">
-        <v>899</v>
+        <v>898</v>
+      </c>
+      <c r="C178" t="s">
+        <v>1150</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B179" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B180" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B181" t="s">
-        <v>824</v>
+        <v>901</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>278</v>
+        <v>246</v>
       </c>
       <c r="B182" t="s">
-        <v>898</v>
-      </c>
-      <c r="C182" t="s">
-        <v>1150</v>
+        <v>824</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>305</v>
+        <v>278</v>
       </c>
       <c r="B183" t="s">
-        <v>306</v>
+        <v>898</v>
+      </c>
+      <c r="C183" t="s">
+        <v>1150</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>595</v>
+        <v>305</v>
       </c>
       <c r="B184" t="s">
-        <v>1145</v>
+        <v>306</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>636</v>
+        <v>595</v>
       </c>
       <c r="B185" t="s">
-        <v>825</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>703</v>
+        <v>636</v>
       </c>
       <c r="B186" t="s">
-        <v>704</v>
-      </c>
-      <c r="C186" t="s">
-        <v>627</v>
+        <v>825</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>716</v>
+        <v>703</v>
       </c>
       <c r="B187" t="s">
-        <v>735</v>
+        <v>704</v>
       </c>
       <c r="C187" t="s">
         <v>627</v>
@@ -9950,809 +9956,809 @@
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>912</v>
+        <v>716</v>
       </c>
       <c r="B188" t="s">
-        <v>913</v>
+        <v>735</v>
+      </c>
+      <c r="C188" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
+        <v>912</v>
+      </c>
+      <c r="B189" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3">
+      <c r="A190" t="s">
         <v>475</v>
       </c>
-      <c r="B189" t="s">
+      <c r="B190" t="s">
         <v>614</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3">
-      <c r="A191" t="s">
-        <v>714</v>
-      </c>
-      <c r="B191" t="s">
-        <v>715</v>
-      </c>
-      <c r="C191" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>468</v>
+        <v>714</v>
       </c>
       <c r="B192" t="s">
-        <v>902</v>
+        <v>715</v>
+      </c>
+      <c r="C192" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
+        <v>468</v>
+      </c>
+      <c r="B193" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3">
+      <c r="A194" t="s">
         <v>248</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B194" t="s">
         <v>903</v>
       </c>
-      <c r="C193" t="s">
+      <c r="C194" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="194" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A194" t="s">
+    <row r="195" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A195" t="s">
         <v>250</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B195" t="s">
         <v>904</v>
       </c>
-      <c r="C194" t="s">
+      <c r="C195" t="s">
         <v>631</v>
-      </c>
-    </row>
-    <row r="195" spans="1:3">
-      <c r="A195" t="s">
-        <v>249</v>
-      </c>
-      <c r="B195" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B196" t="s">
-        <v>251</v>
+        <v>863</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B197" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B198" t="s">
-        <v>255</v>
-      </c>
-      <c r="C198" t="s">
-        <v>597</v>
+        <v>254</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>458</v>
+        <v>256</v>
       </c>
       <c r="B199" t="s">
-        <v>514</v>
+        <v>255</v>
+      </c>
+      <c r="C199" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>257</v>
+        <v>458</v>
       </c>
       <c r="B200" t="s">
-        <v>865</v>
+        <v>514</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B201" t="s">
-        <v>259</v>
+        <v>865</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B202" t="s">
-        <v>866</v>
+        <v>259</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B203" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B204" t="s">
-        <v>905</v>
-      </c>
-      <c r="C204" t="s">
-        <v>597</v>
+        <v>867</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B205" t="s">
-        <v>868</v>
+        <v>905</v>
+      </c>
+      <c r="C205" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B206" t="s">
-        <v>906</v>
-      </c>
-      <c r="C206" t="s">
-        <v>597</v>
+        <v>868</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B207" t="s">
-        <v>869</v>
+        <v>906</v>
+      </c>
+      <c r="C207" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B208" t="s">
-        <v>276</v>
+        <v>869</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B209" t="s">
-        <v>898</v>
-      </c>
-      <c r="C209" t="s">
-        <v>1150</v>
+        <v>276</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B210" t="s">
-        <v>280</v>
+        <v>898</v>
+      </c>
+      <c r="C210" t="s">
+        <v>1150</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>637</v>
+        <v>279</v>
       </c>
       <c r="B211" t="s">
-        <v>825</v>
+        <v>280</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>486</v>
+        <v>637</v>
       </c>
       <c r="B212" t="s">
-        <v>615</v>
+        <v>825</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
+        <v>486</v>
+      </c>
+      <c r="B213" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3">
+      <c r="A214" t="s">
         <v>632</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B214" t="s">
         <v>633</v>
       </c>
-      <c r="C213" t="s">
+      <c r="C214" t="s">
         <v>627</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3">
-      <c r="A215" t="s">
-        <v>469</v>
-      </c>
-      <c r="B215" t="s">
-        <v>826</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>459</v>
+        <v>469</v>
       </c>
       <c r="B216" t="s">
-        <v>515</v>
+        <v>826</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>273</v>
+        <v>459</v>
       </c>
       <c r="B217" t="s">
-        <v>827</v>
+        <v>515</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B218" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="B219" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B220" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B221" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>638</v>
+        <v>283</v>
       </c>
       <c r="B222" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
+        <v>638</v>
+      </c>
+      <c r="B223" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3">
+      <c r="A224" t="s">
         <v>485</v>
       </c>
-      <c r="B223" t="s">
+      <c r="B224" t="s">
         <v>616</v>
-      </c>
-    </row>
-    <row r="225" spans="1:3">
-      <c r="A225" t="s">
-        <v>470</v>
-      </c>
-      <c r="B225" t="s">
-        <v>818</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="B226" t="s">
-        <v>516</v>
+        <v>818</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>286</v>
+        <v>460</v>
       </c>
       <c r="B227" t="s">
-        <v>819</v>
+        <v>516</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B228" t="s">
-        <v>289</v>
+        <v>819</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B229" t="s">
-        <v>820</v>
+        <v>289</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B230" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B231" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B232" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B233" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>639</v>
+        <v>293</v>
       </c>
       <c r="B234" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
+        <v>639</v>
+      </c>
+      <c r="B235" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3">
+      <c r="A236" t="s">
         <v>484</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B236" t="s">
         <v>617</v>
-      </c>
-    </row>
-    <row r="237" spans="1:3">
-      <c r="A237" t="s">
-        <v>471</v>
-      </c>
-      <c r="B237" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>455</v>
+        <v>471</v>
       </c>
       <c r="B238" t="s">
-        <v>299</v>
-      </c>
-      <c r="C238" t="s">
-        <v>532</v>
+        <v>907</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>461</v>
+        <v>455</v>
       </c>
       <c r="B239" t="s">
-        <v>517</v>
+        <v>299</v>
+      </c>
+      <c r="C239" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>297</v>
+        <v>461</v>
       </c>
       <c r="B240" t="s">
-        <v>908</v>
-      </c>
-      <c r="C240" t="s">
-        <v>532</v>
+        <v>517</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B241" t="s">
-        <v>888</v>
+        <v>908</v>
+      </c>
+      <c r="C241" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>454</v>
+        <v>298</v>
       </c>
       <c r="B242" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>300</v>
+        <v>454</v>
       </c>
       <c r="B243" t="s">
-        <v>898</v>
-      </c>
-      <c r="C243" t="s">
-        <v>1147</v>
+        <v>889</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B244" t="s">
-        <v>909</v>
+        <v>898</v>
+      </c>
+      <c r="C244" t="s">
+        <v>1147</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B245" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B246" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B247" t="s">
-        <v>824</v>
+        <v>911</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>640</v>
+        <v>304</v>
       </c>
       <c r="B248" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
+        <v>640</v>
+      </c>
+      <c r="B249" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3">
+      <c r="A250" t="s">
         <v>483</v>
       </c>
-      <c r="B249" t="s">
+      <c r="B250" t="s">
         <v>618</v>
-      </c>
-    </row>
-    <row r="251" spans="1:3">
-      <c r="A251" t="s">
-        <v>674</v>
-      </c>
-      <c r="B251" t="s">
-        <v>675</v>
-      </c>
-      <c r="C251" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>500</v>
+        <v>674</v>
       </c>
       <c r="B252" t="s">
-        <v>503</v>
+        <v>675</v>
       </c>
       <c r="C252" t="s">
-        <v>530</v>
+        <v>627</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B253" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C253" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>529</v>
+        <v>501</v>
       </c>
       <c r="B254" t="s">
-        <v>543</v>
+        <v>502</v>
+      </c>
+      <c r="C254" t="s">
+        <v>531</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>321</v>
+        <v>529</v>
       </c>
       <c r="B255" t="s">
-        <v>307</v>
+        <v>543</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B256" t="s">
-        <v>308</v>
-      </c>
-      <c r="C256" t="s">
-        <v>532</v>
+        <v>307</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>462</v>
+        <v>322</v>
       </c>
       <c r="B257" t="s">
-        <v>518</v>
+        <v>308</v>
+      </c>
+      <c r="C257" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>323</v>
+        <v>462</v>
       </c>
       <c r="B258" t="s">
-        <v>309</v>
+        <v>518</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B259" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B260" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B261" t="s">
-        <v>312</v>
-      </c>
-      <c r="C261" t="s">
-        <v>532</v>
+        <v>311</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B262" t="s">
-        <v>313</v>
+        <v>312</v>
+      </c>
+      <c r="C262" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B263" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B264" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B265" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B266" t="s">
-        <v>317</v>
-      </c>
-      <c r="C266" t="s">
-        <v>532</v>
+        <v>316</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B267" t="s">
-        <v>318</v>
+        <v>317</v>
+      </c>
+      <c r="C267" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B268" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B269" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
+        <v>334</v>
+      </c>
+      <c r="B270" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3">
+      <c r="A271" t="s">
         <v>482</v>
       </c>
-      <c r="B270" t="s">
+      <c r="B271" t="s">
         <v>603</v>
-      </c>
-    </row>
-    <row r="272" spans="1:3">
-      <c r="A272" t="s">
-        <v>547</v>
-      </c>
-      <c r="B272" t="s">
-        <v>548</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>341</v>
+        <v>547</v>
       </c>
       <c r="B273" t="s">
-        <v>359</v>
+        <v>548</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B274" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B275" t="s">
-        <v>357</v>
-      </c>
-      <c r="C275" t="s">
-        <v>532</v>
+        <v>356</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>463</v>
+        <v>343</v>
       </c>
       <c r="B276" t="s">
-        <v>519</v>
+        <v>357</v>
+      </c>
+      <c r="C276" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>360</v>
+        <v>463</v>
       </c>
       <c r="B277" t="s">
-        <v>358</v>
-      </c>
-      <c r="C277" t="s">
-        <v>532</v>
+        <v>519</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="B278" t="s">
-        <v>350</v>
+        <v>358</v>
+      </c>
+      <c r="C278" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>361</v>
+        <v>344</v>
       </c>
       <c r="B279" t="s">
-        <v>351</v>
-      </c>
-      <c r="C279" t="s">
-        <v>509</v>
+        <v>350</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="B280" t="s">
-        <v>352</v>
+        <v>351</v>
+      </c>
+      <c r="C280" t="s">
+        <v>509</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B281" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B282" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B283" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B284" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>1072</v>
+        <v>349</v>
       </c>
       <c r="B285" t="s">
-        <v>1073</v>
-      </c>
-      <c r="C285" t="s">
-        <v>1067</v>
+        <v>352</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="B286" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="C286" t="s">
         <v>1067</v>
@@ -10760,10 +10766,10 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B287" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="C287" t="s">
         <v>1067</v>
@@ -10771,40 +10777,40 @@
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
+        <v>1076</v>
+      </c>
+      <c r="B288" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C288" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3">
+      <c r="A289" t="s">
         <v>481</v>
       </c>
-      <c r="B288" t="s">
+      <c r="B289" t="s">
         <v>619</v>
-      </c>
-    </row>
-    <row r="290" spans="1:3">
-      <c r="A290" t="s">
-        <v>676</v>
-      </c>
-      <c r="B290" t="s">
-        <v>695</v>
-      </c>
-      <c r="C290" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>1065</v>
+        <v>676</v>
       </c>
       <c r="B291" t="s">
-        <v>1066</v>
+        <v>695</v>
       </c>
       <c r="C291" t="s">
-        <v>1067</v>
+        <v>627</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>1068</v>
+        <v>1065</v>
       </c>
       <c r="B292" t="s">
-        <v>1069</v>
+        <v>1066</v>
       </c>
       <c r="C292" t="s">
         <v>1067</v>
@@ -10812,78 +10818,78 @@
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="B293" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="C293" t="s">
         <v>1067</v>
       </c>
     </row>
-    <row r="295" spans="1:3">
-      <c r="A295" t="s">
-        <v>672</v>
-      </c>
-      <c r="B295" t="s">
-        <v>673</v>
-      </c>
-      <c r="C295" t="s">
-        <v>627</v>
+    <row r="294" spans="1:3">
+      <c r="A294" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B294" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C294" t="s">
+        <v>1067</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>472</v>
+        <v>672</v>
       </c>
       <c r="B296" t="s">
-        <v>473</v>
+        <v>673</v>
+      </c>
+      <c r="C296" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>367</v>
+        <v>472</v>
       </c>
       <c r="B297" t="s">
-        <v>378</v>
+        <v>473</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B298" t="s">
-        <v>379</v>
-      </c>
-      <c r="C298" t="s">
-        <v>532</v>
+        <v>378</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>520</v>
+        <v>368</v>
       </c>
       <c r="B299" t="s">
-        <v>521</v>
+        <v>379</v>
+      </c>
+      <c r="C299" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>369</v>
+        <v>520</v>
       </c>
       <c r="B300" t="s">
-        <v>380</v>
-      </c>
-      <c r="C300" t="s">
-        <v>532</v>
+        <v>521</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B301" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C301" t="s">
         <v>532</v>
@@ -10891,139 +10897,139 @@
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B302" t="s">
-        <v>533</v>
+        <v>381</v>
+      </c>
+      <c r="C302" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B303" t="s">
-        <v>382</v>
+        <v>533</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B304" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B305" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B306" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B307" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B308" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>731</v>
+        <v>377</v>
       </c>
       <c r="B309" t="s">
-        <v>1144</v>
-      </c>
-      <c r="C309" t="s">
-        <v>627</v>
+        <v>387</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>479</v>
+        <v>731</v>
       </c>
       <c r="B310" t="s">
-        <v>620</v>
+        <v>1144</v>
+      </c>
+      <c r="C310" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
+        <v>479</v>
+      </c>
+      <c r="B311" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3">
+      <c r="A312" t="s">
         <v>556</v>
       </c>
-      <c r="B311" t="s">
+      <c r="B312" t="s">
         <v>557</v>
-      </c>
-    </row>
-    <row r="313" spans="1:3">
-      <c r="A313" t="s">
-        <v>474</v>
-      </c>
-      <c r="B313" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>394</v>
+        <v>474</v>
       </c>
       <c r="B314" t="s">
-        <v>405</v>
+        <v>473</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B315" t="s">
-        <v>406</v>
-      </c>
-      <c r="C315" t="s">
-        <v>532</v>
+        <v>405</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>464</v>
+        <v>395</v>
       </c>
       <c r="B316" t="s">
-        <v>522</v>
+        <v>406</v>
+      </c>
+      <c r="C316" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>396</v>
+        <v>464</v>
       </c>
       <c r="B317" t="s">
-        <v>407</v>
-      </c>
-      <c r="C317" t="s">
-        <v>532</v>
+        <v>522</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B318" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C318" t="s">
         <v>532</v>
@@ -11031,1362 +11037,1373 @@
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B319" t="s">
-        <v>534</v>
+        <v>408</v>
+      </c>
+      <c r="C319" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B320" t="s">
-        <v>382</v>
+        <v>534</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B321" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B322" t="s">
-        <v>409</v>
+        <v>383</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B323" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B324" t="s">
-        <v>386</v>
+        <v>410</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B325" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>478</v>
+        <v>404</v>
       </c>
       <c r="B326" t="s">
-        <v>620</v>
+        <v>387</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
+        <v>478</v>
+      </c>
+      <c r="B327" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3">
+      <c r="A328" t="s">
         <v>563</v>
       </c>
-      <c r="B327" t="s">
+      <c r="B328" t="s">
         <v>557</v>
-      </c>
-    </row>
-    <row r="329" spans="1:3">
-      <c r="A329" t="s">
-        <v>670</v>
-      </c>
-      <c r="B329" t="s">
-        <v>671</v>
-      </c>
-      <c r="C329" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>388</v>
+        <v>670</v>
       </c>
       <c r="B330" t="s">
-        <v>564</v>
+        <v>671</v>
+      </c>
+      <c r="C330" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B331" t="s">
-        <v>565</v>
-      </c>
-      <c r="C331" t="s">
-        <v>532</v>
+        <v>564</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>465</v>
+        <v>389</v>
       </c>
       <c r="B332" t="s">
-        <v>566</v>
+        <v>565</v>
+      </c>
+      <c r="C332" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>390</v>
+        <v>465</v>
       </c>
       <c r="B333" t="s">
-        <v>591</v>
+        <v>566</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B334" t="s">
-        <v>567</v>
+        <v>591</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B335" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
+        <v>392</v>
+      </c>
+      <c r="B336" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3">
+      <c r="A337" t="s">
         <v>477</v>
       </c>
-      <c r="B336" t="s">
+      <c r="B337" t="s">
         <v>621</v>
-      </c>
-    </row>
-    <row r="338" spans="1:3">
-      <c r="A338" t="s">
-        <v>746</v>
-      </c>
-      <c r="B338" t="s">
-        <v>747</v>
-      </c>
-      <c r="C338" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="339" spans="1:3">
       <c r="A339" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B339" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="C339" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="341" spans="1:3">
-      <c r="A341" t="s">
-        <v>754</v>
-      </c>
-      <c r="B341" t="s">
-        <v>755</v>
+    <row r="340" spans="1:3">
+      <c r="A340" t="s">
+        <v>748</v>
+      </c>
+      <c r="B340" t="s">
+        <v>749</v>
+      </c>
+      <c r="C340" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="B342" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="B343" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B344" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="B345" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="B346" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B347" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B348" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B349" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B350" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="B351" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="B352" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="B353" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="B354" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="B355" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="B356" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>1154</v>
+        <v>784</v>
       </c>
       <c r="B357" t="s">
-        <v>1155</v>
+        <v>785</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>786</v>
+        <v>1154</v>
       </c>
       <c r="B358" t="s">
-        <v>787</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
+        <v>786</v>
+      </c>
+      <c r="B359" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2">
+      <c r="A360" t="s">
         <v>788</v>
       </c>
-      <c r="B359" t="s">
+      <c r="B360" t="s">
         <v>789</v>
-      </c>
-    </row>
-    <row r="361" spans="1:2">
-      <c r="A361" t="s">
-        <v>790</v>
-      </c>
-      <c r="B361" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="B362" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="B363" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="B364" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B365" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="B366" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="B367" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="B368" t="s">
-        <v>320</v>
+        <v>803</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="B369" t="s">
-        <v>806</v>
+        <v>320</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B370" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="B371" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
+        <v>809</v>
+      </c>
+      <c r="B372" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" t="s">
         <v>811</v>
       </c>
-      <c r="B372" t="s">
+      <c r="B373" t="s">
         <v>812</v>
-      </c>
-    </row>
-    <row r="374" spans="1:2">
-      <c r="A374" t="s">
-        <v>813</v>
-      </c>
-      <c r="B374" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="B375" t="s">
-        <v>815</v>
+        <v>313</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="B376" t="s">
-        <v>315</v>
+        <v>815</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
+        <v>816</v>
+      </c>
+      <c r="B377" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2">
+      <c r="A378" t="s">
         <v>817</v>
       </c>
-      <c r="B377" t="s">
+      <c r="B378" t="s">
         <v>316</v>
-      </c>
-    </row>
-    <row r="379" spans="1:2">
-      <c r="A379" t="s">
-        <v>842</v>
-      </c>
-      <c r="B379" t="s">
-        <v>843</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="B380" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
       <c r="B381" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B382" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B383" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
+        <v>833</v>
+      </c>
+      <c r="B384" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" t="s">
         <v>839</v>
       </c>
-      <c r="B384" t="s">
+      <c r="B385" t="s">
         <v>838</v>
-      </c>
-    </row>
-    <row r="386" spans="1:2">
-      <c r="A386" t="s">
-        <v>846</v>
-      </c>
-      <c r="B386" t="s">
-        <v>851</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>854</v>
+        <v>846</v>
       </c>
       <c r="B387" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
       <c r="B388" t="s">
-        <v>835</v>
+        <v>852</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="B389" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B390" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
+        <v>849</v>
+      </c>
+      <c r="B391" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" t="s">
         <v>850</v>
       </c>
-      <c r="B391" t="s">
+      <c r="B392" t="s">
         <v>853</v>
-      </c>
-    </row>
-    <row r="393" spans="1:2">
-      <c r="A393" t="s">
-        <v>859</v>
-      </c>
-      <c r="B393" t="s">
-        <v>860</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="B394" t="s">
-        <v>1136</v>
+        <v>860</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B395" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B396" t="s">
-        <v>1128</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>870</v>
+        <v>864</v>
       </c>
       <c r="B397" t="s">
-        <v>1114</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B398" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B399" t="s">
-        <v>1134</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="B400" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B401" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B402" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B403" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B404" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B405" t="s">
-        <v>869</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B406" t="s">
-        <v>1137</v>
+        <v>869</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B407" t="s">
-        <v>280</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B408" t="s">
-        <v>825</v>
+        <v>280</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>874</v>
+        <v>883</v>
       </c>
       <c r="B409" t="s">
-        <v>633</v>
+        <v>825</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="B410" t="s">
-        <v>1138</v>
+        <v>633</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>1118</v>
+        <v>873</v>
       </c>
       <c r="B411" t="s">
-        <v>1116</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B412" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="B413" t="s">
-        <v>1120</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
       <c r="B414" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="B415" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B416" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>1140</v>
+        <v>1127</v>
       </c>
       <c r="B417" t="s">
-        <v>1139</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
+        <v>1140</v>
+      </c>
+      <c r="B418" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="419" spans="1:2">
+      <c r="A419" t="s">
         <v>1141</v>
       </c>
-      <c r="B418" t="s">
+      <c r="B419" t="s">
         <v>1142</v>
-      </c>
-    </row>
-    <row r="420" spans="1:2">
-      <c r="A420" t="s">
-        <v>947</v>
-      </c>
-      <c r="B420" t="s">
-        <v>926</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>966</v>
+        <v>947</v>
       </c>
       <c r="B421" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B422" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="B423" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="B424" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="B425" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B426" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="B427" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="B428" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="B429" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B430" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>967</v>
+        <v>957</v>
       </c>
       <c r="B431" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>956</v>
+        <v>967</v>
       </c>
       <c r="B432" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="B433" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="B434" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B435" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B436" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B437" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="B438" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B439" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
+        <v>949</v>
+      </c>
+      <c r="B440" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="441" spans="1:2">
+      <c r="A441" t="s">
         <v>948</v>
       </c>
-      <c r="B440" t="s">
+      <c r="B441" t="s">
         <v>946</v>
-      </c>
-    </row>
-    <row r="442" spans="1:2">
-      <c r="A442" t="s">
-        <v>989</v>
-      </c>
-      <c r="B442" t="s">
-        <v>970</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>980</v>
+        <v>989</v>
       </c>
       <c r="B443" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B444" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B445" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>985</v>
+        <v>982</v>
       </c>
       <c r="B446" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="B447" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="B448" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="B449" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="B450" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
+        <v>988</v>
+      </c>
+      <c r="B451" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="452" spans="1:2">
+      <c r="A452" t="s">
         <v>987</v>
       </c>
-      <c r="B451" t="s">
+      <c r="B452" t="s">
         <v>979</v>
-      </c>
-    </row>
-    <row r="453" spans="1:2">
-      <c r="A453" t="s">
-        <v>994</v>
-      </c>
-      <c r="B453" t="s">
-        <v>996</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
+        <v>994</v>
+      </c>
+      <c r="B454" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2">
+      <c r="A455" t="s">
         <v>1005</v>
       </c>
-      <c r="B454" t="s">
+      <c r="B455" t="s">
         <v>1006</v>
-      </c>
-    </row>
-    <row r="456" spans="1:2">
-      <c r="A456" t="s">
-        <v>995</v>
-      </c>
-      <c r="B456" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
+        <v>995</v>
+      </c>
+      <c r="B457" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
         <v>1007</v>
       </c>
-      <c r="B457" t="s">
+      <c r="B458" t="s">
         <v>1008</v>
-      </c>
-    </row>
-    <row r="459" spans="1:2">
-      <c r="A459" t="s">
-        <v>1002</v>
-      </c>
-      <c r="B459" t="s">
-        <v>1000</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B460" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B461" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" t="s">
         <v>999</v>
       </c>
-      <c r="B461" t="s">
+      <c r="B462" t="s">
         <v>1004</v>
-      </c>
-    </row>
-    <row r="463" spans="1:2">
-      <c r="A463" t="s">
-        <v>1017</v>
-      </c>
-      <c r="B463" t="s">
-        <v>1010</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B464" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="B465" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>1064</v>
+        <v>1019</v>
       </c>
       <c r="B466" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>1020</v>
+        <v>1064</v>
       </c>
       <c r="B467" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B468" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" t="s">
         <v>1022</v>
       </c>
-      <c r="B469" t="s">
+      <c r="B470" t="s">
         <v>1016</v>
-      </c>
-    </row>
-    <row r="471" spans="1:2">
-      <c r="A471" t="s">
-        <v>1034</v>
-      </c>
-      <c r="B471" t="s">
-        <v>1028</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1039</v>
+        <v>1034</v>
       </c>
       <c r="B472" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="B473" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="474" spans="1:2">
       <c r="A474" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B474" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B475" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B476" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="477" spans="1:2">
+      <c r="A477" t="s">
         <v>1037</v>
       </c>
-      <c r="B476" t="s">
+      <c r="B477" t="s">
         <v>1033</v>
-      </c>
-    </row>
-    <row r="478" spans="1:2">
-      <c r="A478" t="s">
-        <v>1052</v>
-      </c>
-      <c r="B478" t="s">
-        <v>1040</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="B479" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B480" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B481" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B482" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B483" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="484" spans="1:2">
+      <c r="A484" t="s">
         <v>1051</v>
       </c>
-      <c r="B483" t="s">
+      <c r="B484" t="s">
         <v>1045</v>
-      </c>
-    </row>
-    <row r="485" spans="1:2">
-      <c r="A485" t="s">
-        <v>1053</v>
-      </c>
-      <c r="B485" t="s">
-        <v>1054</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1059</v>
+        <v>1053</v>
       </c>
       <c r="B486" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B487" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B488" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="489" spans="1:2">
       <c r="A489" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B489" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2">
+      <c r="A490" t="s">
         <v>1062</v>
       </c>
-      <c r="B489" t="s">
+      <c r="B490" t="s">
         <v>1058</v>
-      </c>
-    </row>
-    <row r="491" spans="1:2">
-      <c r="A491" t="s">
-        <v>1086</v>
-      </c>
-      <c r="B491" t="s">
-        <v>1087</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1102</v>
+        <v>1086</v>
       </c>
       <c r="B492" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B493" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B494" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1113</v>
+        <v>1104</v>
       </c>
       <c r="B495" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1105</v>
+        <v>1113</v>
       </c>
       <c r="B496" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B497" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="B498" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="B499" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="B500" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B501" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B502" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B503" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B504" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="505" spans="1:2">
+      <c r="A505" t="s">
         <v>1101</v>
       </c>
-      <c r="B504" t="s">
+      <c r="B505" t="s">
         <v>1100</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A459:A460 A456:A457 A442:A451 A453:A454">
+  <conditionalFormatting sqref="A460:A461 A457:A458 A443:A452 A454:A455">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated the code with TX bugs fixes and also Bagi code
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBFD6D62-2842-49D8-9EF7-4740615AC31B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AAB22D-8522-4D2A-80B4-50756F19B86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3522,9 +3522,6 @@
     <t>CZI_PartAYes</t>
   </si>
   <si>
-    <t>One adult answered "Yes" to a question in section A.</t>
-  </si>
-  <si>
     <t>ApplicationIncomplete</t>
   </si>
   <si>
@@ -3538,6 +3535,9 @@
   </si>
   <si>
     <t>General</t>
+  </si>
+  <si>
+    <t>Anticipated income in the next 12 months has been documented as yes for at least one question in Part A of the Certification of Zero Income. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -4036,10 +4036,10 @@
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B12" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -8432,10 +8432,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B5" t="s">
         <v>1161</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1162</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -9586,7 +9586,7 @@
         <v>1159</v>
       </c>
       <c r="B143" t="s">
-        <v>1160</v>
+        <v>1165</v>
       </c>
       <c r="C143" t="s">
         <v>627</v>
@@ -11006,10 +11006,10 @@
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B313" t="s">
         <v>1163</v>
-      </c>
-      <c r="B313" t="s">
-        <v>1164</v>
       </c>
     </row>
     <row r="314" spans="1:3">

</xml_diff>

<commit_message>
ICW findings and config
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8AAB22D-8522-4D2A-80B4-50756F19B86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28F30CF-2BAF-49EB-9C3E-CCA8D561F0CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2496,9 +2496,6 @@
     <t>1040_HasDate</t>
   </si>
   <si>
-    <t>Day Calculator does not exist for Work Number findings</t>
-  </si>
-  <si>
     <t>Employee Name listed on the Work Number, Day Calculator, and ICW do not match.</t>
   </si>
   <si>
@@ -2520,9 +2517,6 @@
     <t>Multiple employment documents provided for same employment. Can't determine which employment document to use to validate Day Calculator. Manual review required.</t>
   </si>
   <si>
-    <t>Day Calculator does not exist for Offer Letter findings</t>
-  </si>
-  <si>
     <t>Employee Name listed on the Offer Letter, Day Calculator, and ICW do not match.</t>
   </si>
   <si>
@@ -2721,9 +2715,6 @@
     <t>The ICW includes multiple employments; however, Day Calculator is not available for all of them.</t>
   </si>
   <si>
-    <t>Day Calculator does not exist for Paystub findings</t>
-  </si>
-  <si>
     <t>Company Name does not match across the Paystub, Day Calculator, and ICW.</t>
   </si>
   <si>
@@ -2748,9 +2739,6 @@
     <t>Gross Pay listed on the Paystub does not match the Day Calculator.</t>
   </si>
   <si>
-    <t>Day Calculator does not exist for Verification of employment findings</t>
-  </si>
-  <si>
     <t>Company Name across the Verification of Employment, Day Calculator, and ICW do not match.</t>
   </si>
   <si>
@@ -2763,9 +2751,6 @@
     <t>The calculated Shift Differential Wage Per Year based on the Verification of Employment does not match the Shift differential Total Per Year on the Day Calculator.</t>
   </si>
   <si>
-    <t>Day Calculator does not exist for Verification services findings</t>
-  </si>
-  <si>
     <t>Employer Name listed on Verification Services, Day Calculator, and ICW do not match.</t>
   </si>
   <si>
@@ -3450,9 +3435,6 @@
     <t>Employment Verification email receipt and clarification verification require manual review.</t>
   </si>
   <si>
-    <t>Day Calculator does not exist for Employment Verification findings.</t>
-  </si>
-  <si>
     <t>Not all fields have been documented appropriately on the Employment Verification.</t>
   </si>
   <si>
@@ -3510,9 +3492,6 @@
     <t>There are more Schedule Cs than CSEI</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>VSI</t>
   </si>
   <si>
@@ -3538,6 +3517,27 @@
   </si>
   <si>
     <t>Anticipated income in the next 12 months has been documented as yes for at least one question in Part A of the Certification of Zero Income. Manual review required.</t>
+  </si>
+  <si>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Paystub</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Verification of employment</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Offer Letter</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Work Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day Calculator does not exist for Verification services </t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Employment Verification.</t>
   </si>
 </sst>
 </file>
@@ -4006,7 +4006,7 @@
         <v>205</v>
       </c>
       <c r="B7" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4036,10 +4036,10 @@
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>1164</v>
+        <v>1157</v>
       </c>
       <c r="B12" t="s">
-        <v>1164</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -4163,7 +4163,7 @@
         <v>411</v>
       </c>
       <c r="B26" t="s">
-        <v>1025</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
@@ -4318,130 +4318,130 @@
         <v>753</v>
       </c>
       <c r="B45" t="s">
-        <v>1025</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="B46" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="B47" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="B48" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="B49" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>924</v>
+        <v>919</v>
       </c>
       <c r="B50" t="s">
-        <v>925</v>
+        <v>920</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1">
       <c r="A51" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="B51" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>990</v>
+        <v>985</v>
       </c>
       <c r="B52" t="s">
-        <v>991</v>
+        <v>986</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>992</v>
+        <v>987</v>
       </c>
       <c r="B53" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>998</v>
+        <v>993</v>
       </c>
       <c r="B54" t="s">
-        <v>1009</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="14.25" customHeight="1">
       <c r="A55" t="s">
-        <v>1023</v>
+        <v>1018</v>
       </c>
       <c r="B55" t="s">
-        <v>1024</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="14.25" customHeight="1">
       <c r="A56" t="s">
-        <v>1026</v>
+        <v>1021</v>
       </c>
       <c r="B56" t="s">
-        <v>1026</v>
+        <v>1021</v>
       </c>
       <c r="C56" t="s">
-        <v>1027</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>1046</v>
+        <v>1041</v>
       </c>
       <c r="B57" t="s">
-        <v>1046</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>1063</v>
+        <v>1058</v>
       </c>
       <c r="B58" t="s">
-        <v>1151</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1">
       <c r="A59" t="s">
-        <v>1157</v>
+        <v>1150</v>
       </c>
       <c r="B59" t="s">
-        <v>1158</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="14.25" customHeight="1">
       <c r="A60" t="s">
-        <v>1084</v>
+        <v>1079</v>
       </c>
       <c r="B60" t="s">
-        <v>1085</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
@@ -7388,50 +7388,50 @@
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>1080</v>
+        <v>1075</v>
       </c>
       <c r="B44" t="s">
-        <v>1080</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>1081</v>
+        <v>1076</v>
       </c>
       <c r="B45" t="s">
-        <v>1081</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>1082</v>
+        <v>1077</v>
       </c>
       <c r="B46" t="s">
-        <v>1082</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>1083</v>
+        <v>1078</v>
       </c>
       <c r="B47" t="s">
-        <v>1083</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>1152</v>
+        <v>1146</v>
       </c>
       <c r="B48" t="s">
-        <v>1152</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>1153</v>
+        <v>1147</v>
       </c>
       <c r="B49" t="s">
-        <v>1153</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8432,10 +8432,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>1160</v>
+        <v>1153</v>
       </c>
       <c r="B5" t="s">
-        <v>1161</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -8623,7 +8623,7 @@
         <v>738</v>
       </c>
       <c r="B26" t="s">
-        <v>1146</v>
+        <v>1140</v>
       </c>
       <c r="C26" t="s">
         <v>627</v>
@@ -8631,10 +8631,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="B27" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -8872,10 +8872,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>1078</v>
+        <v>1073</v>
       </c>
       <c r="B58" t="s">
-        <v>1079</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -9130,7 +9130,7 @@
         <v>185</v>
       </c>
       <c r="B88" t="s">
-        <v>1143</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -9257,10 +9257,10 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
       <c r="B102" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -9306,34 +9306,34 @@
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="B107" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="B108" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="B109" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>923</v>
+        <v>918</v>
       </c>
       <c r="B110" t="s">
-        <v>920</v>
+        <v>915</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -9583,10 +9583,10 @@
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>1159</v>
+        <v>1152</v>
       </c>
       <c r="B143" t="s">
-        <v>1165</v>
+        <v>1158</v>
       </c>
       <c r="C143" t="s">
         <v>627</v>
@@ -9748,7 +9748,7 @@
         <v>592</v>
       </c>
       <c r="B164" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="C164" t="s">
         <v>593</v>
@@ -9770,7 +9770,7 @@
         <v>750</v>
       </c>
       <c r="B166" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="C166" t="s">
         <v>627</v>
@@ -9781,7 +9781,7 @@
         <v>751</v>
       </c>
       <c r="B167" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="C167" t="s">
         <v>627</v>
@@ -9800,13 +9800,13 @@
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>1148</v>
+        <v>1142</v>
       </c>
       <c r="B169" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C169" t="s">
-        <v>1149</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -9814,7 +9814,7 @@
         <v>467</v>
       </c>
       <c r="B171" t="s">
-        <v>893</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="172" spans="1:3">
@@ -9844,7 +9844,7 @@
         <v>238</v>
       </c>
       <c r="B174" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="C174" t="s">
         <v>532</v>
@@ -9855,7 +9855,7 @@
         <v>239</v>
       </c>
       <c r="B175" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -9863,7 +9863,7 @@
         <v>247</v>
       </c>
       <c r="B176" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="C176" t="s">
         <v>590</v>
@@ -9874,7 +9874,7 @@
         <v>717</v>
       </c>
       <c r="B177" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="C177" t="s">
         <v>627</v>
@@ -9901,10 +9901,10 @@
         <v>242</v>
       </c>
       <c r="B180" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C180" t="s">
-        <v>1150</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -9912,7 +9912,7 @@
         <v>243</v>
       </c>
       <c r="B181" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -9920,7 +9920,7 @@
         <v>244</v>
       </c>
       <c r="B182" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -9928,7 +9928,7 @@
         <v>245</v>
       </c>
       <c r="B183" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -9936,7 +9936,7 @@
         <v>246</v>
       </c>
       <c r="B184" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -9944,10 +9944,10 @@
         <v>278</v>
       </c>
       <c r="B185" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C185" t="s">
-        <v>1150</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="186" spans="1:3">
@@ -9963,7 +9963,7 @@
         <v>595</v>
       </c>
       <c r="B187" t="s">
-        <v>1145</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -9971,7 +9971,7 @@
         <v>636</v>
       </c>
       <c r="B188" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="189" spans="1:3">
@@ -9998,10 +9998,10 @@
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="B191" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
     </row>
     <row r="192" spans="1:3">
@@ -10028,7 +10028,7 @@
         <v>468</v>
       </c>
       <c r="B195" t="s">
-        <v>902</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -10036,7 +10036,7 @@
         <v>248</v>
       </c>
       <c r="B196" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="C196" t="s">
         <v>597</v>
@@ -10047,7 +10047,7 @@
         <v>250</v>
       </c>
       <c r="B197" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
       <c r="C197" t="s">
         <v>631</v>
@@ -10058,7 +10058,7 @@
         <v>249</v>
       </c>
       <c r="B198" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="199" spans="1:3">
@@ -10101,7 +10101,7 @@
         <v>257</v>
       </c>
       <c r="B203" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -10117,7 +10117,7 @@
         <v>263</v>
       </c>
       <c r="B205" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -10125,7 +10125,7 @@
         <v>264</v>
       </c>
       <c r="B206" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="207" spans="1:3">
@@ -10133,7 +10133,7 @@
         <v>265</v>
       </c>
       <c r="B207" t="s">
-        <v>905</v>
+        <v>901</v>
       </c>
       <c r="C207" t="s">
         <v>597</v>
@@ -10144,7 +10144,7 @@
         <v>266</v>
       </c>
       <c r="B208" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="209" spans="1:3">
@@ -10152,7 +10152,7 @@
         <v>267</v>
       </c>
       <c r="B209" t="s">
-        <v>906</v>
+        <v>902</v>
       </c>
       <c r="C209" t="s">
         <v>597</v>
@@ -10163,7 +10163,7 @@
         <v>268</v>
       </c>
       <c r="B210" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="211" spans="1:3">
@@ -10179,10 +10179,10 @@
         <v>277</v>
       </c>
       <c r="B212" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C212" t="s">
-        <v>1150</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="213" spans="1:3">
@@ -10198,7 +10198,7 @@
         <v>637</v>
       </c>
       <c r="B214" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="215" spans="1:3">
@@ -10225,7 +10225,7 @@
         <v>469</v>
       </c>
       <c r="B218" t="s">
-        <v>826</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="219" spans="1:3">
@@ -10241,7 +10241,7 @@
         <v>273</v>
       </c>
       <c r="B220" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -10249,7 +10249,7 @@
         <v>274</v>
       </c>
       <c r="B221" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -10257,7 +10257,7 @@
         <v>282</v>
       </c>
       <c r="B222" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
     </row>
     <row r="223" spans="1:3">
@@ -10265,7 +10265,7 @@
         <v>281</v>
       </c>
       <c r="B223" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -10273,7 +10273,7 @@
         <v>283</v>
       </c>
       <c r="B224" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
     </row>
     <row r="225" spans="1:2">
@@ -10281,7 +10281,7 @@
         <v>638</v>
       </c>
       <c r="B225" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="226" spans="1:2">
@@ -10297,7 +10297,7 @@
         <v>470</v>
       </c>
       <c r="B228" t="s">
-        <v>818</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="229" spans="1:2">
@@ -10313,7 +10313,7 @@
         <v>286</v>
       </c>
       <c r="B230" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="231" spans="1:2">
@@ -10329,7 +10329,7 @@
         <v>288</v>
       </c>
       <c r="B232" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
     <row r="233" spans="1:2">
@@ -10337,7 +10337,7 @@
         <v>290</v>
       </c>
       <c r="B233" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="234" spans="1:2">
@@ -10345,7 +10345,7 @@
         <v>291</v>
       </c>
       <c r="B234" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="235" spans="1:2">
@@ -10353,7 +10353,7 @@
         <v>292</v>
       </c>
       <c r="B235" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="236" spans="1:2">
@@ -10361,7 +10361,7 @@
         <v>293</v>
       </c>
       <c r="B236" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="237" spans="1:2">
@@ -10369,7 +10369,7 @@
         <v>639</v>
       </c>
       <c r="B237" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="238" spans="1:2">
@@ -10385,7 +10385,7 @@
         <v>471</v>
       </c>
       <c r="B240" t="s">
-        <v>907</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -10412,7 +10412,7 @@
         <v>297</v>
       </c>
       <c r="B243" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="C243" t="s">
         <v>532</v>
@@ -10423,7 +10423,7 @@
         <v>298</v>
       </c>
       <c r="B244" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -10431,7 +10431,7 @@
         <v>454</v>
       </c>
       <c r="B245" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -10439,10 +10439,10 @@
         <v>300</v>
       </c>
       <c r="B246" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C246" t="s">
-        <v>1147</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -10450,7 +10450,7 @@
         <v>301</v>
       </c>
       <c r="B247" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -10458,7 +10458,7 @@
         <v>302</v>
       </c>
       <c r="B248" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -10466,7 +10466,7 @@
         <v>303</v>
       </c>
       <c r="B249" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
     </row>
     <row r="250" spans="1:3">
@@ -10474,7 +10474,7 @@
         <v>304</v>
       </c>
       <c r="B250" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -10482,7 +10482,7 @@
         <v>640</v>
       </c>
       <c r="B251" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="252" spans="1:3">
@@ -10786,35 +10786,35 @@
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>1072</v>
+        <v>1067</v>
       </c>
       <c r="B288" t="s">
-        <v>1073</v>
+        <v>1068</v>
       </c>
       <c r="C288" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>1074</v>
+        <v>1069</v>
       </c>
       <c r="B289" t="s">
-        <v>1075</v>
+        <v>1070</v>
       </c>
       <c r="C289" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>1076</v>
+        <v>1071</v>
       </c>
       <c r="B290" t="s">
-        <v>1077</v>
+        <v>1072</v>
       </c>
       <c r="C290" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="291" spans="1:3">
@@ -10838,35 +10838,35 @@
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>1065</v>
+        <v>1060</v>
       </c>
       <c r="B294" t="s">
-        <v>1066</v>
+        <v>1061</v>
       </c>
       <c r="C294" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>1068</v>
+        <v>1063</v>
       </c>
       <c r="B295" t="s">
-        <v>1069</v>
+        <v>1064</v>
       </c>
       <c r="C295" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>1070</v>
+        <v>1065</v>
       </c>
       <c r="B296" t="s">
-        <v>1071</v>
+        <v>1066</v>
       </c>
       <c r="C296" t="s">
-        <v>1067</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="298" spans="1:3">
@@ -10998,7 +10998,7 @@
         <v>731</v>
       </c>
       <c r="B312" t="s">
-        <v>1144</v>
+        <v>1138</v>
       </c>
       <c r="C312" t="s">
         <v>627</v>
@@ -11006,10 +11006,10 @@
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>1162</v>
+        <v>1155</v>
       </c>
       <c r="B313" t="s">
-        <v>1163</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="314" spans="1:3">
@@ -11379,10 +11379,10 @@
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>1154</v>
+        <v>1148</v>
       </c>
       <c r="B361" t="s">
-        <v>1155</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="362" spans="1:2">
@@ -11531,215 +11531,215 @@
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="B383" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="B384" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="B385" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="B386" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="B387" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="B388" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="B390" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="B391" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="B392" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="B393" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="B394" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
       <c r="B395" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="B397" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="B398" t="s">
-        <v>1136</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="B399" t="s">
-        <v>1135</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B400" t="s">
-        <v>1128</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="B401" t="s">
-        <v>1114</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="B402" t="s">
-        <v>1115</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="B403" t="s">
-        <v>1134</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="B404" t="s">
-        <v>1133</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="B405" t="s">
-        <v>1132</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="B406" t="s">
-        <v>1131</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="B407" t="s">
-        <v>1130</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="B408" t="s">
-        <v>1129</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="B409" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="B410" t="s">
-        <v>1137</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="B411" t="s">
         <v>280</v>
@@ -11747,15 +11747,15 @@
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="B412" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="B413" t="s">
         <v>633</v>
@@ -11763,682 +11763,682 @@
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="B414" t="s">
-        <v>1138</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1118</v>
+        <v>1113</v>
       </c>
       <c r="B415" t="s">
-        <v>1116</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1119</v>
+        <v>1114</v>
       </c>
       <c r="B416" t="s">
-        <v>1117</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>1121</v>
+        <v>1116</v>
       </c>
       <c r="B417" t="s">
-        <v>1120</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>1125</v>
+        <v>1120</v>
       </c>
       <c r="B418" t="s">
-        <v>1122</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>1126</v>
+        <v>1121</v>
       </c>
       <c r="B419" t="s">
-        <v>1123</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>1127</v>
+        <v>1122</v>
       </c>
       <c r="B420" t="s">
-        <v>1124</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>1140</v>
+        <v>1134</v>
       </c>
       <c r="B421" t="s">
-        <v>1139</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>1141</v>
+        <v>1135</v>
       </c>
       <c r="B422" t="s">
-        <v>1142</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="B424" t="s">
-        <v>926</v>
+        <v>921</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>966</v>
+        <v>961</v>
       </c>
       <c r="B425" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="B426" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="B427" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>963</v>
+        <v>958</v>
       </c>
       <c r="B428" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>962</v>
+        <v>957</v>
       </c>
       <c r="B429" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
       <c r="B430" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>960</v>
+        <v>955</v>
       </c>
       <c r="B431" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="B432" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>958</v>
+        <v>953</v>
       </c>
       <c r="B433" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
       <c r="B434" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>967</v>
+        <v>962</v>
       </c>
       <c r="B435" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="B436" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="B437" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="B438" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="B439" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="B440" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
       <c r="B441" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="B442" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="B443" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="B444" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>989</v>
+        <v>984</v>
       </c>
       <c r="B446" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="B447" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="B448" t="s">
-        <v>972</v>
+        <v>967</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>982</v>
+        <v>977</v>
       </c>
       <c r="B449" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>985</v>
+        <v>980</v>
       </c>
       <c r="B450" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>983</v>
+        <v>978</v>
       </c>
       <c r="B451" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>986</v>
+        <v>981</v>
       </c>
       <c r="B452" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
       <c r="B453" t="s">
-        <v>977</v>
+        <v>972</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>988</v>
+        <v>983</v>
       </c>
       <c r="B454" t="s">
-        <v>978</v>
+        <v>973</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>987</v>
+        <v>982</v>
       </c>
       <c r="B455" t="s">
-        <v>979</v>
+        <v>974</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>994</v>
+        <v>989</v>
       </c>
       <c r="B457" t="s">
-        <v>996</v>
+        <v>991</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="B458" t="s">
-        <v>1006</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
-        <v>995</v>
+        <v>990</v>
       </c>
       <c r="B460" t="s">
-        <v>997</v>
+        <v>992</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>1007</v>
+        <v>1002</v>
       </c>
       <c r="B461" t="s">
-        <v>1008</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>1002</v>
+        <v>997</v>
       </c>
       <c r="B463" t="s">
-        <v>1000</v>
+        <v>995</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>1003</v>
+        <v>998</v>
       </c>
       <c r="B464" t="s">
-        <v>1001</v>
+        <v>996</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
+        <v>994</v>
+      </c>
+      <c r="B465" t="s">
         <v>999</v>
-      </c>
-      <c r="B465" t="s">
-        <v>1004</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>1017</v>
+        <v>1012</v>
       </c>
       <c r="B467" t="s">
-        <v>1010</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1018</v>
+        <v>1013</v>
       </c>
       <c r="B468" t="s">
-        <v>1011</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1019</v>
+        <v>1014</v>
       </c>
       <c r="B469" t="s">
-        <v>1012</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1064</v>
+        <v>1059</v>
       </c>
       <c r="B470" t="s">
-        <v>1013</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1020</v>
+        <v>1015</v>
       </c>
       <c r="B471" t="s">
-        <v>1014</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1021</v>
+        <v>1016</v>
       </c>
       <c r="B472" t="s">
-        <v>1015</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>1022</v>
+        <v>1017</v>
       </c>
       <c r="B473" t="s">
-        <v>1016</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
-        <v>1034</v>
+        <v>1029</v>
       </c>
       <c r="B475" t="s">
-        <v>1028</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1039</v>
+        <v>1034</v>
       </c>
       <c r="B476" t="s">
-        <v>1029</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1035</v>
+        <v>1030</v>
       </c>
       <c r="B477" t="s">
-        <v>1030</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1036</v>
+        <v>1031</v>
       </c>
       <c r="B478" t="s">
-        <v>1031</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1038</v>
+        <v>1033</v>
       </c>
       <c r="B479" t="s">
-        <v>1032</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>1037</v>
+        <v>1032</v>
       </c>
       <c r="B480" t="s">
-        <v>1033</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" t="s">
-        <v>1052</v>
+        <v>1047</v>
       </c>
       <c r="B482" t="s">
-        <v>1040</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>1047</v>
+        <v>1042</v>
       </c>
       <c r="B483" t="s">
-        <v>1041</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>1048</v>
+        <v>1043</v>
       </c>
       <c r="B484" t="s">
-        <v>1042</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1049</v>
+        <v>1044</v>
       </c>
       <c r="B485" t="s">
-        <v>1043</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1050</v>
+        <v>1045</v>
       </c>
       <c r="B486" t="s">
-        <v>1044</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>1051</v>
+        <v>1046</v>
       </c>
       <c r="B487" t="s">
-        <v>1045</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="489" spans="1:2">
       <c r="A489" t="s">
-        <v>1053</v>
+        <v>1048</v>
       </c>
       <c r="B489" t="s">
-        <v>1054</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
-        <v>1059</v>
+        <v>1054</v>
       </c>
       <c r="B490" t="s">
-        <v>1055</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1060</v>
+        <v>1055</v>
       </c>
       <c r="B491" t="s">
-        <v>1056</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1061</v>
+        <v>1056</v>
       </c>
       <c r="B492" t="s">
-        <v>1057</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1062</v>
+        <v>1057</v>
       </c>
       <c r="B493" t="s">
-        <v>1058</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1086</v>
+        <v>1081</v>
       </c>
       <c r="B495" t="s">
-        <v>1087</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1102</v>
+        <v>1097</v>
       </c>
       <c r="B496" t="s">
-        <v>1088</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1103</v>
+        <v>1098</v>
       </c>
       <c r="B497" t="s">
-        <v>1089</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1104</v>
+        <v>1099</v>
       </c>
       <c r="B498" t="s">
-        <v>1090</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
       <c r="B499" t="s">
-        <v>1091</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1105</v>
+        <v>1100</v>
       </c>
       <c r="B500" t="s">
-        <v>1092</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1106</v>
+        <v>1101</v>
       </c>
       <c r="B501" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1107</v>
+        <v>1102</v>
       </c>
       <c r="B502" t="s">
-        <v>1094</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1108</v>
+        <v>1103</v>
       </c>
       <c r="B503" t="s">
-        <v>1095</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
-        <v>1109</v>
+        <v>1104</v>
       </c>
       <c r="B504" t="s">
-        <v>1096</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1110</v>
+        <v>1105</v>
       </c>
       <c r="B505" t="s">
-        <v>1097</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1111</v>
+        <v>1106</v>
       </c>
       <c r="B506" t="s">
-        <v>1098</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1112</v>
+        <v>1107</v>
       </c>
       <c r="B507" t="s">
-        <v>1099</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
-        <v>1101</v>
+        <v>1096</v>
       </c>
       <c r="B508" t="s">
-        <v>1100</v>
+        <v>1095</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes for bagi - VRCC, fixed a finding in Config file
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C80B1186-C05C-45E2-B1F3-2E4B929DCFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C742C6AC-D653-407B-A81F-67E704025175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28350" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="1165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="1168">
   <si>
     <t>Name</t>
   </si>
@@ -2385,9 +2385,6 @@
     <t>Amount listed on the Certification of Self-Employment Income and ICW do not match.</t>
   </si>
   <si>
-    <t>CSEI_findingError</t>
-  </si>
-  <si>
     <t>Unable to validate findings for Certification of Self-Employment Income. Needs manual review.</t>
   </si>
   <si>
@@ -3535,6 +3532,18 @@
   </si>
   <si>
     <t>LLM_Classification_RetryCount</t>
+  </si>
+  <si>
+    <t>CSEI_FindingError</t>
+  </si>
+  <si>
+    <t>VRCC_EmailReceipt</t>
+  </si>
+  <si>
+    <t>Verification of Recurring Cash Contributions email receipt requires manual review.</t>
+  </si>
+  <si>
+    <t>Newly added by Bagi for AZ</t>
   </si>
 </sst>
 </file>
@@ -3970,7 +3979,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -3991,7 +4000,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -4003,7 +4012,7 @@
         <v>203</v>
       </c>
       <c r="B7" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4033,10 +4042,10 @@
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="B12" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -4160,7 +4169,7 @@
         <v>409</v>
       </c>
       <c r="B26" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
@@ -4315,130 +4324,130 @@
         <v>746</v>
       </c>
       <c r="B45" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
+        <v>834</v>
+      </c>
+      <c r="B46" t="s">
         <v>835</v>
-      </c>
-      <c r="B46" t="s">
-        <v>836</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
+        <v>845</v>
+      </c>
+      <c r="B47" t="s">
         <v>846</v>
-      </c>
-      <c r="B47" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
+        <v>847</v>
+      </c>
+      <c r="B48" t="s">
         <v>848</v>
-      </c>
-      <c r="B48" t="s">
-        <v>849</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="14.25" customHeight="1">
       <c r="A49" t="s">
+        <v>874</v>
+      </c>
+      <c r="B49" t="s">
         <v>875</v>
-      </c>
-      <c r="B49" t="s">
-        <v>876</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="14.25" customHeight="1">
       <c r="A50" t="s">
+        <v>911</v>
+      </c>
+      <c r="B50" t="s">
         <v>912</v>
-      </c>
-      <c r="B50" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1">
       <c r="A51" t="s">
+        <v>955</v>
+      </c>
+      <c r="B51" t="s">
         <v>956</v>
-      </c>
-      <c r="B51" t="s">
-        <v>957</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="14.25" customHeight="1">
       <c r="A52" t="s">
+        <v>977</v>
+      </c>
+      <c r="B52" t="s">
         <v>978</v>
-      </c>
-      <c r="B52" t="s">
-        <v>979</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="14.25" customHeight="1">
       <c r="A53" t="s">
+        <v>979</v>
+      </c>
+      <c r="B53" t="s">
         <v>980</v>
-      </c>
-      <c r="B53" t="s">
-        <v>981</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B54" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="14.25" customHeight="1">
       <c r="A55" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B55" t="s">
         <v>1011</v>
-      </c>
-      <c r="B55" t="s">
-        <v>1012</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="14.25" customHeight="1">
       <c r="A56" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C56" t="s">
         <v>1014</v>
-      </c>
-      <c r="B56" t="s">
-        <v>1014</v>
-      </c>
-      <c r="C56" t="s">
-        <v>1015</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B57" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B58" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1">
       <c r="A59" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B59" t="s">
         <v>1143</v>
-      </c>
-      <c r="B59" t="s">
-        <v>1144</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="14.25" customHeight="1">
       <c r="A60" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B60" t="s">
         <v>1072</v>
-      </c>
-      <c r="B60" t="s">
-        <v>1073</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
@@ -7209,10 +7218,10 @@
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B22" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
@@ -7393,50 +7402,50 @@
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B45" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B46" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B47" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B48" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B49" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B50" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8411,7 +8420,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C507"/>
+  <dimension ref="A1:C508"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8437,10 +8446,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B5" t="s">
         <v>1146</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1147</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -8628,7 +8637,7 @@
         <v>731</v>
       </c>
       <c r="B26" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C26" t="s">
         <v>620</v>
@@ -8636,10 +8645,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
+        <v>876</v>
+      </c>
+      <c r="B27" t="s">
         <v>877</v>
-      </c>
-      <c r="B27" t="s">
-        <v>878</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -8877,10 +8886,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B58" t="s">
         <v>1066</v>
-      </c>
-      <c r="B58" t="s">
-        <v>1067</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -9135,7 +9144,7 @@
         <v>183</v>
       </c>
       <c r="B88" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="89" spans="1:3">
@@ -9262,10 +9271,10 @@
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
+        <v>905</v>
+      </c>
+      <c r="B102" t="s">
         <v>906</v>
-      </c>
-      <c r="B102" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -9311,34 +9320,34 @@
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
+        <v>901</v>
+      </c>
+      <c r="B107" t="s">
         <v>902</v>
-      </c>
-      <c r="B107" t="s">
-        <v>903</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
+        <v>903</v>
+      </c>
+      <c r="B108" t="s">
         <v>904</v>
-      </c>
-      <c r="B108" t="s">
-        <v>905</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
+        <v>908</v>
+      </c>
+      <c r="B109" t="s">
         <v>909</v>
-      </c>
-      <c r="B109" t="s">
-        <v>910</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="B110" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -9588,10 +9597,10 @@
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B143" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="C143" t="s">
         <v>620</v>
@@ -9753,7 +9762,7 @@
         <v>590</v>
       </c>
       <c r="B164" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C164" t="s">
         <v>591</v>
@@ -9775,7 +9784,7 @@
         <v>743</v>
       </c>
       <c r="B166" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="C166" t="s">
         <v>620</v>
@@ -9786,7 +9795,7 @@
         <v>744</v>
       </c>
       <c r="B167" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C167" t="s">
         <v>620</v>
@@ -9805,13 +9814,13 @@
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B169" t="s">
+        <v>887</v>
+      </c>
+      <c r="C169" t="s">
         <v>1135</v>
-      </c>
-      <c r="B169" t="s">
-        <v>888</v>
-      </c>
-      <c r="C169" t="s">
-        <v>1136</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -9819,18 +9828,18 @@
         <v>465</v>
       </c>
       <c r="B171" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B172" t="s">
         <v>1159</v>
       </c>
-      <c r="B172" t="s">
+      <c r="C172" t="s">
         <v>1160</v>
-      </c>
-      <c r="C172" t="s">
-        <v>1161</v>
       </c>
     </row>
     <row r="173" spans="1:3">
@@ -9838,7 +9847,7 @@
         <v>236</v>
       </c>
       <c r="B173" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="C173" t="s">
         <v>530</v>
@@ -9849,7 +9858,7 @@
         <v>237</v>
       </c>
       <c r="B174" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -9857,7 +9866,7 @@
         <v>245</v>
       </c>
       <c r="B175" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="C175" t="s">
         <v>588</v>
@@ -9868,7 +9877,7 @@
         <v>710</v>
       </c>
       <c r="B176" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="C176" t="s">
         <v>620</v>
@@ -9895,10 +9904,10 @@
         <v>240</v>
       </c>
       <c r="B179" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C179" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -9906,7 +9915,7 @@
         <v>241</v>
       </c>
       <c r="B180" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -9914,7 +9923,7 @@
         <v>242</v>
       </c>
       <c r="B181" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -9922,7 +9931,7 @@
         <v>243</v>
       </c>
       <c r="B182" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -9930,7 +9939,7 @@
         <v>244</v>
       </c>
       <c r="B183" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -9938,10 +9947,10 @@
         <v>276</v>
       </c>
       <c r="B184" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C184" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -9957,7 +9966,7 @@
         <v>593</v>
       </c>
       <c r="B186" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="187" spans="1:3">
@@ -9965,7 +9974,7 @@
         <v>629</v>
       </c>
       <c r="B187" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -9992,10 +10001,10 @@
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
+        <v>899</v>
+      </c>
+      <c r="B190" t="s">
         <v>900</v>
-      </c>
-      <c r="B190" t="s">
-        <v>901</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -10022,7 +10031,7 @@
         <v>466</v>
       </c>
       <c r="B194" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -10030,7 +10039,7 @@
         <v>246</v>
       </c>
       <c r="B195" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="C195" t="s">
         <v>595</v>
@@ -10041,7 +10050,7 @@
         <v>248</v>
       </c>
       <c r="B196" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="C196" t="s">
         <v>624</v>
@@ -10052,7 +10061,7 @@
         <v>247</v>
       </c>
       <c r="B197" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -10095,7 +10104,7 @@
         <v>255</v>
       </c>
       <c r="B202" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="203" spans="1:3">
@@ -10111,7 +10120,7 @@
         <v>261</v>
       </c>
       <c r="B204" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="205" spans="1:3">
@@ -10119,7 +10128,7 @@
         <v>262</v>
       </c>
       <c r="B205" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -10127,7 +10136,7 @@
         <v>263</v>
       </c>
       <c r="B206" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C206" t="s">
         <v>595</v>
@@ -10138,7 +10147,7 @@
         <v>264</v>
       </c>
       <c r="B207" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -10146,7 +10155,7 @@
         <v>265</v>
       </c>
       <c r="B208" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C208" t="s">
         <v>595</v>
@@ -10157,7 +10166,7 @@
         <v>266</v>
       </c>
       <c r="B209" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -10173,10 +10182,10 @@
         <v>275</v>
       </c>
       <c r="B211" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C211" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="212" spans="1:3">
@@ -10192,7 +10201,7 @@
         <v>630</v>
       </c>
       <c r="B213" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -10219,7 +10228,7 @@
         <v>467</v>
       </c>
       <c r="B217" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -10235,7 +10244,7 @@
         <v>271</v>
       </c>
       <c r="B219" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -10243,7 +10252,7 @@
         <v>272</v>
       </c>
       <c r="B220" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -10251,7 +10260,7 @@
         <v>280</v>
       </c>
       <c r="B221" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -10259,7 +10268,7 @@
         <v>279</v>
       </c>
       <c r="B222" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
     <row r="223" spans="1:3">
@@ -10267,7 +10276,7 @@
         <v>281</v>
       </c>
       <c r="B223" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="224" spans="1:3">
@@ -10275,7 +10284,7 @@
         <v>631</v>
       </c>
       <c r="B224" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -10291,7 +10300,7 @@
         <v>468</v>
       </c>
       <c r="B227" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -10307,7 +10316,7 @@
         <v>284</v>
       </c>
       <c r="B229" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -10323,7 +10332,7 @@
         <v>286</v>
       </c>
       <c r="B231" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -10331,7 +10340,7 @@
         <v>288</v>
       </c>
       <c r="B232" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
     </row>
     <row r="233" spans="1:3">
@@ -10339,7 +10348,7 @@
         <v>289</v>
       </c>
       <c r="B233" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -10347,7 +10356,7 @@
         <v>290</v>
       </c>
       <c r="B234" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
     </row>
     <row r="235" spans="1:3">
@@ -10355,7 +10364,7 @@
         <v>291</v>
       </c>
       <c r="B235" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -10363,7 +10372,7 @@
         <v>632</v>
       </c>
       <c r="B236" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="237" spans="1:3">
@@ -10379,7 +10388,7 @@
         <v>469</v>
       </c>
       <c r="B239" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -10406,7 +10415,7 @@
         <v>295</v>
       </c>
       <c r="B242" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="C242" t="s">
         <v>530</v>
@@ -10417,7 +10426,7 @@
         <v>296</v>
       </c>
       <c r="B243" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -10425,7 +10434,7 @@
         <v>452</v>
       </c>
       <c r="B244" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -10433,10 +10442,10 @@
         <v>298</v>
       </c>
       <c r="B245" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C245" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -10444,7 +10453,7 @@
         <v>299</v>
       </c>
       <c r="B246" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -10452,7 +10461,7 @@
         <v>300</v>
       </c>
       <c r="B247" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -10460,7 +10469,7 @@
         <v>301</v>
       </c>
       <c r="B248" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -10468,7 +10477,7 @@
         <v>302</v>
       </c>
       <c r="B249" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="250" spans="1:3">
@@ -10476,7 +10485,7 @@
         <v>633</v>
       </c>
       <c r="B250" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -10780,35 +10789,35 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B287" t="s">
         <v>1060</v>
       </c>
-      <c r="B287" t="s">
-        <v>1061</v>
-      </c>
       <c r="C287" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B288" t="s">
         <v>1062</v>
       </c>
-      <c r="B288" t="s">
-        <v>1063</v>
-      </c>
       <c r="C288" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B289" t="s">
         <v>1064</v>
       </c>
-      <c r="B289" t="s">
-        <v>1065</v>
-      </c>
       <c r="C289" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="290" spans="1:3">
@@ -10832,35 +10841,35 @@
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B293" t="s">
         <v>1053</v>
       </c>
-      <c r="B293" t="s">
+      <c r="C293" t="s">
         <v>1054</v>
-      </c>
-      <c r="C293" t="s">
-        <v>1055</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B294" t="s">
         <v>1056</v>
       </c>
-      <c r="B294" t="s">
-        <v>1057</v>
-      </c>
       <c r="C294" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B295" t="s">
         <v>1058</v>
       </c>
-      <c r="B295" t="s">
-        <v>1059</v>
-      </c>
       <c r="C295" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="297" spans="1:3">
@@ -10992,7 +11001,7 @@
         <v>724</v>
       </c>
       <c r="B311" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="C311" t="s">
         <v>620</v>
@@ -11000,10 +11009,10 @@
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
+        <v>1147</v>
+      </c>
+      <c r="B312" t="s">
         <v>1148</v>
-      </c>
-      <c r="B312" t="s">
-        <v>1149</v>
       </c>
     </row>
     <row r="313" spans="1:3">
@@ -11215,320 +11224,323 @@
     </row>
     <row r="339" spans="1:3">
       <c r="A339" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B339" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C339" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3">
+      <c r="A340" t="s">
         <v>475</v>
       </c>
-      <c r="B339" t="s">
+      <c r="B340" t="s">
         <v>614</v>
-      </c>
-    </row>
-    <row r="341" spans="1:3">
-      <c r="A341" t="s">
-        <v>739</v>
-      </c>
-      <c r="B341" t="s">
-        <v>740</v>
-      </c>
-      <c r="C341" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="B342" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="C342" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="344" spans="1:3">
-      <c r="A344" t="s">
-        <v>747</v>
-      </c>
-      <c r="B344" t="s">
-        <v>748</v>
+    <row r="343" spans="1:3">
+      <c r="A343" t="s">
+        <v>741</v>
+      </c>
+      <c r="B343" t="s">
+        <v>742</v>
+      </c>
+      <c r="C343" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B345" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="B346" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="B347" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="B348" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="B349" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B350" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="B351" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B352" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B353" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B354" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B355" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B356" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B357" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B358" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B359" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>1141</v>
+        <v>777</v>
       </c>
       <c r="B360" t="s">
-        <v>1142</v>
+        <v>778</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>779</v>
+        <v>1140</v>
       </c>
       <c r="B361" t="s">
-        <v>780</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
+        <v>779</v>
+      </c>
+      <c r="B362" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B363" t="s">
         <v>781</v>
-      </c>
-      <c r="B362" t="s">
-        <v>782</v>
-      </c>
-    </row>
-    <row r="364" spans="1:2">
-      <c r="A364" t="s">
-        <v>783</v>
-      </c>
-      <c r="B364" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="B365" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="B366" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="B367" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="B368" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="B369" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="B370" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="B371" t="s">
-        <v>318</v>
+        <v>795</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B372" t="s">
-        <v>799</v>
+        <v>318</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B373" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="B374" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
+        <v>801</v>
+      </c>
+      <c r="B375" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" t="s">
+        <v>803</v>
+      </c>
+      <c r="B376" t="s">
         <v>804</v>
-      </c>
-      <c r="B375" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="377" spans="1:2">
-      <c r="A377" t="s">
-        <v>806</v>
-      </c>
-      <c r="B377" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="B378" t="s">
-        <v>808</v>
+        <v>311</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="B379" t="s">
-        <v>313</v>
+        <v>807</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="B380" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" t="s">
+        <v>809</v>
+      </c>
+      <c r="B381" t="s">
         <v>314</v>
-      </c>
-    </row>
-    <row r="382" spans="1:2">
-      <c r="A382" t="s">
-        <v>833</v>
-      </c>
-      <c r="B382" t="s">
-        <v>834</v>
       </c>
     </row>
     <row r="383" spans="1:2">
@@ -11536,148 +11548,148 @@
         <v>832</v>
       </c>
       <c r="B383" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="B384" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="B385" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="B386" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>830</v>
+        <v>823</v>
       </c>
       <c r="B387" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2">
+      <c r="A388" t="s">
         <v>829</v>
       </c>
-    </row>
-    <row r="389" spans="1:2">
-      <c r="A389" t="s">
-        <v>837</v>
-      </c>
-      <c r="B389" t="s">
-        <v>842</v>
+      <c r="B388" t="s">
+        <v>828</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>845</v>
+        <v>836</v>
       </c>
       <c r="B390" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="B391" t="s">
-        <v>826</v>
+        <v>842</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="B392" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="B393" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="B394" t="s">
-        <v>844</v>
-      </c>
-    </row>
-    <row r="396" spans="1:2">
-      <c r="A396" t="s">
-        <v>850</v>
-      </c>
-      <c r="B396" t="s">
-        <v>851</v>
+        <v>827</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2">
+      <c r="A395" t="s">
+        <v>840</v>
+      </c>
+      <c r="B395" t="s">
+        <v>843</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="B397" t="s">
-        <v>1158</v>
+        <v>850</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="B398" t="s">
-        <v>1123</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="B399" t="s">
-        <v>1116</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>861</v>
+        <v>854</v>
       </c>
       <c r="B400" t="s">
-        <v>1102</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="B401" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="B402" t="s">
-        <v>1122</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="B403" t="s">
         <v>1121</v>
@@ -11685,7 +11697,7 @@
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="B404" t="s">
         <v>1120</v>
@@ -11693,7 +11705,7 @@
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="B405" t="s">
         <v>1119</v>
@@ -11701,7 +11713,7 @@
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="B406" t="s">
         <v>1118</v>
@@ -11709,7 +11721,7 @@
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="B407" t="s">
         <v>1117</v>
@@ -11717,42 +11729,42 @@
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="B408" t="s">
-        <v>860</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="B409" t="s">
-        <v>1124</v>
+        <v>859</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="B410" t="s">
-        <v>278</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="B411" t="s">
-        <v>817</v>
+        <v>278</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="B412" t="s">
-        <v>626</v>
+        <v>816</v>
       </c>
     </row>
     <row r="413" spans="1:2">
@@ -11760,87 +11772,87 @@
         <v>864</v>
       </c>
       <c r="B413" t="s">
-        <v>1125</v>
+        <v>626</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>1106</v>
+        <v>863</v>
       </c>
       <c r="B414" t="s">
-        <v>1104</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="B415" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="B416" t="s">
-        <v>1108</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
       <c r="B417" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
       <c r="B418" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="B419" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>1127</v>
+        <v>1114</v>
       </c>
       <c r="B420" t="s">
-        <v>1126</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B421" t="s">
+        <v>1125</v>
+      </c>
+    </row>
+    <row r="422" spans="1:2">
+      <c r="A422" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B422" t="s">
         <v>1128</v>
-      </c>
-      <c r="B421" t="s">
-        <v>1129</v>
-      </c>
-    </row>
-    <row r="423" spans="1:2">
-      <c r="A423" t="s">
-        <v>935</v>
-      </c>
-      <c r="B423" t="s">
-        <v>914</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>954</v>
+        <v>934</v>
       </c>
       <c r="B424" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
     </row>
     <row r="425" spans="1:2">
@@ -11848,7 +11860,7 @@
         <v>953</v>
       </c>
       <c r="B425" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
     </row>
     <row r="426" spans="1:2">
@@ -11856,7 +11868,7 @@
         <v>952</v>
       </c>
       <c r="B426" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
     </row>
     <row r="427" spans="1:2">
@@ -11864,7 +11876,7 @@
         <v>951</v>
       </c>
       <c r="B427" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
     </row>
     <row r="428" spans="1:2">
@@ -11872,7 +11884,7 @@
         <v>950</v>
       </c>
       <c r="B428" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
     </row>
     <row r="429" spans="1:2">
@@ -11880,7 +11892,7 @@
         <v>949</v>
       </c>
       <c r="B429" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
     </row>
     <row r="430" spans="1:2">
@@ -11888,7 +11900,7 @@
         <v>948</v>
       </c>
       <c r="B430" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
     </row>
     <row r="431" spans="1:2">
@@ -11896,7 +11908,7 @@
         <v>947</v>
       </c>
       <c r="B431" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
     </row>
     <row r="432" spans="1:2">
@@ -11904,7 +11916,7 @@
         <v>946</v>
       </c>
       <c r="B432" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
     </row>
     <row r="433" spans="1:2">
@@ -11912,23 +11924,23 @@
         <v>945</v>
       </c>
       <c r="B433" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>955</v>
+        <v>944</v>
       </c>
       <c r="B434" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>944</v>
+        <v>954</v>
       </c>
       <c r="B435" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
     </row>
     <row r="436" spans="1:2">
@@ -11936,7 +11948,7 @@
         <v>943</v>
       </c>
       <c r="B436" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
     </row>
     <row r="437" spans="1:2">
@@ -11944,7 +11956,7 @@
         <v>942</v>
       </c>
       <c r="B437" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
     </row>
     <row r="438" spans="1:2">
@@ -11952,7 +11964,7 @@
         <v>941</v>
       </c>
       <c r="B438" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
     </row>
     <row r="439" spans="1:2">
@@ -11960,7 +11972,7 @@
         <v>940</v>
       </c>
       <c r="B439" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
     </row>
     <row r="440" spans="1:2">
@@ -11968,7 +11980,7 @@
         <v>939</v>
       </c>
       <c r="B440" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
     </row>
     <row r="441" spans="1:2">
@@ -11976,7 +11988,7 @@
         <v>938</v>
       </c>
       <c r="B441" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
     </row>
     <row r="442" spans="1:2">
@@ -11984,7 +11996,7 @@
         <v>937</v>
       </c>
       <c r="B442" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
     </row>
     <row r="443" spans="1:2">
@@ -11992,79 +12004,79 @@
         <v>936</v>
       </c>
       <c r="B443" t="s">
-        <v>934</v>
-      </c>
-    </row>
-    <row r="445" spans="1:2">
-      <c r="A445" t="s">
-        <v>977</v>
-      </c>
-      <c r="B445" t="s">
-        <v>958</v>
+        <v>932</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" t="s">
+        <v>935</v>
+      </c>
+      <c r="B444" t="s">
+        <v>933</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>968</v>
+        <v>976</v>
       </c>
       <c r="B446" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="B447" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="B448" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>973</v>
+        <v>969</v>
       </c>
       <c r="B449" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B450" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>974</v>
+        <v>970</v>
       </c>
       <c r="B451" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="B452" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
       <c r="B453" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
     </row>
     <row r="454" spans="1:2">
@@ -12072,159 +12084,159 @@
         <v>975</v>
       </c>
       <c r="B454" t="s">
-        <v>967</v>
-      </c>
-    </row>
-    <row r="456" spans="1:2">
-      <c r="A456" t="s">
-        <v>982</v>
-      </c>
-      <c r="B456" t="s">
-        <v>984</v>
+        <v>965</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2">
+      <c r="A455" t="s">
+        <v>974</v>
+      </c>
+      <c r="B455" t="s">
+        <v>966</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
+        <v>981</v>
+      </c>
+      <c r="B457" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
+        <v>992</v>
+      </c>
+      <c r="B458" t="s">
         <v>993</v>
-      </c>
-      <c r="B457" t="s">
-        <v>994</v>
-      </c>
-    </row>
-    <row r="459" spans="1:2">
-      <c r="A459" t="s">
-        <v>983</v>
-      </c>
-      <c r="B459" t="s">
-        <v>985</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
+        <v>982</v>
+      </c>
+      <c r="B460" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" t="s">
+        <v>994</v>
+      </c>
+      <c r="B461" t="s">
         <v>995</v>
-      </c>
-      <c r="B460" t="s">
-        <v>996</v>
-      </c>
-    </row>
-    <row r="462" spans="1:2">
-      <c r="A462" t="s">
-        <v>990</v>
-      </c>
-      <c r="B462" t="s">
-        <v>988</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="B463" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
       <c r="B464" t="s">
-        <v>992</v>
-      </c>
-    </row>
-    <row r="466" spans="1:2">
-      <c r="A466" t="s">
-        <v>1005</v>
-      </c>
-      <c r="B466" t="s">
-        <v>998</v>
+        <v>988</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" t="s">
+        <v>986</v>
+      </c>
+      <c r="B465" t="s">
+        <v>991</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="B467" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="B468" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1052</v>
+        <v>1006</v>
       </c>
       <c r="B469" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1008</v>
+        <v>1051</v>
       </c>
       <c r="B470" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="B471" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="B472" t="s">
-        <v>1004</v>
-      </c>
-    </row>
-    <row r="474" spans="1:2">
-      <c r="A474" t="s">
-        <v>1022</v>
-      </c>
-      <c r="B474" t="s">
-        <v>1016</v>
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B473" t="s">
+        <v>1003</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
-        <v>1027</v>
+        <v>1021</v>
       </c>
       <c r="B475" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1023</v>
+        <v>1026</v>
       </c>
       <c r="B476" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B477" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1026</v>
+        <v>1023</v>
       </c>
       <c r="B478" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="479" spans="1:2">
@@ -12232,211 +12244,219 @@
         <v>1025</v>
       </c>
       <c r="B479" t="s">
-        <v>1021</v>
-      </c>
-    </row>
-    <row r="481" spans="1:2">
-      <c r="A481" t="s">
-        <v>1040</v>
-      </c>
-      <c r="B481" t="s">
-        <v>1028</v>
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="480" spans="1:2">
+      <c r="A480" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1020</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="B482" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="B483" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="B484" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B485" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="B486" t="s">
-        <v>1033</v>
-      </c>
-    </row>
-    <row r="488" spans="1:2">
-      <c r="A488" t="s">
-        <v>1041</v>
-      </c>
-      <c r="B488" t="s">
-        <v>1042</v>
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="487" spans="1:2">
+      <c r="A487" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1032</v>
       </c>
     </row>
     <row r="489" spans="1:2">
       <c r="A489" t="s">
-        <v>1047</v>
+        <v>1040</v>
       </c>
       <c r="B489" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="B490" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="B491" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="B492" t="s">
-        <v>1046</v>
-      </c>
-    </row>
-    <row r="494" spans="1:2">
-      <c r="A494" t="s">
-        <v>1074</v>
-      </c>
-      <c r="B494" t="s">
-        <v>1075</v>
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="493" spans="1:2">
+      <c r="A493" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1045</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1090</v>
+        <v>1073</v>
       </c>
       <c r="B495" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="B496" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="B497" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1101</v>
+        <v>1091</v>
       </c>
       <c r="B498" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1093</v>
+        <v>1100</v>
       </c>
       <c r="B499" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="B500" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="B501" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="B502" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="B503" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="B504" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="B505" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="B506" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1089</v>
+        <v>1099</v>
       </c>
       <c r="B507" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="508" spans="1:2">
+      <c r="A508" t="s">
         <v>1088</v>
       </c>
+      <c r="B508" t="s">
+        <v>1087</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A462:A463 A459:A460 A445:A454 A456:A457">
+  <conditionalFormatting sqref="A463:A464 A460:A461 A446:A455 A457:A458">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rcv and AS household questions
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C742C6AC-D653-407B-A81F-67E704025175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3CF3893-04F7-4E22-AC3D-DE0ADD26BADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28350" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="1168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1401" uniqueCount="1170">
   <si>
     <t>Name</t>
   </si>
@@ -3544,6 +3544,12 @@
   </si>
   <si>
     <t>Newly added by Bagi for AZ</t>
+  </si>
+  <si>
+    <t>RCV_EmailReceiptAndClarification</t>
+  </si>
+  <si>
+    <t>Regular Contributions Verification email receipt requires manual review.</t>
   </si>
 </sst>
 </file>
@@ -8420,7 +8426,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C508"/>
+  <dimension ref="A1:C509"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -12017,446 +12023,454 @@
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>976</v>
+        <v>1168</v>
       </c>
       <c r="B446" t="s">
-        <v>957</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>967</v>
+        <v>976</v>
       </c>
       <c r="B447" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B448" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B449" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="B450" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="B451" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="B452" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="B453" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="B454" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
+        <v>975</v>
+      </c>
+      <c r="B455" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2">
+      <c r="A456" t="s">
         <v>974</v>
       </c>
-      <c r="B455" t="s">
+      <c r="B456" t="s">
         <v>966</v>
-      </c>
-    </row>
-    <row r="457" spans="1:2">
-      <c r="A457" t="s">
-        <v>981</v>
-      </c>
-      <c r="B457" t="s">
-        <v>983</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
+        <v>981</v>
+      </c>
+      <c r="B458" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" t="s">
         <v>992</v>
       </c>
-      <c r="B458" t="s">
+      <c r="B459" t="s">
         <v>993</v>
-      </c>
-    </row>
-    <row r="460" spans="1:2">
-      <c r="A460" t="s">
-        <v>982</v>
-      </c>
-      <c r="B460" t="s">
-        <v>984</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
+        <v>982</v>
+      </c>
+      <c r="B461" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" t="s">
         <v>994</v>
       </c>
-      <c r="B461" t="s">
+      <c r="B462" t="s">
         <v>995</v>
-      </c>
-    </row>
-    <row r="463" spans="1:2">
-      <c r="A463" t="s">
-        <v>989</v>
-      </c>
-      <c r="B463" t="s">
-        <v>987</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B464" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
+        <v>990</v>
+      </c>
+      <c r="B465" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" t="s">
         <v>986</v>
       </c>
-      <c r="B465" t="s">
+      <c r="B466" t="s">
         <v>991</v>
-      </c>
-    </row>
-    <row r="467" spans="1:2">
-      <c r="A467" t="s">
-        <v>1004</v>
-      </c>
-      <c r="B467" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B468" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B469" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1051</v>
+        <v>1006</v>
       </c>
       <c r="B470" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1007</v>
+        <v>1051</v>
       </c>
       <c r="B471" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B472" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B473" t="s">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2">
+      <c r="A474" t="s">
         <v>1009</v>
       </c>
-      <c r="B473" t="s">
+      <c r="B474" t="s">
         <v>1003</v>
-      </c>
-    </row>
-    <row r="475" spans="1:2">
-      <c r="A475" t="s">
-        <v>1021</v>
-      </c>
-      <c r="B475" t="s">
-        <v>1015</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1026</v>
+        <v>1021</v>
       </c>
       <c r="B476" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="B477" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B478" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="B479" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2">
+      <c r="A481" t="s">
         <v>1024</v>
       </c>
-      <c r="B480" t="s">
+      <c r="B481" t="s">
         <v>1020</v>
-      </c>
-    </row>
-    <row r="482" spans="1:2">
-      <c r="A482" t="s">
-        <v>1039</v>
-      </c>
-      <c r="B482" t="s">
-        <v>1027</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="B483" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B484" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B485" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B486" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2">
+      <c r="A488" t="s">
         <v>1038</v>
       </c>
-      <c r="B487" t="s">
+      <c r="B488" t="s">
         <v>1032</v>
-      </c>
-    </row>
-    <row r="489" spans="1:2">
-      <c r="A489" t="s">
-        <v>1040</v>
-      </c>
-      <c r="B489" t="s">
-        <v>1041</v>
       </c>
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
-        <v>1046</v>
+        <v>1040</v>
       </c>
       <c r="B490" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B491" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B492" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="494" spans="1:2">
+      <c r="A494" t="s">
         <v>1049</v>
       </c>
-      <c r="B493" t="s">
+      <c r="B494" t="s">
         <v>1045</v>
-      </c>
-    </row>
-    <row r="495" spans="1:2">
-      <c r="A495" t="s">
-        <v>1073</v>
-      </c>
-      <c r="B495" t="s">
-        <v>1074</v>
       </c>
     </row>
     <row r="496" spans="1:2">
       <c r="A496" t="s">
-        <v>1089</v>
+        <v>1073</v>
       </c>
       <c r="B496" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="B497" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B498" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1100</v>
+        <v>1091</v>
       </c>
       <c r="B499" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1092</v>
+        <v>1100</v>
       </c>
       <c r="B500" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="B501" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="B502" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B503" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="B504" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="B505" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B506" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B507" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B508" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="509" spans="1:2">
+      <c r="A509" t="s">
         <v>1088</v>
       </c>
-      <c r="B508" t="s">
+      <c r="B509" t="s">
         <v>1087</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A463:A464 A460:A461 A446:A455 A457:A458">
+  <conditionalFormatting sqref="A464:A465 A461:A462 A447:A456 A458:A459">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
redo the changes from earlier
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3CF3893-04F7-4E22-AC3D-DE0ADD26BADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C26B4F9-40A8-4E9C-8F14-7DE7F601D5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1401" uniqueCount="1170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1403" uniqueCount="1172">
   <si>
     <t>Name</t>
   </si>
@@ -1830,63 +1830,6 @@
     <t>removed this check</t>
   </si>
   <si>
-    <t>Unable to validate findings for Self-Employment Certification. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Application Summary. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Member Information Document. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Income &amp; Asset Questionnaire. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Errors in Validating findings for Self Certification of Non Employment. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Asset Self Certification &amp; Worksheet. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Affidavit of Student Financial Assistance. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Student Certification. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Errors in Validating findings for Certification of Zero Income. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for VAWA Acknowledgement. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Screening Document. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Paystub. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Verification of Employment. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Offer Letter. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Work Number. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Verification Services. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Child Support Payment History. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Supplemental Security Income Letter. Needs manual review.</t>
-  </si>
-  <si>
-    <t>Unable to validate findings for Verification of Reccurring Cash Contribution. Needs manual review.</t>
-  </si>
-  <si>
     <t>BusinessAskedToRemovePage2check but on different page</t>
   </si>
   <si>
@@ -1962,9 +1905,6 @@
     <t>AnnualSC_FindingError</t>
   </si>
   <si>
-    <t>Errors in Validating findings for Annual Student Certification since there is Home unit . Needs manual review.</t>
-  </si>
-  <si>
     <t>ICW_UnbornChildDOBListedInThePast</t>
   </si>
   <si>
@@ -2103,9 +2043,6 @@
     <t>HHD_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Housing History Disclosure. Needs manual review.</t>
-  </si>
-  <si>
     <t>Supporting documents have not been provided for Child Support Calcs documented on the Income &amp; Asset Questionnaire.</t>
   </si>
   <si>
@@ -2238,9 +2175,6 @@
     <t>ICW_ZeroAnnualIncome</t>
   </si>
   <si>
-    <t>Unable to validate findings for Income Calculation Worksheet. Needs manual review.</t>
-  </si>
-  <si>
     <t>Annual Income is above the Income Limit listed on the Income Calculation Worksheet.</t>
   </si>
   <si>
@@ -2268,9 +2202,6 @@
     <t>HDR_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Housing Demographic Reporting Form. Needs manual review.</t>
-  </si>
-  <si>
     <t>RDC_BothHourlyIncomeAndPSDocumented</t>
   </si>
   <si>
@@ -2385,9 +2316,6 @@
     <t>Amount listed on the Certification of Self-Employment Income and ICW do not match.</t>
   </si>
   <si>
-    <t>Unable to validate findings for Certification of Self-Employment Income. Needs manual review.</t>
-  </si>
-  <si>
     <t>PL_ApplicantNameCheck</t>
   </si>
   <si>
@@ -2454,9 +2382,6 @@
     <t>PL_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Profit/Loss Statement. Manual review required.</t>
-  </si>
-  <si>
     <t>1040_NameListCheck</t>
   </si>
   <si>
@@ -2526,9 +2451,6 @@
     <t>Dates are not within 120 days of move in.</t>
   </si>
   <si>
-    <t>Unable to validate findings for Application/Tenant Release and Consent. Needs manual review.</t>
-  </si>
-  <si>
     <t>ARC_FindingError</t>
   </si>
   <si>
@@ -2571,9 +2493,6 @@
     <t>Asset type, member name, or asset value does not match Income &amp; Asset Questionnaire for all assets.</t>
   </si>
   <si>
-    <t>Unable to validate findings for Household Asset Breakdown. Needs manual review.</t>
-  </si>
-  <si>
     <t>HAB_NameAndAssetsinIAQ</t>
   </si>
   <si>
@@ -2841,9 +2760,6 @@
     <t>Dates on the Certification of Student Status are not within 120 days of the Move-In date.</t>
   </si>
   <si>
-    <t>Unable to validate findings for the Certification of Student Status. Needs manual review.</t>
-  </si>
-  <si>
     <t>CSSExists</t>
   </si>
   <si>
@@ -2940,9 +2856,6 @@
     <t xml:space="preserve">Frequency of payments checkbox on the Regular Contributions Verification has not been documented appropriately. </t>
   </si>
   <si>
-    <t>Unable to validate findings for Regular Contributions Verification. Needs manual review.</t>
-  </si>
-  <si>
     <t>RCV_RecipientNameCheck</t>
   </si>
   <si>
@@ -3015,21 +2928,12 @@
     <t>VABL_ICWCheck</t>
   </si>
   <si>
-    <t>Unable to validate findings for Veterans Affairs Benefits Letter. Manual review required.</t>
-  </si>
-  <si>
     <t>BS_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Bank Statements. Needs manual review.</t>
-  </si>
-  <si>
     <t>LES_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Leave and Earnings Statement. Needs manual review.</t>
-  </si>
-  <si>
     <t>Veterans Benefits Letter</t>
   </si>
   <si>
@@ -3102,9 +3006,6 @@
     <t>Date on the Tenant Rights and Resource Guide (TRRG) is not within 120 days of the move-in date. </t>
   </si>
   <si>
-    <t>Unable to validate findings for the Tenant Rights and Resource Guide (TRRG). Manual review required. </t>
-  </si>
-  <si>
     <t>TRRG_HeadOfHousehold</t>
   </si>
   <si>
@@ -3138,9 +3039,6 @@
     <t>The date on the TSAHC is not within 120 days of the move-in date. </t>
   </si>
   <si>
-    <t>Unable to validate findings for the TSAHC. Manual review required. </t>
-  </si>
-  <si>
     <t>TSAHC</t>
   </si>
   <si>
@@ -3216,9 +3114,6 @@
     <t>CSC_FindingError</t>
   </si>
   <si>
-    <t>Unable to validate findings for Child Support Calcs. Needs manual review.</t>
-  </si>
-  <si>
     <t>CSPH_PaymentGenerationDate</t>
   </si>
   <si>
@@ -3414,9 +3309,6 @@
     <t>Not all fields have been documented appropriately on the Employment Verification.</t>
   </si>
   <si>
-    <t>Unable to validate findings for Employment Verification. Needs manual review.</t>
-  </si>
-  <si>
     <t>No communication options (Phone #, Fax #, or Email) have been included on the Employment Verification for the Authorized Representative. </t>
   </si>
   <si>
@@ -3550,6 +3442,120 @@
   </si>
   <si>
     <t>Regular Contributions Verification email receipt requires manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Housing History Disclosure. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Income Calculation Worksheet. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Application Summary. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Member Information Document. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Income &amp; Asset Questionnaire. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Asset Self Certification &amp; Worksheet. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Affidavit of Student Financial Assistance. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Student Certification. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate VAWA Acknowledgement. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Screening Document. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Paystub. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Verification of Employment. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Offer Letter. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Work Number. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Verification Services. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Self-Employment Certification. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Child Support Payment History. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Child Support Calcs. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Supplemental Security Income Letter. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Verification of Reccurring Cash Contribution. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Housing Demographic Reporting Form. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Certification of Self-Employment Income. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Profit/Loss Statement. Manual review required.</t>
+  </si>
+  <si>
+    <t>Unable to validate Application/Tenant Release and Consent. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Household Asset Breakdown. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Employment Verification. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate the Certification of Student Status. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Regular Contributions Verification. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Bank Statements. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Leave and Earnings Statement. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Veterans Affairs Benefits Letter. Manual review required.</t>
+  </si>
+  <si>
+    <t>Unable to validate the Tenant Rights and Resource Guide (TRRG). Manual review required. </t>
+  </si>
+  <si>
+    <t>Unable to validate the TSAHC. Manual review required. </t>
+  </si>
+  <si>
+    <t>Unable to validate Self Certification of Non Employment. Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Annual Student Certification since there is Home unit . Needs manual review.</t>
+  </si>
+  <si>
+    <t>Unable to validate Certification of Zero Income. Needs manual review.</t>
+  </si>
+  <si>
+    <t>EV_TX_ApplicantName</t>
+  </si>
+  <si>
+    <t>Applicant Name across the Employment Verification, Day Calculator, and Income Calculation Worksheet do not match.</t>
   </si>
 </sst>
 </file>
@@ -3985,7 +3991,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1161</v>
+        <v>1125</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -4006,7 +4012,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1162</v>
+        <v>1126</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -4018,7 +4024,7 @@
         <v>203</v>
       </c>
       <c r="B7" t="s">
-        <v>1151</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4048,10 +4054,10 @@
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>1149</v>
+        <v>1113</v>
       </c>
       <c r="B12" t="s">
-        <v>1149</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -4072,10 +4078,10 @@
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>634</v>
+        <v>615</v>
       </c>
       <c r="B15" t="s">
-        <v>635</v>
+        <v>616</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
@@ -4175,7 +4181,7 @@
         <v>409</v>
       </c>
       <c r="B26" t="s">
-        <v>1012</v>
+        <v>980</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
@@ -4319,141 +4325,141 @@
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>738</v>
+        <v>716</v>
       </c>
       <c r="B44" t="s">
-        <v>737</v>
+        <v>715</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>746</v>
+        <v>723</v>
       </c>
       <c r="B45" t="s">
-        <v>1012</v>
+        <v>980</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>834</v>
+        <v>808</v>
       </c>
       <c r="B46" t="s">
-        <v>835</v>
+        <v>809</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>845</v>
+        <v>818</v>
       </c>
       <c r="B47" t="s">
-        <v>846</v>
+        <v>819</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>847</v>
+        <v>820</v>
       </c>
       <c r="B48" t="s">
-        <v>848</v>
+        <v>821</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>874</v>
+        <v>847</v>
       </c>
       <c r="B49" t="s">
-        <v>875</v>
+        <v>848</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>911</v>
+        <v>884</v>
       </c>
       <c r="B50" t="s">
-        <v>912</v>
+        <v>885</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1">
       <c r="A51" t="s">
-        <v>955</v>
+        <v>927</v>
       </c>
       <c r="B51" t="s">
-        <v>956</v>
+        <v>928</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>977</v>
+        <v>948</v>
       </c>
       <c r="B52" t="s">
-        <v>978</v>
+        <v>949</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>979</v>
+        <v>950</v>
       </c>
       <c r="B53" t="s">
-        <v>980</v>
+        <v>951</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>985</v>
+        <v>956</v>
       </c>
       <c r="B54" t="s">
-        <v>996</v>
+        <v>964</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="14.25" customHeight="1">
       <c r="A55" t="s">
-        <v>1010</v>
+        <v>978</v>
       </c>
       <c r="B55" t="s">
-        <v>1011</v>
+        <v>979</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="14.25" customHeight="1">
       <c r="A56" t="s">
-        <v>1013</v>
+        <v>981</v>
       </c>
       <c r="B56" t="s">
-        <v>1013</v>
+        <v>981</v>
       </c>
       <c r="C56" t="s">
-        <v>1014</v>
+        <v>982</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>1033</v>
+        <v>999</v>
       </c>
       <c r="B57" t="s">
-        <v>1033</v>
+        <v>999</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>1050</v>
+        <v>1016</v>
       </c>
       <c r="B58" t="s">
-        <v>1137</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1">
       <c r="A59" t="s">
-        <v>1142</v>
+        <v>1106</v>
       </c>
       <c r="B59" t="s">
-        <v>1143</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="14.25" customHeight="1">
       <c r="A60" t="s">
-        <v>1071</v>
+        <v>1036</v>
       </c>
       <c r="B60" t="s">
-        <v>1072</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5747,7 +5753,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>719</v>
+        <v>698</v>
       </c>
       <c r="B42" t="s">
         <v>436</v>
@@ -5950,10 +5956,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>706</v>
+        <v>685</v>
       </c>
       <c r="B20" t="s">
-        <v>706</v>
+        <v>685</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -5966,10 +5972,10 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>658</v>
+        <v>638</v>
       </c>
       <c r="B22" t="s">
-        <v>657</v>
+        <v>637</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -7072,10 +7078,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>736</v>
+        <v>714</v>
       </c>
       <c r="B3" t="s">
-        <v>736</v>
+        <v>714</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -7224,10 +7230,10 @@
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>1163</v>
+        <v>1127</v>
       </c>
       <c r="B22" t="s">
-        <v>1163</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
@@ -7368,90 +7374,90 @@
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>698</v>
+        <v>677</v>
       </c>
       <c r="B40" t="s">
-        <v>698</v>
+        <v>677</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>617</v>
+        <v>598</v>
       </c>
       <c r="B41" t="s">
-        <v>617</v>
+        <v>598</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>655</v>
+        <v>635</v>
       </c>
       <c r="B42" t="s">
-        <v>655</v>
+        <v>635</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>660</v>
+        <v>640</v>
       </c>
       <c r="B43" t="s">
-        <v>660</v>
+        <v>640</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>705</v>
+        <v>684</v>
       </c>
       <c r="B44" t="s">
-        <v>705</v>
+        <v>684</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>1067</v>
+        <v>1032</v>
       </c>
       <c r="B45" t="s">
-        <v>1067</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>1068</v>
+        <v>1033</v>
       </c>
       <c r="B46" t="s">
-        <v>1068</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>1069</v>
+        <v>1034</v>
       </c>
       <c r="B47" t="s">
-        <v>1069</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>1070</v>
+        <v>1035</v>
       </c>
       <c r="B48" t="s">
-        <v>1070</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
-        <v>1138</v>
+        <v>1102</v>
       </c>
       <c r="B49" t="s">
-        <v>1138</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>1139</v>
+        <v>1103</v>
       </c>
       <c r="B50" t="s">
-        <v>1139</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
@@ -8426,7 +8432,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C509"/>
+  <dimension ref="A1:C510"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8452,87 +8458,87 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>1145</v>
+        <v>1109</v>
       </c>
       <c r="B5" t="s">
-        <v>1146</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>651</v>
+        <v>631</v>
       </c>
       <c r="B7" t="s">
-        <v>689</v>
+        <v>668</v>
       </c>
       <c r="C7" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>683</v>
+        <v>663</v>
       </c>
       <c r="B8" t="s">
-        <v>690</v>
+        <v>669</v>
       </c>
       <c r="C8" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>684</v>
+        <v>664</v>
       </c>
       <c r="B9" t="s">
-        <v>691</v>
+        <v>670</v>
       </c>
       <c r="C9" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>685</v>
+        <v>665</v>
       </c>
       <c r="B10" t="s">
-        <v>693</v>
+        <v>672</v>
       </c>
       <c r="C10" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>694</v>
+        <v>673</v>
       </c>
       <c r="B11" t="s">
-        <v>692</v>
+        <v>671</v>
       </c>
       <c r="C11" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>720</v>
+        <v>699</v>
       </c>
       <c r="B12" t="s">
-        <v>721</v>
+        <v>700</v>
       </c>
       <c r="C12" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>686</v>
+        <v>666</v>
       </c>
       <c r="B13" t="s">
-        <v>687</v>
+        <v>1134</v>
       </c>
       <c r="C13" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -8564,7 +8570,7 @@
         <v>75</v>
       </c>
       <c r="B18" t="s">
-        <v>733</v>
+        <v>711</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -8588,73 +8594,73 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>616</v>
+        <v>597</v>
       </c>
       <c r="B21" t="s">
-        <v>725</v>
+        <v>704</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>628</v>
+        <v>609</v>
       </c>
       <c r="B22" t="s">
-        <v>734</v>
+        <v>712</v>
       </c>
       <c r="C22" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>641</v>
+        <v>621</v>
       </c>
       <c r="B23" t="s">
-        <v>642</v>
+        <v>622</v>
       </c>
       <c r="C23" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>654</v>
+        <v>634</v>
       </c>
       <c r="B24" t="s">
-        <v>735</v>
+        <v>713</v>
       </c>
       <c r="C24" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>656</v>
+        <v>636</v>
       </c>
       <c r="B25" t="s">
-        <v>659</v>
+        <v>639</v>
       </c>
       <c r="C25" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>731</v>
+        <v>710</v>
       </c>
       <c r="B26" t="s">
-        <v>1132</v>
+        <v>1096</v>
       </c>
       <c r="C26" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>876</v>
+        <v>849</v>
       </c>
       <c r="B27" t="s">
-        <v>877</v>
+        <v>850</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -8662,7 +8668,7 @@
         <v>478</v>
       </c>
       <c r="B28" t="s">
-        <v>732</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -8710,7 +8716,7 @@
         <v>192</v>
       </c>
       <c r="B35" t="s">
-        <v>717</v>
+        <v>696</v>
       </c>
     </row>
     <row r="36" spans="1:3">
@@ -8718,7 +8724,7 @@
         <v>193</v>
       </c>
       <c r="B36" t="s">
-        <v>718</v>
+        <v>697</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -8766,29 +8772,29 @@
         <v>592</v>
       </c>
       <c r="B42" t="s">
-        <v>727</v>
+        <v>706</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>643</v>
+        <v>623</v>
       </c>
       <c r="B43" t="s">
-        <v>644</v>
+        <v>624</v>
       </c>
       <c r="C43" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>722</v>
+        <v>701</v>
       </c>
       <c r="B44" t="s">
-        <v>723</v>
+        <v>702</v>
       </c>
       <c r="C44" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="45" spans="1:3">
@@ -8796,7 +8802,7 @@
         <v>493</v>
       </c>
       <c r="B45" t="s">
-        <v>597</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -8884,29 +8890,29 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>711</v>
+        <v>690</v>
       </c>
       <c r="B57" t="s">
-        <v>712</v>
+        <v>691</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>1065</v>
+        <v>1030</v>
       </c>
       <c r="B58" t="s">
-        <v>1066</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>621</v>
+        <v>602</v>
       </c>
       <c r="B59" t="s">
-        <v>622</v>
+        <v>603</v>
       </c>
       <c r="C59" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -8914,7 +8920,7 @@
         <v>492</v>
       </c>
       <c r="B60" t="s">
-        <v>598</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -9004,7 +9010,7 @@
         <v>198</v>
       </c>
       <c r="B70" t="s">
-        <v>713</v>
+        <v>692</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -9012,7 +9018,7 @@
         <v>199</v>
       </c>
       <c r="B71" t="s">
-        <v>714</v>
+        <v>693</v>
       </c>
       <c r="C71" t="s">
         <v>530</v>
@@ -9023,7 +9029,7 @@
         <v>521</v>
       </c>
       <c r="B72" t="s">
-        <v>715</v>
+        <v>694</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -9039,7 +9045,7 @@
         <v>502</v>
       </c>
       <c r="B74" t="s">
-        <v>716</v>
+        <v>695</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -9047,18 +9053,18 @@
         <v>491</v>
       </c>
       <c r="B75" t="s">
-        <v>599</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>671</v>
+        <v>651</v>
       </c>
       <c r="B76" t="s">
-        <v>670</v>
+        <v>650</v>
       </c>
       <c r="C76" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="78" spans="1:3">
@@ -9095,46 +9101,46 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>681</v>
+        <v>661</v>
       </c>
       <c r="B82" t="s">
-        <v>682</v>
+        <v>662</v>
       </c>
       <c r="C82" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>701</v>
+        <v>680</v>
       </c>
       <c r="B83" t="s">
-        <v>702</v>
+        <v>681</v>
       </c>
       <c r="C83" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>700</v>
+        <v>679</v>
       </c>
       <c r="B84" t="s">
-        <v>703</v>
+        <v>682</v>
       </c>
       <c r="C84" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>699</v>
+        <v>678</v>
       </c>
       <c r="B85" t="s">
-        <v>704</v>
+        <v>683</v>
       </c>
       <c r="C85" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -9142,7 +9148,7 @@
         <v>490</v>
       </c>
       <c r="B86" t="s">
-        <v>600</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -9150,29 +9156,29 @@
         <v>183</v>
       </c>
       <c r="B88" t="s">
-        <v>1129</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>680</v>
+        <v>660</v>
       </c>
       <c r="B89" t="s">
-        <v>695</v>
+        <v>674</v>
       </c>
       <c r="C89" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>678</v>
+        <v>658</v>
       </c>
       <c r="B90" t="s">
-        <v>679</v>
+        <v>659</v>
       </c>
       <c r="C90" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -9231,7 +9237,7 @@
         <v>448</v>
       </c>
       <c r="C97" t="s">
-        <v>615</v>
+        <v>596</v>
       </c>
     </row>
     <row r="98" spans="1:3">
@@ -9266,54 +9272,54 @@
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>645</v>
+        <v>625</v>
       </c>
       <c r="B101" t="s">
-        <v>646</v>
+        <v>626</v>
       </c>
       <c r="C101" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>905</v>
+        <v>878</v>
       </c>
       <c r="B102" t="s">
-        <v>906</v>
+        <v>879</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>672</v>
+        <v>652</v>
       </c>
       <c r="B103" t="s">
-        <v>673</v>
+        <v>653</v>
       </c>
       <c r="C103" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>675</v>
+        <v>655</v>
       </c>
       <c r="B104" t="s">
-        <v>674</v>
+        <v>654</v>
       </c>
       <c r="C104" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>677</v>
+        <v>657</v>
       </c>
       <c r="B105" t="s">
-        <v>676</v>
+        <v>656</v>
       </c>
       <c r="C105" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="106" spans="1:3">
@@ -9321,39 +9327,39 @@
         <v>489</v>
       </c>
       <c r="B106" t="s">
-        <v>601</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>901</v>
+        <v>874</v>
       </c>
       <c r="B107" t="s">
-        <v>902</v>
+        <v>875</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>903</v>
+        <v>876</v>
       </c>
       <c r="B108" t="s">
-        <v>904</v>
+        <v>877</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>908</v>
+        <v>881</v>
       </c>
       <c r="B109" t="s">
-        <v>909</v>
+        <v>882</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>910</v>
+        <v>883</v>
       </c>
       <c r="B110" t="s">
-        <v>907</v>
+        <v>880</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -9388,12 +9394,12 @@
         <v>522</v>
       </c>
       <c r="C115" t="s">
-        <v>619</v>
+        <v>600</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>618</v>
+        <v>599</v>
       </c>
       <c r="B116" t="s">
         <v>522</v>
@@ -9436,7 +9442,7 @@
         <v>488</v>
       </c>
       <c r="B121" t="s">
-        <v>602</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="123" spans="1:3">
@@ -9473,13 +9479,13 @@
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>730</v>
+        <v>709</v>
       </c>
       <c r="B127" t="s">
-        <v>729</v>
+        <v>708</v>
       </c>
       <c r="C127" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -9503,10 +9509,10 @@
         <v>568</v>
       </c>
       <c r="B130" t="s">
-        <v>623</v>
+        <v>604</v>
       </c>
       <c r="C130" t="s">
-        <v>627</v>
+        <v>608</v>
       </c>
     </row>
     <row r="131" spans="1:3">
@@ -9519,13 +9525,13 @@
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>647</v>
+        <v>627</v>
       </c>
       <c r="B132" t="s">
-        <v>648</v>
+        <v>628</v>
       </c>
       <c r="C132" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -9533,29 +9539,29 @@
         <v>487</v>
       </c>
       <c r="B133" t="s">
-        <v>603</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>636</v>
+        <v>617</v>
       </c>
       <c r="B135" t="s">
-        <v>637</v>
+        <v>618</v>
       </c>
       <c r="C135" t="s">
-        <v>638</v>
+        <v>619</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>639</v>
+        <v>620</v>
       </c>
       <c r="B136" t="s">
-        <v>640</v>
+        <v>1168</v>
       </c>
       <c r="C136" t="s">
-        <v>638</v>
+        <v>619</v>
       </c>
     </row>
     <row r="138" spans="1:3">
@@ -9595,21 +9601,21 @@
         <v>504</v>
       </c>
       <c r="B142" t="s">
-        <v>661</v>
+        <v>641</v>
       </c>
       <c r="C142" t="s">
-        <v>662</v>
+        <v>642</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>1144</v>
+        <v>1108</v>
       </c>
       <c r="B143" t="s">
-        <v>1150</v>
+        <v>1114</v>
       </c>
       <c r="C143" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -9625,7 +9631,7 @@
         <v>486</v>
       </c>
       <c r="B145" t="s">
-        <v>604</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -9665,18 +9671,18 @@
         <v>485</v>
       </c>
       <c r="B151" t="s">
-        <v>605</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>649</v>
+        <v>629</v>
       </c>
       <c r="B152" t="s">
-        <v>650</v>
+        <v>630</v>
       </c>
       <c r="C152" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="154" spans="1:3">
@@ -9760,7 +9766,7 @@
         <v>474</v>
       </c>
       <c r="B162" t="s">
-        <v>606</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="164" spans="1:3">
@@ -9768,7 +9774,7 @@
         <v>590</v>
       </c>
       <c r="B164" t="s">
-        <v>880</v>
+        <v>853</v>
       </c>
       <c r="C164" t="s">
         <v>591</v>
@@ -9776,57 +9782,57 @@
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>652</v>
+        <v>632</v>
       </c>
       <c r="B165" t="s">
-        <v>653</v>
+        <v>633</v>
       </c>
       <c r="C165" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>743</v>
+        <v>720</v>
       </c>
       <c r="B166" t="s">
-        <v>881</v>
+        <v>854</v>
       </c>
       <c r="C166" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>744</v>
+        <v>721</v>
       </c>
       <c r="B167" t="s">
-        <v>882</v>
+        <v>855</v>
       </c>
       <c r="C167" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>745</v>
+        <v>722</v>
       </c>
       <c r="B168" t="s">
-        <v>726</v>
+        <v>705</v>
       </c>
       <c r="C168" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>1134</v>
+        <v>1098</v>
       </c>
       <c r="B169" t="s">
-        <v>887</v>
+        <v>860</v>
       </c>
       <c r="C169" t="s">
-        <v>1135</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -9834,18 +9840,18 @@
         <v>465</v>
       </c>
       <c r="B171" t="s">
-        <v>1152</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>1158</v>
+        <v>1122</v>
       </c>
       <c r="B172" t="s">
-        <v>1159</v>
+        <v>1123</v>
       </c>
       <c r="C172" t="s">
-        <v>1160</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="173" spans="1:3">
@@ -9853,7 +9859,7 @@
         <v>236</v>
       </c>
       <c r="B173" t="s">
-        <v>883</v>
+        <v>856</v>
       </c>
       <c r="C173" t="s">
         <v>530</v>
@@ -9864,7 +9870,7 @@
         <v>237</v>
       </c>
       <c r="B174" t="s">
-        <v>884</v>
+        <v>857</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -9872,7 +9878,7 @@
         <v>245</v>
       </c>
       <c r="B175" t="s">
-        <v>885</v>
+        <v>858</v>
       </c>
       <c r="C175" t="s">
         <v>588</v>
@@ -9880,13 +9886,13 @@
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>710</v>
+        <v>689</v>
       </c>
       <c r="B176" t="s">
-        <v>886</v>
+        <v>859</v>
       </c>
       <c r="C176" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -9910,10 +9916,10 @@
         <v>240</v>
       </c>
       <c r="B179" t="s">
-        <v>887</v>
+        <v>860</v>
       </c>
       <c r="C179" t="s">
-        <v>1136</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="180" spans="1:3">
@@ -9921,7 +9927,7 @@
         <v>241</v>
       </c>
       <c r="B180" t="s">
-        <v>888</v>
+        <v>861</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -9929,7 +9935,7 @@
         <v>242</v>
       </c>
       <c r="B181" t="s">
-        <v>889</v>
+        <v>862</v>
       </c>
     </row>
     <row r="182" spans="1:3">
@@ -9937,7 +9943,7 @@
         <v>243</v>
       </c>
       <c r="B182" t="s">
-        <v>890</v>
+        <v>863</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -9945,7 +9951,7 @@
         <v>244</v>
       </c>
       <c r="B183" t="s">
-        <v>815</v>
+        <v>790</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -9953,10 +9959,10 @@
         <v>276</v>
       </c>
       <c r="B184" t="s">
-        <v>887</v>
+        <v>860</v>
       </c>
       <c r="C184" t="s">
-        <v>1136</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -9972,45 +9978,45 @@
         <v>593</v>
       </c>
       <c r="B186" t="s">
-        <v>1131</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>629</v>
+        <v>610</v>
       </c>
       <c r="B187" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>696</v>
+        <v>675</v>
       </c>
       <c r="B188" t="s">
-        <v>697</v>
+        <v>676</v>
       </c>
       <c r="C188" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>709</v>
+        <v>688</v>
       </c>
       <c r="B189" t="s">
-        <v>728</v>
+        <v>707</v>
       </c>
       <c r="C189" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>899</v>
+        <v>872</v>
       </c>
       <c r="B190" t="s">
-        <v>900</v>
+        <v>873</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -10018,18 +10024,18 @@
         <v>473</v>
       </c>
       <c r="B191" t="s">
-        <v>607</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>707</v>
+        <v>686</v>
       </c>
       <c r="B193" t="s">
-        <v>708</v>
+        <v>687</v>
       </c>
       <c r="C193" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -10037,7 +10043,7 @@
         <v>466</v>
       </c>
       <c r="B194" t="s">
-        <v>1153</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -10045,7 +10051,7 @@
         <v>246</v>
       </c>
       <c r="B195" t="s">
-        <v>891</v>
+        <v>864</v>
       </c>
       <c r="C195" t="s">
         <v>595</v>
@@ -10056,10 +10062,10 @@
         <v>248</v>
       </c>
       <c r="B196" t="s">
-        <v>892</v>
+        <v>865</v>
       </c>
       <c r="C196" t="s">
-        <v>624</v>
+        <v>605</v>
       </c>
     </row>
     <row r="197" spans="1:3">
@@ -10067,7 +10073,7 @@
         <v>247</v>
       </c>
       <c r="B197" t="s">
-        <v>853</v>
+        <v>826</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -10110,7 +10116,7 @@
         <v>255</v>
       </c>
       <c r="B202" t="s">
-        <v>855</v>
+        <v>828</v>
       </c>
     </row>
     <row r="203" spans="1:3">
@@ -10126,7 +10132,7 @@
         <v>261</v>
       </c>
       <c r="B204" t="s">
-        <v>856</v>
+        <v>829</v>
       </c>
     </row>
     <row r="205" spans="1:3">
@@ -10134,7 +10140,7 @@
         <v>262</v>
       </c>
       <c r="B205" t="s">
-        <v>857</v>
+        <v>830</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -10142,7 +10148,7 @@
         <v>263</v>
       </c>
       <c r="B206" t="s">
-        <v>893</v>
+        <v>866</v>
       </c>
       <c r="C206" t="s">
         <v>595</v>
@@ -10153,7 +10159,7 @@
         <v>264</v>
       </c>
       <c r="B207" t="s">
-        <v>858</v>
+        <v>831</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -10161,7 +10167,7 @@
         <v>265</v>
       </c>
       <c r="B208" t="s">
-        <v>894</v>
+        <v>867</v>
       </c>
       <c r="C208" t="s">
         <v>595</v>
@@ -10172,7 +10178,7 @@
         <v>266</v>
       </c>
       <c r="B209" t="s">
-        <v>859</v>
+        <v>832</v>
       </c>
     </row>
     <row r="210" spans="1:3">
@@ -10188,10 +10194,10 @@
         <v>275</v>
       </c>
       <c r="B211" t="s">
-        <v>887</v>
+        <v>860</v>
       </c>
       <c r="C211" t="s">
-        <v>1136</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="212" spans="1:3">
@@ -10204,10 +10210,10 @@
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>630</v>
+        <v>611</v>
       </c>
       <c r="B213" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -10215,18 +10221,18 @@
         <v>484</v>
       </c>
       <c r="B214" t="s">
-        <v>608</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>625</v>
+        <v>606</v>
       </c>
       <c r="B215" t="s">
-        <v>626</v>
+        <v>607</v>
       </c>
       <c r="C215" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="217" spans="1:3">
@@ -10234,7 +10240,7 @@
         <v>467</v>
       </c>
       <c r="B217" t="s">
-        <v>1154</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -10250,7 +10256,7 @@
         <v>271</v>
       </c>
       <c r="B219" t="s">
-        <v>817</v>
+        <v>792</v>
       </c>
     </row>
     <row r="220" spans="1:3">
@@ -10258,7 +10264,7 @@
         <v>272</v>
       </c>
       <c r="B220" t="s">
-        <v>818</v>
+        <v>793</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -10266,7 +10272,7 @@
         <v>280</v>
       </c>
       <c r="B221" t="s">
-        <v>819</v>
+        <v>794</v>
       </c>
     </row>
     <row r="222" spans="1:3">
@@ -10274,7 +10280,7 @@
         <v>279</v>
       </c>
       <c r="B222" t="s">
-        <v>821</v>
+        <v>796</v>
       </c>
     </row>
     <row r="223" spans="1:3">
@@ -10282,15 +10288,15 @@
         <v>281</v>
       </c>
       <c r="B223" t="s">
-        <v>820</v>
+        <v>795</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>631</v>
+        <v>612</v>
       </c>
       <c r="B224" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -10298,7 +10304,7 @@
         <v>483</v>
       </c>
       <c r="B225" t="s">
-        <v>609</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="227" spans="1:3">
@@ -10306,7 +10312,7 @@
         <v>468</v>
       </c>
       <c r="B227" t="s">
-        <v>1155</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="228" spans="1:3">
@@ -10322,7 +10328,7 @@
         <v>284</v>
       </c>
       <c r="B229" t="s">
-        <v>810</v>
+        <v>785</v>
       </c>
     </row>
     <row r="230" spans="1:3">
@@ -10338,7 +10344,7 @@
         <v>286</v>
       </c>
       <c r="B231" t="s">
-        <v>811</v>
+        <v>786</v>
       </c>
     </row>
     <row r="232" spans="1:3">
@@ -10346,7 +10352,7 @@
         <v>288</v>
       </c>
       <c r="B232" t="s">
-        <v>813</v>
+        <v>788</v>
       </c>
     </row>
     <row r="233" spans="1:3">
@@ -10354,7 +10360,7 @@
         <v>289</v>
       </c>
       <c r="B233" t="s">
-        <v>812</v>
+        <v>787</v>
       </c>
     </row>
     <row r="234" spans="1:3">
@@ -10362,7 +10368,7 @@
         <v>290</v>
       </c>
       <c r="B234" t="s">
-        <v>814</v>
+        <v>789</v>
       </c>
     </row>
     <row r="235" spans="1:3">
@@ -10370,15 +10376,15 @@
         <v>291</v>
       </c>
       <c r="B235" t="s">
-        <v>815</v>
+        <v>790</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>632</v>
+        <v>613</v>
       </c>
       <c r="B236" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="237" spans="1:3">
@@ -10386,7 +10392,7 @@
         <v>482</v>
       </c>
       <c r="B237" t="s">
-        <v>610</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="239" spans="1:3">
@@ -10394,7 +10400,7 @@
         <v>469</v>
       </c>
       <c r="B239" t="s">
-        <v>1156</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -10421,7 +10427,7 @@
         <v>295</v>
       </c>
       <c r="B242" t="s">
-        <v>895</v>
+        <v>868</v>
       </c>
       <c r="C242" t="s">
         <v>530</v>
@@ -10432,7 +10438,7 @@
         <v>296</v>
       </c>
       <c r="B243" t="s">
-        <v>878</v>
+        <v>851</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -10440,7 +10446,7 @@
         <v>452</v>
       </c>
       <c r="B244" t="s">
-        <v>879</v>
+        <v>852</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -10448,10 +10454,10 @@
         <v>298</v>
       </c>
       <c r="B245" t="s">
-        <v>887</v>
+        <v>860</v>
       </c>
       <c r="C245" t="s">
-        <v>1133</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="246" spans="1:3">
@@ -10459,7 +10465,7 @@
         <v>299</v>
       </c>
       <c r="B246" t="s">
-        <v>896</v>
+        <v>869</v>
       </c>
     </row>
     <row r="247" spans="1:3">
@@ -10467,7 +10473,7 @@
         <v>300</v>
       </c>
       <c r="B247" t="s">
-        <v>897</v>
+        <v>870</v>
       </c>
     </row>
     <row r="248" spans="1:3">
@@ -10475,7 +10481,7 @@
         <v>301</v>
       </c>
       <c r="B248" t="s">
-        <v>898</v>
+        <v>871</v>
       </c>
     </row>
     <row r="249" spans="1:3">
@@ -10483,15 +10489,15 @@
         <v>302</v>
       </c>
       <c r="B249" t="s">
-        <v>815</v>
+        <v>790</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>633</v>
+        <v>614</v>
       </c>
       <c r="B250" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="251" spans="1:3">
@@ -10499,18 +10505,18 @@
         <v>481</v>
       </c>
       <c r="B251" t="s">
-        <v>611</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>667</v>
+        <v>647</v>
       </c>
       <c r="B253" t="s">
-        <v>668</v>
+        <v>648</v>
       </c>
       <c r="C253" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="254" spans="1:3">
@@ -10677,7 +10683,7 @@
         <v>480</v>
       </c>
       <c r="B272" t="s">
-        <v>596</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="274" spans="1:3">
@@ -10795,35 +10801,35 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>1059</v>
+        <v>1024</v>
       </c>
       <c r="B287" t="s">
-        <v>1060</v>
+        <v>1025</v>
       </c>
       <c r="C287" t="s">
-        <v>1054</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>1061</v>
+        <v>1026</v>
       </c>
       <c r="B288" t="s">
-        <v>1062</v>
+        <v>1027</v>
       </c>
       <c r="C288" t="s">
-        <v>1054</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>1063</v>
+        <v>1028</v>
       </c>
       <c r="B289" t="s">
-        <v>1064</v>
+        <v>1029</v>
       </c>
       <c r="C289" t="s">
-        <v>1054</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="290" spans="1:3">
@@ -10831,62 +10837,62 @@
         <v>479</v>
       </c>
       <c r="B290" t="s">
-        <v>612</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>669</v>
+        <v>649</v>
       </c>
       <c r="B292" t="s">
-        <v>688</v>
+        <v>667</v>
       </c>
       <c r="C292" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>1052</v>
+        <v>1018</v>
       </c>
       <c r="B293" t="s">
-        <v>1053</v>
+        <v>1019</v>
       </c>
       <c r="C293" t="s">
-        <v>1054</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>1055</v>
+        <v>1021</v>
       </c>
       <c r="B294" t="s">
-        <v>1056</v>
+        <v>1022</v>
       </c>
       <c r="C294" t="s">
-        <v>1054</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>1057</v>
+        <v>1023</v>
       </c>
       <c r="B295" t="s">
-        <v>1058</v>
+        <v>1151</v>
       </c>
       <c r="C295" t="s">
-        <v>1054</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>665</v>
+        <v>645</v>
       </c>
       <c r="B297" t="s">
-        <v>666</v>
+        <v>646</v>
       </c>
       <c r="C297" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="298" spans="1:3">
@@ -11004,21 +11010,21 @@
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>724</v>
+        <v>703</v>
       </c>
       <c r="B311" t="s">
-        <v>1130</v>
+        <v>1094</v>
       </c>
       <c r="C311" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>1147</v>
+        <v>1111</v>
       </c>
       <c r="B312" t="s">
-        <v>1148</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="313" spans="1:3">
@@ -11026,7 +11032,7 @@
         <v>477</v>
       </c>
       <c r="B313" t="s">
-        <v>613</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="314" spans="1:3">
@@ -11155,7 +11161,7 @@
         <v>476</v>
       </c>
       <c r="B329" t="s">
-        <v>613</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="330" spans="1:3">
@@ -11168,13 +11174,13 @@
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>663</v>
+        <v>643</v>
       </c>
       <c r="B332" t="s">
-        <v>664</v>
+        <v>644</v>
       </c>
       <c r="C332" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="333" spans="1:3">
@@ -11230,13 +11236,13 @@
     </row>
     <row r="339" spans="1:3">
       <c r="A339" t="s">
-        <v>1165</v>
+        <v>1129</v>
       </c>
       <c r="B339" t="s">
-        <v>1166</v>
+        <v>1130</v>
       </c>
       <c r="C339" t="s">
-        <v>1167</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="340" spans="1:3">
@@ -11244,242 +11250,242 @@
         <v>475</v>
       </c>
       <c r="B340" t="s">
-        <v>614</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>739</v>
+        <v>717</v>
       </c>
       <c r="B342" t="s">
-        <v>740</v>
+        <v>718</v>
       </c>
       <c r="C342" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>741</v>
+        <v>719</v>
       </c>
       <c r="B343" t="s">
-        <v>742</v>
+        <v>1154</v>
       </c>
       <c r="C343" t="s">
-        <v>620</v>
+        <v>601</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>747</v>
+        <v>724</v>
       </c>
       <c r="B345" t="s">
-        <v>748</v>
+        <v>725</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>749</v>
+        <v>726</v>
       </c>
       <c r="B346" t="s">
-        <v>750</v>
+        <v>727</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>751</v>
+        <v>728</v>
       </c>
       <c r="B347" t="s">
-        <v>752</v>
+        <v>729</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>753</v>
+        <v>730</v>
       </c>
       <c r="B348" t="s">
-        <v>754</v>
+        <v>731</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>755</v>
+        <v>732</v>
       </c>
       <c r="B349" t="s">
-        <v>756</v>
+        <v>733</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>757</v>
+        <v>734</v>
       </c>
       <c r="B350" t="s">
-        <v>758</v>
+        <v>735</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>759</v>
+        <v>736</v>
       </c>
       <c r="B351" t="s">
-        <v>760</v>
+        <v>737</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>761</v>
+        <v>738</v>
       </c>
       <c r="B352" t="s">
-        <v>762</v>
+        <v>739</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>763</v>
+        <v>740</v>
       </c>
       <c r="B353" t="s">
-        <v>764</v>
+        <v>741</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>765</v>
+        <v>742</v>
       </c>
       <c r="B354" t="s">
-        <v>766</v>
+        <v>743</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>767</v>
+        <v>744</v>
       </c>
       <c r="B355" t="s">
-        <v>768</v>
+        <v>745</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>769</v>
+        <v>746</v>
       </c>
       <c r="B356" t="s">
-        <v>770</v>
+        <v>747</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>771</v>
+        <v>748</v>
       </c>
       <c r="B357" t="s">
-        <v>772</v>
+        <v>749</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>773</v>
+        <v>750</v>
       </c>
       <c r="B358" t="s">
-        <v>774</v>
+        <v>751</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>775</v>
+        <v>752</v>
       </c>
       <c r="B359" t="s">
-        <v>776</v>
+        <v>753</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>777</v>
+        <v>754</v>
       </c>
       <c r="B360" t="s">
-        <v>778</v>
+        <v>755</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>1140</v>
+        <v>1104</v>
       </c>
       <c r="B361" t="s">
-        <v>1141</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>779</v>
+        <v>756</v>
       </c>
       <c r="B362" t="s">
-        <v>780</v>
+        <v>757</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>1164</v>
+        <v>1128</v>
       </c>
       <c r="B363" t="s">
-        <v>781</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>782</v>
+        <v>758</v>
       </c>
       <c r="B365" t="s">
-        <v>783</v>
+        <v>759</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>784</v>
+        <v>760</v>
       </c>
       <c r="B366" t="s">
-        <v>785</v>
+        <v>761</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>786</v>
+        <v>762</v>
       </c>
       <c r="B367" t="s">
-        <v>787</v>
+        <v>763</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>788</v>
+        <v>764</v>
       </c>
       <c r="B368" t="s">
-        <v>789</v>
+        <v>765</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>790</v>
+        <v>766</v>
       </c>
       <c r="B369" t="s">
-        <v>791</v>
+        <v>767</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>792</v>
+        <v>768</v>
       </c>
       <c r="B370" t="s">
-        <v>793</v>
+        <v>769</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>794</v>
+        <v>770</v>
       </c>
       <c r="B371" t="s">
-        <v>795</v>
+        <v>771</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>796</v>
+        <v>772</v>
       </c>
       <c r="B372" t="s">
         <v>318</v>
@@ -11487,39 +11493,39 @@
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>797</v>
+        <v>773</v>
       </c>
       <c r="B373" t="s">
-        <v>798</v>
+        <v>774</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>799</v>
+        <v>775</v>
       </c>
       <c r="B374" t="s">
-        <v>800</v>
+        <v>776</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>801</v>
+        <v>777</v>
       </c>
       <c r="B375" t="s">
-        <v>802</v>
+        <v>778</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
-        <v>803</v>
+        <v>779</v>
       </c>
       <c r="B376" t="s">
-        <v>804</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>805</v>
+        <v>780</v>
       </c>
       <c r="B378" t="s">
         <v>311</v>
@@ -11527,15 +11533,15 @@
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>806</v>
+        <v>781</v>
       </c>
       <c r="B379" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>808</v>
+        <v>783</v>
       </c>
       <c r="B380" t="s">
         <v>313</v>
@@ -11543,7 +11549,7 @@
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>809</v>
+        <v>784</v>
       </c>
       <c r="B381" t="s">
         <v>314</v>
@@ -11551,215 +11557,215 @@
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>832</v>
+        <v>806</v>
       </c>
       <c r="B383" t="s">
-        <v>833</v>
+        <v>807</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>831</v>
+        <v>805</v>
       </c>
       <c r="B384" t="s">
-        <v>830</v>
+        <v>804</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>824</v>
+        <v>799</v>
       </c>
       <c r="B385" t="s">
-        <v>825</v>
+        <v>800</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>822</v>
+        <v>797</v>
       </c>
       <c r="B386" t="s">
-        <v>826</v>
+        <v>801</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>823</v>
+        <v>798</v>
       </c>
       <c r="B387" t="s">
-        <v>827</v>
+        <v>802</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>829</v>
+        <v>803</v>
       </c>
       <c r="B388" t="s">
-        <v>828</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>836</v>
+        <v>810</v>
       </c>
       <c r="B390" t="s">
-        <v>841</v>
+        <v>815</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>844</v>
+        <v>817</v>
       </c>
       <c r="B391" t="s">
-        <v>842</v>
+        <v>816</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>837</v>
+        <v>811</v>
       </c>
       <c r="B392" t="s">
-        <v>825</v>
+        <v>800</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>838</v>
+        <v>812</v>
       </c>
       <c r="B393" t="s">
-        <v>826</v>
+        <v>801</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>839</v>
+        <v>813</v>
       </c>
       <c r="B394" t="s">
-        <v>827</v>
+        <v>802</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>840</v>
+        <v>814</v>
       </c>
       <c r="B395" t="s">
-        <v>843</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>849</v>
+        <v>822</v>
       </c>
       <c r="B397" t="s">
-        <v>850</v>
+        <v>823</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>851</v>
+        <v>824</v>
       </c>
       <c r="B398" t="s">
-        <v>1157</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>852</v>
+        <v>825</v>
       </c>
       <c r="B399" t="s">
-        <v>1122</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>854</v>
+        <v>827</v>
       </c>
       <c r="B400" t="s">
-        <v>1115</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>860</v>
+        <v>833</v>
       </c>
       <c r="B401" t="s">
-        <v>1101</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>861</v>
+        <v>834</v>
       </c>
       <c r="B402" t="s">
-        <v>1102</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>862</v>
+        <v>835</v>
       </c>
       <c r="B403" t="s">
-        <v>1121</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>865</v>
+        <v>838</v>
       </c>
       <c r="B404" t="s">
-        <v>1120</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>866</v>
+        <v>839</v>
       </c>
       <c r="B405" t="s">
-        <v>1119</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>867</v>
+        <v>840</v>
       </c>
       <c r="B406" t="s">
-        <v>1118</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>868</v>
+        <v>841</v>
       </c>
       <c r="B407" t="s">
-        <v>1117</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>869</v>
+        <v>842</v>
       </c>
       <c r="B408" t="s">
-        <v>1116</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>870</v>
+        <v>843</v>
       </c>
       <c r="B409" t="s">
-        <v>859</v>
+        <v>832</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>871</v>
+        <v>844</v>
       </c>
       <c r="B410" t="s">
-        <v>1123</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>872</v>
+        <v>845</v>
       </c>
       <c r="B411" t="s">
         <v>278</v>
@@ -11767,710 +11773,718 @@
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>873</v>
+        <v>846</v>
       </c>
       <c r="B412" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>864</v>
+        <v>837</v>
       </c>
       <c r="B413" t="s">
-        <v>626</v>
+        <v>607</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>863</v>
+        <v>836</v>
       </c>
       <c r="B414" t="s">
-        <v>1124</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1105</v>
+        <v>1070</v>
       </c>
       <c r="B415" t="s">
-        <v>1103</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1106</v>
+        <v>1071</v>
       </c>
       <c r="B416" t="s">
-        <v>1104</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>1108</v>
+        <v>1073</v>
       </c>
       <c r="B417" t="s">
-        <v>1107</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>1112</v>
+        <v>1077</v>
       </c>
       <c r="B418" t="s">
-        <v>1109</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>1113</v>
+        <v>1078</v>
       </c>
       <c r="B419" t="s">
-        <v>1110</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>1114</v>
+        <v>1079</v>
       </c>
       <c r="B420" t="s">
-        <v>1111</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>1126</v>
+        <v>1090</v>
       </c>
       <c r="B421" t="s">
-        <v>1125</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>1127</v>
+        <v>1091</v>
       </c>
       <c r="B422" t="s">
-        <v>1128</v>
-      </c>
-    </row>
-    <row r="424" spans="1:2">
-      <c r="A424" t="s">
-        <v>934</v>
-      </c>
-      <c r="B424" t="s">
-        <v>913</v>
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="423" spans="1:2">
+      <c r="A423" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1171</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>953</v>
+        <v>906</v>
       </c>
       <c r="B425" t="s">
-        <v>914</v>
+        <v>886</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>952</v>
+        <v>925</v>
       </c>
       <c r="B426" t="s">
-        <v>915</v>
+        <v>887</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>951</v>
+        <v>924</v>
       </c>
       <c r="B427" t="s">
-        <v>916</v>
+        <v>888</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>950</v>
+        <v>923</v>
       </c>
       <c r="B428" t="s">
-        <v>917</v>
+        <v>889</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>949</v>
+        <v>922</v>
       </c>
       <c r="B429" t="s">
-        <v>918</v>
+        <v>890</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>948</v>
+        <v>921</v>
       </c>
       <c r="B430" t="s">
-        <v>919</v>
+        <v>891</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>947</v>
+        <v>920</v>
       </c>
       <c r="B431" t="s">
-        <v>920</v>
+        <v>892</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>946</v>
+        <v>919</v>
       </c>
       <c r="B432" t="s">
-        <v>921</v>
+        <v>893</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>945</v>
+        <v>918</v>
       </c>
       <c r="B433" t="s">
-        <v>922</v>
+        <v>894</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>944</v>
+        <v>917</v>
       </c>
       <c r="B434" t="s">
-        <v>923</v>
+        <v>895</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>954</v>
+        <v>916</v>
       </c>
       <c r="B435" t="s">
-        <v>924</v>
+        <v>896</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>943</v>
+        <v>926</v>
       </c>
       <c r="B436" t="s">
-        <v>925</v>
+        <v>897</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>942</v>
+        <v>915</v>
       </c>
       <c r="B437" t="s">
-        <v>926</v>
+        <v>898</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>941</v>
+        <v>914</v>
       </c>
       <c r="B438" t="s">
-        <v>927</v>
+        <v>899</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>940</v>
+        <v>913</v>
       </c>
       <c r="B439" t="s">
-        <v>928</v>
+        <v>900</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>939</v>
+        <v>912</v>
       </c>
       <c r="B440" t="s">
-        <v>929</v>
+        <v>901</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>938</v>
+        <v>911</v>
       </c>
       <c r="B441" t="s">
-        <v>930</v>
+        <v>902</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>937</v>
+        <v>910</v>
       </c>
       <c r="B442" t="s">
-        <v>931</v>
+        <v>903</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>936</v>
+        <v>909</v>
       </c>
       <c r="B443" t="s">
-        <v>932</v>
+        <v>904</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>935</v>
+        <v>908</v>
       </c>
       <c r="B444" t="s">
-        <v>933</v>
-      </c>
-    </row>
-    <row r="446" spans="1:2">
-      <c r="A446" t="s">
-        <v>1168</v>
-      </c>
-      <c r="B446" t="s">
-        <v>1169</v>
+        <v>905</v>
+      </c>
+    </row>
+    <row r="445" spans="1:2">
+      <c r="A445" t="s">
+        <v>907</v>
+      </c>
+      <c r="B445" t="s">
+        <v>1160</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>976</v>
+        <v>1132</v>
       </c>
       <c r="B447" t="s">
-        <v>957</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>967</v>
+        <v>947</v>
       </c>
       <c r="B448" t="s">
-        <v>958</v>
+        <v>929</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>968</v>
+        <v>938</v>
       </c>
       <c r="B449" t="s">
-        <v>959</v>
+        <v>930</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>969</v>
+        <v>939</v>
       </c>
       <c r="B450" t="s">
-        <v>960</v>
+        <v>931</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>972</v>
+        <v>940</v>
       </c>
       <c r="B451" t="s">
-        <v>961</v>
+        <v>932</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>970</v>
+        <v>943</v>
       </c>
       <c r="B452" t="s">
-        <v>962</v>
+        <v>933</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>973</v>
+        <v>941</v>
       </c>
       <c r="B453" t="s">
-        <v>963</v>
+        <v>934</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>971</v>
+        <v>944</v>
       </c>
       <c r="B454" t="s">
-        <v>964</v>
+        <v>935</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>975</v>
+        <v>942</v>
       </c>
       <c r="B455" t="s">
-        <v>965</v>
+        <v>936</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>974</v>
+        <v>946</v>
       </c>
       <c r="B456" t="s">
-        <v>966</v>
-      </c>
-    </row>
-    <row r="458" spans="1:2">
-      <c r="A458" t="s">
-        <v>981</v>
-      </c>
-      <c r="B458" t="s">
-        <v>983</v>
+        <v>937</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
+        <v>945</v>
+      </c>
+      <c r="B457" t="s">
+        <v>1161</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>992</v>
+        <v>952</v>
       </c>
       <c r="B459" t="s">
-        <v>993</v>
-      </c>
-    </row>
-    <row r="461" spans="1:2">
-      <c r="A461" t="s">
-        <v>982</v>
-      </c>
-      <c r="B461" t="s">
-        <v>984</v>
+        <v>954</v>
+      </c>
+    </row>
+    <row r="460" spans="1:2">
+      <c r="A460" t="s">
+        <v>962</v>
+      </c>
+      <c r="B460" t="s">
+        <v>1162</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>994</v>
+        <v>953</v>
       </c>
       <c r="B462" t="s">
-        <v>995</v>
-      </c>
-    </row>
-    <row r="464" spans="1:2">
-      <c r="A464" t="s">
-        <v>989</v>
-      </c>
-      <c r="B464" t="s">
-        <v>987</v>
+        <v>955</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2">
+      <c r="A463" t="s">
+        <v>963</v>
+      </c>
+      <c r="B463" t="s">
+        <v>1163</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>990</v>
+        <v>960</v>
       </c>
       <c r="B465" t="s">
-        <v>988</v>
+        <v>958</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>986</v>
+        <v>961</v>
       </c>
       <c r="B466" t="s">
-        <v>991</v>
-      </c>
-    </row>
-    <row r="468" spans="1:2">
-      <c r="A468" t="s">
-        <v>1004</v>
-      </c>
-      <c r="B468" t="s">
-        <v>997</v>
+        <v>959</v>
+      </c>
+    </row>
+    <row r="467" spans="1:2">
+      <c r="A467" t="s">
+        <v>957</v>
+      </c>
+      <c r="B467" t="s">
+        <v>1164</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>1005</v>
+        <v>972</v>
       </c>
       <c r="B469" t="s">
-        <v>998</v>
+        <v>965</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>1006</v>
+        <v>973</v>
       </c>
       <c r="B470" t="s">
-        <v>999</v>
+        <v>966</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>1051</v>
+        <v>974</v>
       </c>
       <c r="B471" t="s">
-        <v>1000</v>
+        <v>967</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1007</v>
+        <v>1017</v>
       </c>
       <c r="B472" t="s">
-        <v>1001</v>
+        <v>968</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>1008</v>
+        <v>975</v>
       </c>
       <c r="B473" t="s">
-        <v>1002</v>
+        <v>969</v>
       </c>
     </row>
     <row r="474" spans="1:2">
       <c r="A474" t="s">
-        <v>1009</v>
+        <v>976</v>
       </c>
       <c r="B474" t="s">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="476" spans="1:2">
-      <c r="A476" t="s">
-        <v>1021</v>
-      </c>
-      <c r="B476" t="s">
-        <v>1015</v>
+        <v>970</v>
+      </c>
+    </row>
+    <row r="475" spans="1:2">
+      <c r="A475" t="s">
+        <v>977</v>
+      </c>
+      <c r="B475" t="s">
+        <v>971</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>1026</v>
+        <v>988</v>
       </c>
       <c r="B477" t="s">
-        <v>1016</v>
+        <v>983</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>1022</v>
+        <v>993</v>
       </c>
       <c r="B478" t="s">
-        <v>1017</v>
+        <v>984</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>1023</v>
+        <v>989</v>
       </c>
       <c r="B479" t="s">
-        <v>1018</v>
+        <v>985</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>1025</v>
+        <v>990</v>
       </c>
       <c r="B480" t="s">
-        <v>1019</v>
+        <v>986</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>1024</v>
+        <v>992</v>
       </c>
       <c r="B481" t="s">
-        <v>1020</v>
-      </c>
-    </row>
-    <row r="483" spans="1:2">
-      <c r="A483" t="s">
-        <v>1039</v>
-      </c>
-      <c r="B483" t="s">
-        <v>1027</v>
+        <v>987</v>
+      </c>
+    </row>
+    <row r="482" spans="1:2">
+      <c r="A482" t="s">
+        <v>991</v>
+      </c>
+      <c r="B482" t="s">
+        <v>1165</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>1034</v>
+        <v>1005</v>
       </c>
       <c r="B484" t="s">
-        <v>1028</v>
+        <v>994</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1035</v>
+        <v>1000</v>
       </c>
       <c r="B485" t="s">
-        <v>1029</v>
+        <v>995</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1036</v>
+        <v>1001</v>
       </c>
       <c r="B486" t="s">
-        <v>1030</v>
+        <v>996</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>1037</v>
+        <v>1002</v>
       </c>
       <c r="B487" t="s">
-        <v>1031</v>
+        <v>997</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
-        <v>1038</v>
+        <v>1003</v>
       </c>
       <c r="B488" t="s">
-        <v>1032</v>
-      </c>
-    </row>
-    <row r="490" spans="1:2">
-      <c r="A490" t="s">
-        <v>1040</v>
-      </c>
-      <c r="B490" t="s">
-        <v>1041</v>
+        <v>998</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B489" t="s">
+        <v>1166</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1046</v>
+        <v>1006</v>
       </c>
       <c r="B491" t="s">
-        <v>1042</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1047</v>
+        <v>1012</v>
       </c>
       <c r="B492" t="s">
-        <v>1043</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1048</v>
+        <v>1013</v>
       </c>
       <c r="B493" t="s">
-        <v>1044</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1049</v>
+        <v>1014</v>
       </c>
       <c r="B494" t="s">
-        <v>1045</v>
-      </c>
-    </row>
-    <row r="496" spans="1:2">
-      <c r="A496" t="s">
-        <v>1073</v>
-      </c>
-      <c r="B496" t="s">
-        <v>1074</v>
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="495" spans="1:2">
+      <c r="A495" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B495" t="s">
+        <v>1011</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1089</v>
+        <v>1038</v>
       </c>
       <c r="B497" t="s">
-        <v>1075</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1090</v>
+        <v>1054</v>
       </c>
       <c r="B498" t="s">
-        <v>1076</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1091</v>
+        <v>1055</v>
       </c>
       <c r="B499" t="s">
-        <v>1077</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1100</v>
+        <v>1056</v>
       </c>
       <c r="B500" t="s">
-        <v>1078</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1092</v>
+        <v>1065</v>
       </c>
       <c r="B501" t="s">
-        <v>1079</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1093</v>
+        <v>1057</v>
       </c>
       <c r="B502" t="s">
-        <v>1080</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1094</v>
+        <v>1058</v>
       </c>
       <c r="B503" t="s">
-        <v>1081</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
-        <v>1095</v>
+        <v>1059</v>
       </c>
       <c r="B504" t="s">
-        <v>1082</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1096</v>
+        <v>1060</v>
       </c>
       <c r="B505" t="s">
-        <v>1083</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1097</v>
+        <v>1061</v>
       </c>
       <c r="B506" t="s">
-        <v>1084</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1098</v>
+        <v>1062</v>
       </c>
       <c r="B507" t="s">
-        <v>1085</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
-        <v>1099</v>
+        <v>1063</v>
       </c>
       <c r="B508" t="s">
-        <v>1086</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="509" spans="1:2">
       <c r="A509" t="s">
-        <v>1088</v>
+        <v>1064</v>
       </c>
       <c r="B509" t="s">
-        <v>1087</v>
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="510" spans="1:2">
+      <c r="A510" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1052</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A464:A465 A461:A462 A447:A456 A458:A459">
+  <conditionalFormatting sqref="A465:A466 A462:A463 A448:A457 A459:A460">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
for tickets 2803 and 2842
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C26B4F9-40A8-4E9C-8F14-7DE7F601D5CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B909E6E6-72D3-4A2E-98C5-749798DDCE95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1403" uniqueCount="1172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1406" uniqueCount="1174">
   <si>
     <t>Name</t>
   </si>
@@ -3556,6 +3556,12 @@
   </si>
   <si>
     <t>Applicant Name across the Employment Verification, Day Calculator, and Income Calculation Worksheet do not match.</t>
+  </si>
+  <si>
+    <t>EDC_HighestCalValue</t>
+  </si>
+  <si>
+    <t>Newly added by Harmandeep</t>
   </si>
 </sst>
 </file>
@@ -8432,7 +8438,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C510"/>
+  <dimension ref="A1:C511"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -9771,32 +9777,32 @@
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>590</v>
+        <v>1172</v>
       </c>
       <c r="B164" t="s">
-        <v>853</v>
+        <v>790</v>
       </c>
       <c r="C164" t="s">
-        <v>591</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>632</v>
+        <v>590</v>
       </c>
       <c r="B165" t="s">
-        <v>633</v>
+        <v>853</v>
       </c>
       <c r="C165" t="s">
-        <v>601</v>
+        <v>591</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>720</v>
+        <v>632</v>
       </c>
       <c r="B166" t="s">
-        <v>854</v>
+        <v>633</v>
       </c>
       <c r="C166" t="s">
         <v>601</v>
@@ -9804,10 +9810,10 @@
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B167" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="C167" t="s">
         <v>601</v>
@@ -9815,10 +9821,10 @@
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B168" t="s">
-        <v>705</v>
+        <v>855</v>
       </c>
       <c r="C168" t="s">
         <v>601</v>
@@ -9826,186 +9832,186 @@
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
+        <v>722</v>
+      </c>
+      <c r="B169" t="s">
+        <v>705</v>
+      </c>
+      <c r="C169" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3">
+      <c r="A170" t="s">
         <v>1098</v>
       </c>
-      <c r="B169" t="s">
+      <c r="B170" t="s">
         <v>860</v>
       </c>
-      <c r="C169" t="s">
+      <c r="C170" t="s">
         <v>1099</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3">
-      <c r="A171" t="s">
-        <v>465</v>
-      </c>
-      <c r="B171" t="s">
-        <v>1116</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>1122</v>
+        <v>465</v>
       </c>
       <c r="B172" t="s">
-        <v>1123</v>
-      </c>
-      <c r="C172" t="s">
-        <v>1124</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>236</v>
+        <v>1122</v>
       </c>
       <c r="B173" t="s">
-        <v>856</v>
+        <v>1123</v>
       </c>
       <c r="C173" t="s">
-        <v>530</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B174" t="s">
-        <v>857</v>
+        <v>856</v>
+      </c>
+      <c r="C174" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="B175" t="s">
-        <v>858</v>
-      </c>
-      <c r="C175" t="s">
-        <v>588</v>
+        <v>857</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>689</v>
+        <v>245</v>
       </c>
       <c r="B176" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="C176" t="s">
-        <v>601</v>
+        <v>588</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>239</v>
+        <v>689</v>
       </c>
       <c r="B177" t="s">
-        <v>238</v>
+        <v>859</v>
+      </c>
+      <c r="C177" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>455</v>
+        <v>239</v>
       </c>
       <c r="B178" t="s">
-        <v>464</v>
+        <v>238</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>240</v>
+        <v>455</v>
       </c>
       <c r="B179" t="s">
-        <v>860</v>
-      </c>
-      <c r="C179" t="s">
-        <v>1100</v>
+        <v>464</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B180" t="s">
-        <v>861</v>
+        <v>860</v>
+      </c>
+      <c r="C180" t="s">
+        <v>1100</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B181" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B182" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B183" t="s">
-        <v>790</v>
+        <v>863</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>276</v>
+        <v>244</v>
       </c>
       <c r="B184" t="s">
-        <v>860</v>
-      </c>
-      <c r="C184" t="s">
-        <v>1100</v>
+        <v>790</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>303</v>
+        <v>276</v>
       </c>
       <c r="B185" t="s">
-        <v>304</v>
+        <v>860</v>
+      </c>
+      <c r="C185" t="s">
+        <v>1100</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>593</v>
+        <v>303</v>
       </c>
       <c r="B186" t="s">
-        <v>1095</v>
+        <v>304</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>610</v>
+        <v>593</v>
       </c>
       <c r="B187" t="s">
-        <v>791</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>675</v>
+        <v>610</v>
       </c>
       <c r="B188" t="s">
-        <v>676</v>
-      </c>
-      <c r="C188" t="s">
-        <v>601</v>
+        <v>791</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>688</v>
+        <v>675</v>
       </c>
       <c r="B189" t="s">
-        <v>707</v>
+        <v>676</v>
       </c>
       <c r="C189" t="s">
         <v>601</v>
@@ -10013,809 +10019,809 @@
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>872</v>
+        <v>688</v>
       </c>
       <c r="B190" t="s">
-        <v>873</v>
+        <v>707</v>
+      </c>
+      <c r="C190" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
+        <v>872</v>
+      </c>
+      <c r="B191" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3">
+      <c r="A192" t="s">
         <v>473</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>1144</v>
-      </c>
-    </row>
-    <row r="193" spans="1:3">
-      <c r="A193" t="s">
-        <v>686</v>
-      </c>
-      <c r="B193" t="s">
-        <v>687</v>
-      </c>
-      <c r="C193" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>466</v>
+        <v>686</v>
       </c>
       <c r="B194" t="s">
-        <v>1117</v>
+        <v>687</v>
+      </c>
+      <c r="C194" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
+        <v>466</v>
+      </c>
+      <c r="B195" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3">
+      <c r="A196" t="s">
         <v>246</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B196" t="s">
         <v>864</v>
       </c>
-      <c r="C195" t="s">
+      <c r="C196" t="s">
         <v>595</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A196" t="s">
+    <row r="197" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A197" t="s">
         <v>248</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B197" t="s">
         <v>865</v>
       </c>
-      <c r="C196" t="s">
+      <c r="C197" t="s">
         <v>605</v>
-      </c>
-    </row>
-    <row r="197" spans="1:3">
-      <c r="A197" t="s">
-        <v>247</v>
-      </c>
-      <c r="B197" t="s">
-        <v>826</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B198" t="s">
-        <v>249</v>
+        <v>826</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B199" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B200" t="s">
-        <v>253</v>
-      </c>
-      <c r="C200" t="s">
-        <v>595</v>
+        <v>252</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>456</v>
+        <v>254</v>
       </c>
       <c r="B201" t="s">
-        <v>512</v>
+        <v>253</v>
+      </c>
+      <c r="C201" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>255</v>
+        <v>456</v>
       </c>
       <c r="B202" t="s">
-        <v>828</v>
+        <v>512</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B203" t="s">
-        <v>257</v>
+        <v>828</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B204" t="s">
-        <v>829</v>
+        <v>257</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B205" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B206" t="s">
-        <v>866</v>
-      </c>
-      <c r="C206" t="s">
-        <v>595</v>
+        <v>830</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B207" t="s">
-        <v>831</v>
+        <v>866</v>
+      </c>
+      <c r="C207" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B208" t="s">
-        <v>867</v>
-      </c>
-      <c r="C208" t="s">
-        <v>595</v>
+        <v>831</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B209" t="s">
-        <v>832</v>
+        <v>867</v>
+      </c>
+      <c r="C209" t="s">
+        <v>595</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B210" t="s">
-        <v>274</v>
+        <v>832</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B211" t="s">
-        <v>860</v>
-      </c>
-      <c r="C211" t="s">
-        <v>1100</v>
+        <v>274</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B212" t="s">
-        <v>278</v>
+        <v>860</v>
+      </c>
+      <c r="C212" t="s">
+        <v>1100</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>611</v>
+        <v>277</v>
       </c>
       <c r="B213" t="s">
-        <v>791</v>
+        <v>278</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>484</v>
+        <v>611</v>
       </c>
       <c r="B214" t="s">
-        <v>1145</v>
+        <v>791</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
+        <v>484</v>
+      </c>
+      <c r="B215" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3">
+      <c r="A216" t="s">
         <v>606</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B216" t="s">
         <v>607</v>
       </c>
-      <c r="C215" t="s">
+      <c r="C216" t="s">
         <v>601</v>
-      </c>
-    </row>
-    <row r="217" spans="1:3">
-      <c r="A217" t="s">
-        <v>467</v>
-      </c>
-      <c r="B217" t="s">
-        <v>1118</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
       <c r="B218" t="s">
-        <v>513</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>271</v>
+        <v>457</v>
       </c>
       <c r="B219" t="s">
-        <v>792</v>
+        <v>513</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B220" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="B221" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B222" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B223" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
+        <v>281</v>
+      </c>
+      <c r="B224" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2">
+      <c r="A225" t="s">
         <v>612</v>
       </c>
-      <c r="B224" t="s">
+      <c r="B225" t="s">
         <v>791</v>
       </c>
     </row>
-    <row r="225" spans="1:3">
-      <c r="A225" t="s">
+    <row r="226" spans="1:2">
+      <c r="A226" t="s">
         <v>483</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B226" t="s">
         <v>1146</v>
       </c>
     </row>
-    <row r="227" spans="1:3">
-      <c r="A227" t="s">
+    <row r="228" spans="1:2">
+      <c r="A228" t="s">
         <v>468</v>
       </c>
-      <c r="B227" t="s">
+      <c r="B228" t="s">
         <v>1119</v>
       </c>
     </row>
-    <row r="228" spans="1:3">
-      <c r="A228" t="s">
+    <row r="229" spans="1:2">
+      <c r="A229" t="s">
         <v>458</v>
       </c>
-      <c r="B228" t="s">
+      <c r="B229" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="229" spans="1:3">
-      <c r="A229" t="s">
+    <row r="230" spans="1:2">
+      <c r="A230" t="s">
         <v>284</v>
       </c>
-      <c r="B229" t="s">
+      <c r="B230" t="s">
         <v>785</v>
       </c>
     </row>
-    <row r="230" spans="1:3">
-      <c r="A230" t="s">
+    <row r="231" spans="1:2">
+      <c r="A231" t="s">
         <v>285</v>
       </c>
-      <c r="B230" t="s">
+      <c r="B231" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="231" spans="1:3">
-      <c r="A231" t="s">
+    <row r="232" spans="1:2">
+      <c r="A232" t="s">
         <v>286</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B232" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="232" spans="1:3">
-      <c r="A232" t="s">
+    <row r="233" spans="1:2">
+      <c r="A233" t="s">
         <v>288</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B233" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="233" spans="1:3">
-      <c r="A233" t="s">
+    <row r="234" spans="1:2">
+      <c r="A234" t="s">
         <v>289</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B234" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="234" spans="1:3">
-      <c r="A234" t="s">
+    <row r="235" spans="1:2">
+      <c r="A235" t="s">
         <v>290</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B235" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="235" spans="1:3">
-      <c r="A235" t="s">
+    <row r="236" spans="1:2">
+      <c r="A236" t="s">
         <v>291</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B236" t="s">
         <v>790</v>
       </c>
     </row>
-    <row r="236" spans="1:3">
-      <c r="A236" t="s">
+    <row r="237" spans="1:2">
+      <c r="A237" t="s">
         <v>613</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B237" t="s">
         <v>791</v>
       </c>
     </row>
-    <row r="237" spans="1:3">
-      <c r="A237" t="s">
+    <row r="238" spans="1:2">
+      <c r="A238" t="s">
         <v>482</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B238" t="s">
         <v>1147</v>
       </c>
     </row>
-    <row r="239" spans="1:3">
-      <c r="A239" t="s">
+    <row r="240" spans="1:2">
+      <c r="A240" t="s">
         <v>469</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B240" t="s">
         <v>1120</v>
-      </c>
-    </row>
-    <row r="240" spans="1:3">
-      <c r="A240" t="s">
-        <v>453</v>
-      </c>
-      <c r="B240" t="s">
-        <v>297</v>
-      </c>
-      <c r="C240" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>459</v>
+        <v>453</v>
       </c>
       <c r="B241" t="s">
-        <v>515</v>
+        <v>297</v>
+      </c>
+      <c r="C241" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>295</v>
+        <v>459</v>
       </c>
       <c r="B242" t="s">
-        <v>868</v>
-      </c>
-      <c r="C242" t="s">
-        <v>530</v>
+        <v>515</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B243" t="s">
-        <v>851</v>
+        <v>868</v>
+      </c>
+      <c r="C243" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>452</v>
+        <v>296</v>
       </c>
       <c r="B244" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>298</v>
+        <v>452</v>
       </c>
       <c r="B245" t="s">
-        <v>860</v>
-      </c>
-      <c r="C245" t="s">
-        <v>1097</v>
+        <v>852</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B246" t="s">
-        <v>869</v>
+        <v>860</v>
+      </c>
+      <c r="C246" t="s">
+        <v>1097</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B247" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B248" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B249" t="s">
-        <v>790</v>
+        <v>871</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>614</v>
+        <v>302</v>
       </c>
       <c r="B250" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
+        <v>614</v>
+      </c>
+      <c r="B251" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3">
+      <c r="A252" t="s">
         <v>481</v>
       </c>
-      <c r="B251" t="s">
+      <c r="B252" t="s">
         <v>1148</v>
-      </c>
-    </row>
-    <row r="253" spans="1:3">
-      <c r="A253" t="s">
-        <v>647</v>
-      </c>
-      <c r="B253" t="s">
-        <v>648</v>
-      </c>
-      <c r="C253" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>498</v>
+        <v>647</v>
       </c>
       <c r="B254" t="s">
-        <v>501</v>
+        <v>648</v>
       </c>
       <c r="C254" t="s">
-        <v>528</v>
+        <v>601</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B255" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C255" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>527</v>
+        <v>499</v>
       </c>
       <c r="B256" t="s">
-        <v>541</v>
+        <v>500</v>
+      </c>
+      <c r="C256" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>319</v>
+        <v>527</v>
       </c>
       <c r="B257" t="s">
-        <v>305</v>
+        <v>541</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B258" t="s">
-        <v>306</v>
-      </c>
-      <c r="C258" t="s">
-        <v>530</v>
+        <v>305</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>460</v>
+        <v>320</v>
       </c>
       <c r="B259" t="s">
-        <v>516</v>
+        <v>306</v>
+      </c>
+      <c r="C259" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>321</v>
+        <v>460</v>
       </c>
       <c r="B260" t="s">
-        <v>307</v>
+        <v>516</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B261" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B262" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B263" t="s">
-        <v>310</v>
-      </c>
-      <c r="C263" t="s">
-        <v>530</v>
+        <v>309</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B264" t="s">
-        <v>311</v>
+        <v>310</v>
+      </c>
+      <c r="C264" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B265" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B266" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B267" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B268" t="s">
-        <v>315</v>
-      </c>
-      <c r="C268" t="s">
-        <v>530</v>
+        <v>314</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B269" t="s">
-        <v>316</v>
+        <v>315</v>
+      </c>
+      <c r="C269" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B270" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B271" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
+        <v>332</v>
+      </c>
+      <c r="B272" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3">
+      <c r="A273" t="s">
         <v>480</v>
       </c>
-      <c r="B272" t="s">
+      <c r="B273" t="s">
         <v>1149</v>
-      </c>
-    </row>
-    <row r="274" spans="1:3">
-      <c r="A274" t="s">
-        <v>545</v>
-      </c>
-      <c r="B274" t="s">
-        <v>546</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>339</v>
+        <v>545</v>
       </c>
       <c r="B275" t="s">
-        <v>357</v>
+        <v>546</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B276" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B277" t="s">
-        <v>355</v>
-      </c>
-      <c r="C277" t="s">
-        <v>530</v>
+        <v>354</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>461</v>
+        <v>341</v>
       </c>
       <c r="B278" t="s">
-        <v>517</v>
+        <v>355</v>
+      </c>
+      <c r="C278" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>358</v>
+        <v>461</v>
       </c>
       <c r="B279" t="s">
-        <v>356</v>
-      </c>
-      <c r="C279" t="s">
-        <v>530</v>
+        <v>517</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="B280" t="s">
-        <v>348</v>
+        <v>356</v>
+      </c>
+      <c r="C280" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>359</v>
+        <v>342</v>
       </c>
       <c r="B281" t="s">
-        <v>349</v>
-      </c>
-      <c r="C281" t="s">
-        <v>507</v>
+        <v>348</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="B282" t="s">
-        <v>350</v>
+        <v>349</v>
+      </c>
+      <c r="C282" t="s">
+        <v>507</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B283" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B284" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B285" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B286" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>1024</v>
+        <v>347</v>
       </c>
       <c r="B287" t="s">
-        <v>1025</v>
-      </c>
-      <c r="C287" t="s">
-        <v>1020</v>
+        <v>350</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="B288" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="C288" t="s">
         <v>1020</v>
@@ -10823,10 +10829,10 @@
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="B289" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="C289" t="s">
         <v>1020</v>
@@ -10834,40 +10840,40 @@
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B290" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C290" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3">
+      <c r="A291" t="s">
         <v>479</v>
       </c>
-      <c r="B290" t="s">
+      <c r="B291" t="s">
         <v>1150</v>
-      </c>
-    </row>
-    <row r="292" spans="1:3">
-      <c r="A292" t="s">
-        <v>649</v>
-      </c>
-      <c r="B292" t="s">
-        <v>667</v>
-      </c>
-      <c r="C292" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>1018</v>
+        <v>649</v>
       </c>
       <c r="B293" t="s">
-        <v>1019</v>
+        <v>667</v>
       </c>
       <c r="C293" t="s">
-        <v>1020</v>
+        <v>601</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>1021</v>
+        <v>1018</v>
       </c>
       <c r="B294" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="C294" t="s">
         <v>1020</v>
@@ -10875,78 +10881,78 @@
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="B295" t="s">
-        <v>1151</v>
+        <v>1022</v>
       </c>
       <c r="C295" t="s">
         <v>1020</v>
       </c>
     </row>
-    <row r="297" spans="1:3">
-      <c r="A297" t="s">
-        <v>645</v>
-      </c>
-      <c r="B297" t="s">
-        <v>646</v>
-      </c>
-      <c r="C297" t="s">
-        <v>601</v>
+    <row r="296" spans="1:3">
+      <c r="A296" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B296" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1020</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>470</v>
+        <v>645</v>
       </c>
       <c r="B298" t="s">
-        <v>471</v>
+        <v>646</v>
+      </c>
+      <c r="C298" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>365</v>
+        <v>470</v>
       </c>
       <c r="B299" t="s">
-        <v>376</v>
+        <v>471</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B300" t="s">
-        <v>377</v>
-      </c>
-      <c r="C300" t="s">
-        <v>530</v>
+        <v>376</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>518</v>
+        <v>366</v>
       </c>
       <c r="B301" t="s">
-        <v>519</v>
+        <v>377</v>
+      </c>
+      <c r="C301" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>367</v>
+        <v>518</v>
       </c>
       <c r="B302" t="s">
-        <v>378</v>
-      </c>
-      <c r="C302" t="s">
-        <v>530</v>
+        <v>519</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B303" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C303" t="s">
         <v>530</v>
@@ -10954,147 +10960,147 @@
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B304" t="s">
-        <v>531</v>
+        <v>379</v>
+      </c>
+      <c r="C304" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B305" t="s">
-        <v>380</v>
+        <v>531</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B306" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B307" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B308" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B309" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B310" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>703</v>
+        <v>375</v>
       </c>
       <c r="B311" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C311" t="s">
-        <v>601</v>
+        <v>385</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>1111</v>
+        <v>703</v>
       </c>
       <c r="B312" t="s">
-        <v>1112</v>
+        <v>1094</v>
+      </c>
+      <c r="C312" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>477</v>
+        <v>1111</v>
       </c>
       <c r="B313" t="s">
-        <v>1152</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
+        <v>477</v>
+      </c>
+      <c r="B314" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3">
+      <c r="A315" t="s">
         <v>554</v>
       </c>
-      <c r="B314" t="s">
+      <c r="B315" t="s">
         <v>555</v>
-      </c>
-    </row>
-    <row r="316" spans="1:3">
-      <c r="A316" t="s">
-        <v>472</v>
-      </c>
-      <c r="B316" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>392</v>
+        <v>472</v>
       </c>
       <c r="B317" t="s">
-        <v>403</v>
+        <v>471</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B318" t="s">
-        <v>404</v>
-      </c>
-      <c r="C318" t="s">
-        <v>530</v>
+        <v>403</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>462</v>
+        <v>393</v>
       </c>
       <c r="B319" t="s">
-        <v>520</v>
+        <v>404</v>
+      </c>
+      <c r="C319" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>394</v>
+        <v>462</v>
       </c>
       <c r="B320" t="s">
-        <v>405</v>
-      </c>
-      <c r="C320" t="s">
-        <v>530</v>
+        <v>520</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B321" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C321" t="s">
         <v>530</v>
@@ -11102,1389 +11108,1400 @@
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B322" t="s">
-        <v>532</v>
+        <v>406</v>
+      </c>
+      <c r="C322" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B323" t="s">
-        <v>380</v>
+        <v>532</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B324" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B325" t="s">
-        <v>407</v>
+        <v>381</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B326" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B327" t="s">
-        <v>384</v>
+        <v>408</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B328" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>476</v>
+        <v>402</v>
       </c>
       <c r="B329" t="s">
-        <v>1152</v>
+        <v>385</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
+        <v>476</v>
+      </c>
+      <c r="B330" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3">
+      <c r="A331" t="s">
         <v>561</v>
       </c>
-      <c r="B330" t="s">
+      <c r="B331" t="s">
         <v>555</v>
-      </c>
-    </row>
-    <row r="332" spans="1:3">
-      <c r="A332" t="s">
-        <v>643</v>
-      </c>
-      <c r="B332" t="s">
-        <v>644</v>
-      </c>
-      <c r="C332" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>386</v>
+        <v>643</v>
       </c>
       <c r="B333" t="s">
-        <v>562</v>
+        <v>644</v>
+      </c>
+      <c r="C333" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B334" t="s">
-        <v>563</v>
-      </c>
-      <c r="C334" t="s">
-        <v>530</v>
+        <v>562</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>463</v>
+        <v>387</v>
       </c>
       <c r="B335" t="s">
-        <v>564</v>
+        <v>563</v>
+      </c>
+      <c r="C335" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>388</v>
+        <v>463</v>
       </c>
       <c r="B336" t="s">
-        <v>589</v>
+        <v>564</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B337" t="s">
-        <v>565</v>
+        <v>589</v>
       </c>
     </row>
     <row r="338" spans="1:3">
       <c r="A338" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B338" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="339" spans="1:3">
       <c r="A339" t="s">
-        <v>1129</v>
+        <v>390</v>
       </c>
       <c r="B339" t="s">
-        <v>1130</v>
-      </c>
-      <c r="C339" t="s">
-        <v>1131</v>
+        <v>566</v>
       </c>
     </row>
     <row r="340" spans="1:3">
       <c r="A340" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B340" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C340" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="341" spans="1:3">
+      <c r="A341" t="s">
         <v>475</v>
       </c>
-      <c r="B340" t="s">
+      <c r="B341" t="s">
         <v>1153</v>
-      </c>
-    </row>
-    <row r="342" spans="1:3">
-      <c r="A342" t="s">
-        <v>717</v>
-      </c>
-      <c r="B342" t="s">
-        <v>718</v>
-      </c>
-      <c r="C342" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="B343" t="s">
-        <v>1154</v>
+        <v>718</v>
       </c>
       <c r="C343" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="345" spans="1:3">
-      <c r="A345" t="s">
-        <v>724</v>
-      </c>
-      <c r="B345" t="s">
-        <v>725</v>
+    <row r="344" spans="1:3">
+      <c r="A344" t="s">
+        <v>719</v>
+      </c>
+      <c r="B344" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C344" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B346" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="B347" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="B348" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
     </row>
     <row r="349" spans="1:3">
       <c r="A349" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="B349" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
     </row>
     <row r="350" spans="1:3">
       <c r="A350" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="B350" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="B351" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
     </row>
     <row r="352" spans="1:3">
       <c r="A352" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="B352" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B353" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="B354" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="B355" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B356" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B357" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="B358" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="B359" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="B360" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>1104</v>
+        <v>754</v>
       </c>
       <c r="B361" t="s">
-        <v>1105</v>
+        <v>755</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>756</v>
+        <v>1104</v>
       </c>
       <c r="B362" t="s">
-        <v>757</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
+        <v>756</v>
+      </c>
+      <c r="B363" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" t="s">
         <v>1128</v>
       </c>
-      <c r="B363" t="s">
+      <c r="B364" t="s">
         <v>1155</v>
-      </c>
-    </row>
-    <row r="365" spans="1:2">
-      <c r="A365" t="s">
-        <v>758</v>
-      </c>
-      <c r="B365" t="s">
-        <v>759</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B366" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="B367" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="B368" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B369" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B370" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B371" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B372" t="s">
-        <v>318</v>
+        <v>771</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B373" t="s">
-        <v>774</v>
+        <v>318</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B374" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B375" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
+        <v>777</v>
+      </c>
+      <c r="B376" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="377" spans="1:2">
+      <c r="A377" t="s">
         <v>779</v>
       </c>
-      <c r="B376" t="s">
+      <c r="B377" t="s">
         <v>1156</v>
-      </c>
-    </row>
-    <row r="378" spans="1:2">
-      <c r="A378" t="s">
-        <v>780</v>
-      </c>
-      <c r="B378" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B379" t="s">
-        <v>782</v>
+        <v>311</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B380" t="s">
-        <v>313</v>
+        <v>782</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
+        <v>783</v>
+      </c>
+      <c r="B381" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" t="s">
         <v>784</v>
       </c>
-      <c r="B381" t="s">
+      <c r="B382" t="s">
         <v>314</v>
-      </c>
-    </row>
-    <row r="383" spans="1:2">
-      <c r="A383" t="s">
-        <v>806</v>
-      </c>
-      <c r="B383" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="B384" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="B385" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="B386" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B387" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
+        <v>798</v>
+      </c>
+      <c r="B388" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" t="s">
         <v>803</v>
       </c>
-      <c r="B388" t="s">
+      <c r="B389" t="s">
         <v>1157</v>
-      </c>
-    </row>
-    <row r="390" spans="1:2">
-      <c r="A390" t="s">
-        <v>810</v>
-      </c>
-      <c r="B390" t="s">
-        <v>815</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>817</v>
+        <v>810</v>
       </c>
       <c r="B391" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="B392" t="s">
-        <v>800</v>
+        <v>816</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B393" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B394" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
+        <v>813</v>
+      </c>
+      <c r="B395" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="396" spans="1:2">
+      <c r="A396" t="s">
         <v>814</v>
       </c>
-      <c r="B395" t="s">
+      <c r="B396" t="s">
         <v>1158</v>
-      </c>
-    </row>
-    <row r="397" spans="1:2">
-      <c r="A397" t="s">
-        <v>822</v>
-      </c>
-      <c r="B397" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="B398" t="s">
-        <v>1121</v>
+        <v>823</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B399" t="s">
-        <v>1087</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="B400" t="s">
-        <v>1080</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>833</v>
+        <v>827</v>
       </c>
       <c r="B401" t="s">
-        <v>1066</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B402" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B403" t="s">
-        <v>1086</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="B404" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B405" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B406" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B407" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B408" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B409" t="s">
-        <v>832</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B410" t="s">
-        <v>1088</v>
+        <v>832</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B411" t="s">
-        <v>278</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B412" t="s">
-        <v>791</v>
+        <v>278</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>837</v>
+        <v>846</v>
       </c>
       <c r="B413" t="s">
-        <v>607</v>
+        <v>791</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="B414" t="s">
-        <v>1159</v>
+        <v>607</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>1070</v>
+        <v>836</v>
       </c>
       <c r="B415" t="s">
-        <v>1068</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B416" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="B417" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="B418" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="B419" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B420" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>1090</v>
+        <v>1079</v>
       </c>
       <c r="B421" t="s">
-        <v>1089</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B422" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2">
+      <c r="A424" t="s">
         <v>1170</v>
       </c>
-      <c r="B423" t="s">
+      <c r="B424" t="s">
         <v>1171</v>
-      </c>
-    </row>
-    <row r="425" spans="1:2">
-      <c r="A425" t="s">
-        <v>906</v>
-      </c>
-      <c r="B425" t="s">
-        <v>886</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>925</v>
+        <v>906</v>
       </c>
       <c r="B426" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B427" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="B428" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B429" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="B430" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="B431" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="B432" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B433" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="B434" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B435" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>926</v>
+        <v>916</v>
       </c>
       <c r="B436" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>915</v>
+        <v>926</v>
       </c>
       <c r="B437" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B438" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="B439" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B440" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="B441" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B442" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B443" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B444" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
+        <v>908</v>
+      </c>
+      <c r="B445" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2">
+      <c r="A446" t="s">
         <v>907</v>
       </c>
-      <c r="B445" t="s">
+      <c r="B446" t="s">
         <v>1160</v>
-      </c>
-    </row>
-    <row r="447" spans="1:2">
-      <c r="A447" t="s">
-        <v>1132</v>
-      </c>
-      <c r="B447" t="s">
-        <v>1133</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>947</v>
+        <v>1132</v>
       </c>
       <c r="B448" t="s">
-        <v>929</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>938</v>
+        <v>947</v>
       </c>
       <c r="B449" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="B450" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B451" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
       <c r="B452" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="B453" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="B454" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="B455" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
       <c r="B456" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
+        <v>946</v>
+      </c>
+      <c r="B457" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
         <v>945</v>
       </c>
-      <c r="B457" t="s">
+      <c r="B458" t="s">
         <v>1161</v>
-      </c>
-    </row>
-    <row r="459" spans="1:2">
-      <c r="A459" t="s">
-        <v>952</v>
-      </c>
-      <c r="B459" t="s">
-        <v>954</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
+        <v>952</v>
+      </c>
+      <c r="B460" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" t="s">
         <v>962</v>
       </c>
-      <c r="B460" t="s">
+      <c r="B461" t="s">
         <v>1162</v>
-      </c>
-    </row>
-    <row r="462" spans="1:2">
-      <c r="A462" t="s">
-        <v>953</v>
-      </c>
-      <c r="B462" t="s">
-        <v>955</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
+        <v>953</v>
+      </c>
+      <c r="B463" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2">
+      <c r="A464" t="s">
         <v>963</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B464" t="s">
         <v>1163</v>
-      </c>
-    </row>
-    <row r="465" spans="1:2">
-      <c r="A465" t="s">
-        <v>960</v>
-      </c>
-      <c r="B465" t="s">
-        <v>958</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B466" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
+        <v>961</v>
+      </c>
+      <c r="B467" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" t="s">
         <v>957</v>
       </c>
-      <c r="B467" t="s">
+      <c r="B468" t="s">
         <v>1164</v>
-      </c>
-    </row>
-    <row r="469" spans="1:2">
-      <c r="A469" t="s">
-        <v>972</v>
-      </c>
-      <c r="B469" t="s">
-        <v>965</v>
       </c>
     </row>
     <row r="470" spans="1:2">
       <c r="A470" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B470" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B471" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
-        <v>1017</v>
+        <v>974</v>
       </c>
       <c r="B472" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>975</v>
+        <v>1017</v>
       </c>
       <c r="B473" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="474" spans="1:2">
       <c r="A474" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B474" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
+        <v>976</v>
+      </c>
+      <c r="B475" t="s">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" t="s">
         <v>977</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B476" t="s">
         <v>971</v>
-      </c>
-    </row>
-    <row r="477" spans="1:2">
-      <c r="A477" t="s">
-        <v>988</v>
-      </c>
-      <c r="B477" t="s">
-        <v>983</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>993</v>
+        <v>988</v>
       </c>
       <c r="B478" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="B479" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B480" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B481" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
     </row>
     <row r="482" spans="1:2">
       <c r="A482" t="s">
+        <v>992</v>
+      </c>
+      <c r="B482" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2">
+      <c r="A483" t="s">
         <v>991</v>
       </c>
-      <c r="B482" t="s">
+      <c r="B483" t="s">
         <v>1165</v>
-      </c>
-    </row>
-    <row r="484" spans="1:2">
-      <c r="A484" t="s">
-        <v>1005</v>
-      </c>
-      <c r="B484" t="s">
-        <v>994</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="B485" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B486" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B487" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B488" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
     </row>
     <row r="489" spans="1:2">
       <c r="A489" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B489" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2">
+      <c r="A490" t="s">
         <v>1004</v>
       </c>
-      <c r="B489" t="s">
+      <c r="B490" t="s">
         <v>1166</v>
-      </c>
-    </row>
-    <row r="491" spans="1:2">
-      <c r="A491" t="s">
-        <v>1006</v>
-      </c>
-      <c r="B491" t="s">
-        <v>1007</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1012</v>
+        <v>1006</v>
       </c>
       <c r="B492" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B493" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B494" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B495" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="496" spans="1:2">
+      <c r="A496" t="s">
         <v>1015</v>
       </c>
-      <c r="B495" t="s">
+      <c r="B496" t="s">
         <v>1011</v>
-      </c>
-    </row>
-    <row r="497" spans="1:2">
-      <c r="A497" t="s">
-        <v>1038</v>
-      </c>
-      <c r="B497" t="s">
-        <v>1039</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1054</v>
+        <v>1038</v>
       </c>
       <c r="B498" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B499" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B500" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1065</v>
+        <v>1056</v>
       </c>
       <c r="B501" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
-        <v>1057</v>
+        <v>1065</v>
       </c>
       <c r="B502" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B503" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B504" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B505" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B506" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B507" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B508" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="509" spans="1:2">
       <c r="A509" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="B509" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="510" spans="1:2">
       <c r="A510" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="511" spans="1:2">
+      <c r="A511" t="s">
         <v>1053</v>
       </c>
-      <c r="B510" t="s">
+      <c r="B511" t="s">
         <v>1052</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A465:A466 A462:A463 A448:A457 A459:A460">
+  <conditionalFormatting sqref="A466:A467 A463:A464 A449:A458 A460:A461">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chanbges in IAQ for matching the income typer from ICW
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE7616A7-0ACD-4C1E-96D6-94F7D29C5A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA2FFE25-BBA1-4E66-9E5F-DBF1F6FA0628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21510" windowHeight="9900" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22560" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3387,9 +3387,6 @@
     <t>Anticipated income in the next 12 months has been documented as yes for at least one question in Part A of the Certification of Zero Income. Manual review required.</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Day Calculator does not exist for Paystub</t>
   </si>
   <si>
@@ -3580,6 +3577,9 @@
   </si>
   <si>
     <t>IAQ_NoSupportingDocument</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4015,7 +4015,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -4036,7 +4036,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -4048,7 +4048,7 @@
         <v>203</v>
       </c>
       <c r="B7" t="s">
-        <v>1115</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7254,10 +7254,10 @@
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B22" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
@@ -8559,7 +8559,7 @@
         <v>666</v>
       </c>
       <c r="B13" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="C13" t="s">
         <v>601</v>
@@ -8692,7 +8692,7 @@
         <v>478</v>
       </c>
       <c r="B28" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -8826,7 +8826,7 @@
         <v>493</v>
       </c>
       <c r="B45" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="47" spans="1:3">
@@ -8944,7 +8944,7 @@
         <v>492</v>
       </c>
       <c r="B60" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -9077,7 +9077,7 @@
         <v>491</v>
       </c>
       <c r="B75" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -9093,18 +9093,18 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B77" t="s">
         <v>1176</v>
-      </c>
-      <c r="B77" t="s">
-        <v>1177</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B78" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="80" spans="1:3">
@@ -9188,7 +9188,7 @@
         <v>490</v>
       </c>
       <c r="B88" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -9367,7 +9367,7 @@
         <v>489</v>
       </c>
       <c r="B108" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -9482,7 +9482,7 @@
         <v>488</v>
       </c>
       <c r="B123" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -9579,7 +9579,7 @@
         <v>487</v>
       </c>
       <c r="B135" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -9598,7 +9598,7 @@
         <v>620</v>
       </c>
       <c r="B138" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="C138" t="s">
         <v>619</v>
@@ -9671,7 +9671,7 @@
         <v>486</v>
       </c>
       <c r="B147" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="149" spans="1:3">
@@ -9711,7 +9711,7 @@
         <v>485</v>
       </c>
       <c r="B153" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="154" spans="1:3">
@@ -9806,18 +9806,18 @@
         <v>474</v>
       </c>
       <c r="B164" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B166" t="s">
         <v>790</v>
       </c>
       <c r="C166" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -9891,18 +9891,18 @@
         <v>465</v>
       </c>
       <c r="B174" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B175" t="s">
         <v>1122</v>
       </c>
-      <c r="B175" t="s">
+      <c r="C175" t="s">
         <v>1123</v>
-      </c>
-      <c r="C175" t="s">
-        <v>1124</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -10075,7 +10075,7 @@
         <v>473</v>
       </c>
       <c r="B194" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -10094,7 +10094,7 @@
         <v>466</v>
       </c>
       <c r="B197" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -10272,7 +10272,7 @@
         <v>484</v>
       </c>
       <c r="B217" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="218" spans="1:3">
@@ -10291,7 +10291,7 @@
         <v>467</v>
       </c>
       <c r="B220" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="221" spans="1:3">
@@ -10355,7 +10355,7 @@
         <v>483</v>
       </c>
       <c r="B228" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="230" spans="1:2">
@@ -10363,7 +10363,7 @@
         <v>468</v>
       </c>
       <c r="B230" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="231" spans="1:2">
@@ -10443,7 +10443,7 @@
         <v>482</v>
       </c>
       <c r="B240" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="242" spans="1:3">
@@ -10451,7 +10451,7 @@
         <v>469</v>
       </c>
       <c r="B242" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -10556,7 +10556,7 @@
         <v>481</v>
       </c>
       <c r="B254" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="256" spans="1:3">
@@ -10734,7 +10734,7 @@
         <v>480</v>
       </c>
       <c r="B275" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="277" spans="1:3">
@@ -10888,7 +10888,7 @@
         <v>479</v>
       </c>
       <c r="B293" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="295" spans="1:3">
@@ -10929,7 +10929,7 @@
         <v>1023</v>
       </c>
       <c r="B298" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="C298" t="s">
         <v>1020</v>
@@ -11083,7 +11083,7 @@
         <v>477</v>
       </c>
       <c r="B316" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="317" spans="1:3">
@@ -11212,7 +11212,7 @@
         <v>476</v>
       </c>
       <c r="B332" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="333" spans="1:3">
@@ -11287,13 +11287,13 @@
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B342" t="s">
         <v>1129</v>
       </c>
-      <c r="B342" t="s">
+      <c r="C342" t="s">
         <v>1130</v>
-      </c>
-      <c r="C342" t="s">
-        <v>1131</v>
       </c>
     </row>
     <row r="343" spans="1:3">
@@ -11301,7 +11301,7 @@
         <v>475</v>
       </c>
       <c r="B343" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="345" spans="1:3">
@@ -11320,7 +11320,7 @@
         <v>719</v>
       </c>
       <c r="B346" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C346" t="s">
         <v>601</v>
@@ -11472,10 +11472,10 @@
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B366" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="368" spans="1:2">
@@ -11571,7 +11571,7 @@
         <v>779</v>
       </c>
       <c r="B379" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="381" spans="1:2">
@@ -11651,7 +11651,7 @@
         <v>803</v>
       </c>
       <c r="B391" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="393" spans="1:2">
@@ -11699,7 +11699,7 @@
         <v>814</v>
       </c>
       <c r="B398" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="400" spans="1:2">
@@ -11715,7 +11715,7 @@
         <v>824</v>
       </c>
       <c r="B401" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="402" spans="1:2">
@@ -11843,7 +11843,7 @@
         <v>836</v>
       </c>
       <c r="B417" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="418" spans="1:2">
@@ -11912,10 +11912,10 @@
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B426" t="s">
         <v>1170</v>
-      </c>
-      <c r="B426" t="s">
-        <v>1171</v>
       </c>
     </row>
     <row r="428" spans="1:2">
@@ -12083,23 +12083,23 @@
         <v>907</v>
       </c>
       <c r="B448" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B449" t="s">
         <v>1174</v>
-      </c>
-      <c r="B449" t="s">
-        <v>1175</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B451" t="s">
         <v>1132</v>
-      </c>
-      <c r="B451" t="s">
-        <v>1133</v>
       </c>
     </row>
     <row r="452" spans="1:2">
@@ -12179,7 +12179,7 @@
         <v>945</v>
       </c>
       <c r="B461" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="463" spans="1:2">
@@ -12195,7 +12195,7 @@
         <v>962</v>
       </c>
       <c r="B464" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="466" spans="1:2">
@@ -12211,7 +12211,7 @@
         <v>963</v>
       </c>
       <c r="B467" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="469" spans="1:2">
@@ -12235,7 +12235,7 @@
         <v>957</v>
       </c>
       <c r="B471" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="473" spans="1:2">
@@ -12339,7 +12339,7 @@
         <v>991</v>
       </c>
       <c r="B486" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="488" spans="1:2">
@@ -12387,7 +12387,7 @@
         <v>1004</v>
       </c>
       <c r="B493" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="495" spans="1:2">

</xml_diff>

<commit_message>
Continued working on 2820
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA2FFE25-BBA1-4E66-9E5F-DBF1F6FA0628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4161F9-A722-448D-A6E5-663D84D2B586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="22560" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1412" uniqueCount="1180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1416" uniqueCount="1184">
   <si>
     <t>Name</t>
   </si>
@@ -3579,7 +3579,19 @@
     <t>IAQ_NoSupportingDocument</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>CSEI_NameNotMatchingIAQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-employment income has been indicated, but not all Self Employment documentation has been provided. </t>
+  </si>
+  <si>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>RCV_NameNotMatchingIAQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recurring Monetary Contributions have been indicated, but not all Regular Monetary Contributions documentation has been provided. </t>
   </si>
 </sst>
 </file>
@@ -4048,7 +4060,7 @@
         <v>203</v>
       </c>
       <c r="B7" t="s">
-        <v>1179</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -8456,7 +8468,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C514"/>
+  <dimension ref="A1:C516"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -11478,1072 +11490,1088 @@
         <v>1154</v>
       </c>
     </row>
-    <row r="368" spans="1:2">
-      <c r="A368" t="s">
-        <v>758</v>
-      </c>
-      <c r="B368" t="s">
-        <v>759</v>
+    <row r="367" spans="1:2">
+      <c r="A367" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B367" t="s">
+        <v>1180</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B369" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="B370" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="B371" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B372" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="B373" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B374" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B375" t="s">
-        <v>318</v>
+        <v>771</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B376" t="s">
-        <v>774</v>
+        <v>318</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B377" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B378" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
+        <v>777</v>
+      </c>
+      <c r="B379" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2">
+      <c r="A380" t="s">
         <v>779</v>
       </c>
-      <c r="B379" t="s">
+      <c r="B380" t="s">
         <v>1155</v>
-      </c>
-    </row>
-    <row r="381" spans="1:2">
-      <c r="A381" t="s">
-        <v>780</v>
-      </c>
-      <c r="B381" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B382" t="s">
-        <v>782</v>
+        <v>311</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="B383" t="s">
-        <v>313</v>
+        <v>782</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
+        <v>783</v>
+      </c>
+      <c r="B384" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" t="s">
         <v>784</v>
       </c>
-      <c r="B384" t="s">
+      <c r="B385" t="s">
         <v>314</v>
-      </c>
-    </row>
-    <row r="386" spans="1:2">
-      <c r="A386" t="s">
-        <v>806</v>
-      </c>
-      <c r="B386" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="B387" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
       <c r="B388" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="B389" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="B390" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
+        <v>798</v>
+      </c>
+      <c r="B391" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" t="s">
         <v>803</v>
       </c>
-      <c r="B391" t="s">
+      <c r="B392" t="s">
         <v>1156</v>
-      </c>
-    </row>
-    <row r="393" spans="1:2">
-      <c r="A393" t="s">
-        <v>810</v>
-      </c>
-      <c r="B393" t="s">
-        <v>815</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>817</v>
+        <v>810</v>
       </c>
       <c r="B394" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="B395" t="s">
-        <v>800</v>
+        <v>816</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="B396" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="B397" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
+        <v>813</v>
+      </c>
+      <c r="B398" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="399" spans="1:2">
+      <c r="A399" t="s">
         <v>814</v>
       </c>
-      <c r="B398" t="s">
+      <c r="B399" t="s">
         <v>1157</v>
-      </c>
-    </row>
-    <row r="400" spans="1:2">
-      <c r="A400" t="s">
-        <v>822</v>
-      </c>
-      <c r="B400" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="B401" t="s">
-        <v>1120</v>
+        <v>823</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B402" t="s">
-        <v>1087</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="B403" t="s">
-        <v>1080</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
-        <v>833</v>
+        <v>827</v>
       </c>
       <c r="B404" t="s">
-        <v>1066</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B405" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B406" t="s">
-        <v>1086</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="B407" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B408" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B409" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B410" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B411" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="B412" t="s">
-        <v>832</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="B413" t="s">
-        <v>1088</v>
+        <v>832</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="B414" t="s">
-        <v>278</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="B415" t="s">
-        <v>791</v>
+        <v>278</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>837</v>
+        <v>846</v>
       </c>
       <c r="B416" t="s">
-        <v>607</v>
+        <v>791</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="B417" t="s">
-        <v>1158</v>
+        <v>607</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>1070</v>
+        <v>836</v>
       </c>
       <c r="B418" t="s">
-        <v>1068</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B419" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="B420" t="s">
-        <v>1072</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
       <c r="B421" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="B422" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B423" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>1090</v>
+        <v>1079</v>
       </c>
       <c r="B424" t="s">
-        <v>1089</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="B425" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B426" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2">
+      <c r="A427" t="s">
         <v>1169</v>
       </c>
-      <c r="B426" t="s">
+      <c r="B427" t="s">
         <v>1170</v>
-      </c>
-    </row>
-    <row r="428" spans="1:2">
-      <c r="A428" t="s">
-        <v>906</v>
-      </c>
-      <c r="B428" t="s">
-        <v>886</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>925</v>
+        <v>906</v>
       </c>
       <c r="B429" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B430" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="B431" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="B432" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="B433" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="B434" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="435" spans="1:2">
       <c r="A435" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="B435" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B436" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="B437" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B438" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>926</v>
+        <v>916</v>
       </c>
       <c r="B439" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>915</v>
+        <v>926</v>
       </c>
       <c r="B440" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B441" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="B442" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B443" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="B444" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B445" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="B446" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B447" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="B448" t="s">
-        <v>1159</v>
+        <v>905</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
+        <v>907</v>
+      </c>
+      <c r="B449" t="s">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2">
+      <c r="A450" t="s">
         <v>1173</v>
       </c>
-      <c r="B449" t="s">
+      <c r="B450" t="s">
         <v>1174</v>
-      </c>
-    </row>
-    <row r="451" spans="1:2">
-      <c r="A451" t="s">
-        <v>1131</v>
-      </c>
-      <c r="B451" t="s">
-        <v>1132</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>947</v>
+        <v>1131</v>
       </c>
       <c r="B452" t="s">
-        <v>929</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>938</v>
+        <v>947</v>
       </c>
       <c r="B453" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="B454" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B455" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
       <c r="B456" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
     </row>
     <row r="457" spans="1:2">
       <c r="A457" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="B457" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="458" spans="1:2">
       <c r="A458" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="B458" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="B459" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
       <c r="B460" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
+        <v>946</v>
+      </c>
+      <c r="B461" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" t="s">
         <v>945</v>
       </c>
-      <c r="B461" t="s">
+      <c r="B462" t="s">
         <v>1160</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
+        <v>1182</v>
+      </c>
+      <c r="B463" t="s">
+        <v>1183</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" t="s">
         <v>952</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B465" t="s">
         <v>954</v>
-      </c>
-    </row>
-    <row r="464" spans="1:2">
-      <c r="A464" t="s">
-        <v>962</v>
-      </c>
-      <c r="B464" t="s">
-        <v>1161</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
+        <v>962</v>
+      </c>
+      <c r="B466" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" t="s">
         <v>953</v>
       </c>
-      <c r="B466" t="s">
+      <c r="B468" t="s">
         <v>955</v>
-      </c>
-    </row>
-    <row r="467" spans="1:2">
-      <c r="A467" t="s">
-        <v>963</v>
-      </c>
-      <c r="B467" t="s">
-        <v>1162</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
-        <v>960</v>
+        <v>963</v>
       </c>
       <c r="B469" t="s">
-        <v>958</v>
-      </c>
-    </row>
-    <row r="470" spans="1:2">
-      <c r="A470" t="s">
-        <v>961</v>
-      </c>
-      <c r="B470" t="s">
-        <v>959</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="471" spans="1:2">
       <c r="A471" t="s">
-        <v>957</v>
+        <v>960</v>
       </c>
       <c r="B471" t="s">
-        <v>1163</v>
+        <v>958</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2">
+      <c r="A472" t="s">
+        <v>961</v>
+      </c>
+      <c r="B472" t="s">
+        <v>959</v>
       </c>
     </row>
     <row r="473" spans="1:2">
       <c r="A473" t="s">
-        <v>972</v>
+        <v>957</v>
       </c>
       <c r="B473" t="s">
-        <v>965</v>
-      </c>
-    </row>
-    <row r="474" spans="1:2">
-      <c r="A474" t="s">
-        <v>973</v>
-      </c>
-      <c r="B474" t="s">
-        <v>966</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="B475" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
     </row>
     <row r="476" spans="1:2">
       <c r="A476" t="s">
-        <v>1017</v>
+        <v>973</v>
       </c>
       <c r="B476" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B477" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>976</v>
+        <v>1017</v>
       </c>
       <c r="B478" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="B479" t="s">
-        <v>971</v>
+        <v>969</v>
+      </c>
+    </row>
+    <row r="480" spans="1:2">
+      <c r="A480" t="s">
+        <v>976</v>
+      </c>
+      <c r="B480" t="s">
+        <v>970</v>
       </c>
     </row>
     <row r="481" spans="1:2">
       <c r="A481" t="s">
-        <v>988</v>
+        <v>977</v>
       </c>
       <c r="B481" t="s">
-        <v>983</v>
-      </c>
-    </row>
-    <row r="482" spans="1:2">
-      <c r="A482" t="s">
-        <v>993</v>
-      </c>
-      <c r="B482" t="s">
-        <v>984</v>
+        <v>971</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B483" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>990</v>
+        <v>993</v>
       </c>
       <c r="B484" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>992</v>
+        <v>989</v>
       </c>
       <c r="B485" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B486" t="s">
-        <v>1164</v>
+        <v>986</v>
+      </c>
+    </row>
+    <row r="487" spans="1:2">
+      <c r="A487" t="s">
+        <v>992</v>
+      </c>
+      <c r="B487" t="s">
+        <v>987</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
-        <v>1005</v>
+        <v>991</v>
       </c>
       <c r="B488" t="s">
-        <v>994</v>
-      </c>
-    </row>
-    <row r="489" spans="1:2">
-      <c r="A489" t="s">
-        <v>1000</v>
-      </c>
-      <c r="B489" t="s">
-        <v>995</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="490" spans="1:2">
       <c r="A490" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="B490" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="B491" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="B492" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B493" t="s">
-        <v>1165</v>
+        <v>997</v>
+      </c>
+    </row>
+    <row r="494" spans="1:2">
+      <c r="A494" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B494" t="s">
+        <v>998</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="B495" t="s">
-        <v>1007</v>
-      </c>
-    </row>
-    <row r="496" spans="1:2">
-      <c r="A496" t="s">
-        <v>1012</v>
-      </c>
-      <c r="B496" t="s">
-        <v>1008</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="497" spans="1:2">
       <c r="A497" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="B497" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="B498" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="B499" t="s">
-        <v>1011</v>
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="500" spans="1:2">
+      <c r="A500" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B500" t="s">
+        <v>1010</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>1038</v>
+        <v>1015</v>
       </c>
       <c r="B501" t="s">
-        <v>1039</v>
-      </c>
-    </row>
-    <row r="502" spans="1:2">
-      <c r="A502" t="s">
-        <v>1054</v>
-      </c>
-      <c r="B502" t="s">
-        <v>1040</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="503" spans="1:2">
       <c r="A503" t="s">
-        <v>1055</v>
+        <v>1038</v>
       </c>
       <c r="B503" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="504" spans="1:2">
       <c r="A504" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="B504" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1065</v>
+        <v>1055</v>
       </c>
       <c r="B505" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B506" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1058</v>
+        <v>1065</v>
       </c>
       <c r="B507" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="B508" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="509" spans="1:2">
       <c r="A509" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="B509" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="510" spans="1:2">
       <c r="A510" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="B510" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="511" spans="1:2">
       <c r="A511" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="B511" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="512" spans="1:2">
       <c r="A512" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="B512" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="513" spans="1:2">
       <c r="A513" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="B513" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="514" spans="1:2">
       <c r="A514" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B514" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="515" spans="1:2">
+      <c r="A515" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B515" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="516" spans="1:2">
+      <c r="A516" t="s">
         <v>1053</v>
       </c>
-      <c r="B514" t="s">
+      <c r="B516" t="s">
         <v>1052</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A469:A470 A466:A467 A452:A461 A463:A464">
+  <conditionalFormatting sqref="A471:A472 A468:A469 A453:A463 A465:A466">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
changes for IAQ - TX, because we have more files and we cannot use the same as GA and AZ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847AEAD1-2222-4070-AB8A-7CE3CD6E7BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEFE6E87-4067-493E-9EF4-F2ABF243BAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22560" windowHeight="11655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3600,7 +3600,7 @@
     <t xml:space="preserve">Frequency of payments checkbox on the Regular Contributions Verification has not been documented. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes in IAQ TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B72DCC-C18B-4D26-9C93-2946408377FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B27860D-C2F5-422C-AE52-3D85D446A133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30240" windowHeight="14700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3600,9 +3600,6 @@
     <t xml:space="preserve">Frequency of payments checkbox on the Regular Contributions Verification has not been documented. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>PS_NameNotMatchingIAQ</t>
   </si>
   <si>
@@ -3622,6 +3619,9 @@
   </si>
   <si>
     <t>Child support income has been indicated, but not all Child Support documentation has been provided.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4090,7 +4090,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1186</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7092,10 +7092,10 @@
   <dimension ref="A1:Z1015"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="2" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="65.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -7440,10 +7440,10 @@
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="B40" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
@@ -10139,10 +10139,10 @@
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B196" t="s">
         <v>1187</v>
-      </c>
-      <c r="B196" t="s">
-        <v>1188</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -10960,10 +10960,10 @@
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B296" t="s">
         <v>1192</v>
-      </c>
-      <c r="B296" t="s">
-        <v>1193</v>
       </c>
     </row>
     <row r="298" spans="1:3">
@@ -12331,10 +12331,10 @@
     </row>
     <row r="477" spans="1:2">
       <c r="A477" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B477" t="s">
         <v>1190</v>
-      </c>
-      <c r="B477" t="s">
-        <v>1191</v>
       </c>
     </row>
     <row r="479" spans="1:2">

</xml_diff>

<commit_message>
changes in the IAQ TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C6FEE8-B47F-464E-AB4D-E703ADE32F28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F942496-0D06-4736-BB2F-47BDCE2DDF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30390" windowHeight="15015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3636,7 +3636,7 @@
     <t>Supplemental Security Income has been indicated, but not all Social Security Benefits Letters have been provided. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fix ASC and Profit loss
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F942496-0D06-4736-BB2F-47BDCE2DDF9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13D0BB6-E555-41E4-AA23-B0BCA04A3E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="30390" windowHeight="15015" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="1199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="1201">
   <si>
     <t>Name</t>
   </si>
@@ -3636,7 +3636,13 @@
     <t>Supplemental Security Income has been indicated, but not all Social Security Benefits Letters have been provided. </t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>WN_TotalMatchSum</t>
+  </si>
+  <si>
+    <t>Total Pay listed on the Work Number does not match the sum of each pay type on the Work Number.</t>
   </si>
 </sst>
 </file>
@@ -8522,7 +8528,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C523"/>
+  <dimension ref="A1:C524"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -10528,427 +10534,424 @@
         <v>1137</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
-      <c r="A244" t="s">
-        <v>466</v>
-      </c>
-      <c r="B244" t="s">
-        <v>1110</v>
+    <row r="243" spans="1:3">
+      <c r="A243" t="s">
+        <v>1199</v>
+      </c>
+      <c r="B243" t="s">
+        <v>1200</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="B245" t="s">
-        <v>294</v>
-      </c>
-      <c r="C245" t="s">
-        <v>527</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="B246" t="s">
-        <v>512</v>
+        <v>294</v>
+      </c>
+      <c r="C246" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>292</v>
+        <v>456</v>
       </c>
       <c r="B247" t="s">
-        <v>862</v>
-      </c>
-      <c r="C247" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B248" t="s">
-        <v>845</v>
+        <v>862</v>
+      </c>
+      <c r="C248" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>449</v>
+        <v>293</v>
       </c>
       <c r="B249" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>295</v>
+        <v>449</v>
       </c>
       <c r="B250" t="s">
-        <v>854</v>
-      </c>
-      <c r="C250" t="s">
-        <v>1088</v>
+        <v>846</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B251" t="s">
-        <v>863</v>
+        <v>854</v>
+      </c>
+      <c r="C251" t="s">
+        <v>1088</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B252" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B253" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B254" t="s">
-        <v>784</v>
+        <v>865</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>611</v>
+        <v>299</v>
       </c>
       <c r="B255" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
+        <v>611</v>
+      </c>
+      <c r="B256" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3">
+      <c r="A257" t="s">
         <v>478</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B257" t="s">
         <v>1138</v>
-      </c>
-    </row>
-    <row r="258" spans="1:3">
-      <c r="A258" t="s">
-        <v>644</v>
-      </c>
-      <c r="B258" t="s">
-        <v>645</v>
-      </c>
-      <c r="C258" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>495</v>
+        <v>644</v>
       </c>
       <c r="B259" t="s">
-        <v>498</v>
+        <v>645</v>
       </c>
       <c r="C259" t="s">
-        <v>525</v>
+        <v>598</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B260" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C260" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>524</v>
+        <v>496</v>
       </c>
       <c r="B261" t="s">
-        <v>538</v>
+        <v>497</v>
+      </c>
+      <c r="C261" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>316</v>
+        <v>524</v>
       </c>
       <c r="B262" t="s">
-        <v>302</v>
+        <v>538</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B263" t="s">
-        <v>303</v>
-      </c>
-      <c r="C263" t="s">
-        <v>527</v>
+        <v>302</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>457</v>
+        <v>317</v>
       </c>
       <c r="B264" t="s">
-        <v>513</v>
+        <v>303</v>
+      </c>
+      <c r="C264" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>318</v>
+        <v>457</v>
       </c>
       <c r="B265" t="s">
-        <v>304</v>
+        <v>513</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B266" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B267" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B268" t="s">
-        <v>307</v>
-      </c>
-      <c r="C268" t="s">
-        <v>527</v>
+        <v>306</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B269" t="s">
-        <v>308</v>
+        <v>307</v>
+      </c>
+      <c r="C269" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B270" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B271" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B272" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B273" t="s">
-        <v>312</v>
-      </c>
-      <c r="C273" t="s">
-        <v>527</v>
+        <v>311</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B274" t="s">
-        <v>313</v>
+        <v>312</v>
+      </c>
+      <c r="C274" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B275" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B276" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
+        <v>329</v>
+      </c>
+      <c r="B277" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3">
+      <c r="A278" t="s">
         <v>477</v>
       </c>
-      <c r="B277" t="s">
+      <c r="B278" t="s">
         <v>1139</v>
-      </c>
-    </row>
-    <row r="279" spans="1:3">
-      <c r="A279" t="s">
-        <v>542</v>
-      </c>
-      <c r="B279" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>336</v>
+        <v>542</v>
       </c>
       <c r="B280" t="s">
-        <v>354</v>
+        <v>543</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B281" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B282" t="s">
-        <v>352</v>
-      </c>
-      <c r="C282" t="s">
-        <v>527</v>
+        <v>351</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>458</v>
+        <v>338</v>
       </c>
       <c r="B283" t="s">
-        <v>514</v>
+        <v>352</v>
+      </c>
+      <c r="C283" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>355</v>
+        <v>458</v>
       </c>
       <c r="B284" t="s">
-        <v>353</v>
-      </c>
-      <c r="C284" t="s">
-        <v>527</v>
+        <v>514</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="B285" t="s">
-        <v>345</v>
+        <v>353</v>
+      </c>
+      <c r="C285" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>356</v>
+        <v>339</v>
       </c>
       <c r="B286" t="s">
-        <v>346</v>
-      </c>
-      <c r="C286" t="s">
-        <v>504</v>
+        <v>345</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="B287" t="s">
-        <v>347</v>
+        <v>346</v>
+      </c>
+      <c r="C287" t="s">
+        <v>504</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B288" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B289" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B290" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B291" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>1015</v>
+        <v>344</v>
       </c>
       <c r="B292" t="s">
-        <v>1016</v>
-      </c>
-      <c r="C292" t="s">
-        <v>1011</v>
+        <v>347</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="B293" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="C293" t="s">
         <v>1011</v>
@@ -10956,10 +10959,10 @@
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="B294" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="C294" t="s">
         <v>1011</v>
@@ -10967,48 +10970,48 @@
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>476</v>
+        <v>1019</v>
       </c>
       <c r="B295" t="s">
-        <v>1140</v>
+        <v>1020</v>
+      </c>
+      <c r="C295" t="s">
+        <v>1011</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
+        <v>476</v>
+      </c>
+      <c r="B296" t="s">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3">
+      <c r="A297" t="s">
         <v>1191</v>
       </c>
-      <c r="B296" t="s">
+      <c r="B297" t="s">
         <v>1192</v>
-      </c>
-    </row>
-    <row r="298" spans="1:3">
-      <c r="A298" t="s">
-        <v>646</v>
-      </c>
-      <c r="B298" t="s">
-        <v>664</v>
-      </c>
-      <c r="C298" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>1009</v>
+        <v>646</v>
       </c>
       <c r="B299" t="s">
-        <v>1010</v>
+        <v>664</v>
       </c>
       <c r="C299" t="s">
-        <v>1011</v>
+        <v>598</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>1012</v>
+        <v>1009</v>
       </c>
       <c r="B300" t="s">
-        <v>1013</v>
+        <v>1010</v>
       </c>
       <c r="C300" t="s">
         <v>1011</v>
@@ -11016,78 +11019,78 @@
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="B301" t="s">
-        <v>1141</v>
+        <v>1013</v>
       </c>
       <c r="C301" t="s">
         <v>1011</v>
       </c>
     </row>
-    <row r="303" spans="1:3">
-      <c r="A303" t="s">
-        <v>642</v>
-      </c>
-      <c r="B303" t="s">
-        <v>643</v>
-      </c>
-      <c r="C303" t="s">
-        <v>598</v>
+    <row r="302" spans="1:3">
+      <c r="A302" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B302" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1011</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>467</v>
+        <v>642</v>
       </c>
       <c r="B304" t="s">
-        <v>468</v>
+        <v>643</v>
+      </c>
+      <c r="C304" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>362</v>
+        <v>467</v>
       </c>
       <c r="B305" t="s">
-        <v>373</v>
+        <v>468</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B306" t="s">
-        <v>374</v>
-      </c>
-      <c r="C306" t="s">
-        <v>527</v>
+        <v>373</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>515</v>
+        <v>363</v>
       </c>
       <c r="B307" t="s">
-        <v>516</v>
+        <v>374</v>
+      </c>
+      <c r="C307" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>364</v>
+        <v>515</v>
       </c>
       <c r="B308" t="s">
-        <v>375</v>
-      </c>
-      <c r="C308" t="s">
-        <v>527</v>
+        <v>516</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B309" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C309" t="s">
         <v>527</v>
@@ -11095,155 +11098,155 @@
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B310" t="s">
-        <v>528</v>
+        <v>376</v>
+      </c>
+      <c r="C310" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B311" t="s">
-        <v>377</v>
+        <v>528</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B312" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B313" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B314" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B315" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B316" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>699</v>
+        <v>372</v>
       </c>
       <c r="B317" t="s">
-        <v>1085</v>
-      </c>
-      <c r="C317" t="s">
-        <v>598</v>
+        <v>382</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>1102</v>
+        <v>699</v>
       </c>
       <c r="B318" t="s">
-        <v>1103</v>
+        <v>1085</v>
+      </c>
+      <c r="C318" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>474</v>
+        <v>1102</v>
       </c>
       <c r="B319" t="s">
-        <v>1142</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>551</v>
+        <v>474</v>
       </c>
       <c r="B320" t="s">
-        <v>552</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
+        <v>551</v>
+      </c>
+      <c r="B321" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3">
+      <c r="A322" t="s">
         <v>1194</v>
       </c>
-      <c r="B321" t="s">
+      <c r="B322" t="s">
         <v>1195</v>
-      </c>
-    </row>
-    <row r="323" spans="1:3">
-      <c r="A323" t="s">
-        <v>469</v>
-      </c>
-      <c r="B323" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>389</v>
+        <v>469</v>
       </c>
       <c r="B324" t="s">
-        <v>400</v>
+        <v>468</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B325" t="s">
-        <v>401</v>
-      </c>
-      <c r="C325" t="s">
-        <v>527</v>
+        <v>400</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>459</v>
+        <v>390</v>
       </c>
       <c r="B326" t="s">
-        <v>517</v>
+        <v>401</v>
+      </c>
+      <c r="C326" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>391</v>
+        <v>459</v>
       </c>
       <c r="B327" t="s">
-        <v>402</v>
-      </c>
-      <c r="C327" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B328" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C328" t="s">
         <v>527</v>
@@ -11251,1437 +11254,1448 @@
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B329" t="s">
-        <v>529</v>
+        <v>403</v>
+      </c>
+      <c r="C329" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B330" t="s">
-        <v>377</v>
+        <v>529</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B331" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B332" t="s">
-        <v>404</v>
+        <v>378</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B333" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B334" t="s">
-        <v>381</v>
+        <v>405</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B335" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>473</v>
+        <v>399</v>
       </c>
       <c r="B336" t="s">
-        <v>1142</v>
+        <v>382</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
-        <v>558</v>
+        <v>473</v>
       </c>
       <c r="B337" t="s">
-        <v>552</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="338" spans="1:3">
       <c r="A338" t="s">
+        <v>558</v>
+      </c>
+      <c r="B338" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3">
+      <c r="A339" t="s">
         <v>1196</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B339" t="s">
         <v>1197</v>
-      </c>
-    </row>
-    <row r="340" spans="1:3">
-      <c r="A340" t="s">
-        <v>640</v>
-      </c>
-      <c r="B340" t="s">
-        <v>641</v>
-      </c>
-      <c r="C340" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
-        <v>383</v>
+        <v>640</v>
       </c>
       <c r="B341" t="s">
-        <v>559</v>
+        <v>641</v>
+      </c>
+      <c r="C341" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B342" t="s">
-        <v>560</v>
-      </c>
-      <c r="C342" t="s">
-        <v>527</v>
+        <v>559</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>460</v>
+        <v>384</v>
       </c>
       <c r="B343" t="s">
-        <v>561</v>
+        <v>560</v>
+      </c>
+      <c r="C343" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>385</v>
+        <v>460</v>
       </c>
       <c r="B344" t="s">
-        <v>586</v>
+        <v>561</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B345" t="s">
-        <v>562</v>
+        <v>586</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B346" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>1119</v>
+        <v>387</v>
       </c>
       <c r="B347" t="s">
-        <v>1120</v>
-      </c>
-      <c r="C347" t="s">
-        <v>1121</v>
+        <v>563</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B348" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C348" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3">
+      <c r="A349" t="s">
         <v>472</v>
       </c>
-      <c r="B348" t="s">
+      <c r="B349" t="s">
         <v>1143</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3">
-      <c r="A350" t="s">
-        <v>712</v>
-      </c>
-      <c r="B350" t="s">
-        <v>713</v>
-      </c>
-      <c r="C350" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="B351" t="s">
-        <v>1144</v>
+        <v>713</v>
       </c>
       <c r="C351" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="353" spans="1:2">
-      <c r="A353" t="s">
-        <v>719</v>
-      </c>
-      <c r="B353" t="s">
-        <v>720</v>
+    <row r="352" spans="1:3">
+      <c r="A352" t="s">
+        <v>714</v>
+      </c>
+      <c r="B352" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C352" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="B354" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="B355" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="B356" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="B357" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="B358" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="B359" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="B360" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="B361" t="s">
-        <v>1181</v>
+        <v>734</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B362" t="s">
-        <v>737</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="B363" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B364" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="B365" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="B366" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B367" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B368" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>1095</v>
+        <v>748</v>
       </c>
       <c r="B369" t="s">
-        <v>1096</v>
+        <v>749</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>750</v>
+        <v>1095</v>
       </c>
       <c r="B370" t="s">
-        <v>751</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>1118</v>
+        <v>750</v>
       </c>
       <c r="B371" t="s">
-        <v>1145</v>
+        <v>751</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B372" t="s">
+        <v>1145</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" t="s">
         <v>1169</v>
       </c>
-      <c r="B372" t="s">
+      <c r="B373" t="s">
         <v>1170</v>
-      </c>
-    </row>
-    <row r="374" spans="1:2">
-      <c r="A374" t="s">
-        <v>752</v>
-      </c>
-      <c r="B374" t="s">
-        <v>753</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="B375" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="B376" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="B377" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="B378" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="B379" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="B380" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B381" t="s">
-        <v>315</v>
+        <v>765</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B382" t="s">
-        <v>768</v>
+        <v>315</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B383" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B384" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
+        <v>771</v>
+      </c>
+      <c r="B385" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2">
+      <c r="A386" t="s">
         <v>773</v>
       </c>
-      <c r="B385" t="s">
+      <c r="B386" t="s">
         <v>1146</v>
-      </c>
-    </row>
-    <row r="387" spans="1:2">
-      <c r="A387" t="s">
-        <v>774</v>
-      </c>
-      <c r="B387" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B388" t="s">
-        <v>776</v>
+        <v>308</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="B389" t="s">
-        <v>310</v>
+        <v>776</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
+        <v>777</v>
+      </c>
+      <c r="B390" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" t="s">
         <v>778</v>
       </c>
-      <c r="B390" t="s">
+      <c r="B391" t="s">
         <v>1182</v>
-      </c>
-    </row>
-    <row r="392" spans="1:2">
-      <c r="A392" t="s">
-        <v>800</v>
-      </c>
-      <c r="B392" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="B393" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="B394" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="B395" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B396" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
+        <v>792</v>
+      </c>
+      <c r="B397" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2">
+      <c r="A398" t="s">
         <v>797</v>
       </c>
-      <c r="B397" t="s">
+      <c r="B398" t="s">
         <v>1179</v>
-      </c>
-    </row>
-    <row r="399" spans="1:2">
-      <c r="A399" t="s">
-        <v>804</v>
-      </c>
-      <c r="B399" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="B400" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="B401" t="s">
-        <v>794</v>
+        <v>810</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B402" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B403" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
+        <v>807</v>
+      </c>
+      <c r="B404" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2">
+      <c r="A405" t="s">
         <v>808</v>
       </c>
-      <c r="B404" t="s">
+      <c r="B405" t="s">
         <v>1147</v>
-      </c>
-    </row>
-    <row r="406" spans="1:2">
-      <c r="A406" t="s">
-        <v>816</v>
-      </c>
-      <c r="B406" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="B407" t="s">
-        <v>1111</v>
+        <v>817</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="B408" t="s">
-        <v>1078</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="B409" t="s">
-        <v>1071</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>827</v>
+        <v>821</v>
       </c>
       <c r="B410" t="s">
-        <v>1057</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="B411" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B412" t="s">
-        <v>1077</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B413" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B414" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B415" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B416" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B417" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B418" t="s">
-        <v>826</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B419" t="s">
-        <v>1079</v>
+        <v>826</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B420" t="s">
-        <v>275</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B421" t="s">
-        <v>785</v>
+        <v>275</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>831</v>
+        <v>840</v>
       </c>
       <c r="B422" t="s">
-        <v>604</v>
+        <v>785</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="B423" t="s">
-        <v>1148</v>
+        <v>604</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>1193</v>
+        <v>830</v>
       </c>
       <c r="B424" t="s">
-        <v>1187</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>1061</v>
+        <v>1193</v>
       </c>
       <c r="B425" t="s">
-        <v>1059</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B426" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
       <c r="B427" t="s">
-        <v>1063</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="B428" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B429" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B430" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>1081</v>
+        <v>1070</v>
       </c>
       <c r="B431" t="s">
-        <v>1080</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B432" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B433" t="s">
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2">
+      <c r="A434" t="s">
         <v>1159</v>
       </c>
-      <c r="B433" t="s">
+      <c r="B434" t="s">
         <v>1160</v>
-      </c>
-    </row>
-    <row r="435" spans="1:2">
-      <c r="A435" t="s">
-        <v>900</v>
-      </c>
-      <c r="B435" t="s">
-        <v>880</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>919</v>
+        <v>900</v>
       </c>
       <c r="B436" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>918</v>
+        <v>919</v>
       </c>
       <c r="B437" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>917</v>
+        <v>918</v>
       </c>
       <c r="B438" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>916</v>
+        <v>917</v>
       </c>
       <c r="B439" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="B440" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B441" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="B442" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="B443" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="B444" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B445" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>920</v>
+        <v>910</v>
       </c>
       <c r="B446" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>909</v>
+        <v>920</v>
       </c>
       <c r="B447" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="B448" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="B449" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="B450" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="B451" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="B452" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B453" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="B454" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B455" t="s">
-        <v>1149</v>
+        <v>899</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
+        <v>901</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1149</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
         <v>1163</v>
       </c>
-      <c r="B456" t="s">
+      <c r="B457" t="s">
         <v>1164</v>
-      </c>
-    </row>
-    <row r="458" spans="1:2">
-      <c r="A458" t="s">
-        <v>1122</v>
-      </c>
-      <c r="B458" t="s">
-        <v>1123</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>938</v>
+        <v>1122</v>
       </c>
       <c r="B459" t="s">
-        <v>923</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
-        <v>929</v>
+        <v>938</v>
       </c>
       <c r="B460" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="B461" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B462" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="B463" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="B464" t="s">
-        <v>1183</v>
+        <v>927</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="B465" t="s">
-        <v>928</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="B466" t="s">
-        <v>1184</v>
+        <v>928</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="B467" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="B468" t="s">
-        <v>1150</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
+        <v>936</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" t="s">
         <v>1171</v>
       </c>
-      <c r="B469" t="s">
+      <c r="B470" t="s">
         <v>1172</v>
-      </c>
-    </row>
-    <row r="471" spans="1:2">
-      <c r="A471" t="s">
-        <v>943</v>
-      </c>
-      <c r="B471" t="s">
-        <v>945</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
+        <v>943</v>
+      </c>
+      <c r="B472" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" t="s">
         <v>953</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B473" t="s">
         <v>1151</v>
-      </c>
-    </row>
-    <row r="474" spans="1:2">
-      <c r="A474" t="s">
-        <v>944</v>
-      </c>
-      <c r="B474" t="s">
-        <v>946</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
+        <v>944</v>
+      </c>
+      <c r="B475" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" t="s">
         <v>954</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B476" t="s">
         <v>1152</v>
-      </c>
-    </row>
-    <row r="477" spans="1:2">
-      <c r="A477" t="s">
-        <v>951</v>
-      </c>
-      <c r="B477" t="s">
-        <v>949</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B478" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="B479" t="s">
-        <v>1153</v>
+        <v>950</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
+        <v>948</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2">
+      <c r="A481" t="s">
         <v>1189</v>
       </c>
-      <c r="B480" t="s">
+      <c r="B481" t="s">
         <v>1190</v>
-      </c>
-    </row>
-    <row r="482" spans="1:2">
-      <c r="A482" t="s">
-        <v>963</v>
-      </c>
-      <c r="B482" t="s">
-        <v>956</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B483" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B484" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>1008</v>
+        <v>965</v>
       </c>
       <c r="B485" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>966</v>
+        <v>1008</v>
       </c>
       <c r="B486" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B487" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
+        <v>967</v>
+      </c>
+      <c r="B488" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" t="s">
         <v>968</v>
       </c>
-      <c r="B488" t="s">
+      <c r="B489" t="s">
         <v>962</v>
-      </c>
-    </row>
-    <row r="490" spans="1:2">
-      <c r="A490" t="s">
-        <v>979</v>
-      </c>
-      <c r="B490" t="s">
-        <v>974</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>984</v>
+        <v>979</v>
       </c>
       <c r="B491" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
       <c r="B492" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B493" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="B494" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
+        <v>983</v>
+      </c>
+      <c r="B495" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="496" spans="1:2">
+      <c r="A496" t="s">
         <v>982</v>
       </c>
-      <c r="B495" t="s">
+      <c r="B496" t="s">
         <v>1154</v>
-      </c>
-    </row>
-    <row r="497" spans="1:2">
-      <c r="A497" t="s">
-        <v>996</v>
-      </c>
-      <c r="B497" t="s">
-        <v>985</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="B498" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B499" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B500" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B501" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
+        <v>994</v>
+      </c>
+      <c r="B502" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="503" spans="1:2">
+      <c r="A503" t="s">
         <v>995</v>
       </c>
-      <c r="B502" t="s">
+      <c r="B503" t="s">
         <v>1155</v>
-      </c>
-    </row>
-    <row r="504" spans="1:2">
-      <c r="A504" t="s">
-        <v>997</v>
-      </c>
-      <c r="B504" t="s">
-        <v>998</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>1003</v>
+        <v>997</v>
       </c>
       <c r="B505" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B506" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B507" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B508" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="509" spans="1:2">
+      <c r="A509" t="s">
         <v>1006</v>
       </c>
-      <c r="B508" t="s">
+      <c r="B509" t="s">
         <v>1002</v>
-      </c>
-    </row>
-    <row r="510" spans="1:2">
-      <c r="A510" t="s">
-        <v>1029</v>
-      </c>
-      <c r="B510" t="s">
-        <v>1030</v>
       </c>
     </row>
     <row r="511" spans="1:2">
       <c r="A511" t="s">
-        <v>1045</v>
+        <v>1029</v>
       </c>
       <c r="B511" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="512" spans="1:2">
       <c r="A512" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B512" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="513" spans="1:2">
       <c r="A513" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B513" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="514" spans="1:2">
       <c r="A514" t="s">
-        <v>1056</v>
+        <v>1047</v>
       </c>
       <c r="B514" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="515" spans="1:2">
       <c r="A515" t="s">
-        <v>1048</v>
+        <v>1056</v>
       </c>
       <c r="B515" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="516" spans="1:2">
       <c r="A516" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B516" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="517" spans="1:2">
       <c r="A517" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B517" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="518" spans="1:2">
       <c r="A518" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B518" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="519" spans="1:2">
       <c r="A519" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B519" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="520" spans="1:2">
       <c r="A520" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B520" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="521" spans="1:2">
       <c r="A521" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B521" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="522" spans="1:2">
       <c r="A522" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B522" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="523" spans="1:2">
       <c r="A523" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B523" t="s">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="524" spans="1:2">
+      <c r="A524" t="s">
         <v>1044</v>
       </c>
-      <c r="B523" t="s">
+      <c r="B524" t="s">
         <v>1043</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A477:A478 A474:A475 A459:A469 A471:A472 A480">
+  <conditionalFormatting sqref="A478:A479 A475:A476 A460:A470 A472:A473 A481">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated IAQ for TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13D0BB6-E555-41E4-AA23-B0BCA04A3E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A97E5D3-7C70-492E-AA9F-F1A8444D0FD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3636,13 +3636,13 @@
     <t>Supplemental Security Income has been indicated, but not all Social Security Benefits Letters have been provided. </t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>WN_TotalMatchSum</t>
   </si>
   <si>
     <t>Total Pay listed on the Work Number does not match the sum of each pay type on the Work Number.</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4111,7 +4111,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1198</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -10536,10 +10536,10 @@
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B243" t="s">
         <v>1199</v>
-      </c>
-      <c r="B243" t="s">
-        <v>1200</v>
       </c>
     </row>
     <row r="245" spans="1:3">

</xml_diff>

<commit_message>
changes for log errors for TX
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library_new\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB95B77F-7EEE-4734-B7E2-AE96FC2240EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74066DB-2D3F-474F-A269-8D1FCAC73B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3639,10 +3639,10 @@
     <t>Total Pay listed on the Work Number does not match the sum of each pay type on the Work Number.</t>
   </si>
   <si>
-    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>DocumentTypeUserPrompt_AZ.txt</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4111,7 +4111,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4135,7 +4135,7 @@
         <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Prompt file name updated as AZ for ASC and SEC
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bagi.Elangovan\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471313D9-FD37-4548-BE91-E0B50DF06EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB0FB1A-DE10-42E3-B488-C70298985767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3639,10 +3639,10 @@
     <t>Total Pay listed on the Work Number does not match the sum of each pay type on the Work Number.</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
-    <t>DocumentTypeUserPrompt_GA.txt</t>
+    <t>DocumentTypeUserPrompt_AZ.txt</t>
+  </si>
+  <si>
+    <t>C:\Users\Bagi.Elangovan\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4032,9 +4032,9 @@
   <dimension ref="A1:Z1005"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="64.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="26" width="8.7109375" customWidth="1"/>
   </cols>
@@ -4111,7 +4111,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4135,7 +4135,7 @@
         <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
changes to iaq for real estate check, changes in VSA for assets that don't contain institution name
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{471313D9-FD37-4548-BE91-E0B50DF06EAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D52946-852A-4EAE-8D79-F8E5F0E98E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3639,10 +3639,10 @@
     <t>Total Pay listed on the Work Number does not match the sum of each pay type on the Work Number.</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>DocumentTypeUserPrompt_GA.txt</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4111,7 +4111,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4135,7 +4135,7 @@
         <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
add IAQ check to AZ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38D52946-852A-4EAE-8D79-F8E5F0E98E91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02831545-90A5-4DF1-B517-4C3084B79DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3642,7 +3642,7 @@
     <t>DocumentTypeUserPrompt_GA.txt</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
changes in MID - TX for fuzzy matching names and in Config file to capture newly added assets
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02831545-90A5-4DF1-B517-4C3084B79DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FA7B2D-28BB-429E-A5FF-85B5B670084A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="1201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="1204">
   <si>
     <t>Name</t>
   </si>
@@ -3643,6 +3643,15 @@
   </si>
   <si>
     <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>BackToSiteStates</t>
+  </si>
+  <si>
+    <t>NotBackToSiteStates</t>
+  </si>
+  <si>
+    <t>YardiReviewer</t>
   </si>
 </sst>
 </file>
@@ -7555,9 +7564,30 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1201</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A53" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1202</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A54" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1203</v>
+      </c>
+    </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="57" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
updates to MID fuzzy logic
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Audit-Findings-Library\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FA7B2D-28BB-429E-A5FF-85B5B670084A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0DFDFE-1934-46EA-B1AD-02EC327F59AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3642,9 +3642,6 @@
     <t>DocumentTypeUserPrompt_GA.txt</t>
   </si>
   <si>
-    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>BackToSiteStates</t>
   </si>
   <si>
@@ -3652,6 +3649,9 @@
   </si>
   <si>
     <t>YardiReviewer</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -4120,7 +4120,7 @@
         <v>200</v>
       </c>
       <c r="B7" t="s">
-        <v>1200</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -7566,26 +7566,26 @@
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="B52" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="B53" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="B54" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>